<commit_message>
added a few more servants for testing
</commit_message>
<xml_diff>
--- a/data/Fate-Spreadsheet.xlsx
+++ b/data/Fate-Spreadsheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pixel\Documents\Projects\Fate-Wiki\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{807CE838-7557-4D17-845B-C213D3F85AAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48FB44AB-56B6-46D4-A0D5-481883B29607}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="1" xr2:uid="{B05E798F-9EF6-4508-A0A4-311D06661AED}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{B05E798F-9EF6-4508-A0A4-311D06661AED}"/>
   </bookViews>
   <sheets>
     <sheet name="Servants" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="114">
   <si>
     <t>servant_id</t>
   </si>
@@ -271,6 +271,120 @@
   </si>
   <si>
     <t>quantity</t>
+  </si>
+  <si>
+    <t>S0147</t>
+  </si>
+  <si>
+    <t>Passionlip</t>
+  </si>
+  <si>
+    <t>passionlip</t>
+  </si>
+  <si>
+    <t>Alter Ego</t>
+  </si>
+  <si>
+    <t>2,4,5,5</t>
+  </si>
+  <si>
+    <t>Berserker Strength 7,Berserker Strength 9,Luck,Luck,Surveil</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>Alter Ego Class</t>
+  </si>
+  <si>
+    <t>Durga's Nails</t>
+  </si>
+  <si>
+    <t>Masochistic Nature</t>
+  </si>
+  <si>
+    <t>S0069</t>
+  </si>
+  <si>
+    <t>Euryale</t>
+  </si>
+  <si>
+    <t>euryale</t>
+  </si>
+  <si>
+    <t>Archer</t>
+  </si>
+  <si>
+    <t>Skirmisher</t>
+  </si>
+  <si>
+    <t>2,2,2,3,5</t>
+  </si>
+  <si>
+    <t>Divine Core</t>
+  </si>
+  <si>
+    <t>Divine-Core</t>
+  </si>
+  <si>
+    <t>S0070</t>
+  </si>
+  <si>
+    <t>S0071</t>
+  </si>
+  <si>
+    <t>Archer Class</t>
+  </si>
+  <si>
+    <t>Eye of the Euryale</t>
+  </si>
+  <si>
+    <t>Siren's Song</t>
+  </si>
+  <si>
+    <t>S0108</t>
+  </si>
+  <si>
+    <t>Artoria Avalon</t>
+  </si>
+  <si>
+    <t>artoria-avalon</t>
+  </si>
+  <si>
+    <t>Thrasher</t>
+  </si>
+  <si>
+    <t>2,2,3</t>
+  </si>
+  <si>
+    <t>2,3,3,4,4,5</t>
+  </si>
+  <si>
+    <t>Pilgrim's Call</t>
+  </si>
+  <si>
+    <t>Pilgrim's Respite</t>
+  </si>
+  <si>
+    <t>Pilgrim's Destiny</t>
+  </si>
+  <si>
+    <t>Pilgrims-Call</t>
+  </si>
+  <si>
+    <t>Pilgrims-Respite</t>
+  </si>
+  <si>
+    <t>Pilgrims-Destiny</t>
+  </si>
+  <si>
+    <t>Round of Avalon</t>
+  </si>
+  <si>
+    <t>Around Caliburn</t>
+  </si>
+  <si>
+    <t>Staff of Selection</t>
   </si>
 </sst>
 </file>
@@ -320,11 +434,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -659,7 +774,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E33D7ECC-1EAA-4A40-B4DA-A93E54CBC8B5}">
-  <dimension ref="A1:K6"/>
+  <dimension ref="A1:K9"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="17.1328125" customWidth="1"/>
@@ -670,7 +785,7 @@
     <col min="7" max="7" width="13.73046875" style="2" customWidth="1"/>
     <col min="8" max="8" width="11.73046875" style="2" customWidth="1"/>
     <col min="9" max="9" width="11.796875" style="2" customWidth="1"/>
-    <col min="10" max="10" width="43.06640625" style="2" customWidth="1"/>
+    <col min="10" max="10" width="48.796875" style="2" customWidth="1"/>
     <col min="11" max="11" width="12.59765625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -743,25 +858,28 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>17</v>
+        <v>86</v>
       </c>
       <c r="B3" t="s">
-        <v>18</v>
+        <v>87</v>
       </c>
       <c r="C3" t="s">
-        <v>19</v>
+        <v>88</v>
       </c>
       <c r="D3" t="s">
-        <v>20</v>
+        <v>89</v>
       </c>
       <c r="E3" t="s">
-        <v>8</v>
+        <v>90</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>91</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="J3" s="2" t="s">
-        <v>22</v>
+        <v>42</v>
       </c>
       <c r="K3" t="b">
         <v>1</v>
@@ -769,103 +887,190 @@
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B4" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="C4" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="D4" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="E4" t="s">
         <v>8</v>
       </c>
-      <c r="G4" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>28</v>
+      <c r="I4" s="2" t="s">
+        <v>21</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>70</v>
+        <v>22</v>
       </c>
       <c r="K4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>29</v>
+        <v>99</v>
       </c>
       <c r="B5" t="s">
-        <v>30</v>
+        <v>100</v>
       </c>
       <c r="C5" t="s">
-        <v>31</v>
+        <v>101</v>
       </c>
       <c r="D5" t="s">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="E5" t="s">
-        <v>33</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="H5" s="2">
-        <v>3</v>
+        <v>102</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>103</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="J5" s="2" t="s">
-        <v>35</v>
+        <v>104</v>
       </c>
       <c r="K5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>36</v>
+        <v>76</v>
       </c>
       <c r="B6" t="s">
-        <v>37</v>
+        <v>77</v>
       </c>
       <c r="C6" t="s">
-        <v>38</v>
+        <v>78</v>
       </c>
       <c r="D6" t="s">
-        <v>39</v>
+        <v>79</v>
       </c>
       <c r="E6" t="s">
         <v>40</v>
       </c>
       <c r="G6" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="K6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" t="s">
+        <v>24</v>
+      </c>
+      <c r="C7" t="s">
+        <v>25</v>
+      </c>
+      <c r="D7" t="s">
+        <v>26</v>
+      </c>
+      <c r="E7" t="s">
+        <v>8</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="K7" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A8" t="s">
+        <v>29</v>
+      </c>
+      <c r="B8" t="s">
+        <v>30</v>
+      </c>
+      <c r="C8" t="s">
+        <v>31</v>
+      </c>
+      <c r="D8" t="s">
+        <v>32</v>
+      </c>
+      <c r="E8" t="s">
+        <v>33</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H8" s="2">
+        <v>3</v>
+      </c>
+      <c r="I8" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="K8" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A9" t="s">
+        <v>36</v>
+      </c>
+      <c r="B9" t="s">
+        <v>37</v>
+      </c>
+      <c r="C9" t="s">
+        <v>38</v>
+      </c>
+      <c r="D9" t="s">
+        <v>39</v>
+      </c>
+      <c r="E9" t="s">
+        <v>40</v>
+      </c>
+      <c r="G9" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="H6" s="2" t="s">
+      <c r="H9" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="J6" s="2" t="s">
+      <c r="J9" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="K6" t="b">
+      <c r="K9" t="b">
         <v>1</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError sqref="I6" numberStoredAsText="1"/>
+  </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1BC60D8-44F3-478D-BCC0-4752624457AE}">
-  <dimension ref="A1:F4"/>
+  <dimension ref="A1:F8"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="19" customWidth="1"/>
@@ -894,20 +1099,20 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A2" t="s">
-        <v>17</v>
-      </c>
-      <c r="B2" t="s">
-        <v>18</v>
-      </c>
-      <c r="C2" t="s">
-        <v>47</v>
-      </c>
-      <c r="D2" t="s">
-        <v>72</v>
-      </c>
-      <c r="E2">
+    <row r="2" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="A2" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="E2" s="4">
         <v>2</v>
       </c>
     </row>
@@ -919,40 +1124,110 @@
         <v>18</v>
       </c>
       <c r="C3" t="s">
-        <v>73</v>
+        <v>47</v>
       </c>
       <c r="D3" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="E3">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C4" t="s">
+        <v>73</v>
+      </c>
+      <c r="D4" t="s">
+        <v>74</v>
+      </c>
+      <c r="E4">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
+        <v>99</v>
+      </c>
+      <c r="B5" t="s">
+        <v>100</v>
+      </c>
+      <c r="C5" t="s">
+        <v>105</v>
+      </c>
+      <c r="D5" t="s">
+        <v>108</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
+        <v>99</v>
+      </c>
+      <c r="B6" t="s">
+        <v>100</v>
+      </c>
+      <c r="C6" t="s">
+        <v>106</v>
+      </c>
+      <c r="D6" t="s">
+        <v>109</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A7" t="s">
+        <v>99</v>
+      </c>
+      <c r="B7" t="s">
+        <v>100</v>
+      </c>
+      <c r="C7" t="s">
+        <v>107</v>
+      </c>
+      <c r="D7" t="s">
+        <v>110</v>
+      </c>
+      <c r="E7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A8" t="s">
         <v>36</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B8" t="s">
         <v>37</v>
       </c>
-      <c r="C4" t="s">
+      <c r="C8" t="s">
         <v>48</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D8" t="s">
         <v>48</v>
       </c>
-      <c r="E4">
+      <c r="E8">
         <v>2</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="0" orientation="portrait" horizontalDpi="0" verticalDpi="0" copies="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84E3BB0D-5578-4069-B1C9-C3864EB2A429}">
-  <dimension ref="A1:F16"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="20.59765625" customWidth="1"/>
@@ -1035,10 +1310,10 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>17</v>
+        <v>86</v>
       </c>
       <c r="B5" t="s">
-        <v>18</v>
+        <v>87</v>
       </c>
       <c r="C5">
         <v>1</v>
@@ -1047,15 +1322,15 @@
         <v>1</v>
       </c>
       <c r="E5" t="s">
-        <v>58</v>
+        <v>96</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>17</v>
+        <v>94</v>
       </c>
       <c r="B6" t="s">
-        <v>18</v>
+        <v>87</v>
       </c>
       <c r="C6">
         <v>2</v>
@@ -1064,15 +1339,15 @@
         <v>0</v>
       </c>
       <c r="E6" t="s">
-        <v>59</v>
+        <v>97</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>17</v>
+        <v>95</v>
       </c>
       <c r="B7" t="s">
-        <v>18</v>
+        <v>87</v>
       </c>
       <c r="C7">
         <v>3</v>
@@ -1081,32 +1356,32 @@
         <v>0</v>
       </c>
       <c r="E7" t="s">
-        <v>60</v>
+        <v>98</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B8" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="C8">
         <v>1</v>
       </c>
       <c r="D8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E8" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B9" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="C9">
         <v>2</v>
@@ -1115,15 +1390,15 @@
         <v>0</v>
       </c>
       <c r="E9" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="B10" t="s">
-        <v>24</v>
+        <v>18</v>
       </c>
       <c r="C10">
         <v>3</v>
@@ -1132,15 +1407,15 @@
         <v>0</v>
       </c>
       <c r="E10" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
-        <v>29</v>
+        <v>99</v>
       </c>
       <c r="B11" t="s">
-        <v>30</v>
+        <v>100</v>
       </c>
       <c r="C11">
         <v>1</v>
@@ -1149,15 +1424,15 @@
         <v>0</v>
       </c>
       <c r="E11" t="s">
-        <v>64</v>
+        <v>111</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
-        <v>29</v>
+        <v>99</v>
       </c>
       <c r="B12" t="s">
-        <v>30</v>
+        <v>100</v>
       </c>
       <c r="C12">
         <v>2</v>
@@ -1166,15 +1441,15 @@
         <v>0</v>
       </c>
       <c r="E12" t="s">
-        <v>65</v>
+        <v>112</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
-        <v>29</v>
+        <v>99</v>
       </c>
       <c r="B13" t="s">
-        <v>30</v>
+        <v>100</v>
       </c>
       <c r="C13">
         <v>3</v>
@@ -1183,32 +1458,32 @@
         <v>0</v>
       </c>
       <c r="E13" t="s">
-        <v>66</v>
+        <v>113</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
-        <v>36</v>
+        <v>76</v>
       </c>
       <c r="B14" t="s">
-        <v>37</v>
+        <v>77</v>
       </c>
       <c r="C14">
         <v>1</v>
       </c>
       <c r="D14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E14" t="s">
-        <v>67</v>
+        <v>83</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
-        <v>36</v>
+        <v>76</v>
       </c>
       <c r="B15" t="s">
-        <v>37</v>
+        <v>77</v>
       </c>
       <c r="C15">
         <v>2</v>
@@ -1217,15 +1492,15 @@
         <v>0</v>
       </c>
       <c r="E15" t="s">
-        <v>68</v>
+        <v>84</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
-        <v>36</v>
+        <v>76</v>
       </c>
       <c r="B16" t="s">
-        <v>37</v>
+        <v>77</v>
       </c>
       <c r="C16">
         <v>3</v>
@@ -1234,6 +1509,159 @@
         <v>0</v>
       </c>
       <c r="E16" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A17" t="s">
+        <v>23</v>
+      </c>
+      <c r="B17" t="s">
+        <v>24</v>
+      </c>
+      <c r="C17">
+        <v>1</v>
+      </c>
+      <c r="D17" t="b">
+        <v>0</v>
+      </c>
+      <c r="E17" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A18" t="s">
+        <v>23</v>
+      </c>
+      <c r="B18" t="s">
+        <v>24</v>
+      </c>
+      <c r="C18">
+        <v>2</v>
+      </c>
+      <c r="D18" t="b">
+        <v>0</v>
+      </c>
+      <c r="E18" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A19" t="s">
+        <v>23</v>
+      </c>
+      <c r="B19" t="s">
+        <v>24</v>
+      </c>
+      <c r="C19">
+        <v>3</v>
+      </c>
+      <c r="D19" t="b">
+        <v>0</v>
+      </c>
+      <c r="E19" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A20" t="s">
+        <v>29</v>
+      </c>
+      <c r="B20" t="s">
+        <v>30</v>
+      </c>
+      <c r="C20">
+        <v>1</v>
+      </c>
+      <c r="D20" t="b">
+        <v>0</v>
+      </c>
+      <c r="E20" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A21" t="s">
+        <v>29</v>
+      </c>
+      <c r="B21" t="s">
+        <v>30</v>
+      </c>
+      <c r="C21">
+        <v>2</v>
+      </c>
+      <c r="D21" t="b">
+        <v>0</v>
+      </c>
+      <c r="E21" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A22" t="s">
+        <v>29</v>
+      </c>
+      <c r="B22" t="s">
+        <v>30</v>
+      </c>
+      <c r="C22">
+        <v>3</v>
+      </c>
+      <c r="D22" t="b">
+        <v>0</v>
+      </c>
+      <c r="E22" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A23" t="s">
+        <v>36</v>
+      </c>
+      <c r="B23" t="s">
+        <v>37</v>
+      </c>
+      <c r="C23">
+        <v>1</v>
+      </c>
+      <c r="D23" t="b">
+        <v>0</v>
+      </c>
+      <c r="E23" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A24" t="s">
+        <v>36</v>
+      </c>
+      <c r="B24" t="s">
+        <v>37</v>
+      </c>
+      <c r="C24">
+        <v>2</v>
+      </c>
+      <c r="D24" t="b">
+        <v>0</v>
+      </c>
+      <c r="E24" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A25" t="s">
+        <v>36</v>
+      </c>
+      <c r="B25" t="s">
+        <v>37</v>
+      </c>
+      <c r="C25">
+        <v>3</v>
+      </c>
+      <c r="D25" t="b">
+        <v>0</v>
+      </c>
+      <c r="E25" t="s">
         <v>69</v>
       </c>
     </row>

</xml_diff>

<commit_message>
adding more servants from saber class
</commit_message>
<xml_diff>
--- a/data/Fate-Spreadsheet.xlsx
+++ b/data/Fate-Spreadsheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pixel\Documents\Projects\Fate-Wiki\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B852EF1C-3539-407D-ACE6-F57265693E33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33239780-26C1-4CA1-BB72-800FD4D65CD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{B05E798F-9EF6-4508-A0A4-311D06661AED}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="590" uniqueCount="265">
   <si>
     <t>servant_id</t>
   </si>
@@ -379,6 +379,465 @@
   </si>
   <si>
     <t>Staff of Selection</t>
+  </si>
+  <si>
+    <t>S0002</t>
+  </si>
+  <si>
+    <t>S0003</t>
+  </si>
+  <si>
+    <t>S0004</t>
+  </si>
+  <si>
+    <t>S0005</t>
+  </si>
+  <si>
+    <t>S0006</t>
+  </si>
+  <si>
+    <t>S0007</t>
+  </si>
+  <si>
+    <t>S0008</t>
+  </si>
+  <si>
+    <t>S0009</t>
+  </si>
+  <si>
+    <t>S0010</t>
+  </si>
+  <si>
+    <t>S0011</t>
+  </si>
+  <si>
+    <t>S0012</t>
+  </si>
+  <si>
+    <t>S0013</t>
+  </si>
+  <si>
+    <t>S0014</t>
+  </si>
+  <si>
+    <t>S0015</t>
+  </si>
+  <si>
+    <t>S0016</t>
+  </si>
+  <si>
+    <t>S0017</t>
+  </si>
+  <si>
+    <t>S0018</t>
+  </si>
+  <si>
+    <t>S0019</t>
+  </si>
+  <si>
+    <t>S0020</t>
+  </si>
+  <si>
+    <t>S0021</t>
+  </si>
+  <si>
+    <t>S0022</t>
+  </si>
+  <si>
+    <t>S0023</t>
+  </si>
+  <si>
+    <t>Nero Claudius</t>
+  </si>
+  <si>
+    <t>nero-claudius</t>
+  </si>
+  <si>
+    <t>Mordred</t>
+  </si>
+  <si>
+    <t>Altera</t>
+  </si>
+  <si>
+    <t>Gawain</t>
+  </si>
+  <si>
+    <t>Bedivere</t>
+  </si>
+  <si>
+    <t>Okita Souji</t>
+  </si>
+  <si>
+    <t>Sigurd</t>
+  </si>
+  <si>
+    <t>Siegfried</t>
+  </si>
+  <si>
+    <t>Chevalier d'Eon</t>
+  </si>
+  <si>
+    <t>Senji Muramasa</t>
+  </si>
+  <si>
+    <t>Miyamoto Musashi</t>
+  </si>
+  <si>
+    <t>Charlemagne</t>
+  </si>
+  <si>
+    <t>Jacques de Molay</t>
+  </si>
+  <si>
+    <t>Arthur Pendragon</t>
+  </si>
+  <si>
+    <t>Jason</t>
+  </si>
+  <si>
+    <t>Barghest</t>
+  </si>
+  <si>
+    <t>Saito Hajime</t>
+  </si>
+  <si>
+    <t>Dioscuri</t>
+  </si>
+  <si>
+    <t>Lakshmibai</t>
+  </si>
+  <si>
+    <t>Suzuka Gozen</t>
+  </si>
+  <si>
+    <t>mordred</t>
+  </si>
+  <si>
+    <t>altera</t>
+  </si>
+  <si>
+    <t>gawain</t>
+  </si>
+  <si>
+    <t>bedivere</t>
+  </si>
+  <si>
+    <t>sigurd</t>
+  </si>
+  <si>
+    <t>siegfried</t>
+  </si>
+  <si>
+    <t>charlemagne</t>
+  </si>
+  <si>
+    <t>jason</t>
+  </si>
+  <si>
+    <t>barghest</t>
+  </si>
+  <si>
+    <t>dioscuri</t>
+  </si>
+  <si>
+    <t>lakshmibai</t>
+  </si>
+  <si>
+    <t>okita-souji</t>
+  </si>
+  <si>
+    <t>senji-muramasa</t>
+  </si>
+  <si>
+    <t>miyamoto-musashi</t>
+  </si>
+  <si>
+    <t>arthur-pendragon</t>
+  </si>
+  <si>
+    <t>saito-hajime</t>
+  </si>
+  <si>
+    <t>suzuka-gozen</t>
+  </si>
+  <si>
+    <t>chevalier-deon</t>
+  </si>
+  <si>
+    <t>artoria-pendragon-alter</t>
+  </si>
+  <si>
+    <t>jacques-de-molay</t>
+  </si>
+  <si>
+    <t>okita-souji-alter</t>
+  </si>
+  <si>
+    <t>2,3,4,5,5</t>
+  </si>
+  <si>
+    <t>2,3,4,5</t>
+  </si>
+  <si>
+    <t>Luck</t>
+  </si>
+  <si>
+    <t>2,3,4,5,5,5</t>
+  </si>
+  <si>
+    <t>Luck,Luck,Surveil</t>
+  </si>
+  <si>
+    <t>2,3,3,5,5</t>
+  </si>
+  <si>
+    <t>Surveil,Luck</t>
+  </si>
+  <si>
+    <t>2,2,3,4,5</t>
+  </si>
+  <si>
+    <t>Luck,Preparation</t>
+  </si>
+  <si>
+    <t>4,4</t>
+  </si>
+  <si>
+    <t>2,3,3,4,5,5</t>
+  </si>
+  <si>
+    <t>Luck,Surveil,Surveil</t>
+  </si>
+  <si>
+    <t>3,4,4,5,5</t>
+  </si>
+  <si>
+    <t>Luck,Surveil</t>
+  </si>
+  <si>
+    <t>3,3,4</t>
+  </si>
+  <si>
+    <t>3,4,4</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>3,3,4,5</t>
+  </si>
+  <si>
+    <t>2,3,3,4</t>
+  </si>
+  <si>
+    <t>Luck,Preparation,Preparation</t>
+  </si>
+  <si>
+    <t>2,3,5,5</t>
+  </si>
+  <si>
+    <t>2,4,4</t>
+  </si>
+  <si>
+    <t>Luck,Luck</t>
+  </si>
+  <si>
+    <t>3,3,4,4</t>
+  </si>
+  <si>
+    <t>2,2</t>
+  </si>
+  <si>
+    <t>Luck,Surveil,Preparation</t>
+  </si>
+  <si>
+    <t>2,3,4,4</t>
+  </si>
+  <si>
+    <t>3,4,4,5</t>
+  </si>
+  <si>
+    <t>2,3,3,5</t>
+  </si>
+  <si>
+    <t>2,3,3,4,5</t>
+  </si>
+  <si>
+    <t>Luck,Avenger Class</t>
+  </si>
+  <si>
+    <t>2,2,2</t>
+  </si>
+  <si>
+    <t>Weak Constitution</t>
+  </si>
+  <si>
+    <t>Weak-Constitution</t>
+  </si>
+  <si>
+    <t>Astrapte Argo</t>
+  </si>
+  <si>
+    <t>Astrapte-Argo</t>
+  </si>
+  <si>
+    <t>Misfortune</t>
+  </si>
+  <si>
+    <t>Aestus Domus Aurea</t>
+  </si>
+  <si>
+    <t>Aestus Estus</t>
+  </si>
+  <si>
+    <t>Emperor's Prerogative</t>
+  </si>
+  <si>
+    <t>Clarent</t>
+  </si>
+  <si>
+    <t>Helm of Hidden Infidelity</t>
+  </si>
+  <si>
+    <t>Teardrop Photon Ray</t>
+  </si>
+  <si>
+    <t>Photon Ray</t>
+  </si>
+  <si>
+    <t>Excalibur Galatine</t>
+  </si>
+  <si>
+    <t>Numeral of the Saint</t>
+  </si>
+  <si>
+    <t>Airgetlam</t>
+  </si>
+  <si>
+    <t>Oath of Protection</t>
+  </si>
+  <si>
+    <t>Flag of Sincerity</t>
+  </si>
+  <si>
+    <t>Mumyou Sandan-Zuki</t>
+  </si>
+  <si>
+    <t>Coat of Oaths</t>
+  </si>
+  <si>
+    <t>Gram II</t>
+  </si>
+  <si>
+    <t>Bolverk Gram</t>
+  </si>
+  <si>
+    <t>Ridill &amp; Hrotti</t>
+  </si>
+  <si>
+    <t>Balmung</t>
+  </si>
+  <si>
+    <t>Armour of Fafnir</t>
+  </si>
+  <si>
+    <t>Tarnkappe</t>
+  </si>
+  <si>
+    <t>Self-Suggestion</t>
+  </si>
+  <si>
+    <t>Sword Dance</t>
+  </si>
+  <si>
+    <t>Fleur de Lys</t>
+  </si>
+  <si>
+    <t>Tsumukari Muramasa</t>
+  </si>
+  <si>
+    <t>Imperfect Edge</t>
+  </si>
+  <si>
+    <t>6 Realms, 5 Rings</t>
+  </si>
+  <si>
+    <t>Niten Ichiryu</t>
+  </si>
+  <si>
+    <t>Blackening Curse</t>
+  </si>
+  <si>
+    <t>Excalibur Morgan</t>
+  </si>
+  <si>
+    <t>Charles Patricius</t>
+  </si>
+  <si>
+    <t>Joyeuse Ordre</t>
+  </si>
+  <si>
+    <t>Pilgrim's Reward</t>
+  </si>
+  <si>
+    <t>Mother of Goats</t>
+  </si>
+  <si>
+    <t>The Goat's Invitation</t>
+  </si>
+  <si>
+    <t>Excalibur Proto</t>
+  </si>
+  <si>
+    <t>Heracles</t>
+  </si>
+  <si>
+    <t>Atalante</t>
+  </si>
+  <si>
+    <t>Medea</t>
+  </si>
+  <si>
+    <t>Black Dog Galatine</t>
+  </si>
+  <si>
+    <t>Sun Devourer</t>
+  </si>
+  <si>
+    <t>Demon Chains</t>
+  </si>
+  <si>
+    <t>Formlessness</t>
+  </si>
+  <si>
+    <t>Twin Divinity</t>
+  </si>
+  <si>
+    <t>Dioscures Tyndaridae</t>
+  </si>
+  <si>
+    <t>Gift of Mortality</t>
+  </si>
+  <si>
+    <t>Nahi Doongi</t>
+  </si>
+  <si>
+    <t>Queen of Resistance</t>
+  </si>
+  <si>
+    <t>Boundless Potential</t>
+  </si>
+  <si>
+    <t>Rengoku</t>
+  </si>
+  <si>
+    <t>Trichiliocosm</t>
+  </si>
+  <si>
+    <t>Demonic Sun-Shower</t>
+  </si>
+  <si>
+    <t>Wise Fox</t>
   </si>
 </sst>
 </file>
@@ -428,11 +887,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -767,7 +1227,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E33D7ECC-1EAA-4A40-B4DA-A93E54CBC8B5}">
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:K31"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="17.1328125" customWidth="1"/>
@@ -851,112 +1311,121 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>86</v>
+        <v>112</v>
       </c>
       <c r="B3" t="s">
-        <v>87</v>
+        <v>134</v>
       </c>
       <c r="C3" t="s">
-        <v>88</v>
+        <v>135</v>
       </c>
       <c r="D3" t="s">
-        <v>89</v>
+        <v>7</v>
       </c>
       <c r="E3" t="s">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="G3" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="I3" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="H3" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="I3" s="2" t="s">
-        <v>42</v>
+      <c r="J3" s="2" t="s">
+        <v>178</v>
       </c>
       <c r="K3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>17</v>
+        <v>113</v>
       </c>
       <c r="B4" t="s">
-        <v>18</v>
+        <v>136</v>
       </c>
       <c r="C4" t="s">
-        <v>19</v>
+        <v>155</v>
       </c>
       <c r="D4" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="E4" t="s">
         <v>8</v>
       </c>
-      <c r="I4" s="2" t="s">
-        <v>21</v>
+      <c r="G4" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>101</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>22</v>
+        <v>180</v>
       </c>
       <c r="K4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>97</v>
+        <v>114</v>
       </c>
       <c r="B5" t="s">
-        <v>98</v>
+        <v>137</v>
       </c>
       <c r="C5" t="s">
-        <v>99</v>
+        <v>156</v>
       </c>
       <c r="D5" t="s">
-        <v>20</v>
+        <v>7</v>
       </c>
       <c r="E5" t="s">
-        <v>100</v>
+        <v>8</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>176</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="I5" s="2" t="s">
-        <v>102</v>
+        <v>181</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>182</v>
       </c>
       <c r="K5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>76</v>
+        <v>115</v>
       </c>
       <c r="B6" t="s">
-        <v>77</v>
+        <v>138</v>
       </c>
       <c r="C6" t="s">
-        <v>78</v>
+        <v>157</v>
       </c>
       <c r="D6" t="s">
-        <v>79</v>
+        <v>7</v>
       </c>
       <c r="E6" t="s">
-        <v>40</v>
+        <v>8</v>
       </c>
       <c r="G6" s="2" t="s">
-        <v>80</v>
+        <v>183</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>15</v>
+        <v>177</v>
       </c>
       <c r="I6" s="2" t="s">
         <v>82</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>81</v>
+        <v>184</v>
       </c>
       <c r="K6" t="b">
         <v>0</v>
@@ -964,28 +1433,31 @@
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>23</v>
+        <v>116</v>
       </c>
       <c r="B7" t="s">
-        <v>24</v>
+        <v>139</v>
       </c>
       <c r="C7" t="s">
-        <v>25</v>
+        <v>158</v>
       </c>
       <c r="D7" t="s">
-        <v>26</v>
+        <v>7</v>
       </c>
       <c r="E7" t="s">
         <v>8</v>
       </c>
       <c r="G7" s="2" t="s">
-        <v>27</v>
+        <v>185</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>28</v>
+        <v>186</v>
+      </c>
+      <c r="I7" s="2" t="s">
+        <v>82</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>70</v>
+        <v>187</v>
       </c>
       <c r="K7" t="b">
         <v>0</v>
@@ -993,62 +1465,736 @@
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>29</v>
+        <v>117</v>
       </c>
       <c r="B8" t="s">
-        <v>30</v>
+        <v>140</v>
       </c>
       <c r="C8" t="s">
-        <v>31</v>
+        <v>166</v>
       </c>
       <c r="D8" t="s">
-        <v>32</v>
+        <v>7</v>
       </c>
       <c r="E8" t="s">
-        <v>33</v>
+        <v>90</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>15</v>
+        <v>177</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="I8" s="2" t="s">
-        <v>34</v>
+        <v>188</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>35</v>
+        <v>189</v>
       </c>
       <c r="K8" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
+        <v>118</v>
+      </c>
+      <c r="B9" t="s">
+        <v>141</v>
+      </c>
+      <c r="C9" t="s">
+        <v>159</v>
+      </c>
+      <c r="D9" t="s">
+        <v>7</v>
+      </c>
+      <c r="E9" t="s">
+        <v>90</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="J9" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="K9" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A10" t="s">
+        <v>119</v>
+      </c>
+      <c r="B10" t="s">
+        <v>142</v>
+      </c>
+      <c r="C10" t="s">
+        <v>160</v>
+      </c>
+      <c r="D10" t="s">
+        <v>7</v>
+      </c>
+      <c r="E10" t="s">
+        <v>8</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="J10" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="K10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A11" t="s">
+        <v>120</v>
+      </c>
+      <c r="B11" t="s">
+        <v>143</v>
+      </c>
+      <c r="C11" t="s">
+        <v>172</v>
+      </c>
+      <c r="D11" t="s">
+        <v>7</v>
+      </c>
+      <c r="E11" t="s">
+        <v>90</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="I11" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="J11" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="K11" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A12" t="s">
+        <v>121</v>
+      </c>
+      <c r="B12" t="s">
+        <v>144</v>
+      </c>
+      <c r="C12" t="s">
+        <v>167</v>
+      </c>
+      <c r="D12" t="s">
+        <v>79</v>
+      </c>
+      <c r="E12" t="s">
+        <v>90</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="J12" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="K12" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A13" t="s">
+        <v>122</v>
+      </c>
+      <c r="B13" t="s">
+        <v>145</v>
+      </c>
+      <c r="C13" t="s">
+        <v>168</v>
+      </c>
+      <c r="D13" t="s">
+        <v>7</v>
+      </c>
+      <c r="E13" t="s">
+        <v>100</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="J13" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="K13" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A14" t="s">
+        <v>123</v>
+      </c>
+      <c r="B14" t="s">
+        <v>5</v>
+      </c>
+      <c r="C14" t="s">
+        <v>173</v>
+      </c>
+      <c r="D14" t="s">
+        <v>7</v>
+      </c>
+      <c r="E14" t="s">
+        <v>8</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="J14" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="K14" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A15" t="s">
+        <v>124</v>
+      </c>
+      <c r="B15" t="s">
+        <v>146</v>
+      </c>
+      <c r="C15" t="s">
+        <v>161</v>
+      </c>
+      <c r="D15" t="s">
+        <v>7</v>
+      </c>
+      <c r="E15" t="s">
+        <v>90</v>
+      </c>
+      <c r="G15" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="H15" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="I15" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="J15" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="K15" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A16" t="s">
+        <v>125</v>
+      </c>
+      <c r="B16" t="s">
+        <v>147</v>
+      </c>
+      <c r="C16" t="s">
+        <v>174</v>
+      </c>
+      <c r="D16" t="s">
+        <v>7</v>
+      </c>
+      <c r="E16" t="s">
+        <v>8</v>
+      </c>
+      <c r="G16" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="H16" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="I16" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="J16" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="K16" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A17" t="s">
+        <v>126</v>
+      </c>
+      <c r="B17" t="s">
+        <v>148</v>
+      </c>
+      <c r="C17" t="s">
+        <v>169</v>
+      </c>
+      <c r="D17" t="s">
+        <v>7</v>
+      </c>
+      <c r="E17" t="s">
+        <v>8</v>
+      </c>
+      <c r="G17" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="H17" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I17" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="J17" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="K17" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A18" t="s">
+        <v>127</v>
+      </c>
+      <c r="B18" t="s">
+        <v>149</v>
+      </c>
+      <c r="C18" t="s">
+        <v>162</v>
+      </c>
+      <c r="D18" t="s">
+        <v>7</v>
+      </c>
+      <c r="E18" t="s">
+        <v>90</v>
+      </c>
+      <c r="G18" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="H18" s="2" t="s">
+        <v>202</v>
+      </c>
+      <c r="I18" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="J18" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="K18" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A19" t="s">
+        <v>128</v>
+      </c>
+      <c r="B19" t="s">
+        <v>150</v>
+      </c>
+      <c r="C19" t="s">
+        <v>163</v>
+      </c>
+      <c r="D19" t="s">
+        <v>7</v>
+      </c>
+      <c r="E19" t="s">
+        <v>90</v>
+      </c>
+      <c r="G19" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="H19" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I19" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J19" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="K19" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A20" t="s">
+        <v>129</v>
+      </c>
+      <c r="B20" t="s">
+        <v>151</v>
+      </c>
+      <c r="C20" t="s">
+        <v>170</v>
+      </c>
+      <c r="D20" t="s">
+        <v>7</v>
+      </c>
+      <c r="E20" t="s">
+        <v>90</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="H20" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="J20" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="K20" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A21" t="s">
+        <v>130</v>
+      </c>
+      <c r="B21" t="s">
+        <v>152</v>
+      </c>
+      <c r="C21" t="s">
+        <v>164</v>
+      </c>
+      <c r="D21" t="s">
+        <v>7</v>
+      </c>
+      <c r="E21" t="s">
+        <v>90</v>
+      </c>
+      <c r="G21" s="2" t="s">
+        <v>205</v>
+      </c>
+      <c r="H21" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I21" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="J21" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="K21" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A22" t="s">
+        <v>131</v>
+      </c>
+      <c r="B22" t="s">
+        <v>153</v>
+      </c>
+      <c r="C22" t="s">
+        <v>165</v>
+      </c>
+      <c r="D22" t="s">
+        <v>7</v>
+      </c>
+      <c r="E22" t="s">
+        <v>40</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="H22" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="I22" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="J22" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K22" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A23" t="s">
+        <v>132</v>
+      </c>
+      <c r="B23" t="s">
+        <v>140</v>
+      </c>
+      <c r="C23" t="s">
+        <v>175</v>
+      </c>
+      <c r="D23" t="s">
+        <v>79</v>
+      </c>
+      <c r="E23" t="s">
+        <v>90</v>
+      </c>
+      <c r="G23" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="H23" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="I23" s="2" t="s">
+        <v>207</v>
+      </c>
+      <c r="J23" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="K23" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A24" t="s">
+        <v>133</v>
+      </c>
+      <c r="B24" t="s">
+        <v>154</v>
+      </c>
+      <c r="C24" t="s">
+        <v>171</v>
+      </c>
+      <c r="D24" t="s">
+        <v>7</v>
+      </c>
+      <c r="E24" t="s">
+        <v>90</v>
+      </c>
+      <c r="G24" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H24" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="I24" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="J24" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="K24" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A25" t="s">
+        <v>86</v>
+      </c>
+      <c r="B25" t="s">
+        <v>87</v>
+      </c>
+      <c r="C25" t="s">
+        <v>88</v>
+      </c>
+      <c r="D25" t="s">
+        <v>89</v>
+      </c>
+      <c r="E25" t="s">
+        <v>90</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H25" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="I25" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="K25" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A26" t="s">
+        <v>17</v>
+      </c>
+      <c r="B26" t="s">
+        <v>18</v>
+      </c>
+      <c r="C26" t="s">
+        <v>19</v>
+      </c>
+      <c r="D26" t="s">
+        <v>20</v>
+      </c>
+      <c r="E26" t="s">
+        <v>8</v>
+      </c>
+      <c r="I26" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="J26" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K26" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A27" t="s">
+        <v>97</v>
+      </c>
+      <c r="B27" t="s">
+        <v>98</v>
+      </c>
+      <c r="C27" t="s">
+        <v>99</v>
+      </c>
+      <c r="D27" t="s">
+        <v>20</v>
+      </c>
+      <c r="E27" t="s">
+        <v>100</v>
+      </c>
+      <c r="H27" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="I27" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="K27" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A28" t="s">
+        <v>76</v>
+      </c>
+      <c r="B28" t="s">
+        <v>77</v>
+      </c>
+      <c r="C28" t="s">
+        <v>78</v>
+      </c>
+      <c r="D28" t="s">
+        <v>79</v>
+      </c>
+      <c r="E28" t="s">
+        <v>40</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="H28" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I28" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="J28" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="K28" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A29" t="s">
+        <v>23</v>
+      </c>
+      <c r="B29" t="s">
+        <v>24</v>
+      </c>
+      <c r="C29" t="s">
+        <v>25</v>
+      </c>
+      <c r="D29" t="s">
+        <v>26</v>
+      </c>
+      <c r="E29" t="s">
+        <v>8</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H29" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="J29" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="K29" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A30" t="s">
+        <v>29</v>
+      </c>
+      <c r="B30" t="s">
+        <v>30</v>
+      </c>
+      <c r="C30" t="s">
+        <v>31</v>
+      </c>
+      <c r="D30" t="s">
+        <v>32</v>
+      </c>
+      <c r="E30" t="s">
+        <v>33</v>
+      </c>
+      <c r="G30" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H30" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="I30" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="J30" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="K30" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A31" t="s">
         <v>36</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B31" t="s">
         <v>37</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C31" t="s">
         <v>38</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D31" t="s">
         <v>39</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E31" t="s">
         <v>40</v>
       </c>
-      <c r="G9" s="2" t="s">
+      <c r="G31" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="H9" s="2" t="s">
+      <c r="H31" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="J9" s="2" t="s">
+      <c r="J31" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="K9" t="b">
+      <c r="K31" t="b">
         <v>1</v>
       </c>
     </row>
@@ -1056,14 +2202,14 @@
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="I6 H2 H8" numberStoredAsText="1"/>
+    <ignoredError sqref="H2 I28 H30 I6:I7 I10 I12 H14 I18 I22 I24" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1BC60D8-44F3-478D-BCC0-4752624457AE}">
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="19" customWidth="1"/>
@@ -1092,122 +2238,173 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A2" t="s">
-        <v>86</v>
-      </c>
-      <c r="B2" t="s">
-        <v>87</v>
-      </c>
-      <c r="C2" t="s">
-        <v>92</v>
-      </c>
-      <c r="D2" t="s">
-        <v>93</v>
-      </c>
-      <c r="E2">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A3" t="s">
-        <v>17</v>
-      </c>
-      <c r="B3" t="s">
-        <v>18</v>
-      </c>
-      <c r="C3" t="s">
-        <v>47</v>
-      </c>
-      <c r="D3" t="s">
-        <v>72</v>
-      </c>
-      <c r="E3">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
-      <c r="A4" t="s">
-        <v>17</v>
-      </c>
-      <c r="B4" t="s">
-        <v>18</v>
-      </c>
-      <c r="C4" t="s">
-        <v>73</v>
-      </c>
-      <c r="D4" t="s">
-        <v>74</v>
-      </c>
-      <c r="E4">
-        <v>3</v>
+    <row r="2" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="A2" s="4" t="s">
+        <v>117</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="E2" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="A3" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>210</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="E3" s="4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.45">
+      <c r="A4" s="4" t="s">
+        <v>131</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>153</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="E4" s="4">
+        <v>1</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>97</v>
+        <v>86</v>
       </c>
       <c r="B5" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="C5" t="s">
-        <v>103</v>
+        <v>92</v>
       </c>
       <c r="D5" t="s">
-        <v>106</v>
+        <v>93</v>
       </c>
       <c r="E5">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>97</v>
+        <v>17</v>
       </c>
       <c r="B6" t="s">
-        <v>98</v>
+        <v>18</v>
       </c>
       <c r="C6" t="s">
-        <v>104</v>
+        <v>47</v>
       </c>
       <c r="D6" t="s">
-        <v>107</v>
+        <v>72</v>
       </c>
       <c r="E6">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>97</v>
+        <v>17</v>
       </c>
       <c r="B7" t="s">
-        <v>98</v>
+        <v>18</v>
       </c>
       <c r="C7" t="s">
-        <v>105</v>
+        <v>73</v>
       </c>
       <c r="D7" t="s">
-        <v>108</v>
+        <v>74</v>
       </c>
       <c r="E7">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
+        <v>97</v>
+      </c>
+      <c r="B8" t="s">
+        <v>98</v>
+      </c>
+      <c r="C8" t="s">
+        <v>103</v>
+      </c>
+      <c r="D8" t="s">
+        <v>106</v>
+      </c>
+      <c r="E8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A9" t="s">
+        <v>97</v>
+      </c>
+      <c r="B9" t="s">
+        <v>98</v>
+      </c>
+      <c r="C9" t="s">
+        <v>104</v>
+      </c>
+      <c r="D9" t="s">
+        <v>107</v>
+      </c>
+      <c r="E9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A10" t="s">
+        <v>97</v>
+      </c>
+      <c r="B10" t="s">
+        <v>98</v>
+      </c>
+      <c r="C10" t="s">
+        <v>105</v>
+      </c>
+      <c r="D10" t="s">
+        <v>108</v>
+      </c>
+      <c r="E10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A11" t="s">
         <v>36</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B11" t="s">
         <v>37</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C11" t="s">
         <v>48</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D11" t="s">
         <v>48</v>
       </c>
-      <c r="E8">
+      <c r="E11">
         <v>2</v>
       </c>
     </row>
@@ -1220,13 +2417,13 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84E3BB0D-5578-4069-B1C9-C3864EB2A429}">
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F91"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="20.59765625" customWidth="1"/>
     <col min="3" max="3" width="12.73046875" customWidth="1"/>
     <col min="4" max="4" width="17.06640625" customWidth="1"/>
-    <col min="5" max="5" width="18.1328125" customWidth="1"/>
+    <col min="5" max="5" width="21.59765625" customWidth="1"/>
     <col min="6" max="6" width="15.73046875" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1303,27 +2500,27 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>86</v>
+        <v>112</v>
       </c>
       <c r="B5" t="s">
-        <v>87</v>
+        <v>134</v>
       </c>
       <c r="C5">
         <v>1</v>
       </c>
       <c r="D5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E5" t="s">
-        <v>94</v>
+        <v>213</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>86</v>
+        <v>112</v>
       </c>
       <c r="B6" t="s">
-        <v>87</v>
+        <v>134</v>
       </c>
       <c r="C6">
         <v>2</v>
@@ -1332,15 +2529,15 @@
         <v>0</v>
       </c>
       <c r="E6" t="s">
-        <v>95</v>
+        <v>214</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>86</v>
+        <v>112</v>
       </c>
       <c r="B7" t="s">
-        <v>87</v>
+        <v>134</v>
       </c>
       <c r="C7">
         <v>3</v>
@@ -1349,15 +2546,15 @@
         <v>0</v>
       </c>
       <c r="E7" t="s">
-        <v>96</v>
+        <v>215</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>17</v>
+        <v>113</v>
       </c>
       <c r="B8" t="s">
-        <v>18</v>
+        <v>136</v>
       </c>
       <c r="C8">
         <v>1</v>
@@ -1366,15 +2563,15 @@
         <v>1</v>
       </c>
       <c r="E8" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>17</v>
+        <v>113</v>
       </c>
       <c r="B9" t="s">
-        <v>18</v>
+        <v>136</v>
       </c>
       <c r="C9">
         <v>2</v>
@@ -1383,15 +2580,15 @@
         <v>0</v>
       </c>
       <c r="E9" t="s">
-        <v>59</v>
+        <v>216</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
-        <v>17</v>
+        <v>113</v>
       </c>
       <c r="B10" t="s">
-        <v>18</v>
+        <v>136</v>
       </c>
       <c r="C10">
         <v>3</v>
@@ -1400,32 +2597,32 @@
         <v>0</v>
       </c>
       <c r="E10" t="s">
-        <v>60</v>
+        <v>217</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
-        <v>97</v>
+        <v>114</v>
       </c>
       <c r="B11" t="s">
-        <v>98</v>
+        <v>137</v>
       </c>
       <c r="C11">
         <v>1</v>
       </c>
       <c r="D11" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E11" t="s">
-        <v>109</v>
+        <v>53</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
-        <v>97</v>
+        <v>114</v>
       </c>
       <c r="B12" t="s">
-        <v>98</v>
+        <v>137</v>
       </c>
       <c r="C12">
         <v>2</v>
@@ -1434,15 +2631,15 @@
         <v>0</v>
       </c>
       <c r="E12" t="s">
-        <v>110</v>
+        <v>218</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
-        <v>97</v>
+        <v>114</v>
       </c>
       <c r="B13" t="s">
-        <v>98</v>
+        <v>137</v>
       </c>
       <c r="C13">
         <v>3</v>
@@ -1451,15 +2648,15 @@
         <v>0</v>
       </c>
       <c r="E13" t="s">
-        <v>111</v>
+        <v>219</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
-        <v>76</v>
+        <v>115</v>
       </c>
       <c r="B14" t="s">
-        <v>77</v>
+        <v>138</v>
       </c>
       <c r="C14">
         <v>1</v>
@@ -1468,15 +2665,15 @@
         <v>1</v>
       </c>
       <c r="E14" t="s">
-        <v>83</v>
+        <v>53</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
-        <v>76</v>
+        <v>115</v>
       </c>
       <c r="B15" t="s">
-        <v>77</v>
+        <v>138</v>
       </c>
       <c r="C15">
         <v>2</v>
@@ -1485,15 +2682,15 @@
         <v>0</v>
       </c>
       <c r="E15" t="s">
-        <v>84</v>
+        <v>220</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
-        <v>76</v>
+        <v>115</v>
       </c>
       <c r="B16" t="s">
-        <v>77</v>
+        <v>138</v>
       </c>
       <c r="C16">
         <v>3</v>
@@ -1502,32 +2699,32 @@
         <v>0</v>
       </c>
       <c r="E16" t="s">
-        <v>85</v>
+        <v>221</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
-        <v>23</v>
+        <v>116</v>
       </c>
       <c r="B17" t="s">
-        <v>24</v>
+        <v>139</v>
       </c>
       <c r="C17">
         <v>1</v>
       </c>
       <c r="D17" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E17" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
-        <v>23</v>
+        <v>116</v>
       </c>
       <c r="B18" t="s">
-        <v>24</v>
+        <v>139</v>
       </c>
       <c r="C18">
         <v>2</v>
@@ -1536,15 +2733,15 @@
         <v>0</v>
       </c>
       <c r="E18" t="s">
-        <v>62</v>
+        <v>222</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
-        <v>23</v>
+        <v>116</v>
       </c>
       <c r="B19" t="s">
-        <v>24</v>
+        <v>139</v>
       </c>
       <c r="C19">
         <v>3</v>
@@ -1553,15 +2750,15 @@
         <v>0</v>
       </c>
       <c r="E19" t="s">
-        <v>63</v>
+        <v>223</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
-        <v>29</v>
+        <v>117</v>
       </c>
       <c r="B20" t="s">
-        <v>30</v>
+        <v>140</v>
       </c>
       <c r="C20">
         <v>1</v>
@@ -1570,15 +2767,15 @@
         <v>0</v>
       </c>
       <c r="E20" t="s">
-        <v>64</v>
+        <v>224</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
-        <v>29</v>
+        <v>117</v>
       </c>
       <c r="B21" t="s">
-        <v>30</v>
+        <v>140</v>
       </c>
       <c r="C21">
         <v>2</v>
@@ -1587,15 +2784,15 @@
         <v>0</v>
       </c>
       <c r="E21" t="s">
-        <v>65</v>
+        <v>225</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
-        <v>29</v>
+        <v>117</v>
       </c>
       <c r="B22" t="s">
-        <v>30</v>
+        <v>140</v>
       </c>
       <c r="C22">
         <v>3</v>
@@ -1604,15 +2801,15 @@
         <v>0</v>
       </c>
       <c r="E22" t="s">
-        <v>66</v>
+        <v>226</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
-        <v>36</v>
+        <v>118</v>
       </c>
       <c r="B23" t="s">
-        <v>37</v>
+        <v>141</v>
       </c>
       <c r="C23">
         <v>1</v>
@@ -1621,15 +2818,15 @@
         <v>0</v>
       </c>
       <c r="E23" t="s">
-        <v>67</v>
+        <v>227</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
-        <v>36</v>
+        <v>118</v>
       </c>
       <c r="B24" t="s">
-        <v>37</v>
+        <v>141</v>
       </c>
       <c r="C24">
         <v>2</v>
@@ -1638,15 +2835,15 @@
         <v>0</v>
       </c>
       <c r="E24" t="s">
-        <v>68</v>
+        <v>228</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
-        <v>36</v>
+        <v>118</v>
       </c>
       <c r="B25" t="s">
-        <v>37</v>
+        <v>141</v>
       </c>
       <c r="C25">
         <v>3</v>
@@ -1655,6 +2852,1128 @@
         <v>0</v>
       </c>
       <c r="E25" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A26" t="s">
+        <v>119</v>
+      </c>
+      <c r="B26" t="s">
+        <v>142</v>
+      </c>
+      <c r="C26">
+        <v>1</v>
+      </c>
+      <c r="D26" t="b">
+        <v>0</v>
+      </c>
+      <c r="E26" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A27" t="s">
+        <v>119</v>
+      </c>
+      <c r="B27" t="s">
+        <v>142</v>
+      </c>
+      <c r="C27">
+        <v>2</v>
+      </c>
+      <c r="D27" t="b">
+        <v>0</v>
+      </c>
+      <c r="E27" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A28" t="s">
+        <v>119</v>
+      </c>
+      <c r="B28" t="s">
+        <v>142</v>
+      </c>
+      <c r="C28">
+        <v>3</v>
+      </c>
+      <c r="D28" t="b">
+        <v>0</v>
+      </c>
+      <c r="E28" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A29" t="s">
+        <v>120</v>
+      </c>
+      <c r="B29" t="s">
+        <v>143</v>
+      </c>
+      <c r="C29">
+        <v>1</v>
+      </c>
+      <c r="D29" t="b">
+        <v>0</v>
+      </c>
+      <c r="E29" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A30" t="s">
+        <v>120</v>
+      </c>
+      <c r="B30" t="s">
+        <v>143</v>
+      </c>
+      <c r="C30">
+        <v>2</v>
+      </c>
+      <c r="D30" t="b">
+        <v>0</v>
+      </c>
+      <c r="E30" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A31" t="s">
+        <v>120</v>
+      </c>
+      <c r="B31" t="s">
+        <v>143</v>
+      </c>
+      <c r="C31">
+        <v>3</v>
+      </c>
+      <c r="D31" t="b">
+        <v>0</v>
+      </c>
+      <c r="E31" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A32" t="s">
+        <v>121</v>
+      </c>
+      <c r="B32" t="s">
+        <v>144</v>
+      </c>
+      <c r="C32">
+        <v>1</v>
+      </c>
+      <c r="D32" t="b">
+        <v>1</v>
+      </c>
+      <c r="E32" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A33" t="s">
+        <v>121</v>
+      </c>
+      <c r="B33" t="s">
+        <v>144</v>
+      </c>
+      <c r="C33">
+        <v>2</v>
+      </c>
+      <c r="D33" t="b">
+        <v>0</v>
+      </c>
+      <c r="E33" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A34" t="s">
+        <v>121</v>
+      </c>
+      <c r="B34" t="s">
+        <v>144</v>
+      </c>
+      <c r="C34">
+        <v>3</v>
+      </c>
+      <c r="D34" t="b">
+        <v>0</v>
+      </c>
+      <c r="E34" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A35" t="s">
+        <v>122</v>
+      </c>
+      <c r="B35" t="s">
+        <v>145</v>
+      </c>
+      <c r="C35">
+        <v>1</v>
+      </c>
+      <c r="D35" t="b">
+        <v>1</v>
+      </c>
+      <c r="E35" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A36" t="s">
+        <v>122</v>
+      </c>
+      <c r="B36" t="s">
+        <v>145</v>
+      </c>
+      <c r="C36">
+        <v>2</v>
+      </c>
+      <c r="D36" t="b">
+        <v>0</v>
+      </c>
+      <c r="E36" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A37" t="s">
+        <v>122</v>
+      </c>
+      <c r="B37" t="s">
+        <v>145</v>
+      </c>
+      <c r="C37">
+        <v>3</v>
+      </c>
+      <c r="D37" t="b">
+        <v>0</v>
+      </c>
+      <c r="E37" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A38" t="s">
+        <v>123</v>
+      </c>
+      <c r="B38" t="s">
+        <v>5</v>
+      </c>
+      <c r="C38">
+        <v>1</v>
+      </c>
+      <c r="D38" t="b">
+        <v>1</v>
+      </c>
+      <c r="E38" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A39" t="s">
+        <v>123</v>
+      </c>
+      <c r="B39" t="s">
+        <v>5</v>
+      </c>
+      <c r="C39">
+        <v>2</v>
+      </c>
+      <c r="D39" t="b">
+        <v>0</v>
+      </c>
+      <c r="E39" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A40" t="s">
+        <v>123</v>
+      </c>
+      <c r="B40" t="s">
+        <v>5</v>
+      </c>
+      <c r="C40">
+        <v>3</v>
+      </c>
+      <c r="D40" t="b">
+        <v>0</v>
+      </c>
+      <c r="E40" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A41" t="s">
+        <v>124</v>
+      </c>
+      <c r="B41" t="s">
+        <v>146</v>
+      </c>
+      <c r="C41">
+        <v>1</v>
+      </c>
+      <c r="D41" t="b">
+        <v>1</v>
+      </c>
+      <c r="E41" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A42" t="s">
+        <v>124</v>
+      </c>
+      <c r="B42" t="s">
+        <v>146</v>
+      </c>
+      <c r="C42">
+        <v>2</v>
+      </c>
+      <c r="D42" t="b">
+        <v>0</v>
+      </c>
+      <c r="E42" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A43" t="s">
+        <v>124</v>
+      </c>
+      <c r="B43" t="s">
+        <v>146</v>
+      </c>
+      <c r="C43">
+        <v>3</v>
+      </c>
+      <c r="D43" t="b">
+        <v>0</v>
+      </c>
+      <c r="E43" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="44" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A44" t="s">
+        <v>125</v>
+      </c>
+      <c r="B44" t="s">
+        <v>147</v>
+      </c>
+      <c r="C44">
+        <v>1</v>
+      </c>
+      <c r="D44" t="b">
+        <v>0</v>
+      </c>
+      <c r="E44" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="45" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A45" t="s">
+        <v>125</v>
+      </c>
+      <c r="B45" t="s">
+        <v>147</v>
+      </c>
+      <c r="C45">
+        <v>2</v>
+      </c>
+      <c r="D45" t="b">
+        <v>0</v>
+      </c>
+      <c r="E45" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="46" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A46" t="s">
+        <v>125</v>
+      </c>
+      <c r="B46" t="s">
+        <v>147</v>
+      </c>
+      <c r="C46">
+        <v>3</v>
+      </c>
+      <c r="D46" t="b">
+        <v>0</v>
+      </c>
+      <c r="E46" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="47" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A47" t="s">
+        <v>126</v>
+      </c>
+      <c r="B47" t="s">
+        <v>148</v>
+      </c>
+      <c r="C47">
+        <v>1</v>
+      </c>
+      <c r="D47" t="b">
+        <v>1</v>
+      </c>
+      <c r="E47" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A48" t="s">
+        <v>126</v>
+      </c>
+      <c r="B48" t="s">
+        <v>148</v>
+      </c>
+      <c r="C48">
+        <v>2</v>
+      </c>
+      <c r="D48" t="b">
+        <v>0</v>
+      </c>
+      <c r="E48" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A49" t="s">
+        <v>126</v>
+      </c>
+      <c r="B49" t="s">
+        <v>148</v>
+      </c>
+      <c r="C49">
+        <v>3</v>
+      </c>
+      <c r="D49" t="b">
+        <v>0</v>
+      </c>
+      <c r="E49" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A50" t="s">
+        <v>127</v>
+      </c>
+      <c r="B50" t="s">
+        <v>149</v>
+      </c>
+      <c r="C50">
+        <v>1</v>
+      </c>
+      <c r="D50" t="b">
+        <v>0</v>
+      </c>
+      <c r="E50" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A51" t="s">
+        <v>127</v>
+      </c>
+      <c r="B51" t="s">
+        <v>149</v>
+      </c>
+      <c r="C51">
+        <v>2</v>
+      </c>
+      <c r="D51" t="b">
+        <v>0</v>
+      </c>
+      <c r="E51" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A52" t="s">
+        <v>127</v>
+      </c>
+      <c r="B52" t="s">
+        <v>149</v>
+      </c>
+      <c r="C52">
+        <v>3</v>
+      </c>
+      <c r="D52" t="b">
+        <v>0</v>
+      </c>
+      <c r="E52" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A53" t="s">
+        <v>128</v>
+      </c>
+      <c r="B53" t="s">
+        <v>150</v>
+      </c>
+      <c r="C53">
+        <v>1</v>
+      </c>
+      <c r="D53" t="b">
+        <v>0</v>
+      </c>
+      <c r="E53" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A54" t="s">
+        <v>128</v>
+      </c>
+      <c r="B54" t="s">
+        <v>150</v>
+      </c>
+      <c r="C54">
+        <v>2</v>
+      </c>
+      <c r="D54" t="b">
+        <v>0</v>
+      </c>
+      <c r="E54" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A55" t="s">
+        <v>128</v>
+      </c>
+      <c r="B55" t="s">
+        <v>150</v>
+      </c>
+      <c r="C55">
+        <v>3</v>
+      </c>
+      <c r="D55" t="b">
+        <v>0</v>
+      </c>
+      <c r="E55" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A56" t="s">
+        <v>129</v>
+      </c>
+      <c r="B56" t="s">
+        <v>151</v>
+      </c>
+      <c r="C56">
+        <v>1</v>
+      </c>
+      <c r="D56" t="b">
+        <v>1</v>
+      </c>
+      <c r="E56" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A57" t="s">
+        <v>129</v>
+      </c>
+      <c r="B57" t="s">
+        <v>151</v>
+      </c>
+      <c r="C57">
+        <v>2</v>
+      </c>
+      <c r="D57" t="b">
+        <v>0</v>
+      </c>
+      <c r="E57" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A58" t="s">
+        <v>129</v>
+      </c>
+      <c r="B58" t="s">
+        <v>151</v>
+      </c>
+      <c r="C58">
+        <v>3</v>
+      </c>
+      <c r="D58" t="b">
+        <v>0</v>
+      </c>
+      <c r="E58" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A59" t="s">
+        <v>130</v>
+      </c>
+      <c r="B59" t="s">
+        <v>152</v>
+      </c>
+      <c r="C59">
+        <v>1</v>
+      </c>
+      <c r="D59" t="b">
+        <v>0</v>
+      </c>
+      <c r="E59" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A60" t="s">
+        <v>130</v>
+      </c>
+      <c r="B60" t="s">
+        <v>152</v>
+      </c>
+      <c r="C60">
+        <v>2</v>
+      </c>
+      <c r="D60" t="b">
+        <v>0</v>
+      </c>
+      <c r="E60" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A61" t="s">
+        <v>130</v>
+      </c>
+      <c r="B61" t="s">
+        <v>152</v>
+      </c>
+      <c r="C61">
+        <v>3</v>
+      </c>
+      <c r="D61" t="b">
+        <v>0</v>
+      </c>
+      <c r="E61" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A62" t="s">
+        <v>131</v>
+      </c>
+      <c r="B62" t="s">
+        <v>153</v>
+      </c>
+      <c r="C62">
+        <v>1</v>
+      </c>
+      <c r="D62" t="b">
+        <v>1</v>
+      </c>
+      <c r="E62" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A63" t="s">
+        <v>131</v>
+      </c>
+      <c r="B63" t="s">
+        <v>153</v>
+      </c>
+      <c r="C63">
+        <v>2</v>
+      </c>
+      <c r="D63" t="b">
+        <v>0</v>
+      </c>
+      <c r="E63" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="64" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A64" t="s">
+        <v>131</v>
+      </c>
+      <c r="B64" t="s">
+        <v>153</v>
+      </c>
+      <c r="C64">
+        <v>3</v>
+      </c>
+      <c r="D64" t="b">
+        <v>0</v>
+      </c>
+      <c r="E64" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A65" t="s">
+        <v>132</v>
+      </c>
+      <c r="B65" t="s">
+        <v>140</v>
+      </c>
+      <c r="C65">
+        <v>1</v>
+      </c>
+      <c r="D65" t="b">
+        <v>1</v>
+      </c>
+      <c r="E65" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A66" t="s">
+        <v>132</v>
+      </c>
+      <c r="B66" t="s">
+        <v>140</v>
+      </c>
+      <c r="C66">
+        <v>2</v>
+      </c>
+      <c r="D66" t="b">
+        <v>0</v>
+      </c>
+      <c r="E66" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A67" t="s">
+        <v>132</v>
+      </c>
+      <c r="B67" t="s">
+        <v>140</v>
+      </c>
+      <c r="C67">
+        <v>3</v>
+      </c>
+      <c r="D67" t="b">
+        <v>0</v>
+      </c>
+      <c r="E67" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A68" t="s">
+        <v>133</v>
+      </c>
+      <c r="B68" t="s">
+        <v>154</v>
+      </c>
+      <c r="C68">
+        <v>1</v>
+      </c>
+      <c r="D68" t="b">
+        <v>0</v>
+      </c>
+      <c r="E68" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A69" t="s">
+        <v>133</v>
+      </c>
+      <c r="B69" t="s">
+        <v>154</v>
+      </c>
+      <c r="C69">
+        <v>2</v>
+      </c>
+      <c r="D69" t="b">
+        <v>0</v>
+      </c>
+      <c r="E69" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A70" t="s">
+        <v>133</v>
+      </c>
+      <c r="B70" t="s">
+        <v>154</v>
+      </c>
+      <c r="C70">
+        <v>3</v>
+      </c>
+      <c r="D70" t="b">
+        <v>0</v>
+      </c>
+      <c r="E70" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A71" t="s">
+        <v>86</v>
+      </c>
+      <c r="B71" t="s">
+        <v>87</v>
+      </c>
+      <c r="C71">
+        <v>1</v>
+      </c>
+      <c r="D71" t="b">
+        <v>1</v>
+      </c>
+      <c r="E71" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A72" t="s">
+        <v>86</v>
+      </c>
+      <c r="B72" t="s">
+        <v>87</v>
+      </c>
+      <c r="C72">
+        <v>2</v>
+      </c>
+      <c r="D72" t="b">
+        <v>0</v>
+      </c>
+      <c r="E72" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A73" t="s">
+        <v>86</v>
+      </c>
+      <c r="B73" t="s">
+        <v>87</v>
+      </c>
+      <c r="C73">
+        <v>3</v>
+      </c>
+      <c r="D73" t="b">
+        <v>0</v>
+      </c>
+      <c r="E73" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A74" t="s">
+        <v>17</v>
+      </c>
+      <c r="B74" t="s">
+        <v>18</v>
+      </c>
+      <c r="C74">
+        <v>1</v>
+      </c>
+      <c r="D74" t="b">
+        <v>1</v>
+      </c>
+      <c r="E74" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A75" t="s">
+        <v>17</v>
+      </c>
+      <c r="B75" t="s">
+        <v>18</v>
+      </c>
+      <c r="C75">
+        <v>2</v>
+      </c>
+      <c r="D75" t="b">
+        <v>0</v>
+      </c>
+      <c r="E75" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A76" t="s">
+        <v>17</v>
+      </c>
+      <c r="B76" t="s">
+        <v>18</v>
+      </c>
+      <c r="C76">
+        <v>3</v>
+      </c>
+      <c r="D76" t="b">
+        <v>0</v>
+      </c>
+      <c r="E76" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A77" t="s">
+        <v>97</v>
+      </c>
+      <c r="B77" t="s">
+        <v>98</v>
+      </c>
+      <c r="C77">
+        <v>1</v>
+      </c>
+      <c r="D77" t="b">
+        <v>0</v>
+      </c>
+      <c r="E77" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A78" t="s">
+        <v>97</v>
+      </c>
+      <c r="B78" t="s">
+        <v>98</v>
+      </c>
+      <c r="C78">
+        <v>2</v>
+      </c>
+      <c r="D78" t="b">
+        <v>0</v>
+      </c>
+      <c r="E78" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A79" t="s">
+        <v>97</v>
+      </c>
+      <c r="B79" t="s">
+        <v>98</v>
+      </c>
+      <c r="C79">
+        <v>3</v>
+      </c>
+      <c r="D79" t="b">
+        <v>0</v>
+      </c>
+      <c r="E79" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A80" t="s">
+        <v>76</v>
+      </c>
+      <c r="B80" t="s">
+        <v>77</v>
+      </c>
+      <c r="C80">
+        <v>1</v>
+      </c>
+      <c r="D80" t="b">
+        <v>1</v>
+      </c>
+      <c r="E80" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A81" t="s">
+        <v>76</v>
+      </c>
+      <c r="B81" t="s">
+        <v>77</v>
+      </c>
+      <c r="C81">
+        <v>2</v>
+      </c>
+      <c r="D81" t="b">
+        <v>0</v>
+      </c>
+      <c r="E81" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="82" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A82" t="s">
+        <v>76</v>
+      </c>
+      <c r="B82" t="s">
+        <v>77</v>
+      </c>
+      <c r="C82">
+        <v>3</v>
+      </c>
+      <c r="D82" t="b">
+        <v>0</v>
+      </c>
+      <c r="E82" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A83" t="s">
+        <v>23</v>
+      </c>
+      <c r="B83" t="s">
+        <v>24</v>
+      </c>
+      <c r="C83">
+        <v>1</v>
+      </c>
+      <c r="D83" t="b">
+        <v>0</v>
+      </c>
+      <c r="E83" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="84" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A84" t="s">
+        <v>23</v>
+      </c>
+      <c r="B84" t="s">
+        <v>24</v>
+      </c>
+      <c r="C84">
+        <v>2</v>
+      </c>
+      <c r="D84" t="b">
+        <v>0</v>
+      </c>
+      <c r="E84" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="85" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A85" t="s">
+        <v>23</v>
+      </c>
+      <c r="B85" t="s">
+        <v>24</v>
+      </c>
+      <c r="C85">
+        <v>3</v>
+      </c>
+      <c r="D85" t="b">
+        <v>0</v>
+      </c>
+      <c r="E85" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A86" t="s">
+        <v>29</v>
+      </c>
+      <c r="B86" t="s">
+        <v>30</v>
+      </c>
+      <c r="C86">
+        <v>1</v>
+      </c>
+      <c r="D86" t="b">
+        <v>0</v>
+      </c>
+      <c r="E86" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="87" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A87" t="s">
+        <v>29</v>
+      </c>
+      <c r="B87" t="s">
+        <v>30</v>
+      </c>
+      <c r="C87">
+        <v>2</v>
+      </c>
+      <c r="D87" t="b">
+        <v>0</v>
+      </c>
+      <c r="E87" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="88" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A88" t="s">
+        <v>29</v>
+      </c>
+      <c r="B88" t="s">
+        <v>30</v>
+      </c>
+      <c r="C88">
+        <v>3</v>
+      </c>
+      <c r="D88" t="b">
+        <v>0</v>
+      </c>
+      <c r="E88" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="89" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A89" t="s">
+        <v>36</v>
+      </c>
+      <c r="B89" t="s">
+        <v>37</v>
+      </c>
+      <c r="C89">
+        <v>1</v>
+      </c>
+      <c r="D89" t="b">
+        <v>0</v>
+      </c>
+      <c r="E89" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="90" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A90" t="s">
+        <v>36</v>
+      </c>
+      <c r="B90" t="s">
+        <v>37</v>
+      </c>
+      <c r="C90">
+        <v>2</v>
+      </c>
+      <c r="D90" t="b">
+        <v>0</v>
+      </c>
+      <c r="E90" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="91" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A91" t="s">
+        <v>36</v>
+      </c>
+      <c r="B91" t="s">
+        <v>37</v>
+      </c>
+      <c r="C91">
+        <v>3</v>
+      </c>
+      <c r="D91" t="b">
+        <v>0</v>
+      </c>
+      <c r="E91" t="s">
         <v>69</v>
       </c>
     </row>

</xml_diff>

<commit_message>
added even more servants for testing
</commit_message>
<xml_diff>
--- a/data/Fate-Spreadsheet.xlsx
+++ b/data/Fate-Spreadsheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pixel\Documents\Projects\Fate-Wiki\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33239780-26C1-4CA1-BB72-800FD4D65CD5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81AC9E10-788D-4926-843F-BC146EAE4A45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{B05E798F-9EF6-4508-A0A4-311D06661AED}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="590" uniqueCount="265">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="722" uniqueCount="323">
   <si>
     <t>servant_id</t>
   </si>
@@ -838,6 +838,180 @@
   </si>
   <si>
     <t>Wise Fox</t>
+  </si>
+  <si>
+    <t>S0024</t>
+  </si>
+  <si>
+    <t>Cú Chulainn</t>
+  </si>
+  <si>
+    <t>cu-chulainn</t>
+  </si>
+  <si>
+    <t>Lancer</t>
+  </si>
+  <si>
+    <t>2,4,4,4,5</t>
+  </si>
+  <si>
+    <t>2,4,5</t>
+  </si>
+  <si>
+    <t>Surveil,Surveil</t>
+  </si>
+  <si>
+    <t>S0048</t>
+  </si>
+  <si>
+    <t>Gilgamesh</t>
+  </si>
+  <si>
+    <t>gilgamesh</t>
+  </si>
+  <si>
+    <t>Preparation,Luck,Luck</t>
+  </si>
+  <si>
+    <t>S0070</t>
+  </si>
+  <si>
+    <t>Medusa</t>
+  </si>
+  <si>
+    <t>medusa</t>
+  </si>
+  <si>
+    <t>Rider</t>
+  </si>
+  <si>
+    <t>2,3,5</t>
+  </si>
+  <si>
+    <t>3,3</t>
+  </si>
+  <si>
+    <t>S0093</t>
+  </si>
+  <si>
+    <t>medea</t>
+  </si>
+  <si>
+    <t>Surveil,Luck,Preparation</t>
+  </si>
+  <si>
+    <t>S0101</t>
+  </si>
+  <si>
+    <t>Illyasviel von Einzbern</t>
+  </si>
+  <si>
+    <t>illyasviel-von-einzbern</t>
+  </si>
+  <si>
+    <t>2,2,3,3</t>
+  </si>
+  <si>
+    <t>Saber Install</t>
+  </si>
+  <si>
+    <t>Berserker Install</t>
+  </si>
+  <si>
+    <t>Archer Install</t>
+  </si>
+  <si>
+    <t>Assassin Install</t>
+  </si>
+  <si>
+    <t>Lancer Install</t>
+  </si>
+  <si>
+    <t>Caster Install</t>
+  </si>
+  <si>
+    <t>Rider Install</t>
+  </si>
+  <si>
+    <t>Saber-Install</t>
+  </si>
+  <si>
+    <t>Berserker-Install</t>
+  </si>
+  <si>
+    <t>Archer-Install</t>
+  </si>
+  <si>
+    <t>Assassin-Install</t>
+  </si>
+  <si>
+    <t>Lancer-Install</t>
+  </si>
+  <si>
+    <t>Caster-Install</t>
+  </si>
+  <si>
+    <t>Rider-Install</t>
+  </si>
+  <si>
+    <t>Lancer Class</t>
+  </si>
+  <si>
+    <t>Gae Bolg</t>
+  </si>
+  <si>
+    <t>Enuma Elish</t>
+  </si>
+  <si>
+    <t>Gate of Babylon</t>
+  </si>
+  <si>
+    <t>Rider Class</t>
+  </si>
+  <si>
+    <t>Bellerophon</t>
+  </si>
+  <si>
+    <t>Petrification</t>
+  </si>
+  <si>
+    <t>Rain of Light</t>
+  </si>
+  <si>
+    <t>Rule Breaker</t>
+  </si>
+  <si>
+    <t>Quintett Feuer</t>
+  </si>
+  <si>
+    <t>Schneiden</t>
+  </si>
+  <si>
+    <t>Card Holster</t>
+  </si>
+  <si>
+    <t>S0121</t>
+  </si>
+  <si>
+    <t>Semiramis of Assyria</t>
+  </si>
+  <si>
+    <t>semiramis</t>
+  </si>
+  <si>
+    <t>Assassin</t>
+  </si>
+  <si>
+    <t>2,3,4,4,5</t>
+  </si>
+  <si>
+    <t>Preparation,Preparation,Luck</t>
+  </si>
+  <si>
+    <t>Assassin Class</t>
+  </si>
+  <si>
+    <t>Sikera Usum</t>
   </si>
 </sst>
 </file>
@@ -887,12 +1061,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1227,7 +1400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E33D7ECC-1EAA-4A40-B4DA-A93E54CBC8B5}">
-  <dimension ref="A1:K31"/>
+  <dimension ref="A1:K37"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="17.1328125" customWidth="1"/>
@@ -1997,80 +2170,92 @@
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
-        <v>86</v>
+        <v>265</v>
       </c>
       <c r="B25" t="s">
-        <v>87</v>
+        <v>266</v>
       </c>
       <c r="C25" t="s">
-        <v>88</v>
+        <v>267</v>
       </c>
       <c r="D25" t="s">
-        <v>89</v>
+        <v>268</v>
       </c>
       <c r="E25" t="s">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="G25" s="2" t="s">
         <v>15</v>
       </c>
       <c r="H25" s="2" t="s">
-        <v>91</v>
+        <v>269</v>
       </c>
       <c r="I25" s="2" t="s">
-        <v>42</v>
+        <v>270</v>
+      </c>
+      <c r="J25" s="2" t="s">
+        <v>271</v>
       </c>
       <c r="K25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
-        <v>17</v>
+        <v>272</v>
       </c>
       <c r="B26" t="s">
-        <v>18</v>
+        <v>273</v>
       </c>
       <c r="C26" t="s">
-        <v>19</v>
+        <v>274</v>
       </c>
       <c r="D26" t="s">
-        <v>20</v>
+        <v>89</v>
       </c>
       <c r="E26" t="s">
         <v>8</v>
       </c>
+      <c r="G26" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H26" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="I26" s="2" t="s">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="J26" s="2" t="s">
-        <v>22</v>
+        <v>275</v>
       </c>
       <c r="K26" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
-        <v>97</v>
+        <v>86</v>
       </c>
       <c r="B27" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="C27" t="s">
-        <v>99</v>
+        <v>88</v>
       </c>
       <c r="D27" t="s">
-        <v>20</v>
+        <v>89</v>
       </c>
       <c r="E27" t="s">
-        <v>100</v>
+        <v>90</v>
+      </c>
+      <c r="G27" s="2" t="s">
+        <v>15</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>101</v>
+        <v>91</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>102</v>
+        <v>42</v>
       </c>
       <c r="K27" t="b">
         <v>1</v>
@@ -2078,31 +2263,31 @@
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
-        <v>76</v>
+        <v>276</v>
       </c>
       <c r="B28" t="s">
-        <v>77</v>
+        <v>277</v>
       </c>
       <c r="C28" t="s">
-        <v>78</v>
+        <v>278</v>
       </c>
       <c r="D28" t="s">
-        <v>79</v>
+        <v>279</v>
       </c>
       <c r="E28" t="s">
-        <v>40</v>
+        <v>8</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>80</v>
+        <v>280</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>15</v>
+        <v>205</v>
       </c>
       <c r="I28" s="2" t="s">
-        <v>82</v>
+        <v>281</v>
       </c>
       <c r="J28" s="2" t="s">
-        <v>81</v>
+        <v>43</v>
       </c>
       <c r="K28" t="b">
         <v>0</v>
@@ -2110,28 +2295,28 @@
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
-        <v>23</v>
+        <v>282</v>
       </c>
       <c r="B29" t="s">
-        <v>24</v>
+        <v>250</v>
       </c>
       <c r="C29" t="s">
-        <v>25</v>
+        <v>283</v>
       </c>
       <c r="D29" t="s">
-        <v>26</v>
+        <v>20</v>
       </c>
       <c r="E29" t="s">
-        <v>8</v>
-      </c>
-      <c r="G29" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="H29" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="H29" s="2" t="s">
-        <v>28</v>
+      <c r="I29" s="2" t="s">
+        <v>102</v>
       </c>
       <c r="J29" s="2" t="s">
-        <v>70</v>
+        <v>284</v>
       </c>
       <c r="K29" t="b">
         <v>0</v>
@@ -2139,62 +2324,230 @@
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="B30" t="s">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="C30" t="s">
-        <v>31</v>
+        <v>19</v>
       </c>
       <c r="D30" t="s">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="E30" t="s">
-        <v>33</v>
-      </c>
-      <c r="G30" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="H30" s="2" t="s">
-        <v>82</v>
+        <v>8</v>
       </c>
       <c r="I30" s="2" t="s">
-        <v>34</v>
+        <v>21</v>
       </c>
       <c r="J30" s="2" t="s">
-        <v>35</v>
+        <v>22</v>
       </c>
       <c r="K30" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A31" t="s">
+        <v>285</v>
+      </c>
+      <c r="B31" t="s">
+        <v>286</v>
+      </c>
+      <c r="C31" t="s">
+        <v>287</v>
+      </c>
+      <c r="D31" t="s">
+        <v>20</v>
+      </c>
+      <c r="E31" t="s">
+        <v>8</v>
+      </c>
+      <c r="I31" s="2" t="s">
+        <v>288</v>
+      </c>
+      <c r="J31" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="K31" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A32" t="s">
+        <v>97</v>
+      </c>
+      <c r="B32" t="s">
+        <v>98</v>
+      </c>
+      <c r="C32" t="s">
+        <v>99</v>
+      </c>
+      <c r="D32" t="s">
+        <v>20</v>
+      </c>
+      <c r="E32" t="s">
+        <v>100</v>
+      </c>
+      <c r="H32" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="I32" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="K32" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A33" t="s">
+        <v>315</v>
+      </c>
+      <c r="B33" t="s">
+        <v>316</v>
+      </c>
+      <c r="C33" t="s">
+        <v>317</v>
+      </c>
+      <c r="D33" t="s">
+        <v>318</v>
+      </c>
+      <c r="E33" t="s">
+        <v>33</v>
+      </c>
+      <c r="H33" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="I33" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="J33" s="2" t="s">
+        <v>320</v>
+      </c>
+      <c r="K33" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A34" t="s">
+        <v>76</v>
+      </c>
+      <c r="B34" t="s">
+        <v>77</v>
+      </c>
+      <c r="C34" t="s">
+        <v>78</v>
+      </c>
+      <c r="D34" t="s">
+        <v>79</v>
+      </c>
+      <c r="E34" t="s">
+        <v>40</v>
+      </c>
+      <c r="G34" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="H34" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I34" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="J34" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="K34" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A35" t="s">
+        <v>23</v>
+      </c>
+      <c r="B35" t="s">
+        <v>24</v>
+      </c>
+      <c r="C35" t="s">
+        <v>25</v>
+      </c>
+      <c r="D35" t="s">
+        <v>26</v>
+      </c>
+      <c r="E35" t="s">
+        <v>8</v>
+      </c>
+      <c r="G35" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H35" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="J35" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="K35" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A36" t="s">
+        <v>29</v>
+      </c>
+      <c r="B36" t="s">
+        <v>30</v>
+      </c>
+      <c r="C36" t="s">
+        <v>31</v>
+      </c>
+      <c r="D36" t="s">
+        <v>32</v>
+      </c>
+      <c r="E36" t="s">
+        <v>33</v>
+      </c>
+      <c r="G36" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H36" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="I36" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="J36" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="K36" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="A37" t="s">
         <v>36</v>
       </c>
-      <c r="B31" t="s">
+      <c r="B37" t="s">
         <v>37</v>
       </c>
-      <c r="C31" t="s">
+      <c r="C37" t="s">
         <v>38</v>
       </c>
-      <c r="D31" t="s">
+      <c r="D37" t="s">
         <v>39</v>
       </c>
-      <c r="E31" t="s">
+      <c r="E37" t="s">
         <v>40</v>
       </c>
-      <c r="G31" s="2" t="s">
+      <c r="G37" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="H31" s="2" t="s">
+      <c r="H37" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="J31" s="2" t="s">
+      <c r="J37" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="K31" t="b">
+      <c r="K37" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2202,14 +2555,14 @@
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="H2 I28 H30 I6:I7 I10 I12 H14 I18 I22 I24" numberStoredAsText="1"/>
+    <ignoredError sqref="H2 I34 H36 I6:I7 I10 I12 H14 I18 I22 I24" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1BC60D8-44F3-478D-BCC0-4752624457AE}">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="19" customWidth="1"/>
@@ -2238,54 +2591,54 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="4" t="s">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
         <v>117</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" t="s">
         <v>140</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" t="s">
         <v>208</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" t="s">
         <v>209</v>
       </c>
-      <c r="E2" s="4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A3" s="4" t="s">
+      <c r="E2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
         <v>127</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" t="s">
         <v>149</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" t="s">
         <v>210</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" t="s">
         <v>211</v>
       </c>
-      <c r="E3" s="4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" s="4" customFormat="1" x14ac:dyDescent="0.45">
-      <c r="A4" s="4" t="s">
+      <c r="E3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
         <v>131</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B4" t="s">
         <v>153</v>
       </c>
-      <c r="C4" s="4" t="s">
+      <c r="C4" t="s">
         <v>212</v>
       </c>
-      <c r="D4" s="4" t="s">
+      <c r="D4" t="s">
         <v>212</v>
       </c>
-      <c r="E4" s="4">
+      <c r="E4">
         <v>1</v>
       </c>
     </row>
@@ -2342,16 +2695,16 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>97</v>
+        <v>285</v>
       </c>
       <c r="B8" t="s">
-        <v>98</v>
+        <v>286</v>
       </c>
       <c r="C8" t="s">
-        <v>103</v>
+        <v>289</v>
       </c>
       <c r="D8" t="s">
-        <v>106</v>
+        <v>296</v>
       </c>
       <c r="E8">
         <v>1</v>
@@ -2359,16 +2712,16 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>97</v>
+        <v>285</v>
       </c>
       <c r="B9" t="s">
-        <v>98</v>
+        <v>286</v>
       </c>
       <c r="C9" t="s">
-        <v>104</v>
+        <v>290</v>
       </c>
       <c r="D9" t="s">
-        <v>107</v>
+        <v>297</v>
       </c>
       <c r="E9">
         <v>1</v>
@@ -2376,16 +2729,16 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
-        <v>97</v>
+        <v>285</v>
       </c>
       <c r="B10" t="s">
-        <v>98</v>
+        <v>286</v>
       </c>
       <c r="C10" t="s">
-        <v>105</v>
+        <v>291</v>
       </c>
       <c r="D10" t="s">
-        <v>108</v>
+        <v>298</v>
       </c>
       <c r="E10">
         <v>1</v>
@@ -2393,18 +2746,137 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
+        <v>285</v>
+      </c>
+      <c r="B11" t="s">
+        <v>286</v>
+      </c>
+      <c r="C11" t="s">
+        <v>292</v>
+      </c>
+      <c r="D11" t="s">
+        <v>299</v>
+      </c>
+      <c r="E11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A12" t="s">
+        <v>285</v>
+      </c>
+      <c r="B12" t="s">
+        <v>286</v>
+      </c>
+      <c r="C12" t="s">
+        <v>293</v>
+      </c>
+      <c r="D12" t="s">
+        <v>300</v>
+      </c>
+      <c r="E12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A13" t="s">
+        <v>285</v>
+      </c>
+      <c r="B13" t="s">
+        <v>286</v>
+      </c>
+      <c r="C13" t="s">
+        <v>294</v>
+      </c>
+      <c r="D13" t="s">
+        <v>301</v>
+      </c>
+      <c r="E13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A14" t="s">
+        <v>285</v>
+      </c>
+      <c r="B14" t="s">
+        <v>286</v>
+      </c>
+      <c r="C14" t="s">
+        <v>295</v>
+      </c>
+      <c r="D14" t="s">
+        <v>302</v>
+      </c>
+      <c r="E14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A15" t="s">
+        <v>97</v>
+      </c>
+      <c r="B15" t="s">
+        <v>98</v>
+      </c>
+      <c r="C15" t="s">
+        <v>103</v>
+      </c>
+      <c r="D15" t="s">
+        <v>106</v>
+      </c>
+      <c r="E15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.45">
+      <c r="A16" t="s">
+        <v>97</v>
+      </c>
+      <c r="B16" t="s">
+        <v>98</v>
+      </c>
+      <c r="C16" t="s">
+        <v>104</v>
+      </c>
+      <c r="D16" t="s">
+        <v>107</v>
+      </c>
+      <c r="E16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A17" t="s">
+        <v>97</v>
+      </c>
+      <c r="B17" t="s">
+        <v>98</v>
+      </c>
+      <c r="C17" t="s">
+        <v>105</v>
+      </c>
+      <c r="D17" t="s">
+        <v>108</v>
+      </c>
+      <c r="E17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A18" t="s">
         <v>36</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B18" t="s">
         <v>37</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C18" t="s">
         <v>48</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D18" t="s">
         <v>48</v>
       </c>
-      <c r="E11">
+      <c r="E18">
         <v>2</v>
       </c>
     </row>
@@ -2417,7 +2889,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84E3BB0D-5578-4069-B1C9-C3864EB2A429}">
-  <dimension ref="A1:F91"/>
+  <dimension ref="A1:F109"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="20.59765625" customWidth="1"/>
@@ -3622,10 +4094,10 @@
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A71" t="s">
-        <v>86</v>
+        <v>265</v>
       </c>
       <c r="B71" t="s">
-        <v>87</v>
+        <v>266</v>
       </c>
       <c r="C71">
         <v>1</v>
@@ -3634,15 +4106,15 @@
         <v>1</v>
       </c>
       <c r="E71" t="s">
-        <v>94</v>
+        <v>303</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A72" t="s">
-        <v>86</v>
+        <v>265</v>
       </c>
       <c r="B72" t="s">
-        <v>87</v>
+        <v>266</v>
       </c>
       <c r="C72">
         <v>2</v>
@@ -3651,15 +4123,15 @@
         <v>0</v>
       </c>
       <c r="E72" t="s">
-        <v>95</v>
+        <v>304</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A73" t="s">
-        <v>86</v>
+        <v>265</v>
       </c>
       <c r="B73" t="s">
-        <v>87</v>
+        <v>266</v>
       </c>
       <c r="C73">
         <v>3</v>
@@ -3668,15 +4140,15 @@
         <v>0</v>
       </c>
       <c r="E73" t="s">
-        <v>96</v>
+        <v>304</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A74" t="s">
-        <v>17</v>
+        <v>272</v>
       </c>
       <c r="B74" t="s">
-        <v>18</v>
+        <v>273</v>
       </c>
       <c r="C74">
         <v>1</v>
@@ -3685,15 +4157,15 @@
         <v>1</v>
       </c>
       <c r="E74" t="s">
-        <v>58</v>
+        <v>94</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A75" t="s">
-        <v>17</v>
+        <v>272</v>
       </c>
       <c r="B75" t="s">
-        <v>18</v>
+        <v>273</v>
       </c>
       <c r="C75">
         <v>2</v>
@@ -3702,15 +4174,15 @@
         <v>0</v>
       </c>
       <c r="E75" t="s">
-        <v>59</v>
+        <v>305</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A76" t="s">
-        <v>17</v>
+        <v>272</v>
       </c>
       <c r="B76" t="s">
-        <v>18</v>
+        <v>273</v>
       </c>
       <c r="C76">
         <v>3</v>
@@ -3719,32 +4191,32 @@
         <v>0</v>
       </c>
       <c r="E76" t="s">
-        <v>60</v>
+        <v>306</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A77" t="s">
-        <v>97</v>
+        <v>86</v>
       </c>
       <c r="B77" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="C77">
         <v>1</v>
       </c>
       <c r="D77" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E77" t="s">
-        <v>109</v>
+        <v>94</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A78" t="s">
-        <v>97</v>
+        <v>86</v>
       </c>
       <c r="B78" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="C78">
         <v>2</v>
@@ -3753,15 +4225,15 @@
         <v>0</v>
       </c>
       <c r="E78" t="s">
-        <v>110</v>
+        <v>95</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A79" t="s">
-        <v>97</v>
+        <v>86</v>
       </c>
       <c r="B79" t="s">
-        <v>98</v>
+        <v>87</v>
       </c>
       <c r="C79">
         <v>3</v>
@@ -3770,15 +4242,15 @@
         <v>0</v>
       </c>
       <c r="E79" t="s">
-        <v>111</v>
+        <v>96</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A80" t="s">
-        <v>76</v>
+        <v>276</v>
       </c>
       <c r="B80" t="s">
-        <v>77</v>
+        <v>277</v>
       </c>
       <c r="C80">
         <v>1</v>
@@ -3787,15 +4259,15 @@
         <v>1</v>
       </c>
       <c r="E80" t="s">
-        <v>83</v>
+        <v>307</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A81" t="s">
-        <v>76</v>
+        <v>276</v>
       </c>
       <c r="B81" t="s">
-        <v>77</v>
+        <v>277</v>
       </c>
       <c r="C81">
         <v>2</v>
@@ -3804,15 +4276,15 @@
         <v>0</v>
       </c>
       <c r="E81" t="s">
-        <v>84</v>
+        <v>308</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A82" t="s">
-        <v>76</v>
+        <v>276</v>
       </c>
       <c r="B82" t="s">
-        <v>77</v>
+        <v>277</v>
       </c>
       <c r="C82">
         <v>3</v>
@@ -3821,32 +4293,32 @@
         <v>0</v>
       </c>
       <c r="E82" t="s">
-        <v>85</v>
+        <v>309</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A83" t="s">
-        <v>23</v>
+        <v>282</v>
       </c>
       <c r="B83" t="s">
-        <v>24</v>
+        <v>250</v>
       </c>
       <c r="C83">
         <v>1</v>
       </c>
       <c r="D83" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E83" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A84" t="s">
-        <v>23</v>
+        <v>282</v>
       </c>
       <c r="B84" t="s">
-        <v>24</v>
+        <v>250</v>
       </c>
       <c r="C84">
         <v>2</v>
@@ -3855,15 +4327,15 @@
         <v>0</v>
       </c>
       <c r="E84" t="s">
-        <v>62</v>
+        <v>310</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A85" t="s">
-        <v>23</v>
+        <v>282</v>
       </c>
       <c r="B85" t="s">
-        <v>24</v>
+        <v>250</v>
       </c>
       <c r="C85">
         <v>3</v>
@@ -3872,32 +4344,32 @@
         <v>0</v>
       </c>
       <c r="E85" t="s">
-        <v>63</v>
+        <v>311</v>
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A86" t="s">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="B86" t="s">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="C86">
         <v>1</v>
       </c>
       <c r="D86" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E86" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A87" t="s">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="B87" t="s">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="C87">
         <v>2</v>
@@ -3906,15 +4378,15 @@
         <v>0</v>
       </c>
       <c r="E87" t="s">
-        <v>65</v>
+        <v>59</v>
       </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A88" t="s">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="B88" t="s">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="C88">
         <v>3</v>
@@ -3923,15 +4395,15 @@
         <v>0</v>
       </c>
       <c r="E88" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A89" t="s">
-        <v>36</v>
+        <v>285</v>
       </c>
       <c r="B89" t="s">
-        <v>37</v>
+        <v>286</v>
       </c>
       <c r="C89">
         <v>1</v>
@@ -3940,15 +4412,15 @@
         <v>0</v>
       </c>
       <c r="E89" t="s">
-        <v>67</v>
+        <v>312</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A90" t="s">
-        <v>36</v>
+        <v>285</v>
       </c>
       <c r="B90" t="s">
-        <v>37</v>
+        <v>286</v>
       </c>
       <c r="C90">
         <v>2</v>
@@ -3957,15 +4429,15 @@
         <v>0</v>
       </c>
       <c r="E90" t="s">
-        <v>68</v>
+        <v>313</v>
       </c>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A91" t="s">
-        <v>36</v>
+        <v>285</v>
       </c>
       <c r="B91" t="s">
-        <v>37</v>
+        <v>286</v>
       </c>
       <c r="C91">
         <v>3</v>
@@ -3974,6 +4446,312 @@
         <v>0</v>
       </c>
       <c r="E91" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A92" t="s">
+        <v>97</v>
+      </c>
+      <c r="B92" t="s">
+        <v>98</v>
+      </c>
+      <c r="C92">
+        <v>1</v>
+      </c>
+      <c r="D92" t="b">
+        <v>0</v>
+      </c>
+      <c r="E92" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A93" t="s">
+        <v>97</v>
+      </c>
+      <c r="B93" t="s">
+        <v>98</v>
+      </c>
+      <c r="C93">
+        <v>2</v>
+      </c>
+      <c r="D93" t="b">
+        <v>0</v>
+      </c>
+      <c r="E93" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A94" t="s">
+        <v>97</v>
+      </c>
+      <c r="B94" t="s">
+        <v>98</v>
+      </c>
+      <c r="C94">
+        <v>3</v>
+      </c>
+      <c r="D94" t="b">
+        <v>0</v>
+      </c>
+      <c r="E94" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A95" t="s">
+        <v>315</v>
+      </c>
+      <c r="B95" t="s">
+        <v>316</v>
+      </c>
+      <c r="C95">
+        <v>1</v>
+      </c>
+      <c r="D95" t="b">
+        <v>1</v>
+      </c>
+      <c r="E95" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="96" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A96" t="s">
+        <v>315</v>
+      </c>
+      <c r="B96" t="s">
+        <v>316</v>
+      </c>
+      <c r="C96">
+        <v>2</v>
+      </c>
+      <c r="D96" t="b">
+        <v>1</v>
+      </c>
+      <c r="E96" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="97" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A97" t="s">
+        <v>315</v>
+      </c>
+      <c r="B97" t="s">
+        <v>316</v>
+      </c>
+      <c r="C97">
+        <v>3</v>
+      </c>
+      <c r="D97" t="b">
+        <v>0</v>
+      </c>
+      <c r="E97" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="98" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A98" t="s">
+        <v>76</v>
+      </c>
+      <c r="B98" t="s">
+        <v>77</v>
+      </c>
+      <c r="C98">
+        <v>1</v>
+      </c>
+      <c r="D98" t="b">
+        <v>1</v>
+      </c>
+      <c r="E98" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="99" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A99" t="s">
+        <v>76</v>
+      </c>
+      <c r="B99" t="s">
+        <v>77</v>
+      </c>
+      <c r="C99">
+        <v>2</v>
+      </c>
+      <c r="D99" t="b">
+        <v>0</v>
+      </c>
+      <c r="E99" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="100" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A100" t="s">
+        <v>76</v>
+      </c>
+      <c r="B100" t="s">
+        <v>77</v>
+      </c>
+      <c r="C100">
+        <v>3</v>
+      </c>
+      <c r="D100" t="b">
+        <v>0</v>
+      </c>
+      <c r="E100" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="101" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A101" t="s">
+        <v>23</v>
+      </c>
+      <c r="B101" t="s">
+        <v>24</v>
+      </c>
+      <c r="C101">
+        <v>1</v>
+      </c>
+      <c r="D101" t="b">
+        <v>0</v>
+      </c>
+      <c r="E101" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="102" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A102" t="s">
+        <v>23</v>
+      </c>
+      <c r="B102" t="s">
+        <v>24</v>
+      </c>
+      <c r="C102">
+        <v>2</v>
+      </c>
+      <c r="D102" t="b">
+        <v>0</v>
+      </c>
+      <c r="E102" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="103" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A103" t="s">
+        <v>23</v>
+      </c>
+      <c r="B103" t="s">
+        <v>24</v>
+      </c>
+      <c r="C103">
+        <v>3</v>
+      </c>
+      <c r="D103" t="b">
+        <v>0</v>
+      </c>
+      <c r="E103" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="104" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A104" t="s">
+        <v>29</v>
+      </c>
+      <c r="B104" t="s">
+        <v>30</v>
+      </c>
+      <c r="C104">
+        <v>1</v>
+      </c>
+      <c r="D104" t="b">
+        <v>0</v>
+      </c>
+      <c r="E104" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="105" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A105" t="s">
+        <v>29</v>
+      </c>
+      <c r="B105" t="s">
+        <v>30</v>
+      </c>
+      <c r="C105">
+        <v>2</v>
+      </c>
+      <c r="D105" t="b">
+        <v>0</v>
+      </c>
+      <c r="E105" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="106" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A106" t="s">
+        <v>29</v>
+      </c>
+      <c r="B106" t="s">
+        <v>30</v>
+      </c>
+      <c r="C106">
+        <v>3</v>
+      </c>
+      <c r="D106" t="b">
+        <v>0</v>
+      </c>
+      <c r="E106" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="107" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A107" t="s">
+        <v>36</v>
+      </c>
+      <c r="B107" t="s">
+        <v>37</v>
+      </c>
+      <c r="C107">
+        <v>1</v>
+      </c>
+      <c r="D107" t="b">
+        <v>0</v>
+      </c>
+      <c r="E107" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="108" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A108" t="s">
+        <v>36</v>
+      </c>
+      <c r="B108" t="s">
+        <v>37</v>
+      </c>
+      <c r="C108">
+        <v>2</v>
+      </c>
+      <c r="D108" t="b">
+        <v>0</v>
+      </c>
+      <c r="E108" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="109" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A109" t="s">
+        <v>36</v>
+      </c>
+      <c r="B109" t="s">
+        <v>37</v>
+      </c>
+      <c r="C109">
+        <v>3</v>
+      </c>
+      <c r="D109" t="b">
+        <v>0</v>
+      </c>
+      <c r="E109" t="s">
         <v>69</v>
       </c>
     </row>

</xml_diff>

<commit_message>
spreadsheet update: changed berserker class cards to have underscores, for ease of finding
</commit_message>
<xml_diff>
--- a/data/Fate-Spreadsheet.xlsx
+++ b/data/Fate-Spreadsheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pixel\Documents\Projects\Fate-Wiki\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81AC9E10-788D-4926-843F-BC146EAE4A45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F766361-2887-4A36-9C5B-EE2D635FDC7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{B05E798F-9EF6-4508-A0A4-311D06661AED}"/>
   </bookViews>
@@ -288,9 +288,6 @@
     <t>2,4,5,5</t>
   </si>
   <si>
-    <t>Berserker Strength 7,Berserker Strength 9,Luck,Luck,Surveil</t>
-  </si>
-  <si>
     <t>3</t>
   </si>
   <si>
@@ -1012,6 +1009,9 @@
   </si>
   <si>
     <t>Sikera Usum</t>
+  </si>
+  <si>
+    <t>Berserker_Strength_7,Berserker_Strength_9,Luck,Luck,Surveil</t>
   </si>
 </sst>
 </file>
@@ -1470,7 +1470,7 @@
         <v>14</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="I2" s="2" t="s">
         <v>15</v>
@@ -1484,31 +1484,31 @@
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B3" t="s">
+        <v>133</v>
+      </c>
+      <c r="C3" t="s">
         <v>134</v>
-      </c>
-      <c r="C3" t="s">
-        <v>135</v>
       </c>
       <c r="D3" t="s">
         <v>7</v>
       </c>
       <c r="E3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G3" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="H3" s="2" t="s">
         <v>176</v>
-      </c>
-      <c r="H3" s="2" t="s">
-        <v>177</v>
       </c>
       <c r="I3" s="2" t="s">
         <v>15</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="K3" t="b">
         <v>0</v>
@@ -1516,13 +1516,13 @@
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B4" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C4" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="D4" t="s">
         <v>7</v>
@@ -1531,13 +1531,13 @@
         <v>8</v>
       </c>
       <c r="G4" s="2" t="s">
+        <v>178</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="J4" s="2" t="s">
         <v>179</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="J4" s="2" t="s">
-        <v>180</v>
       </c>
       <c r="K4" t="b">
         <v>0</v>
@@ -1545,13 +1545,13 @@
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B5" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C5" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="D5" t="s">
         <v>7</v>
@@ -1560,13 +1560,13 @@
         <v>8</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="H5" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="J5" s="2" t="s">
         <v>181</v>
-      </c>
-      <c r="J5" s="2" t="s">
-        <v>182</v>
       </c>
       <c r="K5" t="b">
         <v>0</v>
@@ -1574,13 +1574,13 @@
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C6" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="D6" t="s">
         <v>7</v>
@@ -1589,16 +1589,16 @@
         <v>8</v>
       </c>
       <c r="G6" s="2" t="s">
+        <v>182</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="I6" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="J6" s="2" t="s">
         <v>183</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>177</v>
-      </c>
-      <c r="I6" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="J6" s="2" t="s">
-        <v>184</v>
       </c>
       <c r="K6" t="b">
         <v>0</v>
@@ -1606,13 +1606,13 @@
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B7" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C7" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="D7" t="s">
         <v>7</v>
@@ -1621,16 +1621,16 @@
         <v>8</v>
       </c>
       <c r="G7" s="2" t="s">
+        <v>184</v>
+      </c>
+      <c r="H7" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="H7" s="2" t="s">
+      <c r="I7" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="J7" s="2" t="s">
         <v>186</v>
-      </c>
-      <c r="I7" s="2" t="s">
-        <v>82</v>
-      </c>
-      <c r="J7" s="2" t="s">
-        <v>187</v>
       </c>
       <c r="K7" t="b">
         <v>0</v>
@@ -1638,28 +1638,28 @@
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B8" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C8" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D8" t="s">
         <v>7</v>
       </c>
       <c r="E8" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G8" s="2" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="H8" s="2" t="s">
+        <v>187</v>
+      </c>
+      <c r="J8" s="2" t="s">
         <v>188</v>
-      </c>
-      <c r="J8" s="2" t="s">
-        <v>189</v>
       </c>
       <c r="K8" t="b">
         <v>1</v>
@@ -1667,28 +1667,28 @@
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B9" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C9" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="D9" t="s">
         <v>7</v>
       </c>
       <c r="E9" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G9" s="2" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="K9" t="b">
         <v>0</v>
@@ -1696,13 +1696,13 @@
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B10" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C10" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D10" t="s">
         <v>7</v>
@@ -1711,16 +1711,16 @@
         <v>8</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="H10" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="I10" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="I10" s="2" t="s">
-        <v>192</v>
-      </c>
       <c r="J10" s="2" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="K10" t="b">
         <v>0</v>
@@ -1728,31 +1728,31 @@
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B11" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C11" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D11" t="s">
         <v>7</v>
       </c>
       <c r="E11" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G11" s="2" t="s">
         <v>27</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="K11" t="b">
         <v>0</v>
@@ -1760,31 +1760,31 @@
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B12" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C12" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D12" t="s">
         <v>79</v>
       </c>
       <c r="E12" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G12" s="2" t="s">
         <v>80</v>
       </c>
       <c r="H12" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="I12" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="J12" s="2" t="s">
         <v>194</v>
-      </c>
-      <c r="I12" s="2" t="s">
-        <v>192</v>
-      </c>
-      <c r="J12" s="2" t="s">
-        <v>195</v>
       </c>
       <c r="K12" t="b">
         <v>0</v>
@@ -1792,28 +1792,28 @@
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B13" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C13" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D13" t="s">
         <v>7</v>
       </c>
       <c r="E13" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="K13" t="b">
         <v>0</v>
@@ -1821,13 +1821,13 @@
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B14" t="s">
         <v>5</v>
       </c>
       <c r="C14" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D14" t="s">
         <v>7</v>
@@ -1836,16 +1836,16 @@
         <v>8</v>
       </c>
       <c r="G14" s="2" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="K14" t="b">
         <v>0</v>
@@ -1853,31 +1853,31 @@
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B15" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C15" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="D15" t="s">
         <v>7</v>
       </c>
       <c r="E15" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G15" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="H15" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="H15" s="2" t="s">
+      <c r="I15" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="J15" s="2" t="s">
         <v>197</v>
-      </c>
-      <c r="I15" s="2" t="s">
-        <v>101</v>
-      </c>
-      <c r="J15" s="2" t="s">
-        <v>198</v>
       </c>
       <c r="K15" t="b">
         <v>0</v>
@@ -1885,13 +1885,13 @@
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B16" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C16" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D16" t="s">
         <v>7</v>
@@ -1900,16 +1900,16 @@
         <v>8</v>
       </c>
       <c r="G16" s="2" t="s">
+        <v>198</v>
+      </c>
+      <c r="H16" s="2" t="s">
         <v>199</v>
-      </c>
-      <c r="H16" s="2" t="s">
-        <v>200</v>
       </c>
       <c r="I16" s="2" t="s">
         <v>27</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="K16" t="b">
         <v>0</v>
@@ -1917,13 +1917,13 @@
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B17" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C17" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D17" t="s">
         <v>7</v>
@@ -1932,16 +1932,16 @@
         <v>8</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="H17" s="2" t="s">
         <v>15</v>
       </c>
       <c r="I17" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="K17" t="b">
         <v>0</v>
@@ -1949,31 +1949,31 @@
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B18" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C18" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="D18" t="s">
         <v>7</v>
       </c>
       <c r="E18" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G18" s="2" t="s">
         <v>42</v>
       </c>
       <c r="H18" s="2" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="I18" s="2" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="J18" s="2" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="K18" t="b">
         <v>1</v>
@@ -1981,22 +1981,22 @@
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B19" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C19" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D19" t="s">
         <v>7</v>
       </c>
       <c r="E19" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G19" s="2" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="H19" s="2" t="s">
         <v>27</v>
@@ -2005,7 +2005,7 @@
         <v>15</v>
       </c>
       <c r="J19" s="2" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="K19" t="b">
         <v>0</v>
@@ -2013,28 +2013,28 @@
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B20" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C20" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D20" t="s">
         <v>7</v>
       </c>
       <c r="E20" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="J20" s="2" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="K20" t="b">
         <v>0</v>
@@ -2042,31 +2042,31 @@
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B21" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C21" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D21" t="s">
         <v>7</v>
       </c>
       <c r="E21" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="H21" s="2" t="s">
         <v>27</v>
       </c>
       <c r="I21" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="J21" s="2" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="K21" t="b">
         <v>0</v>
@@ -2074,13 +2074,13 @@
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B22" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C22" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D22" t="s">
         <v>7</v>
@@ -2089,13 +2089,13 @@
         <v>40</v>
       </c>
       <c r="G22" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="H22" s="2" t="s">
+        <v>195</v>
+      </c>
+      <c r="I22" s="2" t="s">
         <v>191</v>
-      </c>
-      <c r="H22" s="2" t="s">
-        <v>196</v>
-      </c>
-      <c r="I22" s="2" t="s">
-        <v>192</v>
       </c>
       <c r="J22" s="2" t="s">
         <v>22</v>
@@ -2106,31 +2106,31 @@
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B23" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C23" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D23" t="s">
         <v>79</v>
       </c>
       <c r="E23" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="I23" s="2" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="J23" s="2" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="K23" t="b">
         <v>0</v>
@@ -2138,19 +2138,19 @@
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B24" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C24" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D24" t="s">
         <v>7</v>
       </c>
       <c r="E24" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="G24" s="2" t="s">
         <v>21</v>
@@ -2159,7 +2159,7 @@
         <v>41</v>
       </c>
       <c r="I24" s="2" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="J24" s="2" t="s">
         <v>43</v>
@@ -2170,31 +2170,31 @@
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
+        <v>264</v>
+      </c>
+      <c r="B25" t="s">
         <v>265</v>
       </c>
-      <c r="B25" t="s">
+      <c r="C25" t="s">
         <v>266</v>
       </c>
-      <c r="C25" t="s">
+      <c r="D25" t="s">
         <v>267</v>
       </c>
-      <c r="D25" t="s">
-        <v>268</v>
-      </c>
       <c r="E25" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="G25" s="2" t="s">
         <v>15</v>
       </c>
       <c r="H25" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="I25" s="2" t="s">
         <v>269</v>
       </c>
-      <c r="I25" s="2" t="s">
+      <c r="J25" s="2" t="s">
         <v>270</v>
-      </c>
-      <c r="J25" s="2" t="s">
-        <v>271</v>
       </c>
       <c r="K25" t="b">
         <v>0</v>
@@ -2202,16 +2202,16 @@
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
+        <v>271</v>
+      </c>
+      <c r="B26" t="s">
         <v>272</v>
       </c>
-      <c r="B26" t="s">
+      <c r="C26" t="s">
         <v>273</v>
       </c>
-      <c r="C26" t="s">
-        <v>274</v>
-      </c>
       <c r="D26" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E26" t="s">
         <v>8</v>
@@ -2226,7 +2226,7 @@
         <v>27</v>
       </c>
       <c r="J26" s="2" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="K26" t="b">
         <v>0</v>
@@ -2234,25 +2234,25 @@
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
+        <v>85</v>
+      </c>
+      <c r="B27" t="s">
         <v>86</v>
       </c>
-      <c r="B27" t="s">
+      <c r="C27" t="s">
         <v>87</v>
       </c>
-      <c r="C27" t="s">
+      <c r="D27" t="s">
         <v>88</v>
       </c>
-      <c r="D27" t="s">
+      <c r="E27" t="s">
         <v>89</v>
-      </c>
-      <c r="E27" t="s">
-        <v>90</v>
       </c>
       <c r="G27" s="2" t="s">
         <v>15</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="I27" s="2" t="s">
         <v>42</v>
@@ -2263,28 +2263,28 @@
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
+        <v>275</v>
+      </c>
+      <c r="B28" t="s">
         <v>276</v>
       </c>
-      <c r="B28" t="s">
+      <c r="C28" t="s">
         <v>277</v>
       </c>
-      <c r="C28" t="s">
+      <c r="D28" t="s">
         <v>278</v>
-      </c>
-      <c r="D28" t="s">
-        <v>279</v>
       </c>
       <c r="E28" t="s">
         <v>8</v>
       </c>
       <c r="G28" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="H28" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="I28" s="2" t="s">
         <v>280</v>
-      </c>
-      <c r="H28" s="2" t="s">
-        <v>205</v>
-      </c>
-      <c r="I28" s="2" t="s">
-        <v>281</v>
       </c>
       <c r="J28" s="2" t="s">
         <v>43</v>
@@ -2295,13 +2295,13 @@
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
+        <v>281</v>
+      </c>
+      <c r="B29" t="s">
+        <v>249</v>
+      </c>
+      <c r="C29" t="s">
         <v>282</v>
-      </c>
-      <c r="B29" t="s">
-        <v>250</v>
-      </c>
-      <c r="C29" t="s">
-        <v>283</v>
       </c>
       <c r="D29" t="s">
         <v>20</v>
@@ -2313,10 +2313,10 @@
         <v>27</v>
       </c>
       <c r="I29" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="J29" s="2" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="K29" t="b">
         <v>0</v>
@@ -2350,13 +2350,13 @@
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A31" t="s">
+        <v>284</v>
+      </c>
+      <c r="B31" t="s">
         <v>285</v>
       </c>
-      <c r="B31" t="s">
+      <c r="C31" t="s">
         <v>286</v>
-      </c>
-      <c r="C31" t="s">
-        <v>287</v>
       </c>
       <c r="D31" t="s">
         <v>20</v>
@@ -2365,10 +2365,10 @@
         <v>8</v>
       </c>
       <c r="I31" s="2" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="J31" s="2" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="K31" t="b">
         <v>1</v>
@@ -2376,25 +2376,25 @@
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A32" t="s">
+        <v>96</v>
+      </c>
+      <c r="B32" t="s">
         <v>97</v>
       </c>
-      <c r="B32" t="s">
+      <c r="C32" t="s">
         <v>98</v>
-      </c>
-      <c r="C32" t="s">
-        <v>99</v>
       </c>
       <c r="D32" t="s">
         <v>20</v>
       </c>
       <c r="E32" t="s">
+        <v>99</v>
+      </c>
+      <c r="H32" s="2" t="s">
         <v>100</v>
       </c>
-      <c r="H32" s="2" t="s">
+      <c r="I32" s="2" t="s">
         <v>101</v>
-      </c>
-      <c r="I32" s="2" t="s">
-        <v>102</v>
       </c>
       <c r="K32" t="b">
         <v>1</v>
@@ -2402,16 +2402,16 @@
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.45">
       <c r="A33" t="s">
+        <v>314</v>
+      </c>
+      <c r="B33" t="s">
         <v>315</v>
       </c>
-      <c r="B33" t="s">
+      <c r="C33" t="s">
         <v>316</v>
       </c>
-      <c r="C33" t="s">
+      <c r="D33" t="s">
         <v>317</v>
-      </c>
-      <c r="D33" t="s">
-        <v>318</v>
       </c>
       <c r="E33" t="s">
         <v>33</v>
@@ -2420,10 +2420,10 @@
         <v>21</v>
       </c>
       <c r="I33" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="J33" s="2" t="s">
         <v>319</v>
-      </c>
-      <c r="J33" s="2" t="s">
-        <v>320</v>
       </c>
       <c r="K33" t="b">
         <v>0</v>
@@ -2452,10 +2452,10 @@
         <v>15</v>
       </c>
       <c r="I34" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J34" s="2" t="s">
-        <v>81</v>
+        <v>322</v>
       </c>
       <c r="K34" t="b">
         <v>0</v>
@@ -2510,7 +2510,7 @@
         <v>15</v>
       </c>
       <c r="H36" s="2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="I36" s="2" t="s">
         <v>34</v>
@@ -2593,16 +2593,16 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B2" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C2" t="s">
+        <v>207</v>
+      </c>
+      <c r="D2" t="s">
         <v>208</v>
-      </c>
-      <c r="D2" t="s">
-        <v>209</v>
       </c>
       <c r="E2">
         <v>1</v>
@@ -2610,16 +2610,16 @@
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B3" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C3" t="s">
+        <v>209</v>
+      </c>
+      <c r="D3" t="s">
         <v>210</v>
-      </c>
-      <c r="D3" t="s">
-        <v>211</v>
       </c>
       <c r="E3">
         <v>1</v>
@@ -2627,16 +2627,16 @@
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B4" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C4" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="D4" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="E4">
         <v>1</v>
@@ -2644,16 +2644,16 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
+        <v>85</v>
+      </c>
+      <c r="B5" t="s">
         <v>86</v>
       </c>
-      <c r="B5" t="s">
-        <v>87</v>
-      </c>
       <c r="C5" t="s">
+        <v>91</v>
+      </c>
+      <c r="D5" t="s">
         <v>92</v>
-      </c>
-      <c r="D5" t="s">
-        <v>93</v>
       </c>
       <c r="E5">
         <v>2</v>
@@ -2695,16 +2695,16 @@
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
+        <v>284</v>
+      </c>
+      <c r="B8" t="s">
         <v>285</v>
       </c>
-      <c r="B8" t="s">
-        <v>286</v>
-      </c>
       <c r="C8" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="D8" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="E8">
         <v>1</v>
@@ -2712,16 +2712,16 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
+        <v>284</v>
+      </c>
+      <c r="B9" t="s">
         <v>285</v>
       </c>
-      <c r="B9" t="s">
-        <v>286</v>
-      </c>
       <c r="C9" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="D9" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="E9">
         <v>1</v>
@@ -2729,16 +2729,16 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
+        <v>284</v>
+      </c>
+      <c r="B10" t="s">
         <v>285</v>
       </c>
-      <c r="B10" t="s">
-        <v>286</v>
-      </c>
       <c r="C10" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="D10" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="E10">
         <v>1</v>
@@ -2746,16 +2746,16 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
+        <v>284</v>
+      </c>
+      <c r="B11" t="s">
         <v>285</v>
       </c>
-      <c r="B11" t="s">
-        <v>286</v>
-      </c>
       <c r="C11" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="D11" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="E11">
         <v>1</v>
@@ -2763,16 +2763,16 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
+        <v>284</v>
+      </c>
+      <c r="B12" t="s">
         <v>285</v>
       </c>
-      <c r="B12" t="s">
-        <v>286</v>
-      </c>
       <c r="C12" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="D12" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="E12">
         <v>1</v>
@@ -2780,16 +2780,16 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
+        <v>284</v>
+      </c>
+      <c r="B13" t="s">
         <v>285</v>
       </c>
-      <c r="B13" t="s">
-        <v>286</v>
-      </c>
       <c r="C13" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="D13" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="E13">
         <v>1</v>
@@ -2797,16 +2797,16 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
+        <v>284</v>
+      </c>
+      <c r="B14" t="s">
         <v>285</v>
       </c>
-      <c r="B14" t="s">
-        <v>286</v>
-      </c>
       <c r="C14" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="D14" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="E14">
         <v>1</v>
@@ -2814,16 +2814,16 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
+        <v>96</v>
+      </c>
+      <c r="B15" t="s">
         <v>97</v>
       </c>
-      <c r="B15" t="s">
-        <v>98</v>
-      </c>
       <c r="C15" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D15" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E15">
         <v>1</v>
@@ -2831,16 +2831,16 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
+        <v>96</v>
+      </c>
+      <c r="B16" t="s">
         <v>97</v>
       </c>
-      <c r="B16" t="s">
-        <v>98</v>
-      </c>
       <c r="C16" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D16" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E16">
         <v>1</v>
@@ -2848,16 +2848,16 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
+        <v>96</v>
+      </c>
+      <c r="B17" t="s">
         <v>97</v>
       </c>
-      <c r="B17" t="s">
-        <v>98</v>
-      </c>
       <c r="C17" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D17" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E17">
         <v>1</v>
@@ -2972,10 +2972,10 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B5" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C5">
         <v>1</v>
@@ -2984,15 +2984,15 @@
         <v>0</v>
       </c>
       <c r="E5" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B6" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C6">
         <v>2</v>
@@ -3001,15 +3001,15 @@
         <v>0</v>
       </c>
       <c r="E6" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B7" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="C7">
         <v>3</v>
@@ -3018,15 +3018,15 @@
         <v>0</v>
       </c>
       <c r="E7" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B8" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C8">
         <v>1</v>
@@ -3040,10 +3040,10 @@
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B9" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C9">
         <v>2</v>
@@ -3052,15 +3052,15 @@
         <v>0</v>
       </c>
       <c r="E9" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B10" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C10">
         <v>3</v>
@@ -3069,15 +3069,15 @@
         <v>0</v>
       </c>
       <c r="E10" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B11" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C11">
         <v>1</v>
@@ -3091,10 +3091,10 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B12" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C12">
         <v>2</v>
@@ -3103,15 +3103,15 @@
         <v>0</v>
       </c>
       <c r="E12" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B13" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="C13">
         <v>3</v>
@@ -3120,15 +3120,15 @@
         <v>0</v>
       </c>
       <c r="E13" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B14" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C14">
         <v>1</v>
@@ -3142,10 +3142,10 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B15" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C15">
         <v>2</v>
@@ -3154,15 +3154,15 @@
         <v>0</v>
       </c>
       <c r="E15" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B16" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C16">
         <v>3</v>
@@ -3171,15 +3171,15 @@
         <v>0</v>
       </c>
       <c r="E16" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B17" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C17">
         <v>1</v>
@@ -3193,10 +3193,10 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B18" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C18">
         <v>2</v>
@@ -3205,15 +3205,15 @@
         <v>0</v>
       </c>
       <c r="E18" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B19" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="C19">
         <v>3</v>
@@ -3222,15 +3222,15 @@
         <v>0</v>
       </c>
       <c r="E19" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B20" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C20">
         <v>1</v>
@@ -3239,15 +3239,15 @@
         <v>0</v>
       </c>
       <c r="E20" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B21" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C21">
         <v>2</v>
@@ -3256,15 +3256,15 @@
         <v>0</v>
       </c>
       <c r="E21" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="B22" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C22">
         <v>3</v>
@@ -3273,15 +3273,15 @@
         <v>0</v>
       </c>
       <c r="E22" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B23" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C23">
         <v>1</v>
@@ -3290,15 +3290,15 @@
         <v>0</v>
       </c>
       <c r="E23" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B24" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C24">
         <v>2</v>
@@ -3307,15 +3307,15 @@
         <v>0</v>
       </c>
       <c r="E24" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B25" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C25">
         <v>3</v>
@@ -3324,15 +3324,15 @@
         <v>0</v>
       </c>
       <c r="E25" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B26" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C26">
         <v>1</v>
@@ -3341,15 +3341,15 @@
         <v>0</v>
       </c>
       <c r="E26" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B27" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C27">
         <v>2</v>
@@ -3358,15 +3358,15 @@
         <v>0</v>
       </c>
       <c r="E27" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B28" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C28">
         <v>3</v>
@@ -3375,15 +3375,15 @@
         <v>0</v>
       </c>
       <c r="E28" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B29" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C29">
         <v>1</v>
@@ -3392,15 +3392,15 @@
         <v>0</v>
       </c>
       <c r="E29" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B30" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C30">
         <v>2</v>
@@ -3409,15 +3409,15 @@
         <v>0</v>
       </c>
       <c r="E30" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A31" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B31" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="C31">
         <v>3</v>
@@ -3426,15 +3426,15 @@
         <v>0</v>
       </c>
       <c r="E31" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A32" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B32" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C32">
         <v>1</v>
@@ -3443,15 +3443,15 @@
         <v>1</v>
       </c>
       <c r="E32" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A33" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B33" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C33">
         <v>2</v>
@@ -3460,15 +3460,15 @@
         <v>0</v>
       </c>
       <c r="E33" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A34" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="B34" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C34">
         <v>3</v>
@@ -3477,15 +3477,15 @@
         <v>0</v>
       </c>
       <c r="E34" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A35" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B35" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C35">
         <v>1</v>
@@ -3499,10 +3499,10 @@
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A36" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B36" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C36">
         <v>2</v>
@@ -3511,15 +3511,15 @@
         <v>0</v>
       </c>
       <c r="E36" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A37" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="B37" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C37">
         <v>3</v>
@@ -3528,12 +3528,12 @@
         <v>0</v>
       </c>
       <c r="E37" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A38" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B38" t="s">
         <v>5</v>
@@ -3550,7 +3550,7 @@
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A39" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B39" t="s">
         <v>5</v>
@@ -3562,12 +3562,12 @@
         <v>0</v>
       </c>
       <c r="E39" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A40" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="B40" t="s">
         <v>5</v>
@@ -3579,15 +3579,15 @@
         <v>0</v>
       </c>
       <c r="E40" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A41" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B41" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C41">
         <v>1</v>
@@ -3601,10 +3601,10 @@
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A42" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B42" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C42">
         <v>2</v>
@@ -3613,15 +3613,15 @@
         <v>0</v>
       </c>
       <c r="E42" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A43" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="B43" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C43">
         <v>3</v>
@@ -3630,15 +3630,15 @@
         <v>0</v>
       </c>
       <c r="E43" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A44" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B44" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C44">
         <v>1</v>
@@ -3647,15 +3647,15 @@
         <v>0</v>
       </c>
       <c r="E44" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A45" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B45" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C45">
         <v>2</v>
@@ -3664,15 +3664,15 @@
         <v>0</v>
       </c>
       <c r="E45" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A46" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="B46" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="C46">
         <v>3</v>
@@ -3681,15 +3681,15 @@
         <v>0</v>
       </c>
       <c r="E46" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A47" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B47" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C47">
         <v>1</v>
@@ -3703,10 +3703,10 @@
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A48" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B48" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C48">
         <v>2</v>
@@ -3715,15 +3715,15 @@
         <v>0</v>
       </c>
       <c r="E48" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A49" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B49" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="C49">
         <v>3</v>
@@ -3737,10 +3737,10 @@
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A50" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B50" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C50">
         <v>1</v>
@@ -3749,15 +3749,15 @@
         <v>0</v>
       </c>
       <c r="E50" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A51" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B51" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C51">
         <v>2</v>
@@ -3766,15 +3766,15 @@
         <v>0</v>
       </c>
       <c r="E51" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A52" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B52" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C52">
         <v>3</v>
@@ -3783,15 +3783,15 @@
         <v>0</v>
       </c>
       <c r="E52" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A53" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B53" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C53">
         <v>1</v>
@@ -3800,15 +3800,15 @@
         <v>0</v>
       </c>
       <c r="E53" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A54" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B54" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C54">
         <v>2</v>
@@ -3817,15 +3817,15 @@
         <v>0</v>
       </c>
       <c r="E54" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A55" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B55" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C55">
         <v>3</v>
@@ -3834,15 +3834,15 @@
         <v>0</v>
       </c>
       <c r="E55" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A56" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B56" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C56">
         <v>1</v>
@@ -3856,10 +3856,10 @@
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A57" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B57" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C57">
         <v>2</v>
@@ -3868,15 +3868,15 @@
         <v>0</v>
       </c>
       <c r="E57" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A58" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B58" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C58">
         <v>3</v>
@@ -3885,15 +3885,15 @@
         <v>0</v>
       </c>
       <c r="E58" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A59" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B59" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C59">
         <v>1</v>
@@ -3902,15 +3902,15 @@
         <v>0</v>
       </c>
       <c r="E59" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A60" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B60" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C60">
         <v>2</v>
@@ -3919,15 +3919,15 @@
         <v>0</v>
       </c>
       <c r="E60" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A61" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="B61" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="C61">
         <v>3</v>
@@ -3936,15 +3936,15 @@
         <v>0</v>
       </c>
       <c r="E61" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A62" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B62" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C62">
         <v>1</v>
@@ -3958,10 +3958,10 @@
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A63" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B63" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C63">
         <v>2</v>
@@ -3970,15 +3970,15 @@
         <v>0</v>
       </c>
       <c r="E63" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A64" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="B64" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C64">
         <v>3</v>
@@ -3987,15 +3987,15 @@
         <v>0</v>
       </c>
       <c r="E64" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A65" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B65" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C65">
         <v>1</v>
@@ -4004,15 +4004,15 @@
         <v>1</v>
       </c>
       <c r="E65" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A66" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B66" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C66">
         <v>2</v>
@@ -4021,15 +4021,15 @@
         <v>0</v>
       </c>
       <c r="E66" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A67" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="B67" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C67">
         <v>3</v>
@@ -4038,15 +4038,15 @@
         <v>0</v>
       </c>
       <c r="E67" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A68" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B68" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C68">
         <v>1</v>
@@ -4055,15 +4055,15 @@
         <v>0</v>
       </c>
       <c r="E68" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A69" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B69" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C69">
         <v>2</v>
@@ -4072,15 +4072,15 @@
         <v>0</v>
       </c>
       <c r="E69" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A70" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="B70" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C70">
         <v>3</v>
@@ -4089,16 +4089,16 @@
         <v>0</v>
       </c>
       <c r="E70" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A71" t="s">
+        <v>264</v>
+      </c>
+      <c r="B71" t="s">
         <v>265</v>
       </c>
-      <c r="B71" t="s">
-        <v>266</v>
-      </c>
       <c r="C71">
         <v>1</v>
       </c>
@@ -4106,15 +4106,15 @@
         <v>1</v>
       </c>
       <c r="E71" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A72" t="s">
+        <v>264</v>
+      </c>
+      <c r="B72" t="s">
         <v>265</v>
-      </c>
-      <c r="B72" t="s">
-        <v>266</v>
       </c>
       <c r="C72">
         <v>2</v>
@@ -4123,15 +4123,15 @@
         <v>0</v>
       </c>
       <c r="E72" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A73" t="s">
+        <v>264</v>
+      </c>
+      <c r="B73" t="s">
         <v>265</v>
-      </c>
-      <c r="B73" t="s">
-        <v>266</v>
       </c>
       <c r="C73">
         <v>3</v>
@@ -4140,16 +4140,16 @@
         <v>0</v>
       </c>
       <c r="E73" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A74" t="s">
+        <v>271</v>
+      </c>
+      <c r="B74" t="s">
         <v>272</v>
       </c>
-      <c r="B74" t="s">
-        <v>273</v>
-      </c>
       <c r="C74">
         <v>1</v>
       </c>
@@ -4157,15 +4157,15 @@
         <v>1</v>
       </c>
       <c r="E74" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A75" t="s">
+        <v>271</v>
+      </c>
+      <c r="B75" t="s">
         <v>272</v>
-      </c>
-      <c r="B75" t="s">
-        <v>273</v>
       </c>
       <c r="C75">
         <v>2</v>
@@ -4174,15 +4174,15 @@
         <v>0</v>
       </c>
       <c r="E75" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A76" t="s">
+        <v>271</v>
+      </c>
+      <c r="B76" t="s">
         <v>272</v>
-      </c>
-      <c r="B76" t="s">
-        <v>273</v>
       </c>
       <c r="C76">
         <v>3</v>
@@ -4191,16 +4191,16 @@
         <v>0</v>
       </c>
       <c r="E76" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A77" t="s">
+        <v>85</v>
+      </c>
+      <c r="B77" t="s">
         <v>86</v>
       </c>
-      <c r="B77" t="s">
-        <v>87</v>
-      </c>
       <c r="C77">
         <v>1</v>
       </c>
@@ -4208,15 +4208,15 @@
         <v>1</v>
       </c>
       <c r="E77" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A78" t="s">
+        <v>85</v>
+      </c>
+      <c r="B78" t="s">
         <v>86</v>
-      </c>
-      <c r="B78" t="s">
-        <v>87</v>
       </c>
       <c r="C78">
         <v>2</v>
@@ -4225,15 +4225,15 @@
         <v>0</v>
       </c>
       <c r="E78" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A79" t="s">
+        <v>85</v>
+      </c>
+      <c r="B79" t="s">
         <v>86</v>
-      </c>
-      <c r="B79" t="s">
-        <v>87</v>
       </c>
       <c r="C79">
         <v>3</v>
@@ -4242,16 +4242,16 @@
         <v>0</v>
       </c>
       <c r="E79" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A80" t="s">
+        <v>275</v>
+      </c>
+      <c r="B80" t="s">
         <v>276</v>
       </c>
-      <c r="B80" t="s">
-        <v>277</v>
-      </c>
       <c r="C80">
         <v>1</v>
       </c>
@@ -4259,15 +4259,15 @@
         <v>1</v>
       </c>
       <c r="E80" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A81" t="s">
+        <v>275</v>
+      </c>
+      <c r="B81" t="s">
         <v>276</v>
-      </c>
-      <c r="B81" t="s">
-        <v>277</v>
       </c>
       <c r="C81">
         <v>2</v>
@@ -4276,15 +4276,15 @@
         <v>0</v>
       </c>
       <c r="E81" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A82" t="s">
+        <v>275</v>
+      </c>
+      <c r="B82" t="s">
         <v>276</v>
-      </c>
-      <c r="B82" t="s">
-        <v>277</v>
       </c>
       <c r="C82">
         <v>3</v>
@@ -4293,15 +4293,15 @@
         <v>0</v>
       </c>
       <c r="E82" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A83" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B83" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="C83">
         <v>1</v>
@@ -4315,10 +4315,10 @@
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A84" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B84" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="C84">
         <v>2</v>
@@ -4327,15 +4327,15 @@
         <v>0</v>
       </c>
       <c r="E84" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A85" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="B85" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="C85">
         <v>3</v>
@@ -4344,7 +4344,7 @@
         <v>0</v>
       </c>
       <c r="E85" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.45">
@@ -4400,11 +4400,11 @@
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A89" t="s">
+        <v>284</v>
+      </c>
+      <c r="B89" t="s">
         <v>285</v>
       </c>
-      <c r="B89" t="s">
-        <v>286</v>
-      </c>
       <c r="C89">
         <v>1</v>
       </c>
@@ -4412,15 +4412,15 @@
         <v>0</v>
       </c>
       <c r="E89" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A90" t="s">
+        <v>284</v>
+      </c>
+      <c r="B90" t="s">
         <v>285</v>
-      </c>
-      <c r="B90" t="s">
-        <v>286</v>
       </c>
       <c r="C90">
         <v>2</v>
@@ -4429,15 +4429,15 @@
         <v>0</v>
       </c>
       <c r="E90" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A91" t="s">
+        <v>284</v>
+      </c>
+      <c r="B91" t="s">
         <v>285</v>
-      </c>
-      <c r="B91" t="s">
-        <v>286</v>
       </c>
       <c r="C91">
         <v>3</v>
@@ -4446,16 +4446,16 @@
         <v>0</v>
       </c>
       <c r="E91" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A92" t="s">
+        <v>96</v>
+      </c>
+      <c r="B92" t="s">
         <v>97</v>
       </c>
-      <c r="B92" t="s">
-        <v>98</v>
-      </c>
       <c r="C92">
         <v>1</v>
       </c>
@@ -4463,15 +4463,15 @@
         <v>0</v>
       </c>
       <c r="E92" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A93" t="s">
+        <v>96</v>
+      </c>
+      <c r="B93" t="s">
         <v>97</v>
-      </c>
-      <c r="B93" t="s">
-        <v>98</v>
       </c>
       <c r="C93">
         <v>2</v>
@@ -4480,15 +4480,15 @@
         <v>0</v>
       </c>
       <c r="E93" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A94" t="s">
+        <v>96</v>
+      </c>
+      <c r="B94" t="s">
         <v>97</v>
-      </c>
-      <c r="B94" t="s">
-        <v>98</v>
       </c>
       <c r="C94">
         <v>3</v>
@@ -4497,16 +4497,16 @@
         <v>0</v>
       </c>
       <c r="E94" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A95" t="s">
+        <v>314</v>
+      </c>
+      <c r="B95" t="s">
         <v>315</v>
       </c>
-      <c r="B95" t="s">
-        <v>316</v>
-      </c>
       <c r="C95">
         <v>1</v>
       </c>
@@ -4514,15 +4514,15 @@
         <v>1</v>
       </c>
       <c r="E95" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A96" t="s">
+        <v>314</v>
+      </c>
+      <c r="B96" t="s">
         <v>315</v>
-      </c>
-      <c r="B96" t="s">
-        <v>316</v>
       </c>
       <c r="C96">
         <v>2</v>
@@ -4536,10 +4536,10 @@
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A97" t="s">
+        <v>314</v>
+      </c>
+      <c r="B97" t="s">
         <v>315</v>
-      </c>
-      <c r="B97" t="s">
-        <v>316</v>
       </c>
       <c r="C97">
         <v>3</v>
@@ -4548,7 +4548,7 @@
         <v>0</v>
       </c>
       <c r="E97" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.45">
@@ -4565,7 +4565,7 @@
         <v>1</v>
       </c>
       <c r="E98" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.45">
@@ -4582,7 +4582,7 @@
         <v>0</v>
       </c>
       <c r="E99" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.45">
@@ -4599,7 +4599,7 @@
         <v>0</v>
       </c>
       <c r="E100" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.45">

</xml_diff>

<commit_message>
fixed css sizing stuff and added servant name and servant skill and deck headers
</commit_message>
<xml_diff>
--- a/data/Fate-Spreadsheet.xlsx
+++ b/data/Fate-Spreadsheet.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pixel\Documents\Projects\Fate-Wiki\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Important\Python\Fate-Wiki\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F766361-2887-4A36-9C5B-EE2D635FDC7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{B05E798F-9EF6-4508-A0A4-311D06661AED}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{B05E798F-9EF6-4508-A0A4-311D06661AED}"/>
   </bookViews>
   <sheets>
     <sheet name="Servants" sheetId="1" r:id="rId1"/>
@@ -1401,21 +1401,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E33D7ECC-1EAA-4A40-B4DA-A93E54CBC8B5}">
   <dimension ref="A1:K37"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="17.1328125" customWidth="1"/>
-    <col min="3" max="3" width="21.9296875" customWidth="1"/>
-    <col min="4" max="4" width="12.59765625" customWidth="1"/>
-    <col min="5" max="5" width="11.265625" customWidth="1"/>
-    <col min="6" max="6" width="15.53125" customWidth="1"/>
-    <col min="7" max="7" width="13.73046875" style="2" customWidth="1"/>
-    <col min="8" max="8" width="11.73046875" style="2" customWidth="1"/>
-    <col min="9" max="9" width="11.796875" style="2" customWidth="1"/>
-    <col min="10" max="10" width="48.796875" style="2" customWidth="1"/>
-    <col min="11" max="11" width="12.59765625" customWidth="1"/>
+    <col min="2" max="2" width="17.140625" customWidth="1"/>
+    <col min="3" max="3" width="22" customWidth="1"/>
+    <col min="4" max="4" width="12.5703125" customWidth="1"/>
+    <col min="5" max="5" width="11.28515625" customWidth="1"/>
+    <col min="6" max="6" width="15.5703125" customWidth="1"/>
+    <col min="7" max="7" width="13.7109375" style="2" customWidth="1"/>
+    <col min="8" max="8" width="11.7109375" style="2" customWidth="1"/>
+    <col min="9" max="9" width="11.85546875" style="2" customWidth="1"/>
+    <col min="10" max="10" width="48.85546875" style="2" customWidth="1"/>
+    <col min="11" max="11" width="12.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1450,7 +1450,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -1482,7 +1482,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>111</v>
       </c>
@@ -1514,7 +1514,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>112</v>
       </c>
@@ -1543,7 +1543,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>113</v>
       </c>
@@ -1572,7 +1572,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>114</v>
       </c>
@@ -1604,7 +1604,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>115</v>
       </c>
@@ -1636,7 +1636,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>116</v>
       </c>
@@ -1665,7 +1665,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>117</v>
       </c>
@@ -1694,7 +1694,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>118</v>
       </c>
@@ -1726,7 +1726,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>119</v>
       </c>
@@ -1758,7 +1758,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>120</v>
       </c>
@@ -1790,7 +1790,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>121</v>
       </c>
@@ -1819,7 +1819,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>122</v>
       </c>
@@ -1851,7 +1851,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>123</v>
       </c>
@@ -1883,7 +1883,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>124</v>
       </c>
@@ -1915,7 +1915,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>125</v>
       </c>
@@ -1947,7 +1947,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>126</v>
       </c>
@@ -1979,7 +1979,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>127</v>
       </c>
@@ -2011,7 +2011,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>128</v>
       </c>
@@ -2040,7 +2040,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>129</v>
       </c>
@@ -2072,7 +2072,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>130</v>
       </c>
@@ -2104,7 +2104,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>131</v>
       </c>
@@ -2136,7 +2136,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>132</v>
       </c>
@@ -2168,7 +2168,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>264</v>
       </c>
@@ -2200,7 +2200,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>271</v>
       </c>
@@ -2232,7 +2232,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>85</v>
       </c>
@@ -2261,7 +2261,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>275</v>
       </c>
@@ -2293,7 +2293,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>281</v>
       </c>
@@ -2322,7 +2322,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>17</v>
       </c>
@@ -2348,7 +2348,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>284</v>
       </c>
@@ -2374,7 +2374,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>96</v>
       </c>
@@ -2400,7 +2400,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>314</v>
       </c>
@@ -2429,7 +2429,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>76</v>
       </c>
@@ -2461,7 +2461,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>23</v>
       </c>
@@ -2490,7 +2490,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>29</v>
       </c>
@@ -2522,7 +2522,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>36</v>
       </c>
@@ -2563,15 +2563,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1BC60D8-44F3-478D-BCC0-4752624457AE}">
   <dimension ref="A1:F18"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="19" customWidth="1"/>
-    <col min="3" max="3" width="15.1328125" customWidth="1"/>
-    <col min="4" max="5" width="16.46484375" customWidth="1"/>
-    <col min="6" max="6" width="13.53125" customWidth="1"/>
+    <col min="3" max="3" width="15.140625" customWidth="1"/>
+    <col min="4" max="5" width="16.42578125" customWidth="1"/>
+    <col min="6" max="6" width="13.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2591,7 +2591,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>116</v>
       </c>
@@ -2608,7 +2608,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>126</v>
       </c>
@@ -2625,7 +2625,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>130</v>
       </c>
@@ -2642,7 +2642,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>85</v>
       </c>
@@ -2659,7 +2659,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>17</v>
       </c>
@@ -2676,7 +2676,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>17</v>
       </c>
@@ -2693,7 +2693,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>284</v>
       </c>
@@ -2710,7 +2710,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>284</v>
       </c>
@@ -2727,7 +2727,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>284</v>
       </c>
@@ -2744,7 +2744,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>284</v>
       </c>
@@ -2761,7 +2761,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>284</v>
       </c>
@@ -2778,7 +2778,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>284</v>
       </c>
@@ -2795,7 +2795,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>284</v>
       </c>
@@ -2812,7 +2812,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>96</v>
       </c>
@@ -2829,7 +2829,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>96</v>
       </c>
@@ -2846,7 +2846,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>96</v>
       </c>
@@ -2863,7 +2863,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>36</v>
       </c>
@@ -2890,16 +2890,16 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84E3BB0D-5578-4069-B1C9-C3864EB2A429}">
   <dimension ref="A1:F109"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="20.59765625" customWidth="1"/>
-    <col min="3" max="3" width="12.73046875" customWidth="1"/>
-    <col min="4" max="4" width="17.06640625" customWidth="1"/>
-    <col min="5" max="5" width="21.59765625" customWidth="1"/>
-    <col min="6" max="6" width="15.73046875" customWidth="1"/>
+    <col min="2" max="2" width="20.5703125" customWidth="1"/>
+    <col min="3" max="3" width="12.7109375" customWidth="1"/>
+    <col min="4" max="4" width="17" customWidth="1"/>
+    <col min="5" max="5" width="21.5703125" customWidth="1"/>
+    <col min="6" max="6" width="15.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2919,7 +2919,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -2936,7 +2936,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -2953,7 +2953,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -2970,7 +2970,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>111</v>
       </c>
@@ -2987,7 +2987,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>111</v>
       </c>
@@ -3004,7 +3004,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>111</v>
       </c>
@@ -3021,7 +3021,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>112</v>
       </c>
@@ -3038,7 +3038,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>112</v>
       </c>
@@ -3055,7 +3055,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>112</v>
       </c>
@@ -3072,7 +3072,7 @@
         <v>216</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>113</v>
       </c>
@@ -3089,7 +3089,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>113</v>
       </c>
@@ -3106,7 +3106,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>113</v>
       </c>
@@ -3123,7 +3123,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>114</v>
       </c>
@@ -3140,7 +3140,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>114</v>
       </c>
@@ -3157,7 +3157,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>114</v>
       </c>
@@ -3174,7 +3174,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>115</v>
       </c>
@@ -3191,7 +3191,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>115</v>
       </c>
@@ -3208,7 +3208,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>115</v>
       </c>
@@ -3225,7 +3225,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>116</v>
       </c>
@@ -3242,7 +3242,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>116</v>
       </c>
@@ -3259,7 +3259,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>116</v>
       </c>
@@ -3276,7 +3276,7 @@
         <v>225</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>117</v>
       </c>
@@ -3293,7 +3293,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>117</v>
       </c>
@@ -3310,7 +3310,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>117</v>
       </c>
@@ -3327,7 +3327,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>118</v>
       </c>
@@ -3344,7 +3344,7 @@
         <v>229</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>118</v>
       </c>
@@ -3361,7 +3361,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>118</v>
       </c>
@@ -3378,7 +3378,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>119</v>
       </c>
@@ -3395,7 +3395,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>119</v>
       </c>
@@ -3412,7 +3412,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>119</v>
       </c>
@@ -3429,7 +3429,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>120</v>
       </c>
@@ -3446,7 +3446,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>120</v>
       </c>
@@ -3463,7 +3463,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>120</v>
       </c>
@@ -3480,7 +3480,7 @@
         <v>236</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>121</v>
       </c>
@@ -3497,7 +3497,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>121</v>
       </c>
@@ -3514,7 +3514,7 @@
         <v>237</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>121</v>
       </c>
@@ -3531,7 +3531,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>122</v>
       </c>
@@ -3548,7 +3548,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>122</v>
       </c>
@@ -3565,7 +3565,7 @@
         <v>239</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>122</v>
       </c>
@@ -3582,7 +3582,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>123</v>
       </c>
@@ -3599,7 +3599,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>123</v>
       </c>
@@ -3616,7 +3616,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>123</v>
       </c>
@@ -3633,7 +3633,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>124</v>
       </c>
@@ -3650,7 +3650,7 @@
         <v>243</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>124</v>
       </c>
@@ -3667,7 +3667,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>124</v>
       </c>
@@ -3684,7 +3684,7 @@
         <v>245</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>125</v>
       </c>
@@ -3701,7 +3701,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>125</v>
       </c>
@@ -3718,7 +3718,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>125</v>
       </c>
@@ -3735,7 +3735,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>126</v>
       </c>
@@ -3752,7 +3752,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>126</v>
       </c>
@@ -3769,7 +3769,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>126</v>
       </c>
@@ -3786,7 +3786,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>127</v>
       </c>
@@ -3803,7 +3803,7 @@
         <v>250</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>127</v>
       </c>
@@ -3820,7 +3820,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>127</v>
       </c>
@@ -3837,7 +3837,7 @@
         <v>252</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>128</v>
       </c>
@@ -3854,7 +3854,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>128</v>
       </c>
@@ -3871,7 +3871,7 @@
         <v>223</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>128</v>
       </c>
@@ -3888,7 +3888,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>129</v>
       </c>
@@ -3905,7 +3905,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>129</v>
       </c>
@@ -3922,7 +3922,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>129</v>
       </c>
@@ -3939,7 +3939,7 @@
         <v>256</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>130</v>
       </c>
@@ -3956,7 +3956,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>130</v>
       </c>
@@ -3973,7 +3973,7 @@
         <v>257</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>130</v>
       </c>
@@ -3990,7 +3990,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>131</v>
       </c>
@@ -4007,7 +4007,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>131</v>
       </c>
@@ -4024,7 +4024,7 @@
         <v>259</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>131</v>
       </c>
@@ -4041,7 +4041,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>132</v>
       </c>
@@ -4058,7 +4058,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>132</v>
       </c>
@@ -4075,7 +4075,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>132</v>
       </c>
@@ -4092,7 +4092,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>264</v>
       </c>
@@ -4109,7 +4109,7 @@
         <v>302</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>264</v>
       </c>
@@ -4126,7 +4126,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>264</v>
       </c>
@@ -4143,7 +4143,7 @@
         <v>303</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>271</v>
       </c>
@@ -4160,7 +4160,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>271</v>
       </c>
@@ -4177,7 +4177,7 @@
         <v>304</v>
       </c>
     </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>271</v>
       </c>
@@ -4194,7 +4194,7 @@
         <v>305</v>
       </c>
     </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>85</v>
       </c>
@@ -4211,7 +4211,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>85</v>
       </c>
@@ -4228,7 +4228,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>85</v>
       </c>
@@ -4245,7 +4245,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>275</v>
       </c>
@@ -4262,7 +4262,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="81" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>275</v>
       </c>
@@ -4279,7 +4279,7 @@
         <v>307</v>
       </c>
     </row>
-    <row r="82" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>275</v>
       </c>
@@ -4296,7 +4296,7 @@
         <v>308</v>
       </c>
     </row>
-    <row r="83" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>281</v>
       </c>
@@ -4313,7 +4313,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="84" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>281</v>
       </c>
@@ -4330,7 +4330,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="85" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>281</v>
       </c>
@@ -4347,7 +4347,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>17</v>
       </c>
@@ -4364,7 +4364,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="87" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>17</v>
       </c>
@@ -4381,7 +4381,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="88" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>17</v>
       </c>
@@ -4398,7 +4398,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="89" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>284</v>
       </c>
@@ -4415,7 +4415,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="90" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>284</v>
       </c>
@@ -4432,7 +4432,7 @@
         <v>312</v>
       </c>
     </row>
-    <row r="91" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>284</v>
       </c>
@@ -4449,7 +4449,7 @@
         <v>313</v>
       </c>
     </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>96</v>
       </c>
@@ -4466,7 +4466,7 @@
         <v>108</v>
       </c>
     </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>96</v>
       </c>
@@ -4483,7 +4483,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>96</v>
       </c>
@@ -4500,7 +4500,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>314</v>
       </c>
@@ -4517,7 +4517,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="96" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>314</v>
       </c>
@@ -4534,7 +4534,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>314</v>
       </c>
@@ -4551,7 +4551,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>76</v>
       </c>
@@ -4568,7 +4568,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>76</v>
       </c>
@@ -4585,7 +4585,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>76</v>
       </c>
@@ -4602,7 +4602,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>23</v>
       </c>
@@ -4619,7 +4619,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>23</v>
       </c>
@@ -4636,7 +4636,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>23</v>
       </c>
@@ -4653,7 +4653,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>29</v>
       </c>
@@ -4670,7 +4670,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>29</v>
       </c>
@@ -4687,7 +4687,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>29</v>
       </c>
@@ -4704,7 +4704,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>36</v>
       </c>
@@ -4721,7 +4721,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>36</v>
       </c>
@@ -4738,7 +4738,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>36</v>
       </c>
@@ -4764,7 +4764,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32F3CD10-C054-4484-ABE2-D426F834FC22}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -4773,7 +4773,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{931309AC-3B5D-4169-8BD3-83BC320E154C}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
all of lancer class added
</commit_message>
<xml_diff>
--- a/data/Fate-Spreadsheet.xlsx
+++ b/data/Fate-Spreadsheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Important\Python\Fate-Wiki\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F766361-2887-4A36-9C5B-EE2D635FDC7D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74FB2C1B-B3D2-4F80-982D-47219B1EFE02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{B05E798F-9EF6-4508-A0A4-311D06661AED}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="722" uniqueCount="323">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1141" uniqueCount="476">
   <si>
     <t>servant_id</t>
   </si>
@@ -1012,6 +1012,465 @@
   </si>
   <si>
     <t>Berserker_Strength_7,Berserker_Strength_9,Luck,Luck,Surveil</t>
+  </si>
+  <si>
+    <t>S0025</t>
+  </si>
+  <si>
+    <t>Diarmuid Ua Duibhne</t>
+  </si>
+  <si>
+    <t>diarmuid-ua-duibhne</t>
+  </si>
+  <si>
+    <t>3,4,5</t>
+  </si>
+  <si>
+    <t>2,3,3,4,4,4,5,5</t>
+  </si>
+  <si>
+    <t>Surveil</t>
+  </si>
+  <si>
+    <t>S0026</t>
+  </si>
+  <si>
+    <t>S0027</t>
+  </si>
+  <si>
+    <t>S0028</t>
+  </si>
+  <si>
+    <t>S0029</t>
+  </si>
+  <si>
+    <t>S0030</t>
+  </si>
+  <si>
+    <t>S0031</t>
+  </si>
+  <si>
+    <t>S0032</t>
+  </si>
+  <si>
+    <t>S0033</t>
+  </si>
+  <si>
+    <t>S0034</t>
+  </si>
+  <si>
+    <t>S0035</t>
+  </si>
+  <si>
+    <t>S0036</t>
+  </si>
+  <si>
+    <t>S0037</t>
+  </si>
+  <si>
+    <t>S0038</t>
+  </si>
+  <si>
+    <t>S0039</t>
+  </si>
+  <si>
+    <t>S0040</t>
+  </si>
+  <si>
+    <t>S0041</t>
+  </si>
+  <si>
+    <t>S0042</t>
+  </si>
+  <si>
+    <t>S0043</t>
+  </si>
+  <si>
+    <t>S0044</t>
+  </si>
+  <si>
+    <t>S0045</t>
+  </si>
+  <si>
+    <t>S0046</t>
+  </si>
+  <si>
+    <t>Gae Buidhe</t>
+  </si>
+  <si>
+    <t>Gae Dearg</t>
+  </si>
+  <si>
+    <t>Vasavi Shakti</t>
+  </si>
+  <si>
+    <t>Brahmastra Kundala</t>
+  </si>
+  <si>
+    <t>Kavacha &amp; Kundala</t>
+  </si>
+  <si>
+    <t>Karna</t>
+  </si>
+  <si>
+    <t>Vlad Tepes</t>
+  </si>
+  <si>
+    <t>Elizabeth Bathory</t>
+  </si>
+  <si>
+    <t>scathach</t>
+  </si>
+  <si>
+    <t>elizabeth-bathory</t>
+  </si>
+  <si>
+    <t>vlad-tepes</t>
+  </si>
+  <si>
+    <t>karna</t>
+  </si>
+  <si>
+    <t>Valkyrie</t>
+  </si>
+  <si>
+    <t>valkyrie</t>
+  </si>
+  <si>
+    <t>Ereshkigal</t>
+  </si>
+  <si>
+    <t>ereshkigal</t>
+  </si>
+  <si>
+    <t>Enkidu</t>
+  </si>
+  <si>
+    <t>enkidu</t>
+  </si>
+  <si>
+    <t>Meltryllis</t>
+  </si>
+  <si>
+    <t>meltryllis</t>
+  </si>
+  <si>
+    <t>Brynhildr</t>
+  </si>
+  <si>
+    <t>Caenis</t>
+  </si>
+  <si>
+    <t>Leonidas I</t>
+  </si>
+  <si>
+    <t>leonidas-i</t>
+  </si>
+  <si>
+    <t>caenis</t>
+  </si>
+  <si>
+    <t>brynhildr</t>
+  </si>
+  <si>
+    <t>Romulus</t>
+  </si>
+  <si>
+    <t>Jaguar Man</t>
+  </si>
+  <si>
+    <t>Musashibou Benkei</t>
+  </si>
+  <si>
+    <t>Don Quixote</t>
+  </si>
+  <si>
+    <t>The Lion King</t>
+  </si>
+  <si>
+    <t>Bradamante</t>
+  </si>
+  <si>
+    <t>Gareth</t>
+  </si>
+  <si>
+    <t>Nagao Kagetora</t>
+  </si>
+  <si>
+    <t>Parvati</t>
+  </si>
+  <si>
+    <t>romulus</t>
+  </si>
+  <si>
+    <t>bradamante</t>
+  </si>
+  <si>
+    <t>gareth</t>
+  </si>
+  <si>
+    <t>melusine</t>
+  </si>
+  <si>
+    <t>parvati</t>
+  </si>
+  <si>
+    <t>jaguar-man</t>
+  </si>
+  <si>
+    <t>musashibou-benkei</t>
+  </si>
+  <si>
+    <t>don-quixote</t>
+  </si>
+  <si>
+    <t>nagao-kagetora</t>
+  </si>
+  <si>
+    <t>the-lion-king</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>Luck,Surveil,Preparation,Preparation</t>
+  </si>
+  <si>
+    <t>2,2,4</t>
+  </si>
+  <si>
+    <t>Commander Ortlinde</t>
+  </si>
+  <si>
+    <t>Commander Hildr</t>
+  </si>
+  <si>
+    <t>Commander Thrud</t>
+  </si>
+  <si>
+    <t>Commander-Ortlinde</t>
+  </si>
+  <si>
+    <t>Commander-Hildr</t>
+  </si>
+  <si>
+    <t>Commander-Thrud</t>
+  </si>
+  <si>
+    <t>Kazikli Bey</t>
+  </si>
+  <si>
+    <t>Protector of the Nation</t>
+  </si>
+  <si>
+    <t>Prison Castle Csejte</t>
+  </si>
+  <si>
+    <t>Kilenc Sárkány</t>
+  </si>
+  <si>
+    <t>Torture Techniques</t>
+  </si>
+  <si>
+    <t>Scáthach</t>
+  </si>
+  <si>
+    <t>Gate of Skye</t>
+  </si>
+  <si>
+    <t>Gáe Bolg Alternative</t>
+  </si>
+  <si>
+    <t>Wisdom of Dun Scaith</t>
+  </si>
+  <si>
+    <t>Gungnir</t>
+  </si>
+  <si>
+    <t>Ragnarök</t>
+  </si>
+  <si>
+    <t>Svanhvit</t>
+  </si>
+  <si>
+    <t>2,4</t>
+  </si>
+  <si>
+    <t>Kur Kigal Irkalla</t>
+  </si>
+  <si>
+    <t>Blessing of Kur</t>
+  </si>
+  <si>
+    <t>Enuma Elish (Enkidu)</t>
+  </si>
+  <si>
+    <t>Transfiguration</t>
+  </si>
+  <si>
+    <t>Saraswati Meltout</t>
+  </si>
+  <si>
+    <t>Melt Virus</t>
+  </si>
+  <si>
+    <t>Brynhildr Romantia</t>
+  </si>
+  <si>
+    <t>Hero's Bridesmaid</t>
+  </si>
+  <si>
+    <t>Great Golden Wings</t>
+  </si>
+  <si>
+    <t>Poseidon's Favor</t>
+  </si>
+  <si>
+    <t>Poseidon's Maelstrom</t>
+  </si>
+  <si>
+    <t>Thermopylae Enomotia</t>
+  </si>
+  <si>
+    <t>Spartan War Cry</t>
+  </si>
+  <si>
+    <t>Rear Guard's Pride</t>
+  </si>
+  <si>
+    <t>2,2,3,5</t>
+  </si>
+  <si>
+    <t>Luck,Preparation,Preparation,Preparation</t>
+  </si>
+  <si>
+    <t>Magna Voluisse Magnum</t>
+  </si>
+  <si>
+    <t>Moles Necessrie</t>
+  </si>
+  <si>
+    <t>2,2,4,5</t>
+  </si>
+  <si>
+    <t>Luck,Luck,Preparation</t>
+  </si>
+  <si>
+    <t>Great Death Claw</t>
+  </si>
+  <si>
+    <t>Law of the Jungle</t>
+  </si>
+  <si>
+    <t>2,2,4,4,5</t>
+  </si>
+  <si>
+    <t>Bulwark Stance</t>
+  </si>
+  <si>
+    <t>Evenly Matched</t>
+  </si>
+  <si>
+    <t>3,4,5,5,5</t>
+  </si>
+  <si>
+    <t>3,3,3</t>
+  </si>
+  <si>
+    <t>Valiente Asalto</t>
+  </si>
+  <si>
+    <t>Knight's Fantasy</t>
+  </si>
+  <si>
+    <t>2,2,3,4,4</t>
+  </si>
+  <si>
+    <t>Rhongomyniad</t>
+  </si>
+  <si>
+    <t>Divine Command</t>
+  </si>
+  <si>
+    <t>Dun Stallion</t>
+  </si>
+  <si>
+    <t>2,2,3,4,5,5</t>
+  </si>
+  <si>
+    <t>3,4</t>
+  </si>
+  <si>
+    <t>Bouclier d'Atlante</t>
+  </si>
+  <si>
+    <t>Angelica Cathay</t>
+  </si>
+  <si>
+    <t>2,4,4,5</t>
+  </si>
+  <si>
+    <t>Ira Lupus</t>
+  </si>
+  <si>
+    <t>Gun Lance</t>
+  </si>
+  <si>
+    <t>Ring of Transformation</t>
+  </si>
+  <si>
+    <t>8 Phase Wheel Charge</t>
+  </si>
+  <si>
+    <t>God of War</t>
+  </si>
+  <si>
+    <t>2,2,2,3,3</t>
+  </si>
+  <si>
+    <t>4,4,5,5</t>
+  </si>
+  <si>
+    <t>Mélusine</t>
+  </si>
+  <si>
+    <t>Innocence Arondight</t>
+  </si>
+  <si>
+    <t>Ray Horizon</t>
+  </si>
+  <si>
+    <t>Perl Dancer</t>
+  </si>
+  <si>
+    <t>S0047</t>
+  </si>
+  <si>
+    <t>Emiya</t>
+  </si>
+  <si>
+    <t>emiya</t>
+  </si>
+  <si>
+    <t>Trishula Shakti</t>
+  </si>
+  <si>
+    <t>Imaginary Around</t>
+  </si>
+  <si>
+    <t>Ashes of Kama</t>
+  </si>
+  <si>
+    <t>Caladbolg II</t>
+  </si>
+  <si>
+    <t>Unlimited Blade Works</t>
+  </si>
+  <si>
+    <t>Rho Aias</t>
+  </si>
+  <si>
+    <t>4,4,4</t>
   </si>
 </sst>
 </file>
@@ -1400,16 +1859,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E33D7ECC-1EAA-4A40-B4DA-A93E54CBC8B5}">
-  <dimension ref="A1:K37"/>
+  <dimension ref="A1:K60"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="17.140625" customWidth="1"/>
-    <col min="3" max="3" width="22" customWidth="1"/>
+    <col min="2" max="3" width="22" customWidth="1"/>
     <col min="4" max="4" width="12.5703125" customWidth="1"/>
     <col min="5" max="5" width="11.28515625" customWidth="1"/>
     <col min="6" max="6" width="15.5703125" customWidth="1"/>
     <col min="7" max="7" width="13.7109375" style="2" customWidth="1"/>
-    <col min="8" max="8" width="11.7109375" style="2" customWidth="1"/>
+    <col min="8" max="8" width="16.5703125" style="2" customWidth="1"/>
     <col min="9" max="9" width="11.85546875" style="2" customWidth="1"/>
     <col min="10" max="10" width="48.85546875" style="2" customWidth="1"/>
     <col min="11" max="11" width="12.5703125" customWidth="1"/>
@@ -2202,31 +2660,28 @@
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>271</v>
+        <v>323</v>
       </c>
       <c r="B26" t="s">
-        <v>272</v>
+        <v>324</v>
       </c>
       <c r="C26" t="s">
-        <v>273</v>
+        <v>325</v>
       </c>
       <c r="D26" t="s">
-        <v>88</v>
+        <v>267</v>
       </c>
       <c r="E26" t="s">
-        <v>8</v>
+        <v>99</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>27</v>
+        <v>326</v>
       </c>
       <c r="H26" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="I26" s="2" t="s">
-        <v>27</v>
+        <v>327</v>
       </c>
       <c r="J26" s="2" t="s">
-        <v>274</v>
+        <v>328</v>
       </c>
       <c r="K26" t="b">
         <v>0</v>
@@ -2234,60 +2689,60 @@
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>85</v>
+        <v>329</v>
       </c>
       <c r="B27" t="s">
-        <v>86</v>
+        <v>355</v>
       </c>
       <c r="C27" t="s">
-        <v>87</v>
+        <v>361</v>
       </c>
       <c r="D27" t="s">
-        <v>88</v>
+        <v>267</v>
       </c>
       <c r="E27" t="s">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="G27" s="2" t="s">
-        <v>15</v>
+        <v>269</v>
       </c>
       <c r="H27" s="2" t="s">
-        <v>90</v>
+        <v>204</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>42</v>
+        <v>395</v>
+      </c>
+      <c r="J27" s="2" t="s">
+        <v>200</v>
       </c>
       <c r="K27" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="28" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>275</v>
+        <v>330</v>
       </c>
       <c r="B28" t="s">
-        <v>276</v>
+        <v>356</v>
       </c>
       <c r="C28" t="s">
-        <v>277</v>
+        <v>360</v>
       </c>
       <c r="D28" t="s">
-        <v>278</v>
+        <v>267</v>
       </c>
       <c r="E28" t="s">
-        <v>8</v>
+        <v>89</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>279</v>
+        <v>100</v>
       </c>
       <c r="H28" s="2" t="s">
-        <v>204</v>
-      </c>
-      <c r="I28" s="2" t="s">
-        <v>280</v>
+        <v>182</v>
       </c>
       <c r="J28" s="2" t="s">
-        <v>43</v>
+        <v>396</v>
       </c>
       <c r="K28" t="b">
         <v>0</v>
@@ -2295,28 +2750,31 @@
     </row>
     <row r="29" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>281</v>
+        <v>331</v>
       </c>
       <c r="B29" t="s">
-        <v>249</v>
+        <v>357</v>
       </c>
       <c r="C29" t="s">
-        <v>282</v>
+        <v>359</v>
       </c>
       <c r="D29" t="s">
-        <v>20</v>
+        <v>267</v>
       </c>
       <c r="E29" t="s">
-        <v>33</v>
+        <v>8</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>201</v>
       </c>
       <c r="H29" s="2" t="s">
-        <v>27</v>
+        <v>193</v>
       </c>
       <c r="I29" s="2" t="s">
-        <v>101</v>
+        <v>15</v>
       </c>
       <c r="J29" s="2" t="s">
-        <v>283</v>
+        <v>197</v>
       </c>
       <c r="K29" t="b">
         <v>0</v>
@@ -2324,51 +2782,60 @@
     </row>
     <row r="30" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>17</v>
+        <v>332</v>
       </c>
       <c r="B30" t="s">
-        <v>18</v>
+        <v>409</v>
       </c>
       <c r="C30" t="s">
-        <v>19</v>
+        <v>358</v>
       </c>
       <c r="D30" t="s">
-        <v>20</v>
+        <v>267</v>
       </c>
       <c r="E30" t="s">
-        <v>8</v>
+        <v>99</v>
+      </c>
+      <c r="H30" s="2" t="s">
+        <v>175</v>
       </c>
       <c r="I30" s="2" t="s">
-        <v>21</v>
+        <v>176</v>
       </c>
       <c r="J30" s="2" t="s">
-        <v>22</v>
+        <v>200</v>
       </c>
       <c r="K30" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>284</v>
+        <v>333</v>
       </c>
       <c r="B31" t="s">
-        <v>285</v>
+        <v>362</v>
       </c>
       <c r="C31" t="s">
-        <v>286</v>
+        <v>363</v>
       </c>
       <c r="D31" t="s">
-        <v>20</v>
+        <v>267</v>
       </c>
       <c r="E31" t="s">
-        <v>8</v>
+        <v>89</v>
+      </c>
+      <c r="G31" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H31" s="2" t="s">
+        <v>397</v>
       </c>
       <c r="I31" s="2" t="s">
-        <v>287</v>
+        <v>15</v>
       </c>
       <c r="J31" s="2" t="s">
-        <v>177</v>
+        <v>197</v>
       </c>
       <c r="K31" t="b">
         <v>1</v>
@@ -2376,54 +2843,63 @@
     </row>
     <row r="32" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>96</v>
+        <v>334</v>
       </c>
       <c r="B32" t="s">
-        <v>97</v>
+        <v>364</v>
       </c>
       <c r="C32" t="s">
-        <v>98</v>
+        <v>365</v>
       </c>
       <c r="D32" t="s">
-        <v>20</v>
+        <v>267</v>
       </c>
       <c r="E32" t="s">
-        <v>99</v>
+        <v>8</v>
+      </c>
+      <c r="G32" s="2" t="s">
+        <v>416</v>
       </c>
       <c r="H32" s="2" t="s">
-        <v>100</v>
+        <v>193</v>
       </c>
       <c r="I32" s="2" t="s">
-        <v>101</v>
+        <v>269</v>
+      </c>
+      <c r="J32" s="2" t="s">
+        <v>194</v>
       </c>
       <c r="K32" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="33" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>314</v>
+        <v>335</v>
       </c>
       <c r="B33" t="s">
-        <v>315</v>
+        <v>366</v>
       </c>
       <c r="C33" t="s">
-        <v>316</v>
+        <v>367</v>
       </c>
       <c r="D33" t="s">
-        <v>317</v>
+        <v>267</v>
       </c>
       <c r="E33" t="s">
-        <v>33</v>
+        <v>89</v>
+      </c>
+      <c r="G33" s="2" t="s">
+        <v>27</v>
       </c>
       <c r="H33" s="2" t="s">
-        <v>21</v>
+        <v>190</v>
       </c>
       <c r="I33" s="2" t="s">
-        <v>318</v>
+        <v>27</v>
       </c>
       <c r="J33" s="2" t="s">
-        <v>319</v>
+        <v>200</v>
       </c>
       <c r="K33" t="b">
         <v>0</v>
@@ -2431,13 +2907,13 @@
     </row>
     <row r="34" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>76</v>
+        <v>336</v>
       </c>
       <c r="B34" t="s">
-        <v>77</v>
+        <v>368</v>
       </c>
       <c r="C34" t="s">
-        <v>78</v>
+        <v>369</v>
       </c>
       <c r="D34" t="s">
         <v>79</v>
@@ -2446,16 +2922,16 @@
         <v>40</v>
       </c>
       <c r="G34" s="2" t="s">
-        <v>80</v>
+        <v>191</v>
       </c>
       <c r="H34" s="2" t="s">
-        <v>15</v>
+        <v>204</v>
       </c>
       <c r="I34" s="2" t="s">
-        <v>81</v>
+        <v>27</v>
       </c>
       <c r="J34" s="2" t="s">
-        <v>322</v>
+        <v>186</v>
       </c>
       <c r="K34" t="b">
         <v>0</v>
@@ -2463,28 +2939,31 @@
     </row>
     <row r="35" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
-        <v>23</v>
+        <v>337</v>
       </c>
       <c r="B35" t="s">
-        <v>24</v>
+        <v>370</v>
       </c>
       <c r="C35" t="s">
-        <v>25</v>
+        <v>375</v>
       </c>
       <c r="D35" t="s">
-        <v>26</v>
+        <v>267</v>
       </c>
       <c r="E35" t="s">
         <v>8</v>
       </c>
       <c r="G35" s="2" t="s">
-        <v>27</v>
+        <v>100</v>
       </c>
       <c r="H35" s="2" t="s">
-        <v>28</v>
+        <v>176</v>
+      </c>
+      <c r="I35" s="2" t="s">
+        <v>326</v>
       </c>
       <c r="J35" s="2" t="s">
-        <v>70</v>
+        <v>188</v>
       </c>
       <c r="K35" t="b">
         <v>0</v>
@@ -2492,31 +2971,28 @@
     </row>
     <row r="36" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>29</v>
+        <v>338</v>
       </c>
       <c r="B36" t="s">
-        <v>30</v>
+        <v>371</v>
       </c>
       <c r="C36" t="s">
-        <v>31</v>
+        <v>374</v>
       </c>
       <c r="D36" t="s">
-        <v>32</v>
+        <v>267</v>
       </c>
       <c r="E36" t="s">
-        <v>33</v>
+        <v>89</v>
       </c>
       <c r="G36" s="2" t="s">
-        <v>15</v>
+        <v>175</v>
       </c>
       <c r="H36" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="I36" s="2" t="s">
-        <v>34</v>
+        <v>193</v>
       </c>
       <c r="J36" s="2" t="s">
-        <v>35</v>
+        <v>179</v>
       </c>
       <c r="K36" t="b">
         <v>0</v>
@@ -2524,30 +3000,727 @@
     </row>
     <row r="37" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>36</v>
+        <v>339</v>
       </c>
       <c r="B37" t="s">
-        <v>37</v>
+        <v>372</v>
       </c>
       <c r="C37" t="s">
-        <v>38</v>
+        <v>373</v>
       </c>
       <c r="D37" t="s">
-        <v>39</v>
+        <v>267</v>
       </c>
       <c r="E37" t="s">
         <v>40</v>
       </c>
       <c r="G37" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="H37" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="J37" s="2" t="s">
+        <v>432</v>
+      </c>
+      <c r="K37" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>340</v>
+      </c>
+      <c r="B38" t="s">
+        <v>376</v>
+      </c>
+      <c r="C38" t="s">
+        <v>385</v>
+      </c>
+      <c r="D38" t="s">
+        <v>267</v>
+      </c>
+      <c r="E38" t="s">
+        <v>99</v>
+      </c>
+      <c r="G38" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="H38" s="2" t="s">
+        <v>435</v>
+      </c>
+      <c r="I38" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J38" s="2" t="s">
+        <v>436</v>
+      </c>
+      <c r="K38" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>341</v>
+      </c>
+      <c r="B39" t="s">
+        <v>377</v>
+      </c>
+      <c r="C39" t="s">
+        <v>390</v>
+      </c>
+      <c r="D39" t="s">
+        <v>267</v>
+      </c>
+      <c r="E39" t="s">
+        <v>89</v>
+      </c>
+      <c r="G39" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H39" s="2" t="s">
+        <v>439</v>
+      </c>
+      <c r="J39" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="K39" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>342</v>
+      </c>
+      <c r="B40" t="s">
+        <v>378</v>
+      </c>
+      <c r="C40" t="s">
+        <v>391</v>
+      </c>
+      <c r="D40" t="s">
+        <v>267</v>
+      </c>
+      <c r="E40" t="s">
+        <v>89</v>
+      </c>
+      <c r="G40" s="2" t="s">
+        <v>442</v>
+      </c>
+      <c r="H40" s="2" t="s">
+        <v>443</v>
+      </c>
+      <c r="I40" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="J40" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="K40" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>343</v>
+      </c>
+      <c r="B41" t="s">
+        <v>379</v>
+      </c>
+      <c r="C41" t="s">
+        <v>392</v>
+      </c>
+      <c r="D41" t="s">
+        <v>267</v>
+      </c>
+      <c r="E41" t="s">
+        <v>89</v>
+      </c>
+      <c r="G41" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H41" s="2" t="s">
+        <v>446</v>
+      </c>
+      <c r="J41" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="K41" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>344</v>
+      </c>
+      <c r="B42" t="s">
+        <v>380</v>
+      </c>
+      <c r="C42" t="s">
+        <v>394</v>
+      </c>
+      <c r="D42" t="s">
+        <v>267</v>
+      </c>
+      <c r="E42" t="s">
+        <v>99</v>
+      </c>
+      <c r="G42" s="2" t="s">
+        <v>450</v>
+      </c>
+      <c r="H42" s="2" t="s">
+        <v>451</v>
+      </c>
+      <c r="I42" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="J42" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="K42" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>345</v>
+      </c>
+      <c r="B43" t="s">
+        <v>381</v>
+      </c>
+      <c r="C43" t="s">
+        <v>386</v>
+      </c>
+      <c r="D43" t="s">
+        <v>267</v>
+      </c>
+      <c r="E43" t="s">
+        <v>40</v>
+      </c>
+      <c r="G43" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="H43" s="2" t="s">
+        <v>454</v>
+      </c>
+      <c r="I43" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="J43" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="K43" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>346</v>
+      </c>
+      <c r="B44" t="s">
+        <v>382</v>
+      </c>
+      <c r="C44" t="s">
+        <v>387</v>
+      </c>
+      <c r="D44" t="s">
+        <v>267</v>
+      </c>
+      <c r="E44" t="s">
+        <v>40</v>
+      </c>
+      <c r="G44" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="H44" s="2" t="s">
+        <v>192</v>
+      </c>
+      <c r="I44" s="2" t="s">
+        <v>206</v>
+      </c>
+      <c r="J44" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="K44" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>347</v>
+      </c>
+      <c r="B45" t="s">
+        <v>383</v>
+      </c>
+      <c r="C45" t="s">
+        <v>393</v>
+      </c>
+      <c r="D45" t="s">
+        <v>267</v>
+      </c>
+      <c r="E45" t="s">
+        <v>89</v>
+      </c>
+      <c r="G45" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="H45" s="2" t="s">
+        <v>460</v>
+      </c>
+      <c r="I45" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="J45" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="K45" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>348</v>
+      </c>
+      <c r="B46" t="s">
+        <v>462</v>
+      </c>
+      <c r="C46" t="s">
+        <v>388</v>
+      </c>
+      <c r="D46" t="s">
+        <v>267</v>
+      </c>
+      <c r="E46" t="s">
+        <v>89</v>
+      </c>
+      <c r="G46" s="2" t="s">
+        <v>443</v>
+      </c>
+      <c r="H46" s="2" t="s">
+        <v>461</v>
+      </c>
+      <c r="I46" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J46" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="K46" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>349</v>
+      </c>
+      <c r="B47" t="s">
+        <v>384</v>
+      </c>
+      <c r="C47" t="s">
+        <v>389</v>
+      </c>
+      <c r="D47" t="s">
+        <v>267</v>
+      </c>
+      <c r="E47" t="s">
+        <v>89</v>
+      </c>
+      <c r="G47" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H47" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="I47" s="2" t="s">
+        <v>475</v>
+      </c>
+      <c r="J47" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="K47" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>466</v>
+      </c>
+      <c r="B48" t="s">
+        <v>467</v>
+      </c>
+      <c r="C48" t="s">
+        <v>468</v>
+      </c>
+      <c r="D48" t="s">
+        <v>88</v>
+      </c>
+      <c r="E48" t="s">
+        <v>99</v>
+      </c>
+      <c r="G48" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H48" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="I48" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="J48" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K48" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>271</v>
+      </c>
+      <c r="B49" t="s">
+        <v>272</v>
+      </c>
+      <c r="C49" t="s">
+        <v>273</v>
+      </c>
+      <c r="D49" t="s">
+        <v>88</v>
+      </c>
+      <c r="E49" t="s">
+        <v>8</v>
+      </c>
+      <c r="G49" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H49" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I49" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="J49" s="2" t="s">
+        <v>274</v>
+      </c>
+      <c r="K49" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>85</v>
+      </c>
+      <c r="B50" t="s">
+        <v>86</v>
+      </c>
+      <c r="C50" t="s">
+        <v>87</v>
+      </c>
+      <c r="D50" t="s">
+        <v>88</v>
+      </c>
+      <c r="E50" t="s">
+        <v>89</v>
+      </c>
+      <c r="G50" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H50" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="I50" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="K50" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>275</v>
+      </c>
+      <c r="B51" t="s">
+        <v>276</v>
+      </c>
+      <c r="C51" t="s">
+        <v>277</v>
+      </c>
+      <c r="D51" t="s">
+        <v>278</v>
+      </c>
+      <c r="E51" t="s">
+        <v>8</v>
+      </c>
+      <c r="G51" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="H51" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="I51" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="J51" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="K51" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>281</v>
+      </c>
+      <c r="B52" t="s">
+        <v>249</v>
+      </c>
+      <c r="C52" t="s">
+        <v>282</v>
+      </c>
+      <c r="D52" t="s">
+        <v>20</v>
+      </c>
+      <c r="E52" t="s">
+        <v>33</v>
+      </c>
+      <c r="H52" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I52" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="J52" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="K52" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>17</v>
+      </c>
+      <c r="B53" t="s">
+        <v>18</v>
+      </c>
+      <c r="C53" t="s">
+        <v>19</v>
+      </c>
+      <c r="D53" t="s">
+        <v>20</v>
+      </c>
+      <c r="E53" t="s">
+        <v>8</v>
+      </c>
+      <c r="I53" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="J53" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K53" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>284</v>
+      </c>
+      <c r="B54" t="s">
+        <v>285</v>
+      </c>
+      <c r="C54" t="s">
+        <v>286</v>
+      </c>
+      <c r="D54" t="s">
+        <v>20</v>
+      </c>
+      <c r="E54" t="s">
+        <v>8</v>
+      </c>
+      <c r="I54" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="J54" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="K54" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>96</v>
+      </c>
+      <c r="B55" t="s">
+        <v>97</v>
+      </c>
+      <c r="C55" t="s">
+        <v>98</v>
+      </c>
+      <c r="D55" t="s">
+        <v>20</v>
+      </c>
+      <c r="E55" t="s">
+        <v>99</v>
+      </c>
+      <c r="H55" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="I55" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="K55" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>314</v>
+      </c>
+      <c r="B56" t="s">
+        <v>315</v>
+      </c>
+      <c r="C56" t="s">
+        <v>316</v>
+      </c>
+      <c r="D56" t="s">
+        <v>317</v>
+      </c>
+      <c r="E56" t="s">
+        <v>33</v>
+      </c>
+      <c r="H56" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="I56" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="J56" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="K56" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>76</v>
+      </c>
+      <c r="B57" t="s">
+        <v>77</v>
+      </c>
+      <c r="C57" t="s">
+        <v>78</v>
+      </c>
+      <c r="D57" t="s">
+        <v>79</v>
+      </c>
+      <c r="E57" t="s">
+        <v>40</v>
+      </c>
+      <c r="G57" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="H57" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I57" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="J57" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="K57" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>23</v>
+      </c>
+      <c r="B58" t="s">
+        <v>24</v>
+      </c>
+      <c r="C58" t="s">
+        <v>25</v>
+      </c>
+      <c r="D58" t="s">
+        <v>26</v>
+      </c>
+      <c r="E58" t="s">
+        <v>8</v>
+      </c>
+      <c r="G58" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H58" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="J58" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="K58" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>29</v>
+      </c>
+      <c r="B59" t="s">
+        <v>30</v>
+      </c>
+      <c r="C59" t="s">
+        <v>31</v>
+      </c>
+      <c r="D59" t="s">
+        <v>32</v>
+      </c>
+      <c r="E59" t="s">
+        <v>33</v>
+      </c>
+      <c r="G59" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H59" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="I59" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="J59" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="K59" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>36</v>
+      </c>
+      <c r="B60" t="s">
+        <v>37</v>
+      </c>
+      <c r="C60" t="s">
+        <v>38</v>
+      </c>
+      <c r="D60" t="s">
+        <v>39</v>
+      </c>
+      <c r="E60" t="s">
+        <v>40</v>
+      </c>
+      <c r="G60" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="H37" s="2" t="s">
+      <c r="H60" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="J37" s="2" t="s">
+      <c r="J60" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="K37" t="b">
+      <c r="K60" t="b">
         <v>1</v>
       </c>
     </row>
@@ -2555,19 +3728,20 @@
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="H2 I34 H36 I6:I7 I10 I12 H14 I18 I22 I24" numberStoredAsText="1"/>
+    <ignoredError sqref="H2 I6:I7 I10 I12 H14 I18 I22 I24 I27 G34 I40 I42 I45" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1BC60D8-44F3-478D-BCC0-4752624457AE}">
-  <dimension ref="A1:F18"/>
+  <dimension ref="A1:F21"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="19" customWidth="1"/>
-    <col min="3" max="3" width="15.140625" customWidth="1"/>
-    <col min="4" max="5" width="16.42578125" customWidth="1"/>
+    <col min="3" max="3" width="25.5703125" customWidth="1"/>
+    <col min="4" max="4" width="23.42578125" customWidth="1"/>
+    <col min="5" max="5" width="16.42578125" customWidth="1"/>
     <col min="6" max="6" width="13.5703125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2644,104 +3818,104 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>85</v>
+        <v>333</v>
       </c>
       <c r="B5" t="s">
-        <v>86</v>
+        <v>362</v>
       </c>
       <c r="C5" t="s">
-        <v>91</v>
+        <v>398</v>
       </c>
       <c r="D5" t="s">
-        <v>92</v>
+        <v>401</v>
       </c>
       <c r="E5">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>17</v>
+        <v>333</v>
       </c>
       <c r="B6" t="s">
-        <v>18</v>
+        <v>362</v>
       </c>
       <c r="C6" t="s">
-        <v>47</v>
+        <v>399</v>
       </c>
       <c r="D6" t="s">
-        <v>72</v>
+        <v>402</v>
       </c>
       <c r="E6">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>17</v>
+        <v>333</v>
       </c>
       <c r="B7" t="s">
-        <v>18</v>
+        <v>362</v>
       </c>
       <c r="C7" t="s">
-        <v>73</v>
+        <v>400</v>
       </c>
       <c r="D7" t="s">
-        <v>74</v>
+        <v>403</v>
       </c>
       <c r="E7">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>284</v>
+        <v>85</v>
       </c>
       <c r="B8" t="s">
-        <v>285</v>
+        <v>86</v>
       </c>
       <c r="C8" t="s">
-        <v>288</v>
+        <v>91</v>
       </c>
       <c r="D8" t="s">
-        <v>295</v>
+        <v>92</v>
       </c>
       <c r="E8">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>284</v>
+        <v>17</v>
       </c>
       <c r="B9" t="s">
-        <v>285</v>
+        <v>18</v>
       </c>
       <c r="C9" t="s">
-        <v>289</v>
+        <v>47</v>
       </c>
       <c r="D9" t="s">
-        <v>296</v>
+        <v>72</v>
       </c>
       <c r="E9">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>284</v>
+        <v>17</v>
       </c>
       <c r="B10" t="s">
-        <v>285</v>
+        <v>18</v>
       </c>
       <c r="C10" t="s">
-        <v>290</v>
+        <v>73</v>
       </c>
       <c r="D10" t="s">
-        <v>297</v>
+        <v>74</v>
       </c>
       <c r="E10">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -2752,10 +3926,10 @@
         <v>285</v>
       </c>
       <c r="C11" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="D11" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="E11">
         <v>1</v>
@@ -2769,10 +3943,10 @@
         <v>285</v>
       </c>
       <c r="C12" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="D12" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="E12">
         <v>1</v>
@@ -2786,10 +3960,10 @@
         <v>285</v>
       </c>
       <c r="C13" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="D13" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="E13">
         <v>1</v>
@@ -2803,10 +3977,10 @@
         <v>285</v>
       </c>
       <c r="C14" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="D14" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="E14">
         <v>1</v>
@@ -2814,16 +3988,16 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>96</v>
+        <v>284</v>
       </c>
       <c r="B15" t="s">
-        <v>97</v>
+        <v>285</v>
       </c>
       <c r="C15" t="s">
-        <v>102</v>
+        <v>292</v>
       </c>
       <c r="D15" t="s">
-        <v>105</v>
+        <v>299</v>
       </c>
       <c r="E15">
         <v>1</v>
@@ -2831,16 +4005,16 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>96</v>
+        <v>284</v>
       </c>
       <c r="B16" t="s">
-        <v>97</v>
+        <v>285</v>
       </c>
       <c r="C16" t="s">
-        <v>103</v>
+        <v>293</v>
       </c>
       <c r="D16" t="s">
-        <v>106</v>
+        <v>300</v>
       </c>
       <c r="E16">
         <v>1</v>
@@ -2848,16 +4022,16 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>96</v>
+        <v>284</v>
       </c>
       <c r="B17" t="s">
-        <v>97</v>
+        <v>285</v>
       </c>
       <c r="C17" t="s">
-        <v>104</v>
+        <v>294</v>
       </c>
       <c r="D17" t="s">
-        <v>107</v>
+        <v>301</v>
       </c>
       <c r="E17">
         <v>1</v>
@@ -2865,18 +4039,69 @@
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>96</v>
+      </c>
+      <c r="B18" t="s">
+        <v>97</v>
+      </c>
+      <c r="C18" t="s">
+        <v>102</v>
+      </c>
+      <c r="D18" t="s">
+        <v>105</v>
+      </c>
+      <c r="E18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>96</v>
+      </c>
+      <c r="B19" t="s">
+        <v>97</v>
+      </c>
+      <c r="C19" t="s">
+        <v>103</v>
+      </c>
+      <c r="D19" t="s">
+        <v>106</v>
+      </c>
+      <c r="E19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>96</v>
+      </c>
+      <c r="B20" t="s">
+        <v>97</v>
+      </c>
+      <c r="C20" t="s">
+        <v>104</v>
+      </c>
+      <c r="D20" t="s">
+        <v>107</v>
+      </c>
+      <c r="E20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
         <v>36</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B21" t="s">
         <v>37</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C21" t="s">
         <v>48</v>
       </c>
-      <c r="D18" t="s">
+      <c r="D21" t="s">
         <v>48</v>
       </c>
-      <c r="E18">
+      <c r="E21">
         <v>2</v>
       </c>
     </row>
@@ -2889,13 +4114,13 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84E3BB0D-5578-4069-B1C9-C3864EB2A429}">
-  <dimension ref="A1:F109"/>
+  <dimension ref="A1:F178"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="20.5703125" customWidth="1"/>
     <col min="3" max="3" width="12.7109375" customWidth="1"/>
     <col min="4" max="4" width="17" customWidth="1"/>
-    <col min="5" max="5" width="21.5703125" customWidth="1"/>
+    <col min="5" max="5" width="23.5703125" customWidth="1"/>
     <col min="6" max="6" width="15.7109375" customWidth="1"/>
   </cols>
   <sheetData>
@@ -4145,10 +5370,10 @@
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
-        <v>271</v>
+        <v>323</v>
       </c>
       <c r="B74" t="s">
-        <v>272</v>
+        <v>324</v>
       </c>
       <c r="C74">
         <v>1</v>
@@ -4157,15 +5382,15 @@
         <v>1</v>
       </c>
       <c r="E74" t="s">
-        <v>93</v>
+        <v>302</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
-        <v>271</v>
+        <v>323</v>
       </c>
       <c r="B75" t="s">
-        <v>272</v>
+        <v>324</v>
       </c>
       <c r="C75">
         <v>2</v>
@@ -4174,15 +5399,15 @@
         <v>0</v>
       </c>
       <c r="E75" t="s">
-        <v>304</v>
+        <v>350</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
-        <v>271</v>
+        <v>323</v>
       </c>
       <c r="B76" t="s">
-        <v>272</v>
+        <v>324</v>
       </c>
       <c r="C76">
         <v>3</v>
@@ -4191,32 +5416,32 @@
         <v>0</v>
       </c>
       <c r="E76" t="s">
-        <v>305</v>
+        <v>351</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
-        <v>85</v>
+        <v>329</v>
       </c>
       <c r="B77" t="s">
-        <v>86</v>
+        <v>355</v>
       </c>
       <c r="C77">
         <v>1</v>
       </c>
       <c r="D77" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E77" t="s">
-        <v>93</v>
+        <v>352</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
-        <v>85</v>
+        <v>329</v>
       </c>
       <c r="B78" t="s">
-        <v>86</v>
+        <v>355</v>
       </c>
       <c r="C78">
         <v>2</v>
@@ -4225,15 +5450,15 @@
         <v>0</v>
       </c>
       <c r="E78" t="s">
-        <v>94</v>
+        <v>353</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
-        <v>85</v>
+        <v>329</v>
       </c>
       <c r="B79" t="s">
-        <v>86</v>
+        <v>355</v>
       </c>
       <c r="C79">
         <v>3</v>
@@ -4242,15 +5467,15 @@
         <v>0</v>
       </c>
       <c r="E79" t="s">
-        <v>95</v>
+        <v>354</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
-        <v>275</v>
+        <v>330</v>
       </c>
       <c r="B80" t="s">
-        <v>276</v>
+        <v>356</v>
       </c>
       <c r="C80">
         <v>1</v>
@@ -4259,15 +5484,15 @@
         <v>1</v>
       </c>
       <c r="E80" t="s">
-        <v>306</v>
+        <v>302</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>275</v>
+        <v>330</v>
       </c>
       <c r="B81" t="s">
-        <v>276</v>
+        <v>356</v>
       </c>
       <c r="C81">
         <v>2</v>
@@ -4276,15 +5501,15 @@
         <v>0</v>
       </c>
       <c r="E81" t="s">
-        <v>307</v>
+        <v>404</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
-        <v>275</v>
+        <v>330</v>
       </c>
       <c r="B82" t="s">
-        <v>276</v>
+        <v>356</v>
       </c>
       <c r="C82">
         <v>3</v>
@@ -4293,32 +5518,32 @@
         <v>0</v>
       </c>
       <c r="E82" t="s">
-        <v>308</v>
+        <v>405</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
-        <v>281</v>
+        <v>331</v>
       </c>
       <c r="B83" t="s">
-        <v>249</v>
+        <v>357</v>
       </c>
       <c r="C83">
         <v>1</v>
       </c>
       <c r="D83" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E83" t="s">
-        <v>58</v>
+        <v>406</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
-        <v>281</v>
+        <v>331</v>
       </c>
       <c r="B84" t="s">
-        <v>249</v>
+        <v>357</v>
       </c>
       <c r="C84">
         <v>2</v>
@@ -4327,15 +5552,15 @@
         <v>0</v>
       </c>
       <c r="E84" t="s">
-        <v>309</v>
+        <v>407</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
-        <v>281</v>
+        <v>331</v>
       </c>
       <c r="B85" t="s">
-        <v>249</v>
+        <v>357</v>
       </c>
       <c r="C85">
         <v>3</v>
@@ -4344,32 +5569,32 @@
         <v>0</v>
       </c>
       <c r="E85" t="s">
-        <v>310</v>
+        <v>408</v>
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
-        <v>17</v>
+        <v>332</v>
       </c>
       <c r="B86" t="s">
-        <v>18</v>
+        <v>409</v>
       </c>
       <c r="C86">
         <v>1</v>
       </c>
       <c r="D86" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E86" t="s">
-        <v>58</v>
+        <v>410</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
-        <v>17</v>
+        <v>332</v>
       </c>
       <c r="B87" t="s">
-        <v>18</v>
+        <v>409</v>
       </c>
       <c r="C87">
         <v>2</v>
@@ -4378,15 +5603,15 @@
         <v>0</v>
       </c>
       <c r="E87" t="s">
-        <v>59</v>
+        <v>411</v>
       </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>17</v>
+        <v>332</v>
       </c>
       <c r="B88" t="s">
-        <v>18</v>
+        <v>409</v>
       </c>
       <c r="C88">
         <v>3</v>
@@ -4395,15 +5620,15 @@
         <v>0</v>
       </c>
       <c r="E88" t="s">
-        <v>60</v>
+        <v>412</v>
       </c>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
-        <v>284</v>
+        <v>333</v>
       </c>
       <c r="B89" t="s">
-        <v>285</v>
+        <v>362</v>
       </c>
       <c r="C89">
         <v>1</v>
@@ -4412,15 +5637,15 @@
         <v>0</v>
       </c>
       <c r="E89" t="s">
-        <v>311</v>
+        <v>413</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
-        <v>284</v>
+        <v>333</v>
       </c>
       <c r="B90" t="s">
-        <v>285</v>
+        <v>362</v>
       </c>
       <c r="C90">
         <v>2</v>
@@ -4429,15 +5654,15 @@
         <v>0</v>
       </c>
       <c r="E90" t="s">
-        <v>312</v>
+        <v>414</v>
       </c>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
-        <v>284</v>
+        <v>333</v>
       </c>
       <c r="B91" t="s">
-        <v>285</v>
+        <v>362</v>
       </c>
       <c r="C91">
         <v>3</v>
@@ -4446,32 +5671,32 @@
         <v>0</v>
       </c>
       <c r="E91" t="s">
-        <v>313</v>
+        <v>415</v>
       </c>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
-        <v>96</v>
+        <v>334</v>
       </c>
       <c r="B92" t="s">
-        <v>97</v>
+        <v>364</v>
       </c>
       <c r="C92">
         <v>1</v>
       </c>
       <c r="D92" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E92" t="s">
-        <v>108</v>
+        <v>302</v>
       </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
-        <v>96</v>
+        <v>334</v>
       </c>
       <c r="B93" t="s">
-        <v>97</v>
+        <v>364</v>
       </c>
       <c r="C93">
         <v>2</v>
@@ -4480,15 +5705,15 @@
         <v>0</v>
       </c>
       <c r="E93" t="s">
-        <v>109</v>
+        <v>417</v>
       </c>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
-        <v>96</v>
+        <v>334</v>
       </c>
       <c r="B94" t="s">
-        <v>97</v>
+        <v>364</v>
       </c>
       <c r="C94">
         <v>3</v>
@@ -4497,15 +5722,15 @@
         <v>0</v>
       </c>
       <c r="E94" t="s">
-        <v>110</v>
+        <v>418</v>
       </c>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
-        <v>314</v>
+        <v>335</v>
       </c>
       <c r="B95" t="s">
-        <v>315</v>
+        <v>366</v>
       </c>
       <c r="C95">
         <v>1</v>
@@ -4514,32 +5739,32 @@
         <v>1</v>
       </c>
       <c r="E95" t="s">
-        <v>320</v>
+        <v>302</v>
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
-        <v>314</v>
+        <v>335</v>
       </c>
       <c r="B96" t="s">
-        <v>315</v>
+        <v>366</v>
       </c>
       <c r="C96">
         <v>2</v>
       </c>
       <c r="D96" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E96" t="s">
-        <v>58</v>
+        <v>419</v>
       </c>
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
-        <v>314</v>
+        <v>335</v>
       </c>
       <c r="B97" t="s">
-        <v>315</v>
+        <v>366</v>
       </c>
       <c r="C97">
         <v>3</v>
@@ -4548,15 +5773,15 @@
         <v>0</v>
       </c>
       <c r="E97" t="s">
-        <v>321</v>
+        <v>420</v>
       </c>
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
-        <v>76</v>
+        <v>336</v>
       </c>
       <c r="B98" t="s">
-        <v>77</v>
+        <v>368</v>
       </c>
       <c r="C98">
         <v>1</v>
@@ -4570,10 +5795,10 @@
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
-        <v>76</v>
+        <v>336</v>
       </c>
       <c r="B99" t="s">
-        <v>77</v>
+        <v>368</v>
       </c>
       <c r="C99">
         <v>2</v>
@@ -4582,15 +5807,15 @@
         <v>0</v>
       </c>
       <c r="E99" t="s">
-        <v>83</v>
+        <v>421</v>
       </c>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
-        <v>76</v>
+        <v>336</v>
       </c>
       <c r="B100" t="s">
-        <v>77</v>
+        <v>368</v>
       </c>
       <c r="C100">
         <v>3</v>
@@ -4599,32 +5824,32 @@
         <v>0</v>
       </c>
       <c r="E100" t="s">
-        <v>84</v>
+        <v>422</v>
       </c>
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
-        <v>23</v>
+        <v>337</v>
       </c>
       <c r="B101" t="s">
-        <v>24</v>
+        <v>370</v>
       </c>
       <c r="C101">
         <v>1</v>
       </c>
       <c r="D101" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E101" t="s">
-        <v>61</v>
+        <v>302</v>
       </c>
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
-        <v>23</v>
+        <v>337</v>
       </c>
       <c r="B102" t="s">
-        <v>24</v>
+        <v>370</v>
       </c>
       <c r="C102">
         <v>2</v>
@@ -4633,15 +5858,15 @@
         <v>0</v>
       </c>
       <c r="E102" t="s">
-        <v>62</v>
+        <v>423</v>
       </c>
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
-        <v>23</v>
+        <v>337</v>
       </c>
       <c r="B103" t="s">
-        <v>24</v>
+        <v>370</v>
       </c>
       <c r="C103">
         <v>3</v>
@@ -4650,15 +5875,15 @@
         <v>0</v>
       </c>
       <c r="E103" t="s">
-        <v>63</v>
+        <v>424</v>
       </c>
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
-        <v>29</v>
+        <v>338</v>
       </c>
       <c r="B104" t="s">
-        <v>30</v>
+        <v>371</v>
       </c>
       <c r="C104">
         <v>1</v>
@@ -4667,15 +5892,15 @@
         <v>0</v>
       </c>
       <c r="E104" t="s">
-        <v>64</v>
+        <v>425</v>
       </c>
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
-        <v>29</v>
+        <v>338</v>
       </c>
       <c r="B105" t="s">
-        <v>30</v>
+        <v>371</v>
       </c>
       <c r="C105">
         <v>2</v>
@@ -4684,15 +5909,15 @@
         <v>0</v>
       </c>
       <c r="E105" t="s">
-        <v>65</v>
+        <v>426</v>
       </c>
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
-        <v>29</v>
+        <v>338</v>
       </c>
       <c r="B106" t="s">
-        <v>30</v>
+        <v>371</v>
       </c>
       <c r="C106">
         <v>3</v>
@@ -4701,15 +5926,15 @@
         <v>0</v>
       </c>
       <c r="E106" t="s">
-        <v>66</v>
+        <v>427</v>
       </c>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
-        <v>36</v>
+        <v>339</v>
       </c>
       <c r="B107" t="s">
-        <v>37</v>
+        <v>372</v>
       </c>
       <c r="C107">
         <v>1</v>
@@ -4718,15 +5943,15 @@
         <v>0</v>
       </c>
       <c r="E107" t="s">
-        <v>67</v>
+        <v>428</v>
       </c>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>36</v>
+        <v>339</v>
       </c>
       <c r="B108" t="s">
-        <v>37</v>
+        <v>372</v>
       </c>
       <c r="C108">
         <v>2</v>
@@ -4735,15 +5960,15 @@
         <v>0</v>
       </c>
       <c r="E108" t="s">
-        <v>68</v>
+        <v>429</v>
       </c>
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
-        <v>36</v>
+        <v>339</v>
       </c>
       <c r="B109" t="s">
-        <v>37</v>
+        <v>372</v>
       </c>
       <c r="C109">
         <v>3</v>
@@ -4752,6 +5977,1179 @@
         <v>0</v>
       </c>
       <c r="E109" t="s">
+        <v>430</v>
+      </c>
+    </row>
+    <row r="110" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>340</v>
+      </c>
+      <c r="B110" t="s">
+        <v>376</v>
+      </c>
+      <c r="C110">
+        <v>1</v>
+      </c>
+      <c r="D110" t="b">
+        <v>1</v>
+      </c>
+      <c r="E110" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="111" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>340</v>
+      </c>
+      <c r="B111" t="s">
+        <v>376</v>
+      </c>
+      <c r="C111">
+        <v>2</v>
+      </c>
+      <c r="D111" t="b">
+        <v>0</v>
+      </c>
+      <c r="E111" t="s">
+        <v>433</v>
+      </c>
+    </row>
+    <row r="112" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>340</v>
+      </c>
+      <c r="B112" t="s">
+        <v>376</v>
+      </c>
+      <c r="C112">
+        <v>3</v>
+      </c>
+      <c r="D112" t="b">
+        <v>0</v>
+      </c>
+      <c r="E112" t="s">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="113" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>341</v>
+      </c>
+      <c r="B113" t="s">
+        <v>377</v>
+      </c>
+      <c r="C113">
+        <v>1</v>
+      </c>
+      <c r="D113" t="b">
+        <v>1</v>
+      </c>
+      <c r="E113" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="114" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>341</v>
+      </c>
+      <c r="B114" t="s">
+        <v>377</v>
+      </c>
+      <c r="C114">
+        <v>2</v>
+      </c>
+      <c r="D114" t="b">
+        <v>0</v>
+      </c>
+      <c r="E114" t="s">
+        <v>437</v>
+      </c>
+    </row>
+    <row r="115" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>341</v>
+      </c>
+      <c r="B115" t="s">
+        <v>377</v>
+      </c>
+      <c r="C115">
+        <v>3</v>
+      </c>
+      <c r="D115" t="b">
+        <v>0</v>
+      </c>
+      <c r="E115" t="s">
+        <v>438</v>
+      </c>
+    </row>
+    <row r="116" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>342</v>
+      </c>
+      <c r="B116" t="s">
+        <v>378</v>
+      </c>
+      <c r="C116">
+        <v>1</v>
+      </c>
+      <c r="D116" t="b">
+        <v>1</v>
+      </c>
+      <c r="E116" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="117" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>342</v>
+      </c>
+      <c r="B117" t="s">
+        <v>378</v>
+      </c>
+      <c r="C117">
+        <v>2</v>
+      </c>
+      <c r="D117" t="b">
+        <v>0</v>
+      </c>
+      <c r="E117" t="s">
+        <v>440</v>
+      </c>
+    </row>
+    <row r="118" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>342</v>
+      </c>
+      <c r="B118" t="s">
+        <v>378</v>
+      </c>
+      <c r="C118">
+        <v>3</v>
+      </c>
+      <c r="D118" t="b">
+        <v>0</v>
+      </c>
+      <c r="E118" t="s">
+        <v>441</v>
+      </c>
+    </row>
+    <row r="119" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>343</v>
+      </c>
+      <c r="B119" t="s">
+        <v>379</v>
+      </c>
+      <c r="C119">
+        <v>1</v>
+      </c>
+      <c r="D119" t="b">
+        <v>1</v>
+      </c>
+      <c r="E119" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="120" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>343</v>
+      </c>
+      <c r="B120" t="s">
+        <v>379</v>
+      </c>
+      <c r="C120">
+        <v>2</v>
+      </c>
+      <c r="D120" t="b">
+        <v>0</v>
+      </c>
+      <c r="E120" t="s">
+        <v>444</v>
+      </c>
+    </row>
+    <row r="121" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>343</v>
+      </c>
+      <c r="B121" t="s">
+        <v>379</v>
+      </c>
+      <c r="C121">
+        <v>3</v>
+      </c>
+      <c r="D121" t="b">
+        <v>0</v>
+      </c>
+      <c r="E121" t="s">
+        <v>445</v>
+      </c>
+    </row>
+    <row r="122" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>344</v>
+      </c>
+      <c r="B122" t="s">
+        <v>380</v>
+      </c>
+      <c r="C122">
+        <v>1</v>
+      </c>
+      <c r="D122" t="b">
+        <v>0</v>
+      </c>
+      <c r="E122" t="s">
+        <v>447</v>
+      </c>
+    </row>
+    <row r="123" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>344</v>
+      </c>
+      <c r="B123" t="s">
+        <v>380</v>
+      </c>
+      <c r="C123">
+        <v>2</v>
+      </c>
+      <c r="D123" t="b">
+        <v>0</v>
+      </c>
+      <c r="E123" t="s">
+        <v>448</v>
+      </c>
+    </row>
+    <row r="124" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>344</v>
+      </c>
+      <c r="B124" t="s">
+        <v>380</v>
+      </c>
+      <c r="C124">
+        <v>3</v>
+      </c>
+      <c r="D124" t="b">
+        <v>0</v>
+      </c>
+      <c r="E124" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="125" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>345</v>
+      </c>
+      <c r="B125" t="s">
+        <v>381</v>
+      </c>
+      <c r="C125">
+        <v>1</v>
+      </c>
+      <c r="D125" t="b">
+        <v>1</v>
+      </c>
+      <c r="E125" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="126" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A126" t="s">
+        <v>345</v>
+      </c>
+      <c r="B126" t="s">
+        <v>381</v>
+      </c>
+      <c r="C126">
+        <v>2</v>
+      </c>
+      <c r="D126" t="b">
+        <v>0</v>
+      </c>
+      <c r="E126" t="s">
+        <v>452</v>
+      </c>
+    </row>
+    <row r="127" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A127" t="s">
+        <v>345</v>
+      </c>
+      <c r="B127" t="s">
+        <v>381</v>
+      </c>
+      <c r="C127">
+        <v>3</v>
+      </c>
+      <c r="D127" t="b">
+        <v>0</v>
+      </c>
+      <c r="E127" t="s">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="128" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A128" t="s">
+        <v>346</v>
+      </c>
+      <c r="B128" t="s">
+        <v>382</v>
+      </c>
+      <c r="C128">
+        <v>1</v>
+      </c>
+      <c r="D128" t="b">
+        <v>0</v>
+      </c>
+      <c r="E128" t="s">
+        <v>455</v>
+      </c>
+    </row>
+    <row r="129" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A129" t="s">
+        <v>346</v>
+      </c>
+      <c r="B129" t="s">
+        <v>382</v>
+      </c>
+      <c r="C129">
+        <v>2</v>
+      </c>
+      <c r="D129" t="b">
+        <v>0</v>
+      </c>
+      <c r="E129" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="130" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A130" t="s">
+        <v>346</v>
+      </c>
+      <c r="B130" t="s">
+        <v>382</v>
+      </c>
+      <c r="C130">
+        <v>3</v>
+      </c>
+      <c r="D130" t="b">
+        <v>0</v>
+      </c>
+      <c r="E130" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="131" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A131" t="s">
+        <v>347</v>
+      </c>
+      <c r="B131" t="s">
+        <v>383</v>
+      </c>
+      <c r="C131">
+        <v>1</v>
+      </c>
+      <c r="D131" t="b">
+        <v>1</v>
+      </c>
+      <c r="E131" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="132" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A132" t="s">
+        <v>347</v>
+      </c>
+      <c r="B132" t="s">
+        <v>383</v>
+      </c>
+      <c r="C132">
+        <v>2</v>
+      </c>
+      <c r="D132" t="b">
+        <v>0</v>
+      </c>
+      <c r="E132" t="s">
+        <v>458</v>
+      </c>
+    </row>
+    <row r="133" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A133" t="s">
+        <v>347</v>
+      </c>
+      <c r="B133" t="s">
+        <v>383</v>
+      </c>
+      <c r="C133">
+        <v>3</v>
+      </c>
+      <c r="D133" t="b">
+        <v>0</v>
+      </c>
+      <c r="E133" t="s">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="134" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A134" t="s">
+        <v>348</v>
+      </c>
+      <c r="B134" t="s">
+        <v>462</v>
+      </c>
+      <c r="C134">
+        <v>1</v>
+      </c>
+      <c r="D134" t="b">
+        <v>0</v>
+      </c>
+      <c r="E134" t="s">
+        <v>463</v>
+      </c>
+    </row>
+    <row r="135" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A135" t="s">
+        <v>348</v>
+      </c>
+      <c r="B135" t="s">
+        <v>462</v>
+      </c>
+      <c r="C135">
+        <v>2</v>
+      </c>
+      <c r="D135" t="b">
+        <v>0</v>
+      </c>
+      <c r="E135" t="s">
+        <v>464</v>
+      </c>
+    </row>
+    <row r="136" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A136" t="s">
+        <v>348</v>
+      </c>
+      <c r="B136" t="s">
+        <v>462</v>
+      </c>
+      <c r="C136">
+        <v>3</v>
+      </c>
+      <c r="D136" t="b">
+        <v>0</v>
+      </c>
+      <c r="E136" t="s">
+        <v>465</v>
+      </c>
+    </row>
+    <row r="137" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A137" t="s">
+        <v>349</v>
+      </c>
+      <c r="B137" t="s">
+        <v>384</v>
+      </c>
+      <c r="C137">
+        <v>1</v>
+      </c>
+      <c r="D137" t="b">
+        <v>0</v>
+      </c>
+      <c r="E137" t="s">
+        <v>469</v>
+      </c>
+    </row>
+    <row r="138" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A138" t="s">
+        <v>349</v>
+      </c>
+      <c r="B138" t="s">
+        <v>384</v>
+      </c>
+      <c r="C138">
+        <v>2</v>
+      </c>
+      <c r="D138" t="b">
+        <v>0</v>
+      </c>
+      <c r="E138" t="s">
+        <v>470</v>
+      </c>
+    </row>
+    <row r="139" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A139" t="s">
+        <v>349</v>
+      </c>
+      <c r="B139" t="s">
+        <v>384</v>
+      </c>
+      <c r="C139">
+        <v>3</v>
+      </c>
+      <c r="D139" t="b">
+        <v>0</v>
+      </c>
+      <c r="E139" t="s">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="140" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A140" t="s">
+        <v>466</v>
+      </c>
+      <c r="B140" t="s">
+        <v>467</v>
+      </c>
+      <c r="C140">
+        <v>1</v>
+      </c>
+      <c r="D140" t="b">
+        <v>0</v>
+      </c>
+      <c r="E140" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="141" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A141" t="s">
+        <v>466</v>
+      </c>
+      <c r="B141" t="s">
+        <v>467</v>
+      </c>
+      <c r="C141">
+        <v>2</v>
+      </c>
+      <c r="D141" t="b">
+        <v>0</v>
+      </c>
+      <c r="E141" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="142" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A142" t="s">
+        <v>466</v>
+      </c>
+      <c r="B142" t="s">
+        <v>467</v>
+      </c>
+      <c r="C142">
+        <v>3</v>
+      </c>
+      <c r="D142" t="b">
+        <v>0</v>
+      </c>
+      <c r="E142" t="s">
+        <v>474</v>
+      </c>
+    </row>
+    <row r="143" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A143" t="s">
+        <v>271</v>
+      </c>
+      <c r="B143" t="s">
+        <v>272</v>
+      </c>
+      <c r="C143">
+        <v>1</v>
+      </c>
+      <c r="D143" t="b">
+        <v>1</v>
+      </c>
+      <c r="E143" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="144" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A144" t="s">
+        <v>271</v>
+      </c>
+      <c r="B144" t="s">
+        <v>272</v>
+      </c>
+      <c r="C144">
+        <v>2</v>
+      </c>
+      <c r="D144" t="b">
+        <v>0</v>
+      </c>
+      <c r="E144" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="145" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A145" t="s">
+        <v>271</v>
+      </c>
+      <c r="B145" t="s">
+        <v>272</v>
+      </c>
+      <c r="C145">
+        <v>3</v>
+      </c>
+      <c r="D145" t="b">
+        <v>0</v>
+      </c>
+      <c r="E145" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="146" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A146" t="s">
+        <v>85</v>
+      </c>
+      <c r="B146" t="s">
+        <v>86</v>
+      </c>
+      <c r="C146">
+        <v>1</v>
+      </c>
+      <c r="D146" t="b">
+        <v>1</v>
+      </c>
+      <c r="E146" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="147" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A147" t="s">
+        <v>85</v>
+      </c>
+      <c r="B147" t="s">
+        <v>86</v>
+      </c>
+      <c r="C147">
+        <v>2</v>
+      </c>
+      <c r="D147" t="b">
+        <v>0</v>
+      </c>
+      <c r="E147" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="148" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A148" t="s">
+        <v>85</v>
+      </c>
+      <c r="B148" t="s">
+        <v>86</v>
+      </c>
+      <c r="C148">
+        <v>3</v>
+      </c>
+      <c r="D148" t="b">
+        <v>0</v>
+      </c>
+      <c r="E148" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="149" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A149" t="s">
+        <v>275</v>
+      </c>
+      <c r="B149" t="s">
+        <v>276</v>
+      </c>
+      <c r="C149">
+        <v>1</v>
+      </c>
+      <c r="D149" t="b">
+        <v>1</v>
+      </c>
+      <c r="E149" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="150" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A150" t="s">
+        <v>275</v>
+      </c>
+      <c r="B150" t="s">
+        <v>276</v>
+      </c>
+      <c r="C150">
+        <v>2</v>
+      </c>
+      <c r="D150" t="b">
+        <v>0</v>
+      </c>
+      <c r="E150" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="151" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A151" t="s">
+        <v>275</v>
+      </c>
+      <c r="B151" t="s">
+        <v>276</v>
+      </c>
+      <c r="C151">
+        <v>3</v>
+      </c>
+      <c r="D151" t="b">
+        <v>0</v>
+      </c>
+      <c r="E151" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="152" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A152" t="s">
+        <v>281</v>
+      </c>
+      <c r="B152" t="s">
+        <v>249</v>
+      </c>
+      <c r="C152">
+        <v>1</v>
+      </c>
+      <c r="D152" t="b">
+        <v>1</v>
+      </c>
+      <c r="E152" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="153" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A153" t="s">
+        <v>281</v>
+      </c>
+      <c r="B153" t="s">
+        <v>249</v>
+      </c>
+      <c r="C153">
+        <v>2</v>
+      </c>
+      <c r="D153" t="b">
+        <v>0</v>
+      </c>
+      <c r="E153" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="154" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A154" t="s">
+        <v>281</v>
+      </c>
+      <c r="B154" t="s">
+        <v>249</v>
+      </c>
+      <c r="C154">
+        <v>3</v>
+      </c>
+      <c r="D154" t="b">
+        <v>0</v>
+      </c>
+      <c r="E154" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="155" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A155" t="s">
+        <v>17</v>
+      </c>
+      <c r="B155" t="s">
+        <v>18</v>
+      </c>
+      <c r="C155">
+        <v>1</v>
+      </c>
+      <c r="D155" t="b">
+        <v>1</v>
+      </c>
+      <c r="E155" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="156" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A156" t="s">
+        <v>17</v>
+      </c>
+      <c r="B156" t="s">
+        <v>18</v>
+      </c>
+      <c r="C156">
+        <v>2</v>
+      </c>
+      <c r="D156" t="b">
+        <v>0</v>
+      </c>
+      <c r="E156" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="157" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A157" t="s">
+        <v>17</v>
+      </c>
+      <c r="B157" t="s">
+        <v>18</v>
+      </c>
+      <c r="C157">
+        <v>3</v>
+      </c>
+      <c r="D157" t="b">
+        <v>0</v>
+      </c>
+      <c r="E157" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="158" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A158" t="s">
+        <v>284</v>
+      </c>
+      <c r="B158" t="s">
+        <v>285</v>
+      </c>
+      <c r="C158">
+        <v>1</v>
+      </c>
+      <c r="D158" t="b">
+        <v>0</v>
+      </c>
+      <c r="E158" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="159" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A159" t="s">
+        <v>284</v>
+      </c>
+      <c r="B159" t="s">
+        <v>285</v>
+      </c>
+      <c r="C159">
+        <v>2</v>
+      </c>
+      <c r="D159" t="b">
+        <v>0</v>
+      </c>
+      <c r="E159" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="160" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A160" t="s">
+        <v>284</v>
+      </c>
+      <c r="B160" t="s">
+        <v>285</v>
+      </c>
+      <c r="C160">
+        <v>3</v>
+      </c>
+      <c r="D160" t="b">
+        <v>0</v>
+      </c>
+      <c r="E160" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="161" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A161" t="s">
+        <v>96</v>
+      </c>
+      <c r="B161" t="s">
+        <v>97</v>
+      </c>
+      <c r="C161">
+        <v>1</v>
+      </c>
+      <c r="D161" t="b">
+        <v>0</v>
+      </c>
+      <c r="E161" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="162" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A162" t="s">
+        <v>96</v>
+      </c>
+      <c r="B162" t="s">
+        <v>97</v>
+      </c>
+      <c r="C162">
+        <v>2</v>
+      </c>
+      <c r="D162" t="b">
+        <v>0</v>
+      </c>
+      <c r="E162" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="163" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A163" t="s">
+        <v>96</v>
+      </c>
+      <c r="B163" t="s">
+        <v>97</v>
+      </c>
+      <c r="C163">
+        <v>3</v>
+      </c>
+      <c r="D163" t="b">
+        <v>0</v>
+      </c>
+      <c r="E163" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="164" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A164" t="s">
+        <v>314</v>
+      </c>
+      <c r="B164" t="s">
+        <v>315</v>
+      </c>
+      <c r="C164">
+        <v>1</v>
+      </c>
+      <c r="D164" t="b">
+        <v>1</v>
+      </c>
+      <c r="E164" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="165" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A165" t="s">
+        <v>314</v>
+      </c>
+      <c r="B165" t="s">
+        <v>315</v>
+      </c>
+      <c r="C165">
+        <v>2</v>
+      </c>
+      <c r="D165" t="b">
+        <v>1</v>
+      </c>
+      <c r="E165" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="166" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A166" t="s">
+        <v>314</v>
+      </c>
+      <c r="B166" t="s">
+        <v>315</v>
+      </c>
+      <c r="C166">
+        <v>3</v>
+      </c>
+      <c r="D166" t="b">
+        <v>0</v>
+      </c>
+      <c r="E166" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="167" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A167" t="s">
+        <v>76</v>
+      </c>
+      <c r="B167" t="s">
+        <v>77</v>
+      </c>
+      <c r="C167">
+        <v>1</v>
+      </c>
+      <c r="D167" t="b">
+        <v>1</v>
+      </c>
+      <c r="E167" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="168" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A168" t="s">
+        <v>76</v>
+      </c>
+      <c r="B168" t="s">
+        <v>77</v>
+      </c>
+      <c r="C168">
+        <v>2</v>
+      </c>
+      <c r="D168" t="b">
+        <v>0</v>
+      </c>
+      <c r="E168" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="169" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A169" t="s">
+        <v>76</v>
+      </c>
+      <c r="B169" t="s">
+        <v>77</v>
+      </c>
+      <c r="C169">
+        <v>3</v>
+      </c>
+      <c r="D169" t="b">
+        <v>0</v>
+      </c>
+      <c r="E169" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="170" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A170" t="s">
+        <v>23</v>
+      </c>
+      <c r="B170" t="s">
+        <v>24</v>
+      </c>
+      <c r="C170">
+        <v>1</v>
+      </c>
+      <c r="D170" t="b">
+        <v>0</v>
+      </c>
+      <c r="E170" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="171" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A171" t="s">
+        <v>23</v>
+      </c>
+      <c r="B171" t="s">
+        <v>24</v>
+      </c>
+      <c r="C171">
+        <v>2</v>
+      </c>
+      <c r="D171" t="b">
+        <v>0</v>
+      </c>
+      <c r="E171" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="172" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A172" t="s">
+        <v>23</v>
+      </c>
+      <c r="B172" t="s">
+        <v>24</v>
+      </c>
+      <c r="C172">
+        <v>3</v>
+      </c>
+      <c r="D172" t="b">
+        <v>0</v>
+      </c>
+      <c r="E172" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="173" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A173" t="s">
+        <v>29</v>
+      </c>
+      <c r="B173" t="s">
+        <v>30</v>
+      </c>
+      <c r="C173">
+        <v>1</v>
+      </c>
+      <c r="D173" t="b">
+        <v>0</v>
+      </c>
+      <c r="E173" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="174" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A174" t="s">
+        <v>29</v>
+      </c>
+      <c r="B174" t="s">
+        <v>30</v>
+      </c>
+      <c r="C174">
+        <v>2</v>
+      </c>
+      <c r="D174" t="b">
+        <v>0</v>
+      </c>
+      <c r="E174" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="175" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A175" t="s">
+        <v>29</v>
+      </c>
+      <c r="B175" t="s">
+        <v>30</v>
+      </c>
+      <c r="C175">
+        <v>3</v>
+      </c>
+      <c r="D175" t="b">
+        <v>0</v>
+      </c>
+      <c r="E175" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="176" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A176" t="s">
+        <v>36</v>
+      </c>
+      <c r="B176" t="s">
+        <v>37</v>
+      </c>
+      <c r="C176">
+        <v>1</v>
+      </c>
+      <c r="D176" t="b">
+        <v>0</v>
+      </c>
+      <c r="E176" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="177" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A177" t="s">
+        <v>36</v>
+      </c>
+      <c r="B177" t="s">
+        <v>37</v>
+      </c>
+      <c r="C177">
+        <v>2</v>
+      </c>
+      <c r="D177" t="b">
+        <v>0</v>
+      </c>
+      <c r="E177" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="178" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A178" t="s">
+        <v>36</v>
+      </c>
+      <c r="B178" t="s">
+        <v>37</v>
+      </c>
+      <c r="C178">
+        <v>3</v>
+      </c>
+      <c r="D178" t="b">
+        <v>0</v>
+      </c>
+      <c r="E178" t="s">
         <v>69</v>
       </c>
     </row>

</xml_diff>

<commit_message>
all archer class added
</commit_message>
<xml_diff>
--- a/data/Fate-Spreadsheet.xlsx
+++ b/data/Fate-Spreadsheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Important\Python\Fate-Wiki\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74FB2C1B-B3D2-4F80-982D-47219B1EFE02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAE09173-3834-4445-B317-789F4733B023}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{B05E798F-9EF6-4508-A0A4-311D06661AED}"/>
   </bookViews>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1141" uniqueCount="476">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1515" uniqueCount="622">
   <si>
     <t>servant_id</t>
   </si>
@@ -1471,6 +1471,444 @@
   </si>
   <si>
     <t>4,4,4</t>
+  </si>
+  <si>
+    <t>S0049</t>
+  </si>
+  <si>
+    <t>S0050</t>
+  </si>
+  <si>
+    <t>S0051</t>
+  </si>
+  <si>
+    <t>S0052</t>
+  </si>
+  <si>
+    <t>S0053</t>
+  </si>
+  <si>
+    <t>S0054</t>
+  </si>
+  <si>
+    <t>S0055</t>
+  </si>
+  <si>
+    <t>S0056</t>
+  </si>
+  <si>
+    <t>S0057</t>
+  </si>
+  <si>
+    <t>S0058</t>
+  </si>
+  <si>
+    <t>S0059</t>
+  </si>
+  <si>
+    <t>S0060</t>
+  </si>
+  <si>
+    <t>S0061</t>
+  </si>
+  <si>
+    <t>S0062</t>
+  </si>
+  <si>
+    <t>S0063</t>
+  </si>
+  <si>
+    <t>S0064</t>
+  </si>
+  <si>
+    <t>S0065</t>
+  </si>
+  <si>
+    <t>S0066</t>
+  </si>
+  <si>
+    <t>S0067</t>
+  </si>
+  <si>
+    <t>S0068</t>
+  </si>
+  <si>
+    <t>Oda Nobunaga</t>
+  </si>
+  <si>
+    <t>oda-nobunaga</t>
+  </si>
+  <si>
+    <t>Atalanta</t>
+  </si>
+  <si>
+    <t>Chiron</t>
+  </si>
+  <si>
+    <t>Robin Hood</t>
+  </si>
+  <si>
+    <t>Arjuna</t>
+  </si>
+  <si>
+    <t>Ishtar</t>
+  </si>
+  <si>
+    <t>Mecha Eli-chan</t>
+  </si>
+  <si>
+    <t>Arash</t>
+  </si>
+  <si>
+    <t>Nikola Tesla</t>
+  </si>
+  <si>
+    <t>Billy the Kid</t>
+  </si>
+  <si>
+    <t>Napoleon Bonaparte</t>
+  </si>
+  <si>
+    <t>Chloe von Einzbern</t>
+  </si>
+  <si>
+    <t>Tristan</t>
+  </si>
+  <si>
+    <t>Emiya Shirou</t>
+  </si>
+  <si>
+    <t>emiya-shirou-alter</t>
+  </si>
+  <si>
+    <t>Baobhan Sith</t>
+  </si>
+  <si>
+    <t>Tomoe Gozen</t>
+  </si>
+  <si>
+    <t>Orion</t>
+  </si>
+  <si>
+    <t>James Moriarty</t>
+  </si>
+  <si>
+    <t>Sei Shounagon</t>
+  </si>
+  <si>
+    <t>atalanta</t>
+  </si>
+  <si>
+    <t>chiron</t>
+  </si>
+  <si>
+    <t>arjuna</t>
+  </si>
+  <si>
+    <t>ishtar</t>
+  </si>
+  <si>
+    <t>arash</t>
+  </si>
+  <si>
+    <t>tristan</t>
+  </si>
+  <si>
+    <t>asvatthama</t>
+  </si>
+  <si>
+    <t>orion</t>
+  </si>
+  <si>
+    <t>robin-hood</t>
+  </si>
+  <si>
+    <t>nikola-tesla</t>
+  </si>
+  <si>
+    <t>napoleon-bonaparte</t>
+  </si>
+  <si>
+    <t>baobhan-sith</t>
+  </si>
+  <si>
+    <t>tomoe-gozen</t>
+  </si>
+  <si>
+    <t>james-moriarty</t>
+  </si>
+  <si>
+    <t>sei-shounagon</t>
+  </si>
+  <si>
+    <t>mecha-eli-chan</t>
+  </si>
+  <si>
+    <t>billy-the-kid</t>
+  </si>
+  <si>
+    <t>chloe-von-einzbern</t>
+  </si>
+  <si>
+    <t>S0071</t>
+  </si>
+  <si>
+    <t>S0072</t>
+  </si>
+  <si>
+    <t>S0073</t>
+  </si>
+  <si>
+    <t>S0074</t>
+  </si>
+  <si>
+    <t>S0075</t>
+  </si>
+  <si>
+    <t>S0076</t>
+  </si>
+  <si>
+    <t>S0077</t>
+  </si>
+  <si>
+    <t>S0078</t>
+  </si>
+  <si>
+    <t>S0079</t>
+  </si>
+  <si>
+    <t>S0080</t>
+  </si>
+  <si>
+    <t>S0081</t>
+  </si>
+  <si>
+    <t>S0082</t>
+  </si>
+  <si>
+    <t>S0083</t>
+  </si>
+  <si>
+    <t>S0084</t>
+  </si>
+  <si>
+    <t>S0085</t>
+  </si>
+  <si>
+    <t>S0086</t>
+  </si>
+  <si>
+    <t>S0087</t>
+  </si>
+  <si>
+    <t>S0088</t>
+  </si>
+  <si>
+    <t>S0089</t>
+  </si>
+  <si>
+    <t>S0090</t>
+  </si>
+  <si>
+    <t>S0091</t>
+  </si>
+  <si>
+    <t>S0092</t>
+  </si>
+  <si>
+    <t>2,3,4,4,4</t>
+  </si>
+  <si>
+    <t>Preparation,Preparation,Preparation</t>
+  </si>
+  <si>
+    <t>2,2,3,4,4,4</t>
+  </si>
+  <si>
+    <t>Preparation,Preparation,Surveil</t>
+  </si>
+  <si>
+    <t>2,2,5,5</t>
+  </si>
+  <si>
+    <t>2,2,3,5,5</t>
+  </si>
+  <si>
+    <t>2,2,3,3,3,4</t>
+  </si>
+  <si>
+    <t>Surveil,Surveil,Preparation</t>
+  </si>
+  <si>
+    <t>5,5,5,5</t>
+  </si>
+  <si>
+    <t>2,5,5</t>
+  </si>
+  <si>
+    <t>3,4,5,5</t>
+  </si>
+  <si>
+    <t>2,2,3,3,4</t>
+  </si>
+  <si>
+    <t>5,5,5</t>
+  </si>
+  <si>
+    <t>Luck,Luck,Surveil,Surveil,Preparation</t>
+  </si>
+  <si>
+    <t>Three Line Formation</t>
+  </si>
+  <si>
+    <t>Papiyas</t>
+  </si>
+  <si>
+    <t>Fool of Owari</t>
+  </si>
+  <si>
+    <t>Phoebus Catastrophe</t>
+  </si>
+  <si>
+    <t>Agrius Metamorphosis</t>
+  </si>
+  <si>
+    <t>Antares Snipe</t>
+  </si>
+  <si>
+    <t>Divine Wisdom</t>
+  </si>
+  <si>
+    <t>Yew Bow</t>
+  </si>
+  <si>
+    <t>No Face May King</t>
+  </si>
+  <si>
+    <t>Pashupata</t>
+  </si>
+  <si>
+    <t>Agni Gandiva</t>
+  </si>
+  <si>
+    <t>The Endowed Hero</t>
+  </si>
+  <si>
+    <t>An Gal Ta Kigal She</t>
+  </si>
+  <si>
+    <t>Divine Authority</t>
+  </si>
+  <si>
+    <t>Breast Zero</t>
+  </si>
+  <si>
+    <t>Rocket Fists</t>
+  </si>
+  <si>
+    <t>Stella</t>
+  </si>
+  <si>
+    <t>Solemn Prayer</t>
+  </si>
+  <si>
+    <t>Clairvoyance</t>
+  </si>
+  <si>
+    <t>System Keraunos</t>
+  </si>
+  <si>
+    <t>System Keraunos (Overload)</t>
+  </si>
+  <si>
+    <t>Transhumanism</t>
+  </si>
+  <si>
+    <t>Thunderer (Attack)</t>
+  </si>
+  <si>
+    <t>Thunderer (Passive)</t>
+  </si>
+  <si>
+    <t>Quick Draw</t>
+  </si>
+  <si>
+    <t>Arc de Triomphe</t>
+  </si>
+  <si>
+    <t>Hidden Trump Card</t>
+  </si>
+  <si>
+    <t>Kanshou &amp; Bakuya (Chloe)</t>
+  </si>
+  <si>
+    <t>Projection Magic</t>
+  </si>
+  <si>
+    <t>Unlimited Blade Works (Chloe)</t>
+  </si>
+  <si>
+    <t>Failnaught</t>
+  </si>
+  <si>
+    <t>Soothing Serenade</t>
+  </si>
+  <si>
+    <t>Aśvatthāma</t>
+  </si>
+  <si>
+    <t>Sudarshan Chakra</t>
+  </si>
+  <si>
+    <t>Mahakala Shakti</t>
+  </si>
+  <si>
+    <t>Avatar of Rage</t>
+  </si>
+  <si>
+    <t>Kanshou &amp; Bakuya (Alter)</t>
+  </si>
+  <si>
+    <t>Unlimited Lost Works</t>
+  </si>
+  <si>
+    <t>Fetch Failnaught</t>
+  </si>
+  <si>
+    <t>Part Collector</t>
+  </si>
+  <si>
+    <t>On Arorikya Sowaka</t>
+  </si>
+  <si>
+    <t>Oni Raiders</t>
+  </si>
+  <si>
+    <t>Aegis Eclipse</t>
+  </si>
+  <si>
+    <t>Divine Embrace</t>
+  </si>
+  <si>
+    <t>Moontouched Hunter</t>
+  </si>
+  <si>
+    <t>Dynamics of an Asteroid</t>
+  </si>
+  <si>
+    <t>Wicked Charisma</t>
+  </si>
+  <si>
+    <t>In the Spider's Web</t>
+  </si>
+  <si>
+    <t>Emotional Engine</t>
+  </si>
+  <si>
+    <t>Vivid Sensation</t>
+  </si>
+  <si>
+    <t>Nostalgia Drive</t>
   </si>
 </sst>
 </file>
@@ -1859,7 +2297,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E33D7ECC-1EAA-4A40-B4DA-A93E54CBC8B5}">
-  <dimension ref="A1:K60"/>
+  <dimension ref="A1:K102"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="3" width="22" customWidth="1"/>
@@ -3407,60 +3845,57 @@
     </row>
     <row r="50" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
-        <v>85</v>
+        <v>476</v>
       </c>
       <c r="B50" t="s">
-        <v>86</v>
+        <v>496</v>
       </c>
       <c r="C50" t="s">
-        <v>87</v>
+        <v>497</v>
       </c>
       <c r="D50" t="s">
         <v>88</v>
       </c>
       <c r="E50" t="s">
-        <v>89</v>
+        <v>8</v>
       </c>
       <c r="G50" s="2" t="s">
-        <v>15</v>
+        <v>431</v>
       </c>
       <c r="H50" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="I50" s="2" t="s">
-        <v>42</v>
+        <v>557</v>
+      </c>
+      <c r="J50" s="2" t="s">
+        <v>558</v>
       </c>
       <c r="K50" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
-        <v>275</v>
+        <v>477</v>
       </c>
       <c r="B51" t="s">
-        <v>276</v>
+        <v>498</v>
       </c>
       <c r="C51" t="s">
-        <v>277</v>
+        <v>517</v>
       </c>
       <c r="D51" t="s">
-        <v>278</v>
+        <v>88</v>
       </c>
       <c r="E51" t="s">
-        <v>8</v>
+        <v>33</v>
       </c>
       <c r="G51" s="2" t="s">
-        <v>279</v>
+        <v>100</v>
       </c>
       <c r="H51" s="2" t="s">
-        <v>204</v>
-      </c>
-      <c r="I51" s="2" t="s">
-        <v>280</v>
+        <v>559</v>
       </c>
       <c r="J51" s="2" t="s">
-        <v>43</v>
+        <v>560</v>
       </c>
       <c r="K51" t="b">
         <v>0</v>
@@ -3468,28 +3903,31 @@
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
-        <v>281</v>
+        <v>478</v>
       </c>
       <c r="B52" t="s">
-        <v>249</v>
+        <v>499</v>
       </c>
       <c r="C52" t="s">
-        <v>282</v>
+        <v>518</v>
       </c>
       <c r="D52" t="s">
-        <v>20</v>
+        <v>88</v>
       </c>
       <c r="E52" t="s">
         <v>33</v>
       </c>
+      <c r="G52" s="2" t="s">
+        <v>561</v>
+      </c>
       <c r="H52" s="2" t="s">
-        <v>27</v>
+        <v>562</v>
       </c>
       <c r="I52" s="2" t="s">
-        <v>101</v>
+        <v>191</v>
       </c>
       <c r="J52" s="2" t="s">
-        <v>283</v>
+        <v>188</v>
       </c>
       <c r="K52" t="b">
         <v>0</v>
@@ -3497,106 +3935,124 @@
     </row>
     <row r="53" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
-        <v>17</v>
+        <v>479</v>
       </c>
       <c r="B53" t="s">
-        <v>18</v>
+        <v>500</v>
       </c>
       <c r="C53" t="s">
-        <v>19</v>
+        <v>525</v>
       </c>
       <c r="D53" t="s">
-        <v>20</v>
+        <v>88</v>
       </c>
       <c r="E53" t="s">
-        <v>8</v>
+        <v>33</v>
+      </c>
+      <c r="H53" s="2" t="s">
+        <v>563</v>
       </c>
       <c r="I53" s="2" t="s">
-        <v>21</v>
+        <v>100</v>
       </c>
       <c r="J53" s="2" t="s">
         <v>22</v>
       </c>
       <c r="K53" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="54" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
-        <v>284</v>
+        <v>480</v>
       </c>
       <c r="B54" t="s">
-        <v>285</v>
+        <v>501</v>
       </c>
       <c r="C54" t="s">
-        <v>286</v>
+        <v>519</v>
       </c>
       <c r="D54" t="s">
-        <v>20</v>
+        <v>88</v>
       </c>
       <c r="E54" t="s">
-        <v>8</v>
+        <v>89</v>
+      </c>
+      <c r="G54" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="H54" s="2" t="s">
+        <v>176</v>
       </c>
       <c r="I54" s="2" t="s">
-        <v>287</v>
+        <v>15</v>
       </c>
       <c r="J54" s="2" t="s">
-        <v>177</v>
+        <v>200</v>
       </c>
       <c r="K54" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="55" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
-        <v>96</v>
+        <v>481</v>
       </c>
       <c r="B55" t="s">
-        <v>97</v>
+        <v>502</v>
       </c>
       <c r="C55" t="s">
-        <v>98</v>
+        <v>520</v>
       </c>
       <c r="D55" t="s">
-        <v>20</v>
+        <v>88</v>
       </c>
       <c r="E55" t="s">
-        <v>99</v>
+        <v>33</v>
+      </c>
+      <c r="G55" s="2" t="s">
+        <v>15</v>
       </c>
       <c r="H55" s="2" t="s">
-        <v>100</v>
+        <v>27</v>
       </c>
       <c r="I55" s="2" t="s">
-        <v>101</v>
+        <v>454</v>
+      </c>
+      <c r="J55" s="2" t="s">
+        <v>564</v>
       </c>
       <c r="K55" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
-        <v>314</v>
+        <v>482</v>
       </c>
       <c r="B56" t="s">
-        <v>315</v>
+        <v>503</v>
       </c>
       <c r="C56" t="s">
-        <v>316</v>
+        <v>532</v>
       </c>
       <c r="D56" t="s">
-        <v>317</v>
+        <v>79</v>
       </c>
       <c r="E56" t="s">
-        <v>33</v>
+        <v>8</v>
+      </c>
+      <c r="G56" s="2" t="s">
+        <v>279</v>
       </c>
       <c r="H56" s="2" t="s">
-        <v>21</v>
+        <v>397</v>
       </c>
       <c r="I56" s="2" t="s">
-        <v>318</v>
+        <v>27</v>
       </c>
       <c r="J56" s="2" t="s">
-        <v>319</v>
+        <v>186</v>
       </c>
       <c r="K56" t="b">
         <v>0</v>
@@ -3604,31 +4060,28 @@
     </row>
     <row r="57" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
-        <v>76</v>
+        <v>483</v>
       </c>
       <c r="B57" t="s">
-        <v>77</v>
+        <v>504</v>
       </c>
       <c r="C57" t="s">
-        <v>78</v>
+        <v>521</v>
       </c>
       <c r="D57" t="s">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="E57" t="s">
-        <v>40</v>
+        <v>99</v>
       </c>
       <c r="G57" s="2" t="s">
-        <v>80</v>
+        <v>176</v>
       </c>
       <c r="H57" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="I57" s="2" t="s">
-        <v>81</v>
+        <v>204</v>
       </c>
       <c r="J57" s="2" t="s">
-        <v>322</v>
+        <v>186</v>
       </c>
       <c r="K57" t="b">
         <v>0</v>
@@ -3636,28 +4089,31 @@
     </row>
     <row r="58" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
-        <v>23</v>
+        <v>484</v>
       </c>
       <c r="B58" t="s">
-        <v>24</v>
+        <v>505</v>
       </c>
       <c r="C58" t="s">
-        <v>25</v>
+        <v>526</v>
       </c>
       <c r="D58" t="s">
-        <v>26</v>
+        <v>88</v>
       </c>
       <c r="E58" t="s">
         <v>8</v>
       </c>
       <c r="G58" s="2" t="s">
-        <v>27</v>
+        <v>199</v>
       </c>
       <c r="H58" s="2" t="s">
-        <v>28</v>
+        <v>287</v>
+      </c>
+      <c r="I58" s="2" t="s">
+        <v>565</v>
       </c>
       <c r="J58" s="2" t="s">
-        <v>70</v>
+        <v>183</v>
       </c>
       <c r="K58" t="b">
         <v>0</v>
@@ -3665,31 +4121,28 @@
     </row>
     <row r="59" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
-        <v>29</v>
+        <v>485</v>
       </c>
       <c r="B59" t="s">
-        <v>30</v>
+        <v>506</v>
       </c>
       <c r="C59" t="s">
-        <v>31</v>
+        <v>533</v>
       </c>
       <c r="D59" t="s">
-        <v>32</v>
+        <v>88</v>
       </c>
       <c r="E59" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="G59" s="2" t="s">
-        <v>15</v>
+        <v>100</v>
       </c>
       <c r="H59" s="2" t="s">
-        <v>81</v>
-      </c>
-      <c r="I59" s="2" t="s">
-        <v>34</v>
+        <v>101</v>
       </c>
       <c r="J59" s="2" t="s">
-        <v>35</v>
+        <v>200</v>
       </c>
       <c r="K59" t="b">
         <v>0</v>
@@ -3697,30 +4150,741 @@
     </row>
     <row r="60" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
+        <v>486</v>
+      </c>
+      <c r="B60" t="s">
+        <v>507</v>
+      </c>
+      <c r="C60" t="s">
+        <v>527</v>
+      </c>
+      <c r="D60" t="s">
+        <v>88</v>
+      </c>
+      <c r="E60" t="s">
+        <v>33</v>
+      </c>
+      <c r="G60" s="2" t="s">
+        <v>450</v>
+      </c>
+      <c r="H60" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="J60" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="K60" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>487</v>
+      </c>
+      <c r="B61" t="s">
+        <v>508</v>
+      </c>
+      <c r="C61" t="s">
+        <v>534</v>
+      </c>
+      <c r="D61" t="s">
+        <v>88</v>
+      </c>
+      <c r="E61" t="s">
+        <v>89</v>
+      </c>
+      <c r="G61" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="H61" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="I61" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="J61" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="K61" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>488</v>
+      </c>
+      <c r="B62" t="s">
+        <v>509</v>
+      </c>
+      <c r="C62" t="s">
+        <v>522</v>
+      </c>
+      <c r="D62" t="s">
+        <v>88</v>
+      </c>
+      <c r="E62" t="s">
+        <v>8</v>
+      </c>
+      <c r="G62" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="H62" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="I62" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="J62" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="K62" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>489</v>
+      </c>
+      <c r="B63" t="s">
+        <v>603</v>
+      </c>
+      <c r="C63" t="s">
+        <v>523</v>
+      </c>
+      <c r="D63" t="s">
+        <v>88</v>
+      </c>
+      <c r="E63" t="s">
+        <v>8</v>
+      </c>
+      <c r="G63" s="2" t="s">
+        <v>196</v>
+      </c>
+      <c r="H63" s="2" t="s">
+        <v>435</v>
+      </c>
+      <c r="I63" s="2" t="s">
+        <v>326</v>
+      </c>
+      <c r="J63" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="K63" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>490</v>
+      </c>
+      <c r="B64" t="s">
+        <v>510</v>
+      </c>
+      <c r="C64" t="s">
+        <v>511</v>
+      </c>
+      <c r="D64" t="s">
+        <v>88</v>
+      </c>
+      <c r="E64" t="s">
+        <v>89</v>
+      </c>
+      <c r="G64" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H64" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="I64" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="J64" s="2" t="s">
+        <v>564</v>
+      </c>
+      <c r="K64" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="65" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A65" t="s">
+        <v>491</v>
+      </c>
+      <c r="B65" t="s">
+        <v>512</v>
+      </c>
+      <c r="C65" t="s">
+        <v>528</v>
+      </c>
+      <c r="D65" t="s">
+        <v>88</v>
+      </c>
+      <c r="E65" t="s">
+        <v>8</v>
+      </c>
+      <c r="G65" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="H65" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="I65" s="2" t="s">
+        <v>566</v>
+      </c>
+      <c r="J65" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K65" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A66" t="s">
+        <v>492</v>
+      </c>
+      <c r="B66" t="s">
+        <v>513</v>
+      </c>
+      <c r="C66" t="s">
+        <v>529</v>
+      </c>
+      <c r="D66" t="s">
+        <v>88</v>
+      </c>
+      <c r="E66" t="s">
+        <v>89</v>
+      </c>
+      <c r="G66" s="2" t="s">
+        <v>567</v>
+      </c>
+      <c r="H66" s="2" t="s">
+        <v>568</v>
+      </c>
+      <c r="J66" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="K66" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A67" t="s">
+        <v>493</v>
+      </c>
+      <c r="B67" t="s">
+        <v>514</v>
+      </c>
+      <c r="C67" t="s">
+        <v>524</v>
+      </c>
+      <c r="D67" t="s">
+        <v>88</v>
+      </c>
+      <c r="E67" t="s">
+        <v>89</v>
+      </c>
+      <c r="G67" s="2" t="s">
+        <v>569</v>
+      </c>
+      <c r="H67" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="J67" s="2" t="s">
+        <v>570</v>
+      </c>
+      <c r="K67" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="68" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A68" t="s">
+        <v>494</v>
+      </c>
+      <c r="B68" t="s">
+        <v>515</v>
+      </c>
+      <c r="C68" t="s">
+        <v>530</v>
+      </c>
+      <c r="D68" t="s">
+        <v>88</v>
+      </c>
+      <c r="E68" t="s">
+        <v>8</v>
+      </c>
+      <c r="G68" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H68" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="I68" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="J68" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K68" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A69" t="s">
+        <v>495</v>
+      </c>
+      <c r="B69" t="s">
+        <v>516</v>
+      </c>
+      <c r="C69" t="s">
+        <v>531</v>
+      </c>
+      <c r="D69" t="s">
+        <v>88</v>
+      </c>
+      <c r="E69" t="s">
+        <v>89</v>
+      </c>
+      <c r="G69" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="H69" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="I69" s="2" t="s">
+        <v>190</v>
+      </c>
+      <c r="J69" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="K69" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A70" t="s">
+        <v>85</v>
+      </c>
+      <c r="B70" t="s">
+        <v>86</v>
+      </c>
+      <c r="C70" t="s">
+        <v>87</v>
+      </c>
+      <c r="D70" t="s">
+        <v>88</v>
+      </c>
+      <c r="E70" t="s">
+        <v>89</v>
+      </c>
+      <c r="G70" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H70" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="I70" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="K70" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="71" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A71" t="s">
+        <v>275</v>
+      </c>
+      <c r="B71" t="s">
+        <v>276</v>
+      </c>
+      <c r="C71" t="s">
+        <v>277</v>
+      </c>
+      <c r="D71" t="s">
+        <v>278</v>
+      </c>
+      <c r="E71" t="s">
+        <v>8</v>
+      </c>
+      <c r="G71" s="2" t="s">
+        <v>279</v>
+      </c>
+      <c r="H71" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="I71" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="J71" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="K71" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A72" t="s">
+        <v>535</v>
+      </c>
+    </row>
+    <row r="73" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A73" t="s">
+        <v>536</v>
+      </c>
+    </row>
+    <row r="74" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A74" t="s">
+        <v>537</v>
+      </c>
+    </row>
+    <row r="75" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A75" t="s">
+        <v>538</v>
+      </c>
+    </row>
+    <row r="76" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A76" t="s">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="77" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A77" t="s">
+        <v>540</v>
+      </c>
+    </row>
+    <row r="78" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A78" t="s">
+        <v>541</v>
+      </c>
+    </row>
+    <row r="79" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A79" t="s">
+        <v>542</v>
+      </c>
+    </row>
+    <row r="80" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A80" t="s">
+        <v>543</v>
+      </c>
+    </row>
+    <row r="81" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A81" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="82" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A82" t="s">
+        <v>545</v>
+      </c>
+    </row>
+    <row r="83" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A83" t="s">
+        <v>546</v>
+      </c>
+    </row>
+    <row r="84" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A84" t="s">
+        <v>547</v>
+      </c>
+    </row>
+    <row r="85" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A85" t="s">
+        <v>548</v>
+      </c>
+    </row>
+    <row r="86" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A86" t="s">
+        <v>549</v>
+      </c>
+    </row>
+    <row r="87" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A87" t="s">
+        <v>550</v>
+      </c>
+    </row>
+    <row r="88" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A88" t="s">
+        <v>551</v>
+      </c>
+    </row>
+    <row r="89" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A89" t="s">
+        <v>552</v>
+      </c>
+    </row>
+    <row r="90" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A90" t="s">
+        <v>553</v>
+      </c>
+    </row>
+    <row r="91" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A91" t="s">
+        <v>554</v>
+      </c>
+    </row>
+    <row r="92" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A92" t="s">
+        <v>555</v>
+      </c>
+    </row>
+    <row r="93" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A93" t="s">
+        <v>556</v>
+      </c>
+    </row>
+    <row r="94" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A94" t="s">
+        <v>281</v>
+      </c>
+      <c r="B94" t="s">
+        <v>249</v>
+      </c>
+      <c r="C94" t="s">
+        <v>282</v>
+      </c>
+      <c r="D94" t="s">
+        <v>20</v>
+      </c>
+      <c r="E94" t="s">
+        <v>33</v>
+      </c>
+      <c r="H94" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I94" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="J94" s="2" t="s">
+        <v>283</v>
+      </c>
+      <c r="K94" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="95" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A95" t="s">
+        <v>17</v>
+      </c>
+      <c r="B95" t="s">
+        <v>18</v>
+      </c>
+      <c r="C95" t="s">
+        <v>19</v>
+      </c>
+      <c r="D95" t="s">
+        <v>20</v>
+      </c>
+      <c r="E95" t="s">
+        <v>8</v>
+      </c>
+      <c r="I95" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="J95" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="K95" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="96" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A96" t="s">
+        <v>284</v>
+      </c>
+      <c r="B96" t="s">
+        <v>285</v>
+      </c>
+      <c r="C96" t="s">
+        <v>286</v>
+      </c>
+      <c r="D96" t="s">
+        <v>20</v>
+      </c>
+      <c r="E96" t="s">
+        <v>8</v>
+      </c>
+      <c r="I96" s="2" t="s">
+        <v>287</v>
+      </c>
+      <c r="J96" s="2" t="s">
+        <v>177</v>
+      </c>
+      <c r="K96" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="97" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A97" t="s">
+        <v>96</v>
+      </c>
+      <c r="B97" t="s">
+        <v>97</v>
+      </c>
+      <c r="C97" t="s">
+        <v>98</v>
+      </c>
+      <c r="D97" t="s">
+        <v>20</v>
+      </c>
+      <c r="E97" t="s">
+        <v>99</v>
+      </c>
+      <c r="H97" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="I97" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="K97" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="98" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A98" t="s">
+        <v>314</v>
+      </c>
+      <c r="B98" t="s">
+        <v>315</v>
+      </c>
+      <c r="C98" t="s">
+        <v>316</v>
+      </c>
+      <c r="D98" t="s">
+        <v>317</v>
+      </c>
+      <c r="E98" t="s">
+        <v>33</v>
+      </c>
+      <c r="H98" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="I98" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="J98" s="2" t="s">
+        <v>319</v>
+      </c>
+      <c r="K98" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="99" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A99" t="s">
+        <v>76</v>
+      </c>
+      <c r="B99" t="s">
+        <v>77</v>
+      </c>
+      <c r="C99" t="s">
+        <v>78</v>
+      </c>
+      <c r="D99" t="s">
+        <v>79</v>
+      </c>
+      <c r="E99" t="s">
+        <v>40</v>
+      </c>
+      <c r="G99" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="H99" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I99" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="J99" s="2" t="s">
+        <v>322</v>
+      </c>
+      <c r="K99" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="100" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A100" t="s">
+        <v>23</v>
+      </c>
+      <c r="B100" t="s">
+        <v>24</v>
+      </c>
+      <c r="C100" t="s">
+        <v>25</v>
+      </c>
+      <c r="D100" t="s">
+        <v>26</v>
+      </c>
+      <c r="E100" t="s">
+        <v>8</v>
+      </c>
+      <c r="G100" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H100" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="J100" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="K100" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="101" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A101" t="s">
+        <v>29</v>
+      </c>
+      <c r="B101" t="s">
+        <v>30</v>
+      </c>
+      <c r="C101" t="s">
+        <v>31</v>
+      </c>
+      <c r="D101" t="s">
+        <v>32</v>
+      </c>
+      <c r="E101" t="s">
+        <v>33</v>
+      </c>
+      <c r="G101" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H101" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="I101" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="J101" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="K101" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="102" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A102" t="s">
         <v>36</v>
       </c>
-      <c r="B60" t="s">
+      <c r="B102" t="s">
         <v>37</v>
       </c>
-      <c r="C60" t="s">
+      <c r="C102" t="s">
         <v>38</v>
       </c>
-      <c r="D60" t="s">
+      <c r="D102" t="s">
         <v>39</v>
       </c>
-      <c r="E60" t="s">
+      <c r="E102" t="s">
         <v>40</v>
       </c>
-      <c r="G60" s="2" t="s">
+      <c r="G102" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="H60" s="2" t="s">
+      <c r="H102" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="J60" s="2" t="s">
+      <c r="J102" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="K60" t="b">
+      <c r="K102" t="b">
         <v>1</v>
       </c>
     </row>
@@ -3728,7 +4892,7 @@
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="H2 I6:I7 I10 I12 H14 I18 I22 I24 I27 G34 I40 I42 I45" numberStoredAsText="1"/>
+    <ignoredError sqref="H2 I6:I7 I10 I12 H14 I18 I22 I24 I27 G34 I40 I42 I45 I52 I62" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -4114,13 +5278,13 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84E3BB0D-5578-4069-B1C9-C3864EB2A429}">
-  <dimension ref="A1:F178"/>
+  <dimension ref="A1:F238"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="20.5703125" customWidth="1"/>
     <col min="3" max="3" width="12.7109375" customWidth="1"/>
     <col min="4" max="4" width="17" customWidth="1"/>
-    <col min="5" max="5" width="23.5703125" customWidth="1"/>
+    <col min="5" max="5" width="29.5703125" customWidth="1"/>
     <col min="6" max="6" width="15.7109375" customWidth="1"/>
   </cols>
   <sheetData>
@@ -6594,27 +7758,27 @@
     </row>
     <row r="146" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
-        <v>85</v>
+        <v>476</v>
       </c>
       <c r="B146" t="s">
-        <v>86</v>
+        <v>496</v>
       </c>
       <c r="C146">
         <v>1</v>
       </c>
       <c r="D146" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E146" t="s">
-        <v>93</v>
+        <v>571</v>
       </c>
     </row>
     <row r="147" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
-        <v>85</v>
+        <v>476</v>
       </c>
       <c r="B147" t="s">
-        <v>86</v>
+        <v>496</v>
       </c>
       <c r="C147">
         <v>2</v>
@@ -6623,15 +7787,15 @@
         <v>0</v>
       </c>
       <c r="E147" t="s">
-        <v>94</v>
+        <v>572</v>
       </c>
     </row>
     <row r="148" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
-        <v>85</v>
+        <v>476</v>
       </c>
       <c r="B148" t="s">
-        <v>86</v>
+        <v>496</v>
       </c>
       <c r="C148">
         <v>3</v>
@@ -6640,15 +7804,15 @@
         <v>0</v>
       </c>
       <c r="E148" t="s">
-        <v>95</v>
+        <v>573</v>
       </c>
     </row>
     <row r="149" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
-        <v>275</v>
+        <v>477</v>
       </c>
       <c r="B149" t="s">
-        <v>276</v>
+        <v>498</v>
       </c>
       <c r="C149">
         <v>1</v>
@@ -6657,15 +7821,15 @@
         <v>1</v>
       </c>
       <c r="E149" t="s">
-        <v>306</v>
+        <v>93</v>
       </c>
     </row>
     <row r="150" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
-        <v>275</v>
+        <v>477</v>
       </c>
       <c r="B150" t="s">
-        <v>276</v>
+        <v>498</v>
       </c>
       <c r="C150">
         <v>2</v>
@@ -6674,15 +7838,15 @@
         <v>0</v>
       </c>
       <c r="E150" t="s">
-        <v>307</v>
+        <v>574</v>
       </c>
     </row>
     <row r="151" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
-        <v>275</v>
+        <v>477</v>
       </c>
       <c r="B151" t="s">
-        <v>276</v>
+        <v>498</v>
       </c>
       <c r="C151">
         <v>3</v>
@@ -6691,15 +7855,15 @@
         <v>0</v>
       </c>
       <c r="E151" t="s">
-        <v>308</v>
+        <v>575</v>
       </c>
     </row>
     <row r="152" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
-        <v>281</v>
+        <v>478</v>
       </c>
       <c r="B152" t="s">
-        <v>249</v>
+        <v>499</v>
       </c>
       <c r="C152">
         <v>1</v>
@@ -6708,15 +7872,15 @@
         <v>1</v>
       </c>
       <c r="E152" t="s">
-        <v>58</v>
+        <v>93</v>
       </c>
     </row>
     <row r="153" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
-        <v>281</v>
+        <v>478</v>
       </c>
       <c r="B153" t="s">
-        <v>249</v>
+        <v>499</v>
       </c>
       <c r="C153">
         <v>2</v>
@@ -6725,15 +7889,15 @@
         <v>0</v>
       </c>
       <c r="E153" t="s">
-        <v>309</v>
+        <v>576</v>
       </c>
     </row>
     <row r="154" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
-        <v>281</v>
+        <v>478</v>
       </c>
       <c r="B154" t="s">
-        <v>249</v>
+        <v>499</v>
       </c>
       <c r="C154">
         <v>3</v>
@@ -6742,15 +7906,15 @@
         <v>0</v>
       </c>
       <c r="E154" t="s">
-        <v>310</v>
+        <v>577</v>
       </c>
     </row>
     <row r="155" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
-        <v>17</v>
+        <v>479</v>
       </c>
       <c r="B155" t="s">
-        <v>18</v>
+        <v>500</v>
       </c>
       <c r="C155">
         <v>1</v>
@@ -6759,15 +7923,15 @@
         <v>1</v>
       </c>
       <c r="E155" t="s">
-        <v>58</v>
+        <v>93</v>
       </c>
     </row>
     <row r="156" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
-        <v>17</v>
+        <v>479</v>
       </c>
       <c r="B156" t="s">
-        <v>18</v>
+        <v>500</v>
       </c>
       <c r="C156">
         <v>2</v>
@@ -6776,15 +7940,15 @@
         <v>0</v>
       </c>
       <c r="E156" t="s">
-        <v>59</v>
+        <v>578</v>
       </c>
     </row>
     <row r="157" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
-        <v>17</v>
+        <v>479</v>
       </c>
       <c r="B157" t="s">
-        <v>18</v>
+        <v>500</v>
       </c>
       <c r="C157">
         <v>3</v>
@@ -6793,15 +7957,15 @@
         <v>0</v>
       </c>
       <c r="E157" t="s">
-        <v>60</v>
+        <v>579</v>
       </c>
     </row>
     <row r="158" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
-        <v>284</v>
+        <v>480</v>
       </c>
       <c r="B158" t="s">
-        <v>285</v>
+        <v>501</v>
       </c>
       <c r="C158">
         <v>1</v>
@@ -6810,15 +7974,15 @@
         <v>0</v>
       </c>
       <c r="E158" t="s">
-        <v>311</v>
+        <v>580</v>
       </c>
     </row>
     <row r="159" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
-        <v>284</v>
+        <v>480</v>
       </c>
       <c r="B159" t="s">
-        <v>285</v>
+        <v>501</v>
       </c>
       <c r="C159">
         <v>2</v>
@@ -6827,15 +7991,15 @@
         <v>0</v>
       </c>
       <c r="E159" t="s">
-        <v>312</v>
+        <v>581</v>
       </c>
     </row>
     <row r="160" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
-        <v>284</v>
+        <v>480</v>
       </c>
       <c r="B160" t="s">
-        <v>285</v>
+        <v>501</v>
       </c>
       <c r="C160">
         <v>3</v>
@@ -6844,32 +8008,32 @@
         <v>0</v>
       </c>
       <c r="E160" t="s">
-        <v>313</v>
+        <v>582</v>
       </c>
     </row>
     <row r="161" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
-        <v>96</v>
+        <v>481</v>
       </c>
       <c r="B161" t="s">
-        <v>97</v>
+        <v>502</v>
       </c>
       <c r="C161">
         <v>1</v>
       </c>
       <c r="D161" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E161" t="s">
-        <v>108</v>
+        <v>93</v>
       </c>
     </row>
     <row r="162" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
-        <v>96</v>
+        <v>481</v>
       </c>
       <c r="B162" t="s">
-        <v>97</v>
+        <v>502</v>
       </c>
       <c r="C162">
         <v>2</v>
@@ -6878,15 +8042,15 @@
         <v>0</v>
       </c>
       <c r="E162" t="s">
-        <v>109</v>
+        <v>583</v>
       </c>
     </row>
     <row r="163" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
-        <v>96</v>
+        <v>481</v>
       </c>
       <c r="B163" t="s">
-        <v>97</v>
+        <v>502</v>
       </c>
       <c r="C163">
         <v>3</v>
@@ -6895,15 +8059,15 @@
         <v>0</v>
       </c>
       <c r="E163" t="s">
-        <v>110</v>
+        <v>584</v>
       </c>
     </row>
     <row r="164" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
-        <v>314</v>
+        <v>482</v>
       </c>
       <c r="B164" t="s">
-        <v>315</v>
+        <v>503</v>
       </c>
       <c r="C164">
         <v>1</v>
@@ -6912,32 +8076,32 @@
         <v>1</v>
       </c>
       <c r="E164" t="s">
-        <v>320</v>
+        <v>82</v>
       </c>
     </row>
     <row r="165" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
-        <v>314</v>
+        <v>482</v>
       </c>
       <c r="B165" t="s">
-        <v>315</v>
+        <v>503</v>
       </c>
       <c r="C165">
         <v>2</v>
       </c>
       <c r="D165" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E165" t="s">
-        <v>58</v>
+        <v>585</v>
       </c>
     </row>
     <row r="166" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
-        <v>314</v>
+        <v>482</v>
       </c>
       <c r="B166" t="s">
-        <v>315</v>
+        <v>503</v>
       </c>
       <c r="C166">
         <v>3</v>
@@ -6946,32 +8110,32 @@
         <v>0</v>
       </c>
       <c r="E166" t="s">
-        <v>321</v>
+        <v>586</v>
       </c>
     </row>
     <row r="167" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
-        <v>76</v>
+        <v>483</v>
       </c>
       <c r="B167" t="s">
-        <v>77</v>
+        <v>504</v>
       </c>
       <c r="C167">
         <v>1</v>
       </c>
       <c r="D167" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E167" t="s">
-        <v>82</v>
+        <v>587</v>
       </c>
     </row>
     <row r="168" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
-        <v>76</v>
+        <v>483</v>
       </c>
       <c r="B168" t="s">
-        <v>77</v>
+        <v>504</v>
       </c>
       <c r="C168">
         <v>2</v>
@@ -6980,15 +8144,15 @@
         <v>0</v>
       </c>
       <c r="E168" t="s">
-        <v>83</v>
+        <v>588</v>
       </c>
     </row>
     <row r="169" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
-        <v>76</v>
+        <v>483</v>
       </c>
       <c r="B169" t="s">
-        <v>77</v>
+        <v>504</v>
       </c>
       <c r="C169">
         <v>3</v>
@@ -6997,15 +8161,15 @@
         <v>0</v>
       </c>
       <c r="E169" t="s">
-        <v>84</v>
+        <v>589</v>
       </c>
     </row>
     <row r="170" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
-        <v>23</v>
+        <v>484</v>
       </c>
       <c r="B170" t="s">
-        <v>24</v>
+        <v>505</v>
       </c>
       <c r="C170">
         <v>1</v>
@@ -7014,15 +8178,15 @@
         <v>0</v>
       </c>
       <c r="E170" t="s">
-        <v>61</v>
+        <v>590</v>
       </c>
     </row>
     <row r="171" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
-        <v>23</v>
+        <v>484</v>
       </c>
       <c r="B171" t="s">
-        <v>24</v>
+        <v>505</v>
       </c>
       <c r="C171">
         <v>2</v>
@@ -7031,15 +8195,15 @@
         <v>0</v>
       </c>
       <c r="E171" t="s">
-        <v>62</v>
+        <v>591</v>
       </c>
     </row>
     <row r="172" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
-        <v>23</v>
+        <v>484</v>
       </c>
       <c r="B172" t="s">
-        <v>24</v>
+        <v>505</v>
       </c>
       <c r="C172">
         <v>3</v>
@@ -7048,15 +8212,15 @@
         <v>0</v>
       </c>
       <c r="E172" t="s">
-        <v>63</v>
+        <v>592</v>
       </c>
     </row>
     <row r="173" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
-        <v>29</v>
+        <v>485</v>
       </c>
       <c r="B173" t="s">
-        <v>30</v>
+        <v>506</v>
       </c>
       <c r="C173">
         <v>1</v>
@@ -7065,15 +8229,15 @@
         <v>0</v>
       </c>
       <c r="E173" t="s">
-        <v>64</v>
+        <v>593</v>
       </c>
     </row>
     <row r="174" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
-        <v>29</v>
+        <v>485</v>
       </c>
       <c r="B174" t="s">
-        <v>30</v>
+        <v>506</v>
       </c>
       <c r="C174">
         <v>2</v>
@@ -7082,15 +8246,15 @@
         <v>0</v>
       </c>
       <c r="E174" t="s">
-        <v>65</v>
+        <v>594</v>
       </c>
     </row>
     <row r="175" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
-        <v>29</v>
+        <v>485</v>
       </c>
       <c r="B175" t="s">
-        <v>30</v>
+        <v>506</v>
       </c>
       <c r="C175">
         <v>3</v>
@@ -7099,32 +8263,32 @@
         <v>0</v>
       </c>
       <c r="E175" t="s">
-        <v>66</v>
+        <v>595</v>
       </c>
     </row>
     <row r="176" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
-        <v>36</v>
+        <v>486</v>
       </c>
       <c r="B176" t="s">
-        <v>37</v>
+        <v>507</v>
       </c>
       <c r="C176">
         <v>1</v>
       </c>
       <c r="D176" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E176" t="s">
-        <v>67</v>
+        <v>93</v>
       </c>
     </row>
     <row r="177" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
-        <v>36</v>
+        <v>486</v>
       </c>
       <c r="B177" t="s">
-        <v>37</v>
+        <v>507</v>
       </c>
       <c r="C177">
         <v>2</v>
@@ -7133,15 +8297,15 @@
         <v>0</v>
       </c>
       <c r="E177" t="s">
-        <v>68</v>
+        <v>596</v>
       </c>
     </row>
     <row r="178" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
-        <v>36</v>
+        <v>486</v>
       </c>
       <c r="B178" t="s">
-        <v>37</v>
+        <v>507</v>
       </c>
       <c r="C178">
         <v>3</v>
@@ -7150,6 +8314,1026 @@
         <v>0</v>
       </c>
       <c r="E178" t="s">
+        <v>597</v>
+      </c>
+    </row>
+    <row r="179" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A179" t="s">
+        <v>487</v>
+      </c>
+      <c r="B179" t="s">
+        <v>508</v>
+      </c>
+      <c r="C179">
+        <v>1</v>
+      </c>
+      <c r="D179" t="b">
+        <v>0</v>
+      </c>
+      <c r="E179" t="s">
+        <v>598</v>
+      </c>
+    </row>
+    <row r="180" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A180" t="s">
+        <v>487</v>
+      </c>
+      <c r="B180" t="s">
+        <v>508</v>
+      </c>
+      <c r="C180">
+        <v>2</v>
+      </c>
+      <c r="D180" t="b">
+        <v>0</v>
+      </c>
+      <c r="E180" t="s">
+        <v>599</v>
+      </c>
+    </row>
+    <row r="181" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A181" t="s">
+        <v>487</v>
+      </c>
+      <c r="B181" t="s">
+        <v>508</v>
+      </c>
+      <c r="C181">
+        <v>3</v>
+      </c>
+      <c r="D181" t="b">
+        <v>0</v>
+      </c>
+      <c r="E181" t="s">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="182" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A182" t="s">
+        <v>488</v>
+      </c>
+      <c r="B182" t="s">
+        <v>509</v>
+      </c>
+      <c r="C182">
+        <v>1</v>
+      </c>
+      <c r="D182" t="b">
+        <v>1</v>
+      </c>
+      <c r="E182" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="183" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A183" t="s">
+        <v>488</v>
+      </c>
+      <c r="B183" t="s">
+        <v>509</v>
+      </c>
+      <c r="C183">
+        <v>2</v>
+      </c>
+      <c r="D183" t="b">
+        <v>0</v>
+      </c>
+      <c r="E183" t="s">
+        <v>601</v>
+      </c>
+    </row>
+    <row r="184" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A184" t="s">
+        <v>488</v>
+      </c>
+      <c r="B184" t="s">
+        <v>509</v>
+      </c>
+      <c r="C184">
+        <v>3</v>
+      </c>
+      <c r="D184" t="b">
+        <v>0</v>
+      </c>
+      <c r="E184" t="s">
+        <v>602</v>
+      </c>
+    </row>
+    <row r="185" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A185" t="s">
+        <v>489</v>
+      </c>
+      <c r="B185" t="s">
+        <v>603</v>
+      </c>
+      <c r="C185">
+        <v>1</v>
+      </c>
+      <c r="D185" t="b">
+        <v>0</v>
+      </c>
+      <c r="E185" t="s">
+        <v>604</v>
+      </c>
+    </row>
+    <row r="186" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A186" t="s">
+        <v>489</v>
+      </c>
+      <c r="B186" t="s">
+        <v>603</v>
+      </c>
+      <c r="C186">
+        <v>2</v>
+      </c>
+      <c r="D186" t="b">
+        <v>0</v>
+      </c>
+      <c r="E186" t="s">
+        <v>605</v>
+      </c>
+    </row>
+    <row r="187" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A187" t="s">
+        <v>489</v>
+      </c>
+      <c r="B187" t="s">
+        <v>603</v>
+      </c>
+      <c r="C187">
+        <v>3</v>
+      </c>
+      <c r="D187" t="b">
+        <v>0</v>
+      </c>
+      <c r="E187" t="s">
+        <v>606</v>
+      </c>
+    </row>
+    <row r="188" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A188" t="s">
+        <v>490</v>
+      </c>
+      <c r="B188" t="s">
+        <v>510</v>
+      </c>
+      <c r="C188">
+        <v>1</v>
+      </c>
+      <c r="D188" t="b">
+        <v>1</v>
+      </c>
+      <c r="E188" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="189" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A189" t="s">
+        <v>490</v>
+      </c>
+      <c r="B189" t="s">
+        <v>510</v>
+      </c>
+      <c r="C189">
+        <v>2</v>
+      </c>
+      <c r="D189" t="b">
+        <v>0</v>
+      </c>
+      <c r="E189" t="s">
+        <v>607</v>
+      </c>
+    </row>
+    <row r="190" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A190" t="s">
+        <v>490</v>
+      </c>
+      <c r="B190" t="s">
+        <v>510</v>
+      </c>
+      <c r="C190">
+        <v>3</v>
+      </c>
+      <c r="D190" t="b">
+        <v>0</v>
+      </c>
+      <c r="E190" t="s">
+        <v>608</v>
+      </c>
+    </row>
+    <row r="191" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A191" t="s">
+        <v>491</v>
+      </c>
+      <c r="B191" t="s">
+        <v>512</v>
+      </c>
+      <c r="C191">
+        <v>1</v>
+      </c>
+      <c r="D191" t="b">
+        <v>1</v>
+      </c>
+      <c r="E191" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="192" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A192" t="s">
+        <v>491</v>
+      </c>
+      <c r="B192" t="s">
+        <v>512</v>
+      </c>
+      <c r="C192">
+        <v>2</v>
+      </c>
+      <c r="D192" t="b">
+        <v>0</v>
+      </c>
+      <c r="E192" t="s">
+        <v>609</v>
+      </c>
+    </row>
+    <row r="193" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A193" t="s">
+        <v>491</v>
+      </c>
+      <c r="B193" t="s">
+        <v>512</v>
+      </c>
+      <c r="C193">
+        <v>3</v>
+      </c>
+      <c r="D193" t="b">
+        <v>0</v>
+      </c>
+      <c r="E193" t="s">
+        <v>610</v>
+      </c>
+    </row>
+    <row r="194" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A194" t="s">
+        <v>492</v>
+      </c>
+      <c r="B194" t="s">
+        <v>513</v>
+      </c>
+      <c r="C194">
+        <v>1</v>
+      </c>
+      <c r="D194" t="b">
+        <v>1</v>
+      </c>
+      <c r="E194" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="195" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A195" t="s">
+        <v>492</v>
+      </c>
+      <c r="B195" t="s">
+        <v>513</v>
+      </c>
+      <c r="C195">
+        <v>2</v>
+      </c>
+      <c r="D195" t="b">
+        <v>0</v>
+      </c>
+      <c r="E195" t="s">
+        <v>611</v>
+      </c>
+    </row>
+    <row r="196" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A196" t="s">
+        <v>492</v>
+      </c>
+      <c r="B196" t="s">
+        <v>513</v>
+      </c>
+      <c r="C196">
+        <v>3</v>
+      </c>
+      <c r="D196" t="b">
+        <v>0</v>
+      </c>
+      <c r="E196" t="s">
+        <v>612</v>
+      </c>
+    </row>
+    <row r="197" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A197" t="s">
+        <v>493</v>
+      </c>
+      <c r="B197" t="s">
+        <v>514</v>
+      </c>
+      <c r="C197">
+        <v>1</v>
+      </c>
+      <c r="D197" t="b">
+        <v>0</v>
+      </c>
+      <c r="E197" t="s">
+        <v>613</v>
+      </c>
+    </row>
+    <row r="198" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A198" t="s">
+        <v>493</v>
+      </c>
+      <c r="B198" t="s">
+        <v>514</v>
+      </c>
+      <c r="C198">
+        <v>2</v>
+      </c>
+      <c r="D198" t="b">
+        <v>0</v>
+      </c>
+      <c r="E198" t="s">
+        <v>614</v>
+      </c>
+    </row>
+    <row r="199" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A199" t="s">
+        <v>493</v>
+      </c>
+      <c r="B199" t="s">
+        <v>514</v>
+      </c>
+      <c r="C199">
+        <v>3</v>
+      </c>
+      <c r="D199" t="b">
+        <v>0</v>
+      </c>
+      <c r="E199" t="s">
+        <v>615</v>
+      </c>
+    </row>
+    <row r="200" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A200" t="s">
+        <v>494</v>
+      </c>
+      <c r="B200" t="s">
+        <v>515</v>
+      </c>
+      <c r="C200">
+        <v>1</v>
+      </c>
+      <c r="D200" t="b">
+        <v>0</v>
+      </c>
+      <c r="E200" t="s">
+        <v>616</v>
+      </c>
+    </row>
+    <row r="201" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A201" t="s">
+        <v>494</v>
+      </c>
+      <c r="B201" t="s">
+        <v>515</v>
+      </c>
+      <c r="C201">
+        <v>2</v>
+      </c>
+      <c r="D201" t="b">
+        <v>0</v>
+      </c>
+      <c r="E201" t="s">
+        <v>617</v>
+      </c>
+    </row>
+    <row r="202" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A202" t="s">
+        <v>494</v>
+      </c>
+      <c r="B202" t="s">
+        <v>515</v>
+      </c>
+      <c r="C202">
+        <v>3</v>
+      </c>
+      <c r="D202" t="b">
+        <v>0</v>
+      </c>
+      <c r="E202" t="s">
+        <v>618</v>
+      </c>
+    </row>
+    <row r="203" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A203" t="s">
+        <v>495</v>
+      </c>
+      <c r="B203" t="s">
+        <v>516</v>
+      </c>
+      <c r="C203">
+        <v>1</v>
+      </c>
+      <c r="D203" t="b">
+        <v>0</v>
+      </c>
+      <c r="E203" t="s">
+        <v>619</v>
+      </c>
+    </row>
+    <row r="204" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A204" t="s">
+        <v>495</v>
+      </c>
+      <c r="B204" t="s">
+        <v>516</v>
+      </c>
+      <c r="C204">
+        <v>2</v>
+      </c>
+      <c r="D204" t="b">
+        <v>0</v>
+      </c>
+      <c r="E204" t="s">
+        <v>620</v>
+      </c>
+    </row>
+    <row r="205" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A205" t="s">
+        <v>495</v>
+      </c>
+      <c r="B205" t="s">
+        <v>516</v>
+      </c>
+      <c r="C205">
+        <v>3</v>
+      </c>
+      <c r="D205" t="b">
+        <v>0</v>
+      </c>
+      <c r="E205" t="s">
+        <v>621</v>
+      </c>
+    </row>
+    <row r="206" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A206" t="s">
+        <v>85</v>
+      </c>
+      <c r="B206" t="s">
+        <v>86</v>
+      </c>
+      <c r="C206">
+        <v>1</v>
+      </c>
+      <c r="D206" t="b">
+        <v>1</v>
+      </c>
+      <c r="E206" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="207" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A207" t="s">
+        <v>85</v>
+      </c>
+      <c r="B207" t="s">
+        <v>86</v>
+      </c>
+      <c r="C207">
+        <v>2</v>
+      </c>
+      <c r="D207" t="b">
+        <v>0</v>
+      </c>
+      <c r="E207" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="208" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A208" t="s">
+        <v>85</v>
+      </c>
+      <c r="B208" t="s">
+        <v>86</v>
+      </c>
+      <c r="C208">
+        <v>3</v>
+      </c>
+      <c r="D208" t="b">
+        <v>0</v>
+      </c>
+      <c r="E208" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="209" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A209" t="s">
+        <v>275</v>
+      </c>
+      <c r="B209" t="s">
+        <v>276</v>
+      </c>
+      <c r="C209">
+        <v>1</v>
+      </c>
+      <c r="D209" t="b">
+        <v>1</v>
+      </c>
+      <c r="E209" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="210" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A210" t="s">
+        <v>275</v>
+      </c>
+      <c r="B210" t="s">
+        <v>276</v>
+      </c>
+      <c r="C210">
+        <v>2</v>
+      </c>
+      <c r="D210" t="b">
+        <v>0</v>
+      </c>
+      <c r="E210" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="211" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A211" t="s">
+        <v>275</v>
+      </c>
+      <c r="B211" t="s">
+        <v>276</v>
+      </c>
+      <c r="C211">
+        <v>3</v>
+      </c>
+      <c r="D211" t="b">
+        <v>0</v>
+      </c>
+      <c r="E211" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="212" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A212" t="s">
+        <v>281</v>
+      </c>
+      <c r="B212" t="s">
+        <v>249</v>
+      </c>
+      <c r="C212">
+        <v>1</v>
+      </c>
+      <c r="D212" t="b">
+        <v>1</v>
+      </c>
+      <c r="E212" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="213" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A213" t="s">
+        <v>281</v>
+      </c>
+      <c r="B213" t="s">
+        <v>249</v>
+      </c>
+      <c r="C213">
+        <v>2</v>
+      </c>
+      <c r="D213" t="b">
+        <v>0</v>
+      </c>
+      <c r="E213" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="214" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A214" t="s">
+        <v>281</v>
+      </c>
+      <c r="B214" t="s">
+        <v>249</v>
+      </c>
+      <c r="C214">
+        <v>3</v>
+      </c>
+      <c r="D214" t="b">
+        <v>0</v>
+      </c>
+      <c r="E214" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="215" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A215" t="s">
+        <v>17</v>
+      </c>
+      <c r="B215" t="s">
+        <v>18</v>
+      </c>
+      <c r="C215">
+        <v>1</v>
+      </c>
+      <c r="D215" t="b">
+        <v>1</v>
+      </c>
+      <c r="E215" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="216" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A216" t="s">
+        <v>17</v>
+      </c>
+      <c r="B216" t="s">
+        <v>18</v>
+      </c>
+      <c r="C216">
+        <v>2</v>
+      </c>
+      <c r="D216" t="b">
+        <v>0</v>
+      </c>
+      <c r="E216" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="217" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A217" t="s">
+        <v>17</v>
+      </c>
+      <c r="B217" t="s">
+        <v>18</v>
+      </c>
+      <c r="C217">
+        <v>3</v>
+      </c>
+      <c r="D217" t="b">
+        <v>0</v>
+      </c>
+      <c r="E217" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="218" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A218" t="s">
+        <v>284</v>
+      </c>
+      <c r="B218" t="s">
+        <v>285</v>
+      </c>
+      <c r="C218">
+        <v>1</v>
+      </c>
+      <c r="D218" t="b">
+        <v>0</v>
+      </c>
+      <c r="E218" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="219" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A219" t="s">
+        <v>284</v>
+      </c>
+      <c r="B219" t="s">
+        <v>285</v>
+      </c>
+      <c r="C219">
+        <v>2</v>
+      </c>
+      <c r="D219" t="b">
+        <v>0</v>
+      </c>
+      <c r="E219" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="220" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A220" t="s">
+        <v>284</v>
+      </c>
+      <c r="B220" t="s">
+        <v>285</v>
+      </c>
+      <c r="C220">
+        <v>3</v>
+      </c>
+      <c r="D220" t="b">
+        <v>0</v>
+      </c>
+      <c r="E220" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="221" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A221" t="s">
+        <v>96</v>
+      </c>
+      <c r="B221" t="s">
+        <v>97</v>
+      </c>
+      <c r="C221">
+        <v>1</v>
+      </c>
+      <c r="D221" t="b">
+        <v>0</v>
+      </c>
+      <c r="E221" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="222" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A222" t="s">
+        <v>96</v>
+      </c>
+      <c r="B222" t="s">
+        <v>97</v>
+      </c>
+      <c r="C222">
+        <v>2</v>
+      </c>
+      <c r="D222" t="b">
+        <v>0</v>
+      </c>
+      <c r="E222" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="223" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A223" t="s">
+        <v>96</v>
+      </c>
+      <c r="B223" t="s">
+        <v>97</v>
+      </c>
+      <c r="C223">
+        <v>3</v>
+      </c>
+      <c r="D223" t="b">
+        <v>0</v>
+      </c>
+      <c r="E223" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="224" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A224" t="s">
+        <v>314</v>
+      </c>
+      <c r="B224" t="s">
+        <v>315</v>
+      </c>
+      <c r="C224">
+        <v>1</v>
+      </c>
+      <c r="D224" t="b">
+        <v>1</v>
+      </c>
+      <c r="E224" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="225" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A225" t="s">
+        <v>314</v>
+      </c>
+      <c r="B225" t="s">
+        <v>315</v>
+      </c>
+      <c r="C225">
+        <v>2</v>
+      </c>
+      <c r="D225" t="b">
+        <v>1</v>
+      </c>
+      <c r="E225" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="226" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A226" t="s">
+        <v>314</v>
+      </c>
+      <c r="B226" t="s">
+        <v>315</v>
+      </c>
+      <c r="C226">
+        <v>3</v>
+      </c>
+      <c r="D226" t="b">
+        <v>0</v>
+      </c>
+      <c r="E226" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="227" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A227" t="s">
+        <v>76</v>
+      </c>
+      <c r="B227" t="s">
+        <v>77</v>
+      </c>
+      <c r="C227">
+        <v>1</v>
+      </c>
+      <c r="D227" t="b">
+        <v>1</v>
+      </c>
+      <c r="E227" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="228" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A228" t="s">
+        <v>76</v>
+      </c>
+      <c r="B228" t="s">
+        <v>77</v>
+      </c>
+      <c r="C228">
+        <v>2</v>
+      </c>
+      <c r="D228" t="b">
+        <v>0</v>
+      </c>
+      <c r="E228" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="229" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A229" t="s">
+        <v>76</v>
+      </c>
+      <c r="B229" t="s">
+        <v>77</v>
+      </c>
+      <c r="C229">
+        <v>3</v>
+      </c>
+      <c r="D229" t="b">
+        <v>0</v>
+      </c>
+      <c r="E229" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="230" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A230" t="s">
+        <v>23</v>
+      </c>
+      <c r="B230" t="s">
+        <v>24</v>
+      </c>
+      <c r="C230">
+        <v>1</v>
+      </c>
+      <c r="D230" t="b">
+        <v>0</v>
+      </c>
+      <c r="E230" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="231" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A231" t="s">
+        <v>23</v>
+      </c>
+      <c r="B231" t="s">
+        <v>24</v>
+      </c>
+      <c r="C231">
+        <v>2</v>
+      </c>
+      <c r="D231" t="b">
+        <v>0</v>
+      </c>
+      <c r="E231" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="232" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A232" t="s">
+        <v>23</v>
+      </c>
+      <c r="B232" t="s">
+        <v>24</v>
+      </c>
+      <c r="C232">
+        <v>3</v>
+      </c>
+      <c r="D232" t="b">
+        <v>0</v>
+      </c>
+      <c r="E232" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="233" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A233" t="s">
+        <v>29</v>
+      </c>
+      <c r="B233" t="s">
+        <v>30</v>
+      </c>
+      <c r="C233">
+        <v>1</v>
+      </c>
+      <c r="D233" t="b">
+        <v>0</v>
+      </c>
+      <c r="E233" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="234" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A234" t="s">
+        <v>29</v>
+      </c>
+      <c r="B234" t="s">
+        <v>30</v>
+      </c>
+      <c r="C234">
+        <v>2</v>
+      </c>
+      <c r="D234" t="b">
+        <v>0</v>
+      </c>
+      <c r="E234" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="235" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A235" t="s">
+        <v>29</v>
+      </c>
+      <c r="B235" t="s">
+        <v>30</v>
+      </c>
+      <c r="C235">
+        <v>3</v>
+      </c>
+      <c r="D235" t="b">
+        <v>0</v>
+      </c>
+      <c r="E235" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="236" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A236" t="s">
+        <v>36</v>
+      </c>
+      <c r="B236" t="s">
+        <v>37</v>
+      </c>
+      <c r="C236">
+        <v>1</v>
+      </c>
+      <c r="D236" t="b">
+        <v>0</v>
+      </c>
+      <c r="E236" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="237" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A237" t="s">
+        <v>36</v>
+      </c>
+      <c r="B237" t="s">
+        <v>37</v>
+      </c>
+      <c r="C237">
+        <v>2</v>
+      </c>
+      <c r="D237" t="b">
+        <v>0</v>
+      </c>
+      <c r="E237" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="238" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A238" t="s">
+        <v>36</v>
+      </c>
+      <c r="B238" t="s">
+        <v>37</v>
+      </c>
+      <c r="C238">
+        <v>3</v>
+      </c>
+      <c r="D238" t="b">
+        <v>0</v>
+      </c>
+      <c r="E238" t="s">
         <v>69</v>
       </c>
     </row>

</xml_diff>

<commit_message>
added rider class and pretender card in skills
</commit_message>
<xml_diff>
--- a/data/Fate-Spreadsheet.xlsx
+++ b/data/Fate-Spreadsheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Important\Python\Fate-Wiki\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BAE09173-3834-4445-B317-789F4733B023}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74414681-1B7E-4E20-8CB8-128DF038A562}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{B05E798F-9EF6-4508-A0A4-311D06661AED}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{B05E798F-9EF6-4508-A0A4-311D06661AED}"/>
   </bookViews>
   <sheets>
     <sheet name="Servants" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1515" uniqueCount="622">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1860" uniqueCount="717">
   <si>
     <t>servant_id</t>
   </si>
@@ -1909,6 +1909,291 @@
   </si>
   <si>
     <t>Nostalgia Drive</t>
+  </si>
+  <si>
+    <t>Iskander of Macedonia</t>
+  </si>
+  <si>
+    <t>iskander-of-macedonia</t>
+  </si>
+  <si>
+    <t>2,2,3,3,4,5</t>
+  </si>
+  <si>
+    <t>Astolfo</t>
+  </si>
+  <si>
+    <t>Achilles</t>
+  </si>
+  <si>
+    <t>Ivan the Terrible</t>
+  </si>
+  <si>
+    <t>Francis Drake</t>
+  </si>
+  <si>
+    <t>Ushiwakamaru</t>
+  </si>
+  <si>
+    <t>Ozymandias</t>
+  </si>
+  <si>
+    <t>Sitonai</t>
+  </si>
+  <si>
+    <t>Odysseus</t>
+  </si>
+  <si>
+    <t>Queen Medb</t>
+  </si>
+  <si>
+    <t>Bartholomew Roberts</t>
+  </si>
+  <si>
+    <t>Boudica</t>
+  </si>
+  <si>
+    <t>Quetzalcoatl</t>
+  </si>
+  <si>
+    <t>Hephaistion</t>
+  </si>
+  <si>
+    <t>Sakamoto Ryouma</t>
+  </si>
+  <si>
+    <t>Edward Teach</t>
+  </si>
+  <si>
+    <t>Mandricardo</t>
+  </si>
+  <si>
+    <t>Saint Martha</t>
+  </si>
+  <si>
+    <t>Saint Georgios</t>
+  </si>
+  <si>
+    <t>Captain Nemo</t>
+  </si>
+  <si>
+    <t>Taisui Xingjun</t>
+  </si>
+  <si>
+    <t>Constantine XI</t>
+  </si>
+  <si>
+    <t>Pretender</t>
+  </si>
+  <si>
+    <t>3,3,3,4,5,5</t>
+  </si>
+  <si>
+    <t>3,3,3,5</t>
+  </si>
+  <si>
+    <t>Luck,Surveil,Surveil,Surveil</t>
+  </si>
+  <si>
+    <t>Surveil,Surveil,Preparation,Preparation</t>
+  </si>
+  <si>
+    <t>Luck,Surveil,Preparation,Berserker_Strength_9</t>
+  </si>
+  <si>
+    <t>3,3,3,4</t>
+  </si>
+  <si>
+    <t>Surveil,Surveil,Surveil,Luck,Luck</t>
+  </si>
+  <si>
+    <t>2,3,3,3</t>
+  </si>
+  <si>
+    <t>2,3,3,3,4</t>
+  </si>
+  <si>
+    <t>2,5,5,5</t>
+  </si>
+  <si>
+    <t>3,3,5</t>
+  </si>
+  <si>
+    <t>2,2,2,3,3,4</t>
+  </si>
+  <si>
+    <t>2,2,3,3,5,5</t>
+  </si>
+  <si>
+    <t>2,3,3,3,5</t>
+  </si>
+  <si>
+    <t>2,2,3,4,4,5</t>
+  </si>
+  <si>
+    <t>3,5</t>
+  </si>
+  <si>
+    <t>Luck,Luck,Surveil,Surveil,Preparation,Preparation</t>
+  </si>
+  <si>
+    <t>3,3,5,5</t>
+  </si>
+  <si>
+    <t>Luck,Luck,Surveil,Preparation</t>
+  </si>
+  <si>
+    <t>Ionian Hetairoi</t>
+  </si>
+  <si>
+    <t>Gordius Wheel</t>
+  </si>
+  <si>
+    <t>Casseur de Logistille</t>
+  </si>
+  <si>
+    <t>La Lune Noire</t>
+  </si>
+  <si>
+    <t>Trap of Argalia</t>
+  </si>
+  <si>
+    <t>Diatrekhon Aster Lonkhe</t>
+  </si>
+  <si>
+    <t>Akhilleus Kosmos</t>
+  </si>
+  <si>
+    <t>Andreias Amarantos</t>
+  </si>
+  <si>
+    <t>Oprichniki</t>
+  </si>
+  <si>
+    <t>Monstrous Form</t>
+  </si>
+  <si>
+    <t>The Golden Hind</t>
+  </si>
+  <si>
+    <t>Privateer's Glory</t>
+  </si>
+  <si>
+    <t>Eight Boat Leap</t>
+  </si>
+  <si>
+    <t>Icicle Cutter</t>
+  </si>
+  <si>
+    <t>Abu el-Hol Sphinx</t>
+  </si>
+  <si>
+    <t>Dendera Electric Bulb</t>
+  </si>
+  <si>
+    <t>Ramesseum Tentyris</t>
+  </si>
+  <si>
+    <t>Pohjola Fimbul</t>
+  </si>
+  <si>
+    <t>Combination Attack</t>
+  </si>
+  <si>
+    <t>Aigis</t>
+  </si>
+  <si>
+    <t>Troia Hippos</t>
+  </si>
+  <si>
+    <t>Chariot My Love</t>
+  </si>
+  <si>
+    <t>My Red Mead</t>
+  </si>
+  <si>
+    <t>The Royal Rover</t>
+  </si>
+  <si>
+    <t>Pirate's Code</t>
+  </si>
+  <si>
+    <t>Sword of Boudica</t>
+  </si>
+  <si>
+    <t>Chariot of Boudica</t>
+  </si>
+  <si>
+    <t>Piedra del Sol</t>
+  </si>
+  <si>
+    <t>Quetzalcoatlus</t>
+  </si>
+  <si>
+    <t>Blood Frenzy</t>
+  </si>
+  <si>
+    <t>Pretender Class</t>
+  </si>
+  <si>
+    <t>Hecatic Wheel</t>
+  </si>
+  <si>
+    <t>Like a Soaring Dragon</t>
+  </si>
+  <si>
+    <t>Dragon of Restoration</t>
+  </si>
+  <si>
+    <t>Blade of Restoration</t>
+  </si>
+  <si>
+    <t>Queen Anne's Revenge</t>
+  </si>
+  <si>
+    <t>Deviant Tastes</t>
+  </si>
+  <si>
+    <t>Serment de Durandal</t>
+  </si>
+  <si>
+    <t>Wooden Sword</t>
+  </si>
+  <si>
+    <t>Tarasque</t>
+  </si>
+  <si>
+    <t>Divine Obedience</t>
+  </si>
+  <si>
+    <t>Ascalon</t>
+  </si>
+  <si>
+    <t>Bayard</t>
+  </si>
+  <si>
+    <t>Martyr's Soul</t>
+  </si>
+  <si>
+    <t>The Nautilus</t>
+  </si>
+  <si>
+    <t>Memory Partition</t>
+  </si>
+  <si>
+    <t>Triton's Favour</t>
+  </si>
+  <si>
+    <t>Taisu Awaken</t>
+  </si>
+  <si>
+    <t>God of Calamity</t>
+  </si>
+  <si>
+    <t>Theodosios Constantinos</t>
+  </si>
+  <si>
+    <t>Twilit Empire</t>
   </si>
 </sst>
 </file>
@@ -4524,110 +4809,617 @@
       <c r="A72" t="s">
         <v>535</v>
       </c>
+      <c r="B72" t="s">
+        <v>622</v>
+      </c>
+      <c r="C72" t="s">
+        <v>623</v>
+      </c>
+      <c r="D72" t="s">
+        <v>278</v>
+      </c>
+      <c r="E72" t="s">
+        <v>8</v>
+      </c>
+      <c r="G72" s="2" t="s">
+        <v>624</v>
+      </c>
+      <c r="H72" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I72" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="J72" s="2" t="s">
+        <v>181</v>
+      </c>
+      <c r="K72" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="73" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>536</v>
       </c>
+      <c r="B73" t="s">
+        <v>625</v>
+      </c>
+      <c r="D73" t="s">
+        <v>278</v>
+      </c>
+      <c r="E73" t="s">
+        <v>89</v>
+      </c>
+      <c r="G73" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H73" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="I73" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="J73" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="K73" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="74" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>537</v>
       </c>
+      <c r="B74" t="s">
+        <v>626</v>
+      </c>
+      <c r="D74" t="s">
+        <v>278</v>
+      </c>
+      <c r="E74" t="s">
+        <v>40</v>
+      </c>
+      <c r="G74" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="H74" s="2" t="s">
+        <v>318</v>
+      </c>
+      <c r="J74" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="K74" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="75" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>538</v>
       </c>
+      <c r="B75" t="s">
+        <v>627</v>
+      </c>
+      <c r="D75" t="s">
+        <v>278</v>
+      </c>
+      <c r="E75" t="s">
+        <v>40</v>
+      </c>
+      <c r="G75" s="2" t="s">
+        <v>647</v>
+      </c>
+      <c r="I75" s="2" t="s">
+        <v>648</v>
+      </c>
+      <c r="J75" s="2" t="s">
+        <v>183</v>
+      </c>
+      <c r="K75" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="76" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>539</v>
       </c>
+      <c r="B76" t="s">
+        <v>628</v>
+      </c>
+      <c r="D76" t="s">
+        <v>278</v>
+      </c>
+      <c r="E76" t="s">
+        <v>8</v>
+      </c>
+      <c r="G76" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="H76" s="2" t="s">
+        <v>204</v>
+      </c>
+      <c r="J76" s="2" t="s">
+        <v>649</v>
+      </c>
+      <c r="K76" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="77" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>540</v>
       </c>
+      <c r="B77" t="s">
+        <v>629</v>
+      </c>
+      <c r="D77" t="s">
+        <v>278</v>
+      </c>
+      <c r="E77" t="s">
+        <v>89</v>
+      </c>
+      <c r="G77" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H77" s="2" t="s">
+        <v>624</v>
+      </c>
+      <c r="J77" s="2" t="s">
+        <v>650</v>
+      </c>
+      <c r="K77" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="78" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>541</v>
       </c>
+      <c r="B78" t="s">
+        <v>630</v>
+      </c>
+      <c r="D78" t="s">
+        <v>278</v>
+      </c>
+      <c r="E78" t="s">
+        <v>40</v>
+      </c>
+      <c r="G78" s="2" t="s">
+        <v>176</v>
+      </c>
+      <c r="H78" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I78" s="2" t="s">
+        <v>269</v>
+      </c>
+      <c r="J78" s="2" t="s">
+        <v>436</v>
+      </c>
+      <c r="K78" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="79" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>542</v>
       </c>
+      <c r="B79" t="s">
+        <v>631</v>
+      </c>
+      <c r="D79" t="s">
+        <v>79</v>
+      </c>
+      <c r="E79" t="s">
+        <v>99</v>
+      </c>
+      <c r="G79" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="H79" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="I79" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="J79" s="2" t="s">
+        <v>651</v>
+      </c>
+      <c r="K79" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="80" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>543</v>
       </c>
+      <c r="B80" t="s">
+        <v>632</v>
+      </c>
+      <c r="D80" t="s">
+        <v>278</v>
+      </c>
+      <c r="E80" t="s">
+        <v>8</v>
+      </c>
+      <c r="G80" s="2" t="s">
+        <v>652</v>
+      </c>
+      <c r="H80" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I80" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="J80" s="2" t="s">
+        <v>653</v>
+      </c>
+      <c r="K80" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="81" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>544</v>
       </c>
+      <c r="B81" t="s">
+        <v>633</v>
+      </c>
+      <c r="D81" t="s">
+        <v>278</v>
+      </c>
+      <c r="E81" t="s">
+        <v>33</v>
+      </c>
+      <c r="G81" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="H81" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="I81" s="2" t="s">
+        <v>280</v>
+      </c>
+      <c r="J81" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="K81" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="82" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>545</v>
       </c>
+      <c r="B82" t="s">
+        <v>634</v>
+      </c>
+      <c r="D82" t="s">
+        <v>278</v>
+      </c>
+      <c r="E82" t="s">
+        <v>33</v>
+      </c>
+      <c r="G82" s="2" t="s">
+        <v>654</v>
+      </c>
+      <c r="H82" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="J82" s="2" t="s">
+        <v>186</v>
+      </c>
+      <c r="K82" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="83" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>546</v>
       </c>
+      <c r="B83" t="s">
+        <v>635</v>
+      </c>
+      <c r="D83" t="s">
+        <v>278</v>
+      </c>
+      <c r="E83" t="s">
+        <v>89</v>
+      </c>
+      <c r="G83" s="2" t="s">
+        <v>431</v>
+      </c>
+      <c r="H83" s="2" t="s">
+        <v>655</v>
+      </c>
+      <c r="J83" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="K83" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="84" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>547</v>
       </c>
+      <c r="B84" t="s">
+        <v>636</v>
+      </c>
+      <c r="D84" t="s">
+        <v>278</v>
+      </c>
+      <c r="E84" t="s">
+        <v>89</v>
+      </c>
+      <c r="G84" s="2" t="s">
+        <v>656</v>
+      </c>
+      <c r="H84" s="2" t="s">
+        <v>460</v>
+      </c>
+      <c r="I84" s="2" t="s">
+        <v>395</v>
+      </c>
+      <c r="J84" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="K84" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="85" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>548</v>
       </c>
+      <c r="B85" t="s">
+        <v>637</v>
+      </c>
+      <c r="D85" t="s">
+        <v>646</v>
+      </c>
+      <c r="E85" t="s">
+        <v>8</v>
+      </c>
+      <c r="G85" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="H85" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="I85" s="2" t="s">
+        <v>657</v>
+      </c>
+      <c r="J85" s="2" t="s">
+        <v>200</v>
+      </c>
+      <c r="K85" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="86" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>549</v>
       </c>
+      <c r="B86" t="s">
+        <v>638</v>
+      </c>
+      <c r="D86" t="s">
+        <v>278</v>
+      </c>
+      <c r="E86" t="s">
+        <v>89</v>
+      </c>
+      <c r="G86" s="2" t="s">
+        <v>203</v>
+      </c>
+      <c r="H86" s="2" t="s">
+        <v>658</v>
+      </c>
+      <c r="J86" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="K86" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="87" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>550</v>
       </c>
+      <c r="B87" t="s">
+        <v>639</v>
+      </c>
+      <c r="D87" t="s">
+        <v>278</v>
+      </c>
+      <c r="E87" t="s">
+        <v>99</v>
+      </c>
+      <c r="G87" s="2" t="s">
+        <v>659</v>
+      </c>
+      <c r="H87" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="J87" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="K87" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="88" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>551</v>
       </c>
+      <c r="B88" t="s">
+        <v>640</v>
+      </c>
+      <c r="D88" t="s">
+        <v>278</v>
+      </c>
+      <c r="E88" t="s">
+        <v>99</v>
+      </c>
+      <c r="G88" s="2" t="s">
+        <v>660</v>
+      </c>
+      <c r="H88" s="2" t="s">
+        <v>652</v>
+      </c>
+      <c r="I88" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="J88" s="2" t="s">
+        <v>188</v>
+      </c>
+      <c r="K88" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="89" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>552</v>
       </c>
+      <c r="B89" t="s">
+        <v>641</v>
+      </c>
+      <c r="D89" t="s">
+        <v>278</v>
+      </c>
+      <c r="E89" t="s">
+        <v>8</v>
+      </c>
+      <c r="G89" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="H89" s="2" t="s">
+        <v>451</v>
+      </c>
+      <c r="I89" s="2" t="s">
+        <v>657</v>
+      </c>
+      <c r="J89" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="K89" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="90" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>553</v>
       </c>
+      <c r="B90" t="s">
+        <v>642</v>
+      </c>
+      <c r="D90" t="s">
+        <v>278</v>
+      </c>
+      <c r="E90" t="s">
+        <v>8</v>
+      </c>
+      <c r="G90" s="2" t="s">
+        <v>661</v>
+      </c>
+      <c r="H90" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="I90" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="J90" s="2" t="s">
+        <v>197</v>
+      </c>
+      <c r="K90" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="91" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>554</v>
       </c>
+      <c r="B91" t="s">
+        <v>643</v>
+      </c>
+      <c r="D91" t="s">
+        <v>278</v>
+      </c>
+      <c r="E91" t="s">
+        <v>8</v>
+      </c>
+      <c r="G91" s="2" t="s">
+        <v>191</v>
+      </c>
+      <c r="H91" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="I91" s="2" t="s">
+        <v>662</v>
+      </c>
+      <c r="J91" s="2" t="s">
+        <v>663</v>
+      </c>
+      <c r="K91" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="92" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>555</v>
       </c>
+      <c r="B92" t="s">
+        <v>644</v>
+      </c>
+      <c r="D92" t="s">
+        <v>79</v>
+      </c>
+      <c r="E92" t="s">
+        <v>89</v>
+      </c>
+      <c r="G92" s="2" t="s">
+        <v>664</v>
+      </c>
+      <c r="H92" s="2" t="s">
+        <v>199</v>
+      </c>
+      <c r="I92" s="2" t="s">
+        <v>451</v>
+      </c>
+      <c r="J92" s="2" t="s">
+        <v>665</v>
+      </c>
+      <c r="K92" t="b">
+        <v>0</v>
+      </c>
     </row>
     <row r="93" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>556</v>
+      </c>
+      <c r="B93" t="s">
+        <v>645</v>
+      </c>
+      <c r="D93" t="s">
+        <v>278</v>
+      </c>
+      <c r="E93" t="s">
+        <v>40</v>
+      </c>
+      <c r="G93" s="2" t="s">
+        <v>201</v>
+      </c>
+      <c r="H93" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="I93" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="J93" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="K93" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="94" spans="1:11" x14ac:dyDescent="0.25">
@@ -4892,7 +5684,7 @@
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="H2 I6:I7 I10 I12 H14 I18 I22 I24 I27 G34 I40 I42 I45 I52 I62" numberStoredAsText="1"/>
+    <ignoredError sqref="H2 I6:I7 I10 I12 H14 I18 I22 I24 I27 G34 I40 I42 I45 I52 I62 I72 H79 I80 I84 I88 I90 G91" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -5278,7 +6070,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84E3BB0D-5578-4069-B1C9-C3864EB2A429}">
-  <dimension ref="A1:F238"/>
+  <dimension ref="A1:F304"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="20.5703125" customWidth="1"/>
@@ -8880,10 +9672,10 @@
     </row>
     <row r="212" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A212" t="s">
-        <v>281</v>
+        <v>535</v>
       </c>
       <c r="B212" t="s">
-        <v>249</v>
+        <v>622</v>
       </c>
       <c r="C212">
         <v>1</v>
@@ -8892,15 +9684,15 @@
         <v>1</v>
       </c>
       <c r="E212" t="s">
-        <v>58</v>
+        <v>306</v>
       </c>
     </row>
     <row r="213" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A213" t="s">
-        <v>281</v>
+        <v>535</v>
       </c>
       <c r="B213" t="s">
-        <v>249</v>
+        <v>622</v>
       </c>
       <c r="C213">
         <v>2</v>
@@ -8909,15 +9701,15 @@
         <v>0</v>
       </c>
       <c r="E213" t="s">
-        <v>309</v>
+        <v>666</v>
       </c>
     </row>
     <row r="214" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A214" t="s">
-        <v>281</v>
+        <v>535</v>
       </c>
       <c r="B214" t="s">
-        <v>249</v>
+        <v>622</v>
       </c>
       <c r="C214">
         <v>3</v>
@@ -8926,32 +9718,32 @@
         <v>0</v>
       </c>
       <c r="E214" t="s">
-        <v>310</v>
+        <v>667</v>
       </c>
     </row>
     <row r="215" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A215" t="s">
-        <v>17</v>
+        <v>536</v>
       </c>
       <c r="B215" t="s">
-        <v>18</v>
+        <v>625</v>
       </c>
       <c r="C215">
         <v>1</v>
       </c>
       <c r="D215" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E215" t="s">
-        <v>58</v>
+        <v>668</v>
       </c>
     </row>
     <row r="216" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A216" t="s">
-        <v>17</v>
+        <v>536</v>
       </c>
       <c r="B216" t="s">
-        <v>18</v>
+        <v>625</v>
       </c>
       <c r="C216">
         <v>2</v>
@@ -8960,15 +9752,15 @@
         <v>0</v>
       </c>
       <c r="E216" t="s">
-        <v>59</v>
+        <v>669</v>
       </c>
     </row>
     <row r="217" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A217" t="s">
-        <v>17</v>
+        <v>536</v>
       </c>
       <c r="B217" t="s">
-        <v>18</v>
+        <v>625</v>
       </c>
       <c r="C217">
         <v>3</v>
@@ -8977,15 +9769,15 @@
         <v>0</v>
       </c>
       <c r="E217" t="s">
-        <v>60</v>
+        <v>670</v>
       </c>
     </row>
     <row r="218" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A218" t="s">
-        <v>284</v>
+        <v>537</v>
       </c>
       <c r="B218" t="s">
-        <v>285</v>
+        <v>626</v>
       </c>
       <c r="C218">
         <v>1</v>
@@ -8994,15 +9786,15 @@
         <v>0</v>
       </c>
       <c r="E218" t="s">
-        <v>311</v>
+        <v>671</v>
       </c>
     </row>
     <row r="219" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A219" t="s">
-        <v>284</v>
+        <v>537</v>
       </c>
       <c r="B219" t="s">
-        <v>285</v>
+        <v>626</v>
       </c>
       <c r="C219">
         <v>2</v>
@@ -9011,15 +9803,15 @@
         <v>0</v>
       </c>
       <c r="E219" t="s">
-        <v>312</v>
+        <v>672</v>
       </c>
     </row>
     <row r="220" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A220" t="s">
-        <v>284</v>
+        <v>537</v>
       </c>
       <c r="B220" t="s">
-        <v>285</v>
+        <v>626</v>
       </c>
       <c r="C220">
         <v>3</v>
@@ -9028,32 +9820,32 @@
         <v>0</v>
       </c>
       <c r="E220" t="s">
-        <v>313</v>
+        <v>673</v>
       </c>
     </row>
     <row r="221" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A221" t="s">
-        <v>96</v>
+        <v>538</v>
       </c>
       <c r="B221" t="s">
-        <v>97</v>
+        <v>627</v>
       </c>
       <c r="C221">
         <v>1</v>
       </c>
       <c r="D221" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E221" t="s">
-        <v>108</v>
+        <v>306</v>
       </c>
     </row>
     <row r="222" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A222" t="s">
-        <v>96</v>
+        <v>538</v>
       </c>
       <c r="B222" t="s">
-        <v>97</v>
+        <v>627</v>
       </c>
       <c r="C222">
         <v>2</v>
@@ -9062,15 +9854,15 @@
         <v>0</v>
       </c>
       <c r="E222" t="s">
-        <v>109</v>
+        <v>674</v>
       </c>
     </row>
     <row r="223" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A223" t="s">
-        <v>96</v>
+        <v>538</v>
       </c>
       <c r="B223" t="s">
-        <v>97</v>
+        <v>627</v>
       </c>
       <c r="C223">
         <v>3</v>
@@ -9079,15 +9871,15 @@
         <v>0</v>
       </c>
       <c r="E223" t="s">
-        <v>110</v>
+        <v>675</v>
       </c>
     </row>
     <row r="224" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A224" t="s">
-        <v>314</v>
+        <v>539</v>
       </c>
       <c r="B224" t="s">
-        <v>315</v>
+        <v>628</v>
       </c>
       <c r="C224">
         <v>1</v>
@@ -9096,32 +9888,32 @@
         <v>1</v>
       </c>
       <c r="E224" t="s">
-        <v>320</v>
+        <v>306</v>
       </c>
     </row>
     <row r="225" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A225" t="s">
-        <v>314</v>
+        <v>539</v>
       </c>
       <c r="B225" t="s">
-        <v>315</v>
+        <v>628</v>
       </c>
       <c r="C225">
         <v>2</v>
       </c>
       <c r="D225" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E225" t="s">
-        <v>58</v>
+        <v>676</v>
       </c>
     </row>
     <row r="226" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A226" t="s">
-        <v>314</v>
+        <v>539</v>
       </c>
       <c r="B226" t="s">
-        <v>315</v>
+        <v>628</v>
       </c>
       <c r="C226">
         <v>3</v>
@@ -9130,15 +9922,15 @@
         <v>0</v>
       </c>
       <c r="E226" t="s">
-        <v>321</v>
+        <v>677</v>
       </c>
     </row>
     <row r="227" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A227" t="s">
-        <v>76</v>
+        <v>540</v>
       </c>
       <c r="B227" t="s">
-        <v>77</v>
+        <v>629</v>
       </c>
       <c r="C227">
         <v>1</v>
@@ -9147,15 +9939,15 @@
         <v>1</v>
       </c>
       <c r="E227" t="s">
-        <v>82</v>
+        <v>306</v>
       </c>
     </row>
     <row r="228" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A228" t="s">
-        <v>76</v>
+        <v>540</v>
       </c>
       <c r="B228" t="s">
-        <v>77</v>
+        <v>629</v>
       </c>
       <c r="C228">
         <v>2</v>
@@ -9164,15 +9956,15 @@
         <v>0</v>
       </c>
       <c r="E228" t="s">
-        <v>83</v>
+        <v>678</v>
       </c>
     </row>
     <row r="229" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A229" t="s">
-        <v>76</v>
+        <v>540</v>
       </c>
       <c r="B229" t="s">
-        <v>77</v>
+        <v>629</v>
       </c>
       <c r="C229">
         <v>3</v>
@@ -9181,15 +9973,15 @@
         <v>0</v>
       </c>
       <c r="E229" t="s">
-        <v>84</v>
+        <v>679</v>
       </c>
     </row>
     <row r="230" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A230" t="s">
-        <v>23</v>
+        <v>541</v>
       </c>
       <c r="B230" t="s">
-        <v>24</v>
+        <v>630</v>
       </c>
       <c r="C230">
         <v>1</v>
@@ -9198,15 +9990,15 @@
         <v>0</v>
       </c>
       <c r="E230" t="s">
-        <v>61</v>
+        <v>680</v>
       </c>
     </row>
     <row r="231" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A231" t="s">
-        <v>23</v>
+        <v>541</v>
       </c>
       <c r="B231" t="s">
-        <v>24</v>
+        <v>630</v>
       </c>
       <c r="C231">
         <v>2</v>
@@ -9215,15 +10007,15 @@
         <v>0</v>
       </c>
       <c r="E231" t="s">
-        <v>62</v>
+        <v>681</v>
       </c>
     </row>
     <row r="232" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A232" t="s">
-        <v>23</v>
+        <v>541</v>
       </c>
       <c r="B232" t="s">
-        <v>24</v>
+        <v>630</v>
       </c>
       <c r="C232">
         <v>3</v>
@@ -9232,32 +10024,32 @@
         <v>0</v>
       </c>
       <c r="E232" t="s">
-        <v>63</v>
+        <v>682</v>
       </c>
     </row>
     <row r="233" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A233" t="s">
-        <v>29</v>
+        <v>542</v>
       </c>
       <c r="B233" t="s">
-        <v>30</v>
+        <v>631</v>
       </c>
       <c r="C233">
         <v>1</v>
       </c>
       <c r="D233" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E233" t="s">
-        <v>64</v>
+        <v>82</v>
       </c>
     </row>
     <row r="234" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A234" t="s">
-        <v>29</v>
+        <v>542</v>
       </c>
       <c r="B234" t="s">
-        <v>30</v>
+        <v>631</v>
       </c>
       <c r="C234">
         <v>2</v>
@@ -9266,15 +10058,15 @@
         <v>0</v>
       </c>
       <c r="E234" t="s">
-        <v>65</v>
+        <v>683</v>
       </c>
     </row>
     <row r="235" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A235" t="s">
-        <v>29</v>
+        <v>542</v>
       </c>
       <c r="B235" t="s">
-        <v>30</v>
+        <v>631</v>
       </c>
       <c r="C235">
         <v>3</v>
@@ -9283,32 +10075,32 @@
         <v>0</v>
       </c>
       <c r="E235" t="s">
-        <v>66</v>
+        <v>684</v>
       </c>
     </row>
     <row r="236" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A236" t="s">
-        <v>36</v>
+        <v>543</v>
       </c>
       <c r="B236" t="s">
-        <v>37</v>
+        <v>632</v>
       </c>
       <c r="C236">
         <v>1</v>
       </c>
       <c r="D236" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E236" t="s">
-        <v>67</v>
+        <v>306</v>
       </c>
     </row>
     <row r="237" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A237" t="s">
-        <v>36</v>
+        <v>543</v>
       </c>
       <c r="B237" t="s">
-        <v>37</v>
+        <v>632</v>
       </c>
       <c r="C237">
         <v>2</v>
@@ -9317,15 +10109,15 @@
         <v>0</v>
       </c>
       <c r="E237" t="s">
-        <v>68</v>
+        <v>685</v>
       </c>
     </row>
     <row r="238" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A238" t="s">
-        <v>36</v>
+        <v>543</v>
       </c>
       <c r="B238" t="s">
-        <v>37</v>
+        <v>632</v>
       </c>
       <c r="C238">
         <v>3</v>
@@ -9334,6 +10126,1128 @@
         <v>0</v>
       </c>
       <c r="E238" t="s">
+        <v>686</v>
+      </c>
+    </row>
+    <row r="239" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A239" t="s">
+        <v>544</v>
+      </c>
+      <c r="B239" t="s">
+        <v>633</v>
+      </c>
+      <c r="C239">
+        <v>1</v>
+      </c>
+      <c r="D239" t="b">
+        <v>1</v>
+      </c>
+      <c r="E239" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="240" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A240" t="s">
+        <v>544</v>
+      </c>
+      <c r="B240" t="s">
+        <v>633</v>
+      </c>
+      <c r="C240">
+        <v>2</v>
+      </c>
+      <c r="D240" t="b">
+        <v>0</v>
+      </c>
+      <c r="E240" t="s">
+        <v>687</v>
+      </c>
+    </row>
+    <row r="241" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A241" t="s">
+        <v>544</v>
+      </c>
+      <c r="B241" t="s">
+        <v>633</v>
+      </c>
+      <c r="C241">
+        <v>3</v>
+      </c>
+      <c r="D241" t="b">
+        <v>0</v>
+      </c>
+      <c r="E241" t="s">
+        <v>688</v>
+      </c>
+    </row>
+    <row r="242" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A242" t="s">
+        <v>545</v>
+      </c>
+      <c r="B242" t="s">
+        <v>634</v>
+      </c>
+      <c r="C242">
+        <v>1</v>
+      </c>
+      <c r="D242" t="b">
+        <v>1</v>
+      </c>
+      <c r="E242" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="243" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A243" t="s">
+        <v>545</v>
+      </c>
+      <c r="B243" t="s">
+        <v>634</v>
+      </c>
+      <c r="C243">
+        <v>2</v>
+      </c>
+      <c r="D243" t="b">
+        <v>0</v>
+      </c>
+      <c r="E243" t="s">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="244" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A244" t="s">
+        <v>545</v>
+      </c>
+      <c r="B244" t="s">
+        <v>634</v>
+      </c>
+      <c r="C244">
+        <v>3</v>
+      </c>
+      <c r="D244" t="b">
+        <v>0</v>
+      </c>
+      <c r="E244" t="s">
+        <v>690</v>
+      </c>
+    </row>
+    <row r="245" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A245" t="s">
+        <v>546</v>
+      </c>
+      <c r="B245" t="s">
+        <v>635</v>
+      </c>
+      <c r="C245">
+        <v>1</v>
+      </c>
+      <c r="D245" t="b">
+        <v>1</v>
+      </c>
+      <c r="E245" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="246" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A246" t="s">
+        <v>546</v>
+      </c>
+      <c r="B246" t="s">
+        <v>635</v>
+      </c>
+      <c r="C246">
+        <v>2</v>
+      </c>
+      <c r="D246" t="b">
+        <v>0</v>
+      </c>
+      <c r="E246" t="s">
+        <v>691</v>
+      </c>
+    </row>
+    <row r="247" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A247" t="s">
+        <v>546</v>
+      </c>
+      <c r="B247" t="s">
+        <v>635</v>
+      </c>
+      <c r="C247">
+        <v>3</v>
+      </c>
+      <c r="D247" t="b">
+        <v>0</v>
+      </c>
+      <c r="E247" t="s">
+        <v>692</v>
+      </c>
+    </row>
+    <row r="248" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A248" t="s">
+        <v>547</v>
+      </c>
+      <c r="B248" t="s">
+        <v>636</v>
+      </c>
+      <c r="C248">
+        <v>1</v>
+      </c>
+      <c r="D248" t="b">
+        <v>0</v>
+      </c>
+      <c r="E248" t="s">
+        <v>693</v>
+      </c>
+    </row>
+    <row r="249" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A249" t="s">
+        <v>547</v>
+      </c>
+      <c r="B249" t="s">
+        <v>636</v>
+      </c>
+      <c r="C249">
+        <v>2</v>
+      </c>
+      <c r="D249" t="b">
+        <v>0</v>
+      </c>
+      <c r="E249" t="s">
+        <v>694</v>
+      </c>
+    </row>
+    <row r="250" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A250" t="s">
+        <v>547</v>
+      </c>
+      <c r="B250" t="s">
+        <v>636</v>
+      </c>
+      <c r="C250">
+        <v>3</v>
+      </c>
+      <c r="D250" t="b">
+        <v>0</v>
+      </c>
+      <c r="E250" t="s">
+        <v>695</v>
+      </c>
+    </row>
+    <row r="251" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A251" t="s">
+        <v>548</v>
+      </c>
+      <c r="B251" t="s">
+        <v>637</v>
+      </c>
+      <c r="C251">
+        <v>1</v>
+      </c>
+      <c r="D251" t="b">
+        <v>1</v>
+      </c>
+      <c r="E251" t="s">
+        <v>696</v>
+      </c>
+    </row>
+    <row r="252" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A252" t="s">
+        <v>548</v>
+      </c>
+      <c r="B252" t="s">
+        <v>637</v>
+      </c>
+      <c r="C252">
+        <v>2</v>
+      </c>
+      <c r="D252" t="b">
+        <v>1</v>
+      </c>
+      <c r="E252" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="253" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A253" t="s">
+        <v>548</v>
+      </c>
+      <c r="B253" t="s">
+        <v>637</v>
+      </c>
+      <c r="C253">
+        <v>3</v>
+      </c>
+      <c r="D253" t="b">
+        <v>0</v>
+      </c>
+      <c r="E253" t="s">
+        <v>697</v>
+      </c>
+    </row>
+    <row r="254" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A254" t="s">
+        <v>549</v>
+      </c>
+      <c r="B254" t="s">
+        <v>638</v>
+      </c>
+      <c r="C254">
+        <v>1</v>
+      </c>
+      <c r="D254" t="b">
+        <v>0</v>
+      </c>
+      <c r="E254" t="s">
+        <v>698</v>
+      </c>
+    </row>
+    <row r="255" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A255" t="s">
+        <v>549</v>
+      </c>
+      <c r="B255" t="s">
+        <v>638</v>
+      </c>
+      <c r="C255">
+        <v>2</v>
+      </c>
+      <c r="D255" t="b">
+        <v>0</v>
+      </c>
+      <c r="E255" t="s">
+        <v>699</v>
+      </c>
+    </row>
+    <row r="256" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A256" t="s">
+        <v>549</v>
+      </c>
+      <c r="B256" t="s">
+        <v>638</v>
+      </c>
+      <c r="C256">
+        <v>3</v>
+      </c>
+      <c r="D256" t="b">
+        <v>0</v>
+      </c>
+      <c r="E256" t="s">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="257" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A257" t="s">
+        <v>550</v>
+      </c>
+      <c r="B257" t="s">
+        <v>639</v>
+      </c>
+      <c r="C257">
+        <v>1</v>
+      </c>
+      <c r="D257" t="b">
+        <v>1</v>
+      </c>
+      <c r="E257" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="258" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A258" t="s">
+        <v>550</v>
+      </c>
+      <c r="B258" t="s">
+        <v>639</v>
+      </c>
+      <c r="C258">
+        <v>2</v>
+      </c>
+      <c r="D258" t="b">
+        <v>0</v>
+      </c>
+      <c r="E258" t="s">
+        <v>701</v>
+      </c>
+    </row>
+    <row r="259" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A259" t="s">
+        <v>550</v>
+      </c>
+      <c r="B259" t="s">
+        <v>639</v>
+      </c>
+      <c r="C259">
+        <v>3</v>
+      </c>
+      <c r="D259" t="b">
+        <v>0</v>
+      </c>
+      <c r="E259" t="s">
+        <v>702</v>
+      </c>
+    </row>
+    <row r="260" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A260" t="s">
+        <v>551</v>
+      </c>
+      <c r="B260" t="s">
+        <v>640</v>
+      </c>
+      <c r="C260">
+        <v>1</v>
+      </c>
+      <c r="D260" t="b">
+        <v>1</v>
+      </c>
+      <c r="E260" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="261" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A261" t="s">
+        <v>551</v>
+      </c>
+      <c r="B261" t="s">
+        <v>640</v>
+      </c>
+      <c r="C261">
+        <v>2</v>
+      </c>
+      <c r="D261" t="b">
+        <v>0</v>
+      </c>
+      <c r="E261" t="s">
+        <v>703</v>
+      </c>
+    </row>
+    <row r="262" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A262" t="s">
+        <v>551</v>
+      </c>
+      <c r="B262" t="s">
+        <v>640</v>
+      </c>
+      <c r="C262">
+        <v>3</v>
+      </c>
+      <c r="D262" t="b">
+        <v>0</v>
+      </c>
+      <c r="E262" t="s">
+        <v>704</v>
+      </c>
+    </row>
+    <row r="263" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A263" t="s">
+        <v>552</v>
+      </c>
+      <c r="B263" t="s">
+        <v>641</v>
+      </c>
+      <c r="C263">
+        <v>1</v>
+      </c>
+      <c r="D263" t="b">
+        <v>1</v>
+      </c>
+      <c r="E263" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="264" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A264" t="s">
+        <v>552</v>
+      </c>
+      <c r="B264" t="s">
+        <v>641</v>
+      </c>
+      <c r="C264">
+        <v>2</v>
+      </c>
+      <c r="D264" t="b">
+        <v>0</v>
+      </c>
+      <c r="E264" t="s">
+        <v>705</v>
+      </c>
+    </row>
+    <row r="265" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A265" t="s">
+        <v>552</v>
+      </c>
+      <c r="B265" t="s">
+        <v>641</v>
+      </c>
+      <c r="C265">
+        <v>3</v>
+      </c>
+      <c r="D265" t="b">
+        <v>0</v>
+      </c>
+      <c r="E265" t="s">
+        <v>706</v>
+      </c>
+    </row>
+    <row r="266" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A266" t="s">
+        <v>553</v>
+      </c>
+      <c r="B266" t="s">
+        <v>642</v>
+      </c>
+      <c r="C266">
+        <v>1</v>
+      </c>
+      <c r="D266" t="b">
+        <v>0</v>
+      </c>
+      <c r="E266" t="s">
+        <v>707</v>
+      </c>
+    </row>
+    <row r="267" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A267" t="s">
+        <v>553</v>
+      </c>
+      <c r="B267" t="s">
+        <v>642</v>
+      </c>
+      <c r="C267">
+        <v>2</v>
+      </c>
+      <c r="D267" t="b">
+        <v>0</v>
+      </c>
+      <c r="E267" t="s">
+        <v>708</v>
+      </c>
+    </row>
+    <row r="268" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A268" t="s">
+        <v>553</v>
+      </c>
+      <c r="B268" t="s">
+        <v>642</v>
+      </c>
+      <c r="C268">
+        <v>3</v>
+      </c>
+      <c r="D268" t="b">
+        <v>0</v>
+      </c>
+      <c r="E268" t="s">
+        <v>709</v>
+      </c>
+    </row>
+    <row r="269" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A269" t="s">
+        <v>554</v>
+      </c>
+      <c r="B269" t="s">
+        <v>643</v>
+      </c>
+      <c r="C269">
+        <v>1</v>
+      </c>
+      <c r="D269" t="b">
+        <v>0</v>
+      </c>
+      <c r="E269" t="s">
+        <v>710</v>
+      </c>
+    </row>
+    <row r="270" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A270" t="s">
+        <v>554</v>
+      </c>
+      <c r="B270" t="s">
+        <v>643</v>
+      </c>
+      <c r="C270">
+        <v>2</v>
+      </c>
+      <c r="D270" t="b">
+        <v>0</v>
+      </c>
+      <c r="E270" t="s">
+        <v>711</v>
+      </c>
+    </row>
+    <row r="271" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A271" t="s">
+        <v>554</v>
+      </c>
+      <c r="B271" t="s">
+        <v>643</v>
+      </c>
+      <c r="C271">
+        <v>3</v>
+      </c>
+      <c r="D271" t="b">
+        <v>0</v>
+      </c>
+      <c r="E271" t="s">
+        <v>712</v>
+      </c>
+    </row>
+    <row r="272" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A272" t="s">
+        <v>555</v>
+      </c>
+      <c r="B272" t="s">
+        <v>644</v>
+      </c>
+      <c r="C272">
+        <v>1</v>
+      </c>
+      <c r="D272" t="b">
+        <v>1</v>
+      </c>
+      <c r="E272" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="273" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A273" t="s">
+        <v>555</v>
+      </c>
+      <c r="B273" t="s">
+        <v>644</v>
+      </c>
+      <c r="C273">
+        <v>2</v>
+      </c>
+      <c r="D273" t="b">
+        <v>0</v>
+      </c>
+      <c r="E273" t="s">
+        <v>713</v>
+      </c>
+    </row>
+    <row r="274" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A274" t="s">
+        <v>555</v>
+      </c>
+      <c r="B274" t="s">
+        <v>644</v>
+      </c>
+      <c r="C274">
+        <v>3</v>
+      </c>
+      <c r="D274" t="b">
+        <v>0</v>
+      </c>
+      <c r="E274" t="s">
+        <v>714</v>
+      </c>
+    </row>
+    <row r="275" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A275" t="s">
+        <v>556</v>
+      </c>
+      <c r="B275" t="s">
+        <v>645</v>
+      </c>
+      <c r="C275">
+        <v>1</v>
+      </c>
+      <c r="D275" t="b">
+        <v>1</v>
+      </c>
+      <c r="E275" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="276" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A276" t="s">
+        <v>556</v>
+      </c>
+      <c r="B276" t="s">
+        <v>645</v>
+      </c>
+      <c r="C276">
+        <v>2</v>
+      </c>
+      <c r="D276" t="b">
+        <v>0</v>
+      </c>
+      <c r="E276" t="s">
+        <v>715</v>
+      </c>
+    </row>
+    <row r="277" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A277" t="s">
+        <v>556</v>
+      </c>
+      <c r="B277" t="s">
+        <v>645</v>
+      </c>
+      <c r="C277">
+        <v>3</v>
+      </c>
+      <c r="D277" t="b">
+        <v>0</v>
+      </c>
+      <c r="E277" t="s">
+        <v>716</v>
+      </c>
+    </row>
+    <row r="278" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A278" t="s">
+        <v>281</v>
+      </c>
+      <c r="B278" t="s">
+        <v>249</v>
+      </c>
+      <c r="C278">
+        <v>1</v>
+      </c>
+      <c r="D278" t="b">
+        <v>1</v>
+      </c>
+      <c r="E278" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="279" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A279" t="s">
+        <v>281</v>
+      </c>
+      <c r="B279" t="s">
+        <v>249</v>
+      </c>
+      <c r="C279">
+        <v>2</v>
+      </c>
+      <c r="D279" t="b">
+        <v>0</v>
+      </c>
+      <c r="E279" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="280" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A280" t="s">
+        <v>281</v>
+      </c>
+      <c r="B280" t="s">
+        <v>249</v>
+      </c>
+      <c r="C280">
+        <v>3</v>
+      </c>
+      <c r="D280" t="b">
+        <v>0</v>
+      </c>
+      <c r="E280" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="281" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A281" t="s">
+        <v>17</v>
+      </c>
+      <c r="B281" t="s">
+        <v>18</v>
+      </c>
+      <c r="C281">
+        <v>1</v>
+      </c>
+      <c r="D281" t="b">
+        <v>1</v>
+      </c>
+      <c r="E281" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="282" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A282" t="s">
+        <v>17</v>
+      </c>
+      <c r="B282" t="s">
+        <v>18</v>
+      </c>
+      <c r="C282">
+        <v>2</v>
+      </c>
+      <c r="D282" t="b">
+        <v>0</v>
+      </c>
+      <c r="E282" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="283" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A283" t="s">
+        <v>17</v>
+      </c>
+      <c r="B283" t="s">
+        <v>18</v>
+      </c>
+      <c r="C283">
+        <v>3</v>
+      </c>
+      <c r="D283" t="b">
+        <v>0</v>
+      </c>
+      <c r="E283" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="284" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A284" t="s">
+        <v>284</v>
+      </c>
+      <c r="B284" t="s">
+        <v>285</v>
+      </c>
+      <c r="C284">
+        <v>1</v>
+      </c>
+      <c r="D284" t="b">
+        <v>0</v>
+      </c>
+      <c r="E284" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="285" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A285" t="s">
+        <v>284</v>
+      </c>
+      <c r="B285" t="s">
+        <v>285</v>
+      </c>
+      <c r="C285">
+        <v>2</v>
+      </c>
+      <c r="D285" t="b">
+        <v>0</v>
+      </c>
+      <c r="E285" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="286" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A286" t="s">
+        <v>284</v>
+      </c>
+      <c r="B286" t="s">
+        <v>285</v>
+      </c>
+      <c r="C286">
+        <v>3</v>
+      </c>
+      <c r="D286" t="b">
+        <v>0</v>
+      </c>
+      <c r="E286" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="287" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A287" t="s">
+        <v>96</v>
+      </c>
+      <c r="B287" t="s">
+        <v>97</v>
+      </c>
+      <c r="C287">
+        <v>1</v>
+      </c>
+      <c r="D287" t="b">
+        <v>0</v>
+      </c>
+      <c r="E287" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="288" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A288" t="s">
+        <v>96</v>
+      </c>
+      <c r="B288" t="s">
+        <v>97</v>
+      </c>
+      <c r="C288">
+        <v>2</v>
+      </c>
+      <c r="D288" t="b">
+        <v>0</v>
+      </c>
+      <c r="E288" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="289" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A289" t="s">
+        <v>96</v>
+      </c>
+      <c r="B289" t="s">
+        <v>97</v>
+      </c>
+      <c r="C289">
+        <v>3</v>
+      </c>
+      <c r="D289" t="b">
+        <v>0</v>
+      </c>
+      <c r="E289" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="290" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A290" t="s">
+        <v>314</v>
+      </c>
+      <c r="B290" t="s">
+        <v>315</v>
+      </c>
+      <c r="C290">
+        <v>1</v>
+      </c>
+      <c r="D290" t="b">
+        <v>1</v>
+      </c>
+      <c r="E290" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="291" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A291" t="s">
+        <v>314</v>
+      </c>
+      <c r="B291" t="s">
+        <v>315</v>
+      </c>
+      <c r="C291">
+        <v>2</v>
+      </c>
+      <c r="D291" t="b">
+        <v>1</v>
+      </c>
+      <c r="E291" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="292" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A292" t="s">
+        <v>314</v>
+      </c>
+      <c r="B292" t="s">
+        <v>315</v>
+      </c>
+      <c r="C292">
+        <v>3</v>
+      </c>
+      <c r="D292" t="b">
+        <v>0</v>
+      </c>
+      <c r="E292" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="293" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A293" t="s">
+        <v>76</v>
+      </c>
+      <c r="B293" t="s">
+        <v>77</v>
+      </c>
+      <c r="C293">
+        <v>1</v>
+      </c>
+      <c r="D293" t="b">
+        <v>1</v>
+      </c>
+      <c r="E293" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="294" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A294" t="s">
+        <v>76</v>
+      </c>
+      <c r="B294" t="s">
+        <v>77</v>
+      </c>
+      <c r="C294">
+        <v>2</v>
+      </c>
+      <c r="D294" t="b">
+        <v>0</v>
+      </c>
+      <c r="E294" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="295" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A295" t="s">
+        <v>76</v>
+      </c>
+      <c r="B295" t="s">
+        <v>77</v>
+      </c>
+      <c r="C295">
+        <v>3</v>
+      </c>
+      <c r="D295" t="b">
+        <v>0</v>
+      </c>
+      <c r="E295" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="296" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A296" t="s">
+        <v>23</v>
+      </c>
+      <c r="B296" t="s">
+        <v>24</v>
+      </c>
+      <c r="C296">
+        <v>1</v>
+      </c>
+      <c r="D296" t="b">
+        <v>0</v>
+      </c>
+      <c r="E296" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="297" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A297" t="s">
+        <v>23</v>
+      </c>
+      <c r="B297" t="s">
+        <v>24</v>
+      </c>
+      <c r="C297">
+        <v>2</v>
+      </c>
+      <c r="D297" t="b">
+        <v>0</v>
+      </c>
+      <c r="E297" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="298" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A298" t="s">
+        <v>23</v>
+      </c>
+      <c r="B298" t="s">
+        <v>24</v>
+      </c>
+      <c r="C298">
+        <v>3</v>
+      </c>
+      <c r="D298" t="b">
+        <v>0</v>
+      </c>
+      <c r="E298" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="299" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A299" t="s">
+        <v>29</v>
+      </c>
+      <c r="B299" t="s">
+        <v>30</v>
+      </c>
+      <c r="C299">
+        <v>1</v>
+      </c>
+      <c r="D299" t="b">
+        <v>0</v>
+      </c>
+      <c r="E299" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="300" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A300" t="s">
+        <v>29</v>
+      </c>
+      <c r="B300" t="s">
+        <v>30</v>
+      </c>
+      <c r="C300">
+        <v>2</v>
+      </c>
+      <c r="D300" t="b">
+        <v>0</v>
+      </c>
+      <c r="E300" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="301" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A301" t="s">
+        <v>29</v>
+      </c>
+      <c r="B301" t="s">
+        <v>30</v>
+      </c>
+      <c r="C301">
+        <v>3</v>
+      </c>
+      <c r="D301" t="b">
+        <v>0</v>
+      </c>
+      <c r="E301" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="302" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A302" t="s">
+        <v>36</v>
+      </c>
+      <c r="B302" t="s">
+        <v>37</v>
+      </c>
+      <c r="C302">
+        <v>1</v>
+      </c>
+      <c r="D302" t="b">
+        <v>0</v>
+      </c>
+      <c r="E302" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="303" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A303" t="s">
+        <v>36</v>
+      </c>
+      <c r="B303" t="s">
+        <v>37</v>
+      </c>
+      <c r="C303">
+        <v>2</v>
+      </c>
+      <c r="D303" t="b">
+        <v>0</v>
+      </c>
+      <c r="E303" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="304" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A304" t="s">
+        <v>36</v>
+      </c>
+      <c r="B304" t="s">
+        <v>37</v>
+      </c>
+      <c r="C304">
+        <v>3</v>
+      </c>
+      <c r="D304" t="b">
+        <v>0</v>
+      </c>
+      <c r="E304" t="s">
         <v>69</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fixed spreadsheet to add rider slugs
</commit_message>
<xml_diff>
--- a/data/Fate-Spreadsheet.xlsx
+++ b/data/Fate-Spreadsheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Important\Python\Fate-Wiki\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{74414681-1B7E-4E20-8CB8-128DF038A562}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF92ED3E-3185-4BAF-9CCD-CBCFD6240792}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="2" xr2:uid="{B05E798F-9EF6-4508-A0A4-311D06661AED}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{B05E798F-9EF6-4508-A0A4-311D06661AED}"/>
   </bookViews>
   <sheets>
     <sheet name="Servants" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1860" uniqueCount="717">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1881" uniqueCount="738">
   <si>
     <t>servant_id</t>
   </si>
@@ -2194,6 +2194,69 @@
   </si>
   <si>
     <t>Twilit Empire</t>
+  </si>
+  <si>
+    <t>astolfo</t>
+  </si>
+  <si>
+    <t>achilles</t>
+  </si>
+  <si>
+    <t>ushiwakamaru</t>
+  </si>
+  <si>
+    <t>ozymandias</t>
+  </si>
+  <si>
+    <t>sitonai</t>
+  </si>
+  <si>
+    <t>odysseus</t>
+  </si>
+  <si>
+    <t>boudica</t>
+  </si>
+  <si>
+    <t>quetzalcoatl</t>
+  </si>
+  <si>
+    <t>hephaistion</t>
+  </si>
+  <si>
+    <t>mandricardo</t>
+  </si>
+  <si>
+    <t>ivan-the-terrible</t>
+  </si>
+  <si>
+    <t>edward-teach</t>
+  </si>
+  <si>
+    <t>saint-georgios</t>
+  </si>
+  <si>
+    <t>francis-drake</t>
+  </si>
+  <si>
+    <t>queen-medb</t>
+  </si>
+  <si>
+    <t>bartholomew-roberts</t>
+  </si>
+  <si>
+    <t>sakamoto-ryouma</t>
+  </si>
+  <si>
+    <t>saint-martha</t>
+  </si>
+  <si>
+    <t>captain-nemo</t>
+  </si>
+  <si>
+    <t>taisui-xingjun</t>
+  </si>
+  <si>
+    <t>constantine-xi</t>
   </si>
 </sst>
 </file>
@@ -4844,6 +4907,9 @@
       <c r="B73" t="s">
         <v>625</v>
       </c>
+      <c r="C73" t="s">
+        <v>717</v>
+      </c>
       <c r="D73" t="s">
         <v>278</v>
       </c>
@@ -4873,6 +4939,9 @@
       <c r="B74" t="s">
         <v>626</v>
       </c>
+      <c r="C74" t="s">
+        <v>718</v>
+      </c>
       <c r="D74" t="s">
         <v>278</v>
       </c>
@@ -4899,6 +4968,9 @@
       <c r="B75" t="s">
         <v>627</v>
       </c>
+      <c r="C75" t="s">
+        <v>727</v>
+      </c>
       <c r="D75" t="s">
         <v>278</v>
       </c>
@@ -4925,6 +4997,9 @@
       <c r="B76" t="s">
         <v>628</v>
       </c>
+      <c r="C76" t="s">
+        <v>730</v>
+      </c>
       <c r="D76" t="s">
         <v>278</v>
       </c>
@@ -4951,6 +5026,9 @@
       <c r="B77" t="s">
         <v>629</v>
       </c>
+      <c r="C77" t="s">
+        <v>719</v>
+      </c>
       <c r="D77" t="s">
         <v>278</v>
       </c>
@@ -4977,6 +5055,9 @@
       <c r="B78" t="s">
         <v>630</v>
       </c>
+      <c r="C78" t="s">
+        <v>720</v>
+      </c>
       <c r="D78" t="s">
         <v>278</v>
       </c>
@@ -5006,6 +5087,9 @@
       <c r="B79" t="s">
         <v>631</v>
       </c>
+      <c r="C79" t="s">
+        <v>721</v>
+      </c>
       <c r="D79" t="s">
         <v>79</v>
       </c>
@@ -5035,6 +5119,9 @@
       <c r="B80" t="s">
         <v>632</v>
       </c>
+      <c r="C80" t="s">
+        <v>722</v>
+      </c>
       <c r="D80" t="s">
         <v>278</v>
       </c>
@@ -5064,6 +5151,9 @@
       <c r="B81" t="s">
         <v>633</v>
       </c>
+      <c r="C81" t="s">
+        <v>731</v>
+      </c>
       <c r="D81" t="s">
         <v>278</v>
       </c>
@@ -5093,6 +5183,9 @@
       <c r="B82" t="s">
         <v>634</v>
       </c>
+      <c r="C82" t="s">
+        <v>732</v>
+      </c>
       <c r="D82" t="s">
         <v>278</v>
       </c>
@@ -5119,6 +5212,9 @@
       <c r="B83" t="s">
         <v>635</v>
       </c>
+      <c r="C83" t="s">
+        <v>723</v>
+      </c>
       <c r="D83" t="s">
         <v>278</v>
       </c>
@@ -5145,6 +5241,9 @@
       <c r="B84" t="s">
         <v>636</v>
       </c>
+      <c r="C84" t="s">
+        <v>724</v>
+      </c>
       <c r="D84" t="s">
         <v>278</v>
       </c>
@@ -5174,6 +5273,9 @@
       <c r="B85" t="s">
         <v>637</v>
       </c>
+      <c r="C85" t="s">
+        <v>725</v>
+      </c>
       <c r="D85" t="s">
         <v>646</v>
       </c>
@@ -5203,6 +5305,9 @@
       <c r="B86" t="s">
         <v>638</v>
       </c>
+      <c r="C86" t="s">
+        <v>733</v>
+      </c>
       <c r="D86" t="s">
         <v>278</v>
       </c>
@@ -5229,6 +5334,9 @@
       <c r="B87" t="s">
         <v>639</v>
       </c>
+      <c r="C87" t="s">
+        <v>728</v>
+      </c>
       <c r="D87" t="s">
         <v>278</v>
       </c>
@@ -5255,6 +5363,9 @@
       <c r="B88" t="s">
         <v>640</v>
       </c>
+      <c r="C88" t="s">
+        <v>726</v>
+      </c>
       <c r="D88" t="s">
         <v>278</v>
       </c>
@@ -5284,6 +5395,9 @@
       <c r="B89" t="s">
         <v>641</v>
       </c>
+      <c r="C89" t="s">
+        <v>734</v>
+      </c>
       <c r="D89" t="s">
         <v>278</v>
       </c>
@@ -5313,6 +5427,9 @@
       <c r="B90" t="s">
         <v>642</v>
       </c>
+      <c r="C90" t="s">
+        <v>729</v>
+      </c>
       <c r="D90" t="s">
         <v>278</v>
       </c>
@@ -5342,6 +5459,9 @@
       <c r="B91" t="s">
         <v>643</v>
       </c>
+      <c r="C91" t="s">
+        <v>735</v>
+      </c>
       <c r="D91" t="s">
         <v>278</v>
       </c>
@@ -5371,6 +5491,9 @@
       <c r="B92" t="s">
         <v>644</v>
       </c>
+      <c r="C92" t="s">
+        <v>736</v>
+      </c>
       <c r="D92" t="s">
         <v>79</v>
       </c>
@@ -5399,6 +5522,9 @@
       </c>
       <c r="B93" t="s">
         <v>645</v>
+      </c>
+      <c r="C93" t="s">
+        <v>737</v>
       </c>
       <c r="D93" t="s">
         <v>278</v>

</xml_diff>

<commit_message>
added masters to spreadsheet
</commit_message>
<xml_diff>
--- a/data/Fate-Spreadsheet.xlsx
+++ b/data/Fate-Spreadsheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pixel\Documents\Projects\Fate-Wiki\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFFB8807-7EA1-489A-B2D9-DACB6B2DF62F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1173C242-17D1-4877-8E86-FD83C74B9C4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{B05E798F-9EF6-4508-A0A4-311D06661AED}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="2" xr2:uid="{B05E798F-9EF6-4508-A0A4-311D06661AED}"/>
   </bookViews>
   <sheets>
     <sheet name="Servants" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3373" uniqueCount="1271">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3641" uniqueCount="1472">
   <si>
     <t>servant_id</t>
   </si>
@@ -3856,6 +3856,609 @@
   </si>
   <si>
     <t>form_magic</t>
+  </si>
+  <si>
+    <t>master_id</t>
+  </si>
+  <si>
+    <t>M001</t>
+  </si>
+  <si>
+    <t>M002</t>
+  </si>
+  <si>
+    <t>M003</t>
+  </si>
+  <si>
+    <t>M004</t>
+  </si>
+  <si>
+    <t>M005</t>
+  </si>
+  <si>
+    <t>M006</t>
+  </si>
+  <si>
+    <t>M007</t>
+  </si>
+  <si>
+    <t>M008</t>
+  </si>
+  <si>
+    <t>M009</t>
+  </si>
+  <si>
+    <t>M010</t>
+  </si>
+  <si>
+    <t>M011</t>
+  </si>
+  <si>
+    <t>M012</t>
+  </si>
+  <si>
+    <t>M013</t>
+  </si>
+  <si>
+    <t>M014</t>
+  </si>
+  <si>
+    <t>M015</t>
+  </si>
+  <si>
+    <t>M016</t>
+  </si>
+  <si>
+    <t>M017</t>
+  </si>
+  <si>
+    <t>M018</t>
+  </si>
+  <si>
+    <t>M019</t>
+  </si>
+  <si>
+    <t>M020</t>
+  </si>
+  <si>
+    <t>M021</t>
+  </si>
+  <si>
+    <t>M022</t>
+  </si>
+  <si>
+    <t>M023</t>
+  </si>
+  <si>
+    <t>M024</t>
+  </si>
+  <si>
+    <t>M025</t>
+  </si>
+  <si>
+    <t>M026</t>
+  </si>
+  <si>
+    <t>M027</t>
+  </si>
+  <si>
+    <t>M028</t>
+  </si>
+  <si>
+    <t>M029</t>
+  </si>
+  <si>
+    <t>M030</t>
+  </si>
+  <si>
+    <t>M031</t>
+  </si>
+  <si>
+    <t>M032</t>
+  </si>
+  <si>
+    <t>M033</t>
+  </si>
+  <si>
+    <t>M034</t>
+  </si>
+  <si>
+    <t>M035</t>
+  </si>
+  <si>
+    <t>M036</t>
+  </si>
+  <si>
+    <t>M037</t>
+  </si>
+  <si>
+    <t>M038</t>
+  </si>
+  <si>
+    <t>M039</t>
+  </si>
+  <si>
+    <t>M040</t>
+  </si>
+  <si>
+    <t>M041</t>
+  </si>
+  <si>
+    <t>M042</t>
+  </si>
+  <si>
+    <t>M043</t>
+  </si>
+  <si>
+    <t>M044</t>
+  </si>
+  <si>
+    <t>M045</t>
+  </si>
+  <si>
+    <t>M046</t>
+  </si>
+  <si>
+    <t>M047</t>
+  </si>
+  <si>
+    <t>M048</t>
+  </si>
+  <si>
+    <t>M049</t>
+  </si>
+  <si>
+    <t>M050</t>
+  </si>
+  <si>
+    <t>M051</t>
+  </si>
+  <si>
+    <t>M052</t>
+  </si>
+  <si>
+    <t>M053</t>
+  </si>
+  <si>
+    <t>M054</t>
+  </si>
+  <si>
+    <t>M055</t>
+  </si>
+  <si>
+    <t>M056</t>
+  </si>
+  <si>
+    <t>M057</t>
+  </si>
+  <si>
+    <t>M058</t>
+  </si>
+  <si>
+    <t>M059</t>
+  </si>
+  <si>
+    <t>M060</t>
+  </si>
+  <si>
+    <t>M061</t>
+  </si>
+  <si>
+    <t>M062</t>
+  </si>
+  <si>
+    <t>M063</t>
+  </si>
+  <si>
+    <t>M064</t>
+  </si>
+  <si>
+    <t>M065</t>
+  </si>
+  <si>
+    <t>M066</t>
+  </si>
+  <si>
+    <t>master_name</t>
+  </si>
+  <si>
+    <t>mechanic</t>
+  </si>
+  <si>
+    <t>Tohsaka Rin</t>
+  </si>
+  <si>
+    <t>Combat</t>
+  </si>
+  <si>
+    <t>Utility</t>
+  </si>
+  <si>
+    <t>Mana Gain</t>
+  </si>
+  <si>
+    <t>End Game</t>
+  </si>
+  <si>
+    <t>VP Gain</t>
+  </si>
+  <si>
+    <t>Matou Shinji</t>
+  </si>
+  <si>
+    <t>Matou Sakura</t>
+  </si>
+  <si>
+    <t>Illyasviel Von Einzbern</t>
+  </si>
+  <si>
+    <t>Kuzuki Soichirou</t>
+  </si>
+  <si>
+    <t>Kotomine Kirei</t>
+  </si>
+  <si>
+    <t>Matou Zouken</t>
+  </si>
+  <si>
+    <t>Fujimura Taiga</t>
+  </si>
+  <si>
+    <t>Bazett Fraga McRemitz</t>
+  </si>
+  <si>
+    <t>Caren Hortensia</t>
+  </si>
+  <si>
+    <t>Emiya Kiritsugu</t>
+  </si>
+  <si>
+    <t>Irisviel von Einzbern</t>
+  </si>
+  <si>
+    <t>Tohsaka Tokiomi</t>
+  </si>
+  <si>
+    <t>Matou Kariya</t>
+  </si>
+  <si>
+    <t>Waver Velvet</t>
+  </si>
+  <si>
+    <t>Kayneth Archibald</t>
+  </si>
+  <si>
+    <t>Uryuu Ryuunosuke</t>
+  </si>
+  <si>
+    <t>Kishinami Hakuno (Male)</t>
+  </si>
+  <si>
+    <t>Kishinami Hakuno (Female)</t>
+  </si>
+  <si>
+    <t>Rani VIII</t>
+  </si>
+  <si>
+    <t>Jinako Carigiri</t>
+  </si>
+  <si>
+    <t>Dan Blackmore</t>
+  </si>
+  <si>
+    <t>Alice</t>
+  </si>
+  <si>
+    <t>Julius Belisk Harwey</t>
+  </si>
+  <si>
+    <t>Leonardo Bistario Harwey</t>
+  </si>
+  <si>
+    <t>Sesshouin Kiara</t>
+  </si>
+  <si>
+    <t>Twice H. Pieceman</t>
+  </si>
+  <si>
+    <t>Darnic Prestone</t>
+  </si>
+  <si>
+    <t>Fiore Forvedge</t>
+  </si>
+  <si>
+    <t>Caules Forvedge</t>
+  </si>
+  <si>
+    <t>Roche Frain</t>
+  </si>
+  <si>
+    <t>Celenike Icecolle</t>
+  </si>
+  <si>
+    <t>Sieg</t>
+  </si>
+  <si>
+    <t>Kotomine Shirou</t>
+  </si>
+  <si>
+    <t>Shishigou Kairi</t>
+  </si>
+  <si>
+    <t>Fujimaru Ritsuka (Female)</t>
+  </si>
+  <si>
+    <t>Servant Enhancement</t>
+  </si>
+  <si>
+    <t>Fujimaru Ritsuka (Male)</t>
+  </si>
+  <si>
+    <t>Goredolf Musik</t>
+  </si>
+  <si>
+    <t>Sion Sokaris</t>
+  </si>
+  <si>
+    <t>Fou</t>
+  </si>
+  <si>
+    <t>Kadoc Zemplupus</t>
+  </si>
+  <si>
+    <t>Ophelia Phamrsolone</t>
+  </si>
+  <si>
+    <t>Akuta Hinako</t>
+  </si>
+  <si>
+    <t>Scandinavia Peperoncino</t>
+  </si>
+  <si>
+    <t>Kirschtaria Wodime</t>
+  </si>
+  <si>
+    <t>Demon God Goetia</t>
+  </si>
+  <si>
+    <t>Tiamat</t>
+  </si>
+  <si>
+    <t>Reines Archisorte</t>
+  </si>
+  <si>
+    <t>Magical Ruby</t>
+  </si>
+  <si>
+    <t>Magical Sapphire</t>
+  </si>
+  <si>
+    <t>Nanaya Shiki</t>
+  </si>
+  <si>
+    <t>Tohno Akiha</t>
+  </si>
+  <si>
+    <t>Ciel</t>
+  </si>
+  <si>
+    <t>Magical Amber</t>
+  </si>
+  <si>
+    <t>Brainwash Detective Hisui</t>
+  </si>
+  <si>
+    <t>Nrvnqsr Chaos</t>
+  </si>
+  <si>
+    <t>The Serpent of Akasha</t>
+  </si>
+  <si>
+    <t>Tohno SHIKI</t>
+  </si>
+  <si>
+    <t>The Night of Wallachia</t>
+  </si>
+  <si>
+    <t>Ryougi Shiki</t>
+  </si>
+  <si>
+    <t>Asagami Fujino</t>
+  </si>
+  <si>
+    <t>Araya Souren</t>
+  </si>
+  <si>
+    <t>master_slug</t>
+  </si>
+  <si>
+    <t>emiya-shirou</t>
+  </si>
+  <si>
+    <t>tohsaka-rin</t>
+  </si>
+  <si>
+    <t>matou-shinji</t>
+  </si>
+  <si>
+    <t>matou-sakura</t>
+  </si>
+  <si>
+    <t>kuzuki-soichirou</t>
+  </si>
+  <si>
+    <t>kotomine-kirei</t>
+  </si>
+  <si>
+    <t>matou-zouken</t>
+  </si>
+  <si>
+    <t>fujimura-taiga</t>
+  </si>
+  <si>
+    <t>caren-hortensia</t>
+  </si>
+  <si>
+    <t>emiya-kiritsugu</t>
+  </si>
+  <si>
+    <t>tohsaka-tokiomi</t>
+  </si>
+  <si>
+    <t>matou-kariya</t>
+  </si>
+  <si>
+    <t>waver-velvet</t>
+  </si>
+  <si>
+    <t>kayneth-archibald</t>
+  </si>
+  <si>
+    <t>uryuu-ryuunosuke</t>
+  </si>
+  <si>
+    <t>rani-viii</t>
+  </si>
+  <si>
+    <t>jinako-carigiri</t>
+  </si>
+  <si>
+    <t>dan-blackmore</t>
+  </si>
+  <si>
+    <t>sesshouin-kiara</t>
+  </si>
+  <si>
+    <t>darnic-prestone</t>
+  </si>
+  <si>
+    <t>fiore-forvedge</t>
+  </si>
+  <si>
+    <t>caules-forvedge</t>
+  </si>
+  <si>
+    <t>roche-frain</t>
+  </si>
+  <si>
+    <t>celenike-icecolle</t>
+  </si>
+  <si>
+    <t>kotomine-shirou</t>
+  </si>
+  <si>
+    <t>shishigou-kairi</t>
+  </si>
+  <si>
+    <t>goredolf-musik</t>
+  </si>
+  <si>
+    <t>sion-sokaris</t>
+  </si>
+  <si>
+    <t>kadoc-zemplupus</t>
+  </si>
+  <si>
+    <t>ophelia-phamrsolone</t>
+  </si>
+  <si>
+    <t>akuta-hinako</t>
+  </si>
+  <si>
+    <t>scandinavia-peperoncino</t>
+  </si>
+  <si>
+    <t>kirschtaria-wodime</t>
+  </si>
+  <si>
+    <t>reines-archisorte</t>
+  </si>
+  <si>
+    <t>magical-ruby</t>
+  </si>
+  <si>
+    <t>magical-sapphire</t>
+  </si>
+  <si>
+    <t>nanaya-shiki</t>
+  </si>
+  <si>
+    <t>tohno-akiha</t>
+  </si>
+  <si>
+    <t>magical-amber</t>
+  </si>
+  <si>
+    <t>nrvnqsr-chaos</t>
+  </si>
+  <si>
+    <t>tohno-shiki</t>
+  </si>
+  <si>
+    <t>ryougi-shiki</t>
+  </si>
+  <si>
+    <t>asagami-fujino</t>
+  </si>
+  <si>
+    <t>araya-souren</t>
+  </si>
+  <si>
+    <t>bazett-fraga-mcremitz</t>
+  </si>
+  <si>
+    <t>irisviel-von-einzbern</t>
+  </si>
+  <si>
+    <t>julius-belisk-harwey</t>
+  </si>
+  <si>
+    <t>leonardo-bistario-harwey</t>
+  </si>
+  <si>
+    <t>twice-h-pieceman</t>
+  </si>
+  <si>
+    <t>demon-god-goetia</t>
+  </si>
+  <si>
+    <t>brainwash-detective-hisui</t>
+  </si>
+  <si>
+    <t>kishinami-hakuno-male</t>
+  </si>
+  <si>
+    <t>kishinami-hakuno-female</t>
+  </si>
+  <si>
+    <t>fujimaru-ritsuka-female</t>
+  </si>
+  <si>
+    <t>fujimaru-ritsuka-male</t>
+  </si>
+  <si>
+    <t>the-serpent-of-akasha</t>
+  </si>
+  <si>
+    <t>the-night-of-wallachia</t>
+  </si>
+  <si>
+    <t>sieg</t>
+  </si>
+  <si>
+    <t>alice</t>
+  </si>
+  <si>
+    <t>fou</t>
+  </si>
+  <si>
+    <t>tiamat</t>
+  </si>
+  <si>
+    <t>ciel</t>
+  </si>
+  <si>
+    <t>emiya-shirou-cook</t>
   </si>
 </sst>
 </file>
@@ -19913,9 +20516,956 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32F3CD10-C054-4484-ABE2-D426F834FC22}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:E67"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="13.3984375" customWidth="1"/>
+    <col min="2" max="3" width="26" customWidth="1"/>
+    <col min="4" max="4" width="20.46484375" customWidth="1"/>
+    <col min="5" max="5" width="14.6640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A1" s="1" t="s">
+        <v>1271</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1338</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>1408</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>1339</v>
+      </c>
+      <c r="E1" s="1"/>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>1272</v>
+      </c>
+      <c r="B2" t="s">
+        <v>510</v>
+      </c>
+      <c r="C2" t="s">
+        <v>1409</v>
+      </c>
+      <c r="D2" t="s">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>1273</v>
+      </c>
+      <c r="B3" t="s">
+        <v>1340</v>
+      </c>
+      <c r="C3" t="s">
+        <v>1410</v>
+      </c>
+      <c r="D3" t="s">
+        <v>1342</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>1274</v>
+      </c>
+      <c r="B4" t="s">
+        <v>1346</v>
+      </c>
+      <c r="C4" t="s">
+        <v>1411</v>
+      </c>
+      <c r="D4" t="s">
+        <v>1343</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
+        <v>1275</v>
+      </c>
+      <c r="B5" t="s">
+        <v>1347</v>
+      </c>
+      <c r="C5" t="s">
+        <v>1412</v>
+      </c>
+      <c r="D5" t="s">
+        <v>1344</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
+        <v>1276</v>
+      </c>
+      <c r="B6" t="s">
+        <v>1348</v>
+      </c>
+      <c r="C6" t="s">
+        <v>286</v>
+      </c>
+      <c r="D6" t="s">
+        <v>1343</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A7" t="s">
+        <v>1277</v>
+      </c>
+      <c r="B7" t="s">
+        <v>1349</v>
+      </c>
+      <c r="C7" t="s">
+        <v>1413</v>
+      </c>
+      <c r="D7" t="s">
+        <v>1345</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A8" t="s">
+        <v>1278</v>
+      </c>
+      <c r="B8" t="s">
+        <v>1350</v>
+      </c>
+      <c r="C8" t="s">
+        <v>1414</v>
+      </c>
+      <c r="D8" t="s">
+        <v>1345</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A9" t="s">
+        <v>1279</v>
+      </c>
+      <c r="B9" t="s">
+        <v>1351</v>
+      </c>
+      <c r="C9" t="s">
+        <v>1415</v>
+      </c>
+      <c r="D9" t="s">
+        <v>1343</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A10" t="s">
+        <v>1280</v>
+      </c>
+      <c r="B10" t="s">
+        <v>1352</v>
+      </c>
+      <c r="C10" t="s">
+        <v>1416</v>
+      </c>
+      <c r="D10" t="s">
+        <v>1345</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A11" t="s">
+        <v>1281</v>
+      </c>
+      <c r="B11" t="s">
+        <v>1353</v>
+      </c>
+      <c r="C11" t="s">
+        <v>1453</v>
+      </c>
+      <c r="D11" t="s">
+        <v>1345</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A12" t="s">
+        <v>1282</v>
+      </c>
+      <c r="B12" t="s">
+        <v>1354</v>
+      </c>
+      <c r="C12" t="s">
+        <v>1417</v>
+      </c>
+      <c r="D12" t="s">
+        <v>1345</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A13" t="s">
+        <v>1283</v>
+      </c>
+      <c r="B13" t="s">
+        <v>5</v>
+      </c>
+      <c r="C13" t="s">
+        <v>6</v>
+      </c>
+      <c r="D13" t="s">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A14" t="s">
+        <v>1284</v>
+      </c>
+      <c r="B14" t="s">
+        <v>1355</v>
+      </c>
+      <c r="C14" t="s">
+        <v>1418</v>
+      </c>
+      <c r="D14" t="s">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A15" t="s">
+        <v>1285</v>
+      </c>
+      <c r="B15" t="s">
+        <v>1356</v>
+      </c>
+      <c r="C15" t="s">
+        <v>1454</v>
+      </c>
+      <c r="D15" t="s">
+        <v>1343</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A16" t="s">
+        <v>1286</v>
+      </c>
+      <c r="B16" t="s">
+        <v>1357</v>
+      </c>
+      <c r="C16" t="s">
+        <v>1419</v>
+      </c>
+      <c r="D16" t="s">
+        <v>1345</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A17" t="s">
+        <v>1287</v>
+      </c>
+      <c r="B17" t="s">
+        <v>1358</v>
+      </c>
+      <c r="C17" t="s">
+        <v>1420</v>
+      </c>
+      <c r="D17" t="s">
+        <v>1343</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A18" t="s">
+        <v>1288</v>
+      </c>
+      <c r="B18" t="s">
+        <v>1359</v>
+      </c>
+      <c r="C18" t="s">
+        <v>1421</v>
+      </c>
+      <c r="D18" t="s">
+        <v>1342</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A19" t="s">
+        <v>1289</v>
+      </c>
+      <c r="B19" t="s">
+        <v>1360</v>
+      </c>
+      <c r="C19" t="s">
+        <v>1422</v>
+      </c>
+      <c r="D19" t="s">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A20" t="s">
+        <v>1290</v>
+      </c>
+      <c r="B20" t="s">
+        <v>1361</v>
+      </c>
+      <c r="C20" t="s">
+        <v>1423</v>
+      </c>
+      <c r="D20" t="s">
+        <v>1343</v>
+      </c>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A21" t="s">
+        <v>1291</v>
+      </c>
+      <c r="B21" t="s">
+        <v>1362</v>
+      </c>
+      <c r="C21" t="s">
+        <v>1460</v>
+      </c>
+      <c r="D21" t="s">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A22" t="s">
+        <v>1292</v>
+      </c>
+      <c r="B22" t="s">
+        <v>1363</v>
+      </c>
+      <c r="C22" t="s">
+        <v>1461</v>
+      </c>
+      <c r="D22" t="s">
+        <v>1342</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A23" t="s">
+        <v>1293</v>
+      </c>
+      <c r="B23" t="s">
+        <v>1364</v>
+      </c>
+      <c r="C23" t="s">
+        <v>1424</v>
+      </c>
+      <c r="D23" t="s">
+        <v>1345</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A24" t="s">
+        <v>1294</v>
+      </c>
+      <c r="B24" t="s">
+        <v>1365</v>
+      </c>
+      <c r="C24" t="s">
+        <v>1425</v>
+      </c>
+      <c r="D24" t="s">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A25" t="s">
+        <v>1295</v>
+      </c>
+      <c r="B25" t="s">
+        <v>1366</v>
+      </c>
+      <c r="C25" t="s">
+        <v>1426</v>
+      </c>
+      <c r="D25" t="s">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A26" t="s">
+        <v>1296</v>
+      </c>
+      <c r="B26" t="s">
+        <v>1367</v>
+      </c>
+      <c r="C26" t="s">
+        <v>1467</v>
+      </c>
+      <c r="D26" t="s">
+        <v>1345</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A27" t="s">
+        <v>1297</v>
+      </c>
+      <c r="B27" t="s">
+        <v>1368</v>
+      </c>
+      <c r="C27" t="s">
+        <v>1455</v>
+      </c>
+      <c r="D27" t="s">
+        <v>1342</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A28" t="s">
+        <v>1298</v>
+      </c>
+      <c r="B28" t="s">
+        <v>1369</v>
+      </c>
+      <c r="C28" t="s">
+        <v>1456</v>
+      </c>
+      <c r="D28" t="s">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A29" t="s">
+        <v>1299</v>
+      </c>
+      <c r="B29" t="s">
+        <v>1370</v>
+      </c>
+      <c r="C29" t="s">
+        <v>1427</v>
+      </c>
+      <c r="D29" t="s">
+        <v>1344</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A30" t="s">
+        <v>1300</v>
+      </c>
+      <c r="B30" t="s">
+        <v>1371</v>
+      </c>
+      <c r="C30" t="s">
+        <v>1457</v>
+      </c>
+      <c r="D30" t="s">
+        <v>1342</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A31" t="s">
+        <v>1301</v>
+      </c>
+      <c r="B31" t="s">
+        <v>1372</v>
+      </c>
+      <c r="C31" t="s">
+        <v>1428</v>
+      </c>
+      <c r="D31" t="s">
+        <v>1343</v>
+      </c>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A32" t="s">
+        <v>1302</v>
+      </c>
+      <c r="B32" t="s">
+        <v>1373</v>
+      </c>
+      <c r="C32" t="s">
+        <v>1429</v>
+      </c>
+      <c r="D32" t="s">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="33" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A33" t="s">
+        <v>1303</v>
+      </c>
+      <c r="B33" t="s">
+        <v>1374</v>
+      </c>
+      <c r="C33" t="s">
+        <v>1430</v>
+      </c>
+      <c r="D33" t="s">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="34" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A34" t="s">
+        <v>1304</v>
+      </c>
+      <c r="B34" t="s">
+        <v>1375</v>
+      </c>
+      <c r="C34" t="s">
+        <v>1431</v>
+      </c>
+      <c r="D34" t="s">
+        <v>1345</v>
+      </c>
+    </row>
+    <row r="35" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A35" t="s">
+        <v>1305</v>
+      </c>
+      <c r="B35" t="s">
+        <v>1376</v>
+      </c>
+      <c r="C35" t="s">
+        <v>1432</v>
+      </c>
+      <c r="D35" t="s">
+        <v>1343</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A36" t="s">
+        <v>1306</v>
+      </c>
+      <c r="B36" t="s">
+        <v>1377</v>
+      </c>
+      <c r="C36" t="s">
+        <v>1466</v>
+      </c>
+      <c r="D36" t="s">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A37" t="s">
+        <v>1307</v>
+      </c>
+      <c r="B37" t="s">
+        <v>1378</v>
+      </c>
+      <c r="C37" t="s">
+        <v>1433</v>
+      </c>
+      <c r="D37" t="s">
+        <v>1342</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A38" t="s">
+        <v>1308</v>
+      </c>
+      <c r="B38" t="s">
+        <v>1379</v>
+      </c>
+      <c r="C38" t="s">
+        <v>1434</v>
+      </c>
+      <c r="D38" t="s">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A39" t="s">
+        <v>1309</v>
+      </c>
+      <c r="B39" t="s">
+        <v>1380</v>
+      </c>
+      <c r="C39" t="s">
+        <v>1462</v>
+      </c>
+      <c r="D39" t="s">
+        <v>1381</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A40" t="s">
+        <v>1310</v>
+      </c>
+      <c r="B40" t="s">
+        <v>1382</v>
+      </c>
+      <c r="C40" t="s">
+        <v>1463</v>
+      </c>
+      <c r="D40" t="s">
+        <v>1342</v>
+      </c>
+    </row>
+    <row r="41" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A41" t="s">
+        <v>1311</v>
+      </c>
+      <c r="B41" t="s">
+        <v>1383</v>
+      </c>
+      <c r="C41" t="s">
+        <v>1435</v>
+      </c>
+      <c r="D41" t="s">
+        <v>1345</v>
+      </c>
+    </row>
+    <row r="42" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A42" t="s">
+        <v>1312</v>
+      </c>
+      <c r="B42" t="s">
+        <v>1384</v>
+      </c>
+      <c r="C42" t="s">
+        <v>1436</v>
+      </c>
+      <c r="D42" t="s">
+        <v>1381</v>
+      </c>
+    </row>
+    <row r="43" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A43" t="s">
+        <v>1313</v>
+      </c>
+      <c r="B43" t="s">
+        <v>1385</v>
+      </c>
+      <c r="C43" t="s">
+        <v>1468</v>
+      </c>
+      <c r="D43" t="s">
+        <v>1343</v>
+      </c>
+    </row>
+    <row r="44" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A44" t="s">
+        <v>1314</v>
+      </c>
+      <c r="B44" t="s">
+        <v>1386</v>
+      </c>
+      <c r="C44" t="s">
+        <v>1437</v>
+      </c>
+      <c r="D44" t="s">
+        <v>1342</v>
+      </c>
+    </row>
+    <row r="45" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A45" t="s">
+        <v>1315</v>
+      </c>
+      <c r="B45" t="s">
+        <v>1387</v>
+      </c>
+      <c r="C45" t="s">
+        <v>1438</v>
+      </c>
+      <c r="D45" t="s">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A46" t="s">
+        <v>1316</v>
+      </c>
+      <c r="B46" t="s">
+        <v>1388</v>
+      </c>
+      <c r="C46" t="s">
+        <v>1439</v>
+      </c>
+      <c r="D46" t="s">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A47" t="s">
+        <v>1317</v>
+      </c>
+      <c r="B47" t="s">
+        <v>1389</v>
+      </c>
+      <c r="C47" t="s">
+        <v>1440</v>
+      </c>
+      <c r="D47" t="s">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="48" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A48" t="s">
+        <v>1318</v>
+      </c>
+      <c r="B48" t="s">
+        <v>1390</v>
+      </c>
+      <c r="C48" t="s">
+        <v>1441</v>
+      </c>
+      <c r="D48" t="s">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="49" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A49" t="s">
+        <v>1319</v>
+      </c>
+      <c r="B49" t="s">
+        <v>1391</v>
+      </c>
+      <c r="C49" t="s">
+        <v>1458</v>
+      </c>
+      <c r="D49" t="s">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A50" t="s">
+        <v>1320</v>
+      </c>
+      <c r="B50" t="s">
+        <v>1392</v>
+      </c>
+      <c r="C50" t="s">
+        <v>1469</v>
+      </c>
+      <c r="D50" t="s">
+        <v>1344</v>
+      </c>
+    </row>
+    <row r="51" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A51" t="s">
+        <v>1321</v>
+      </c>
+      <c r="B51" t="s">
+        <v>510</v>
+      </c>
+      <c r="C51" t="s">
+        <v>1471</v>
+      </c>
+      <c r="D51" t="s">
+        <v>1343</v>
+      </c>
+    </row>
+    <row r="52" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A52" t="s">
+        <v>1322</v>
+      </c>
+      <c r="B52" t="s">
+        <v>1393</v>
+      </c>
+      <c r="C52" t="s">
+        <v>1442</v>
+      </c>
+      <c r="D52" t="s">
+        <v>1342</v>
+      </c>
+    </row>
+    <row r="53" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A53" t="s">
+        <v>1323</v>
+      </c>
+      <c r="B53" t="s">
+        <v>1394</v>
+      </c>
+      <c r="C53" t="s">
+        <v>1443</v>
+      </c>
+      <c r="D53" t="s">
+        <v>1342</v>
+      </c>
+    </row>
+    <row r="54" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A54" t="s">
+        <v>1324</v>
+      </c>
+      <c r="B54" t="s">
+        <v>1395</v>
+      </c>
+      <c r="C54" t="s">
+        <v>1444</v>
+      </c>
+      <c r="D54" t="s">
+        <v>1381</v>
+      </c>
+    </row>
+    <row r="55" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A55" t="s">
+        <v>1325</v>
+      </c>
+      <c r="B55" t="s">
+        <v>1396</v>
+      </c>
+      <c r="C55" t="s">
+        <v>1445</v>
+      </c>
+      <c r="D55" t="s">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="56" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A56" t="s">
+        <v>1326</v>
+      </c>
+      <c r="B56" t="s">
+        <v>1397</v>
+      </c>
+      <c r="C56" t="s">
+        <v>1446</v>
+      </c>
+      <c r="D56" t="s">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="57" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A57" t="s">
+        <v>1327</v>
+      </c>
+      <c r="B57" t="s">
+        <v>1021</v>
+      </c>
+      <c r="C57" t="s">
+        <v>1022</v>
+      </c>
+      <c r="D57" t="s">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="58" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A58" t="s">
+        <v>1328</v>
+      </c>
+      <c r="B58" t="s">
+        <v>1398</v>
+      </c>
+      <c r="C58" t="s">
+        <v>1470</v>
+      </c>
+      <c r="D58" t="s">
+        <v>1342</v>
+      </c>
+    </row>
+    <row r="59" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A59" t="s">
+        <v>1329</v>
+      </c>
+      <c r="B59" t="s">
+        <v>1399</v>
+      </c>
+      <c r="C59" t="s">
+        <v>1447</v>
+      </c>
+      <c r="D59" t="s">
+        <v>1342</v>
+      </c>
+    </row>
+    <row r="60" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A60" t="s">
+        <v>1330</v>
+      </c>
+      <c r="B60" t="s">
+        <v>1400</v>
+      </c>
+      <c r="C60" t="s">
+        <v>1459</v>
+      </c>
+      <c r="D60" t="s">
+        <v>1342</v>
+      </c>
+    </row>
+    <row r="61" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A61" t="s">
+        <v>1331</v>
+      </c>
+      <c r="B61" t="s">
+        <v>1401</v>
+      </c>
+      <c r="C61" t="s">
+        <v>1448</v>
+      </c>
+      <c r="D61" t="s">
+        <v>1342</v>
+      </c>
+    </row>
+    <row r="62" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A62" t="s">
+        <v>1332</v>
+      </c>
+      <c r="B62" t="s">
+        <v>1402</v>
+      </c>
+      <c r="C62" t="s">
+        <v>1464</v>
+      </c>
+      <c r="D62" t="s">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="63" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A63" t="s">
+        <v>1333</v>
+      </c>
+      <c r="B63" t="s">
+        <v>1403</v>
+      </c>
+      <c r="C63" t="s">
+        <v>1449</v>
+      </c>
+      <c r="D63" t="s">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="64" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A64" t="s">
+        <v>1334</v>
+      </c>
+      <c r="B64" t="s">
+        <v>1404</v>
+      </c>
+      <c r="C64" t="s">
+        <v>1465</v>
+      </c>
+      <c r="D64" t="s">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="65" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A65" t="s">
+        <v>1335</v>
+      </c>
+      <c r="B65" t="s">
+        <v>1405</v>
+      </c>
+      <c r="C65" t="s">
+        <v>1450</v>
+      </c>
+      <c r="D65" t="s">
+        <v>1341</v>
+      </c>
+    </row>
+    <row r="66" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A66" t="s">
+        <v>1336</v>
+      </c>
+      <c r="B66" t="s">
+        <v>1406</v>
+      </c>
+      <c r="C66" t="s">
+        <v>1451</v>
+      </c>
+      <c r="D66" t="s">
+        <v>1343</v>
+      </c>
+    </row>
+    <row r="67" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A67" t="s">
+        <v>1337</v>
+      </c>
+      <c r="B67" t="s">
+        <v>1407</v>
+      </c>
+      <c r="C67" t="s">
+        <v>1452</v>
+      </c>
+      <c r="D67" t="s">
+        <v>1343</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
fixed the servant assets not being hidden
</commit_message>
<xml_diff>
--- a/data/Fate-Spreadsheet.xlsx
+++ b/data/Fate-Spreadsheet.xlsx
@@ -8,17 +8,18 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pixel\Documents\Projects\Fate-Wiki\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A8AEC5F-F014-4DE0-B160-E5C74668FC87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6975E217-4937-4962-9F68-2043D1A69F68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="3" xr2:uid="{B05E798F-9EF6-4508-A0A4-311D06661AED}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{B05E798F-9EF6-4508-A0A4-311D06661AED}"/>
   </bookViews>
   <sheets>
     <sheet name="Servants" sheetId="1" r:id="rId1"/>
-    <sheet name="Unique Deck Cards" sheetId="4" r:id="rId2"/>
-    <sheet name="Servant Skills" sheetId="3" r:id="rId3"/>
-    <sheet name="Servant Misc Cards" sheetId="7" r:id="rId4"/>
-    <sheet name="Masters" sheetId="5" r:id="rId5"/>
-    <sheet name="Master Cards" sheetId="6" r:id="rId6"/>
+    <sheet name="Servant Traits List" sheetId="8" r:id="rId2"/>
+    <sheet name="Unique Deck Cards" sheetId="4" r:id="rId3"/>
+    <sheet name="Servant Skills" sheetId="3" r:id="rId4"/>
+    <sheet name="Servant Misc Cards" sheetId="7" r:id="rId5"/>
+    <sheet name="Masters" sheetId="5" r:id="rId6"/>
+    <sheet name="Master Cards" sheetId="6" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -44,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3752" uniqueCount="1509">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4216" uniqueCount="1884">
   <si>
     <t>servant_id</t>
   </si>
@@ -4571,6 +4572,1131 @@
   </si>
   <si>
     <t>Albions-Remnant</t>
+  </si>
+  <si>
+    <t>Power Negation,High Power,VP Negation</t>
+  </si>
+  <si>
+    <t>NP Reliant</t>
+  </si>
+  <si>
+    <t>Win Streak VP Gain,Turn Order Manipulation</t>
+  </si>
+  <si>
+    <t>High Risk,Setup Reliant,NP Reliant</t>
+  </si>
+  <si>
+    <t>traits_pros</t>
+  </si>
+  <si>
+    <t>traits_cons</t>
+  </si>
+  <si>
+    <t>servant_pros</t>
+  </si>
+  <si>
+    <t>servant_cons</t>
+  </si>
+  <si>
+    <t>High Power,Combat Plays</t>
+  </si>
+  <si>
+    <t>Mana Hungry,NP Reliant</t>
+  </si>
+  <si>
+    <t>Power Negation</t>
+  </si>
+  <si>
+    <t>High Power</t>
+  </si>
+  <si>
+    <t>VP Negation</t>
+  </si>
+  <si>
+    <t>Win Streak VP Gain</t>
+  </si>
+  <si>
+    <t>Turn Order Manipulation</t>
+  </si>
+  <si>
+    <t>Combat Plays</t>
+  </si>
+  <si>
+    <t>High Risk</t>
+  </si>
+  <si>
+    <t>Setup Reliant</t>
+  </si>
+  <si>
+    <t>Mana Hungry</t>
+  </si>
+  <si>
+    <t>High Power,Objective Manipulation</t>
+  </si>
+  <si>
+    <t>Objective Manipulation</t>
+  </si>
+  <si>
+    <t>High Power,VP Gain</t>
+  </si>
+  <si>
+    <t>High Power,Cheap Power,Ability Negation</t>
+  </si>
+  <si>
+    <t>Cheap Power</t>
+  </si>
+  <si>
+    <t>Ability Negation</t>
+  </si>
+  <si>
+    <t>Deck Destruction</t>
+  </si>
+  <si>
+    <t>Fading Power</t>
+  </si>
+  <si>
+    <t>Deck Destruction,Fading Power</t>
+  </si>
+  <si>
+    <t>Good Scaling,Cheap Power</t>
+  </si>
+  <si>
+    <t>Chance Reliant</t>
+  </si>
+  <si>
+    <t>Good Scaling</t>
+  </si>
+  <si>
+    <t>Good Scaling,Cheap Power,High Power</t>
+  </si>
+  <si>
+    <t>VP Loss</t>
+  </si>
+  <si>
+    <t>NP Reliant,VP Loss,Card Reliant</t>
+  </si>
+  <si>
+    <t>Card Reliant</t>
+  </si>
+  <si>
+    <t>Prediction Reliant</t>
+  </si>
+  <si>
+    <t>Cheap Power,Card Negation</t>
+  </si>
+  <si>
+    <t>Card Reliant,Prediction Reliant</t>
+  </si>
+  <si>
+    <t>Card Negation</t>
+  </si>
+  <si>
+    <t>Combat Plays,Cheap Power</t>
+  </si>
+  <si>
+    <t>Card Reliant,Setup Reliant,Limited Use</t>
+  </si>
+  <si>
+    <t>Limited Use</t>
+  </si>
+  <si>
+    <t>Growing Power</t>
+  </si>
+  <si>
+    <t>Low Power</t>
+  </si>
+  <si>
+    <t>Needs Combat Wins</t>
+  </si>
+  <si>
+    <t>Growing Power,Cheap Power</t>
+  </si>
+  <si>
+    <t>Low Power,Needs Combat Wins</t>
+  </si>
+  <si>
+    <t>Control,High Power</t>
+  </si>
+  <si>
+    <t>Setup Reliant,Mana Hungry</t>
+  </si>
+  <si>
+    <t>Control</t>
+  </si>
+  <si>
+    <t>Objective Recycling</t>
+  </si>
+  <si>
+    <t>Good Scaling,High Power,Objective Recycling</t>
+  </si>
+  <si>
+    <t>Mana Hungry,Card Reliant</t>
+  </si>
+  <si>
+    <t>High Power,Foreigner Transform,Special Hate</t>
+  </si>
+  <si>
+    <t>Foreigner Transform</t>
+  </si>
+  <si>
+    <t>Special Hate</t>
+  </si>
+  <si>
+    <t>High Risk,Mana Hungry,Setup Reliant</t>
+  </si>
+  <si>
+    <t>Adaptable</t>
+  </si>
+  <si>
+    <t>Power Negation,High Power,Adaptable</t>
+  </si>
+  <si>
+    <t>Cheap Power,Good Scaling,Free Card Plays</t>
+  </si>
+  <si>
+    <t>Free Card Plays</t>
+  </si>
+  <si>
+    <t>Setup Reliant,Card Reliant,Chance Reliant</t>
+  </si>
+  <si>
+    <t>High Power,Cheap Power,Power Negation</t>
+  </si>
+  <si>
+    <t>Immobile</t>
+  </si>
+  <si>
+    <t>Chance Reliant,Immobile,Card Reliant</t>
+  </si>
+  <si>
+    <t>Power Negation,Good Scaling</t>
+  </si>
+  <si>
+    <t>Low Power,NP Reliant,Buff Reliant</t>
+  </si>
+  <si>
+    <t>Buff Reliant</t>
+  </si>
+  <si>
+    <t>Buff Reliant,Mana Hungry,Card Reliant</t>
+  </si>
+  <si>
+    <t>Gank Protection,VP Negation,Good Scaling</t>
+  </si>
+  <si>
+    <t>Gank Protection</t>
+  </si>
+  <si>
+    <t>Reactive</t>
+  </si>
+  <si>
+    <t>Positioning Reliant</t>
+  </si>
+  <si>
+    <t>No Luck</t>
+  </si>
+  <si>
+    <t>Reactive,Positioning Reliant,No Luck</t>
+  </si>
+  <si>
+    <t>Luck Reliant,Setup Reliant</t>
+  </si>
+  <si>
+    <t>Luck Reliant</t>
+  </si>
+  <si>
+    <t>Card Reliant,Setup Reliant</t>
+  </si>
+  <si>
+    <t>Target Defeat,VP Theft</t>
+  </si>
+  <si>
+    <t>Target Defeat</t>
+  </si>
+  <si>
+    <t>VP Theft</t>
+  </si>
+  <si>
+    <t>NP Reliant,Low Power,No Luck</t>
+  </si>
+  <si>
+    <t>Power Negation,Skill Removal,Combat Plays</t>
+  </si>
+  <si>
+    <t>Low Power,No Luck</t>
+  </si>
+  <si>
+    <t>Skill Removal</t>
+  </si>
+  <si>
+    <t>Player Removal</t>
+  </si>
+  <si>
+    <t>Power Negation,High Power,Player Removal</t>
+  </si>
+  <si>
+    <t>Mana Hungry,VP Loss</t>
+  </si>
+  <si>
+    <t>Cheap Power,Gank Protection,Good Scaling</t>
+  </si>
+  <si>
+    <t>Growing Power,VP Gain</t>
+  </si>
+  <si>
+    <t>Immobile,NP Reliant,Mana Hungry</t>
+  </si>
+  <si>
+    <t>Adaptable,Group Defeat,High Power</t>
+  </si>
+  <si>
+    <t>Group Defeat</t>
+  </si>
+  <si>
+    <t>High Mobility</t>
+  </si>
+  <si>
+    <t>Difficult Mechanics</t>
+  </si>
+  <si>
+    <t>High Mobility,Cheap Power,High Power</t>
+  </si>
+  <si>
+    <t>High Risk,Card Reliant,Difficult Mechanics</t>
+  </si>
+  <si>
+    <t>Objective Inversion</t>
+  </si>
+  <si>
+    <t>Buff Reliant,Setup Reliant</t>
+  </si>
+  <si>
+    <t>Good Scaling,Adaptable,Control</t>
+  </si>
+  <si>
+    <t>Setup Reliant,Card Reliant,Difficult Mechanics</t>
+  </si>
+  <si>
+    <t>Power Negation,Skill Theft,Control</t>
+  </si>
+  <si>
+    <t>Skill Theft</t>
+  </si>
+  <si>
+    <t>Setup Reliant,Chance Reliant</t>
+  </si>
+  <si>
+    <t>Adaptable,VP Gain,Cheap Power</t>
+  </si>
+  <si>
+    <t>Positioning Reliant,Setup Reliant,NP Reliant</t>
+  </si>
+  <si>
+    <t>Adaptable,High Mobility,Cheap Power</t>
+  </si>
+  <si>
+    <t>Control,Combat Plays,Gank Protection</t>
+  </si>
+  <si>
+    <t>Immobile,Low Power</t>
+  </si>
+  <si>
+    <t>Gank Protection,VP Gain,High Power</t>
+  </si>
+  <si>
+    <t>Good Scaling,Cheap Power,High Mobility</t>
+  </si>
+  <si>
+    <t>Buff Reliant,Positioning Reliant,Setup Reliant</t>
+  </si>
+  <si>
+    <t>Control,Skill Theft,Growing Power</t>
+  </si>
+  <si>
+    <t>Low Power,Setup Reliant</t>
+  </si>
+  <si>
+    <t>VP Gain,Growing Power</t>
+  </si>
+  <si>
+    <t>Low Power,NP Reliant</t>
+  </si>
+  <si>
+    <t>Alternate Win Con</t>
+  </si>
+  <si>
+    <t>High Power,Alternate Win Con,Cheap Power</t>
+  </si>
+  <si>
+    <t>NP Reliant,Mana Hungry,VP Loss</t>
+  </si>
+  <si>
+    <t>Ability Negation,Buff Negation,Combat Plays</t>
+  </si>
+  <si>
+    <t>Buff Negation</t>
+  </si>
+  <si>
+    <t>NP Reliant,Low Power</t>
+  </si>
+  <si>
+    <t>Low Power,Card Reliant,Setup Reliant</t>
+  </si>
+  <si>
+    <t>Cheap Power,VP Gain,Good Scaling</t>
+  </si>
+  <si>
+    <t>Control Loss,Gives VP</t>
+  </si>
+  <si>
+    <t>Control Loss</t>
+  </si>
+  <si>
+    <t>Gives VP</t>
+  </si>
+  <si>
+    <t>Transform,Cheap Power,Good Scaling</t>
+  </si>
+  <si>
+    <t>VP Loss,NP Reliant</t>
+  </si>
+  <si>
+    <t>Transform</t>
+  </si>
+  <si>
+    <t>Good Scaling,Target Defeat,Card Draw</t>
+  </si>
+  <si>
+    <t>Card Draw</t>
+  </si>
+  <si>
+    <t>Good Scaling,Agility Negation,VP Gain</t>
+  </si>
+  <si>
+    <t>Setup Reliant,Positioning Reliant,No Luck</t>
+  </si>
+  <si>
+    <t>Agility Negation</t>
+  </si>
+  <si>
+    <t>Growing Power,Power Reduction,Group Defeat</t>
+  </si>
+  <si>
+    <t>Power Reduction</t>
+  </si>
+  <si>
+    <t>Low Power,High Risk,No Luck</t>
+  </si>
+  <si>
+    <t>VP Gain,Good Scaling,Adaptable</t>
+  </si>
+  <si>
+    <t>NP Reliant,Positioning Reliant,No Luck</t>
+  </si>
+  <si>
+    <t>Combat Plays,VP Gain</t>
+  </si>
+  <si>
+    <t>VP Gain,Group Defeat</t>
+  </si>
+  <si>
+    <t>Low Power,Setup Reliant,No Luck</t>
+  </si>
+  <si>
+    <t>Cheap Power,High Power,Control</t>
+  </si>
+  <si>
+    <t>Combat Plays,VP Gain,High Mobility</t>
+  </si>
+  <si>
+    <t>High Power,Gank Protection,Enemy Displacement</t>
+  </si>
+  <si>
+    <t>Enemy Displacement</t>
+  </si>
+  <si>
+    <t>Positioning Reliant,Setup Reliant</t>
+  </si>
+  <si>
+    <t>High Power,Cheap Power,VP Gain</t>
+  </si>
+  <si>
+    <t>High Risk,Dies</t>
+  </si>
+  <si>
+    <t>Dies</t>
+  </si>
+  <si>
+    <t>High Power,Mana Gain</t>
+  </si>
+  <si>
+    <t>Donates Mana</t>
+  </si>
+  <si>
+    <t>Donates Mana,Setup Reliant,Difficult Mechanics</t>
+  </si>
+  <si>
+    <t>Good Scaling,Combat Plays</t>
+  </si>
+  <si>
+    <t>VP Gain,Combat Negation</t>
+  </si>
+  <si>
+    <t>Combat Negation</t>
+  </si>
+  <si>
+    <t>Card Reliant,Limited Use</t>
+  </si>
+  <si>
+    <t>Cheap Power,Good Scaling</t>
+  </si>
+  <si>
+    <t>VP Gain,Power Negation</t>
+  </si>
+  <si>
+    <t>Event Manipulation,Cheap Power,Good Scaling</t>
+  </si>
+  <si>
+    <t>Setup Reliant,Positioning Reliant,Card Reliant</t>
+  </si>
+  <si>
+    <t>Event Manipulation</t>
+  </si>
+  <si>
+    <t>Cheap Power,VP Gain,Target Defeat</t>
+  </si>
+  <si>
+    <t>Setup Reliant,Card Reliant,No Luck</t>
+  </si>
+  <si>
+    <t>Target Defeat,VP Gain</t>
+  </si>
+  <si>
+    <t>Setup Reliant,Low Power,No Luck</t>
+  </si>
+  <si>
+    <t>VP Gain,Control</t>
+  </si>
+  <si>
+    <t>Positioning Reliant,Mana Hungry</t>
+  </si>
+  <si>
+    <t>High Power,Cheap Power</t>
+  </si>
+  <si>
+    <t>Card Reliant,Chance Reliant,Mana Hungry</t>
+  </si>
+  <si>
+    <t>Cheap Power,Skill Theft,VP Theft</t>
+  </si>
+  <si>
+    <t>NP Reliant,Limited Use,No Luck</t>
+  </si>
+  <si>
+    <t>VP Gain,Cheap Power,Good Scaling</t>
+  </si>
+  <si>
+    <t>NP Reliant,Setup Reliant,Card Reliant</t>
+  </si>
+  <si>
+    <t>VP Gain,Cheap Power</t>
+  </si>
+  <si>
+    <t>High Risk,Card Reliant</t>
+  </si>
+  <si>
+    <t>High Power,Group Defeat</t>
+  </si>
+  <si>
+    <t>Mana Hungry,No Luck</t>
+  </si>
+  <si>
+    <t>High Power,Good Scaling,Objective Manipulation</t>
+  </si>
+  <si>
+    <t>Mana Hungry,Buff Reliant,NP Reliant</t>
+  </si>
+  <si>
+    <t>Power Negation,Control,Gank Protection</t>
+  </si>
+  <si>
+    <t>High Risk,Low Power,NP Reliant</t>
+  </si>
+  <si>
+    <t>VP Denial</t>
+  </si>
+  <si>
+    <t>VP Denial,VP Gain,Enemy Displacement</t>
+  </si>
+  <si>
+    <t>Immobile,Card Reliant</t>
+  </si>
+  <si>
+    <t>High Mobility,High Power,VP Gain</t>
+  </si>
+  <si>
+    <t>Good Scaling,Enemy Displacement,High Mobility</t>
+  </si>
+  <si>
+    <t>Buff Reliant,Card Reliant,No Luck</t>
+  </si>
+  <si>
+    <t>Control,Gank Protection</t>
+  </si>
+  <si>
+    <t>Setup Reliant,NP Reliant</t>
+  </si>
+  <si>
+    <t>Cheap Power,VP Gain,Control</t>
+  </si>
+  <si>
+    <t>Card Reliant,Buff Reliant,Setup Reliant</t>
+  </si>
+  <si>
+    <t>Enemy Displacement,VP Theft,High Mobility</t>
+  </si>
+  <si>
+    <t>Setup Reliant,Mana Hungry,Low Power</t>
+  </si>
+  <si>
+    <t>Weak Duelist,NP Reliant</t>
+  </si>
+  <si>
+    <t>Weak Duelist</t>
+  </si>
+  <si>
+    <t>High Mobility,Cheap Power,VP Gain</t>
+  </si>
+  <si>
+    <t>Weak Duelist,Buff Reliant,NP Reliant</t>
+  </si>
+  <si>
+    <t>Cheap Power,High Mobility</t>
+  </si>
+  <si>
+    <t>NP Reliant,High Risk</t>
+  </si>
+  <si>
+    <t>High Power,Good Scaling,High Mobility</t>
+  </si>
+  <si>
+    <t>Setup Reliant,Difficult Mechanics</t>
+  </si>
+  <si>
+    <t>VP Gain,Card Negation,Good Scaling</t>
+  </si>
+  <si>
+    <t>Limited Early Game,NP Reliant,Mana Hungry</t>
+  </si>
+  <si>
+    <t>Limited Early Game</t>
+  </si>
+  <si>
+    <t>No Utility,Buff Reliant</t>
+  </si>
+  <si>
+    <t>No Utility</t>
+  </si>
+  <si>
+    <t>Growing Power,VP Gain,Deck Destruction</t>
+  </si>
+  <si>
+    <t>NP Reliant,Needs Combat Wins</t>
+  </si>
+  <si>
+    <t>Cheap Power,VP Gain,Combat Plays</t>
+  </si>
+  <si>
+    <t>Limited Use,Weak Climax</t>
+  </si>
+  <si>
+    <t>Weak Climax</t>
+  </si>
+  <si>
+    <t>High Power,Enemy Displacement,VP Gain</t>
+  </si>
+  <si>
+    <t>High Power,High Mobility,Cheap Power</t>
+  </si>
+  <si>
+    <t>Mana Hungry,Card Reliant,Setup Reliant</t>
+  </si>
+  <si>
+    <t>High Mobility,Adaptable,Cheap Power</t>
+  </si>
+  <si>
+    <t>Setup Reliant,Low Power,Card Reliant</t>
+  </si>
+  <si>
+    <t>Group Defeat,Cheap Power,VP Theft</t>
+  </si>
+  <si>
+    <t>Poor Matchups</t>
+  </si>
+  <si>
+    <t>Setup Reliant,Weak Climax,Poor Matchups</t>
+  </si>
+  <si>
+    <t>Cheap Power,VP Gain</t>
+  </si>
+  <si>
+    <t>VP Gain,Target Defeat</t>
+  </si>
+  <si>
+    <t>VP Gain,Good Scaling,High Power</t>
+  </si>
+  <si>
+    <t>High Risk,Setup Reliant,No Luck</t>
+  </si>
+  <si>
+    <t>Growing Power,Good Scaling,Magic Penetration</t>
+  </si>
+  <si>
+    <t>Magic Penetration</t>
+  </si>
+  <si>
+    <t>NP Reliant,Mana Hungry,Card Reliant</t>
+  </si>
+  <si>
+    <t>VP Gain,Kingmaking</t>
+  </si>
+  <si>
+    <t>Low Power,Prediction Reliant,Setup Reliant</t>
+  </si>
+  <si>
+    <t>Kingmaking</t>
+  </si>
+  <si>
+    <t>VP Gain,Growing Power,High Power</t>
+  </si>
+  <si>
+    <t>Setup Reliant,High Risk,Mana Hungry,No Luck</t>
+  </si>
+  <si>
+    <t>VP Gain,Unlocks Master Ascension</t>
+  </si>
+  <si>
+    <t>Unlocks Master Ascension</t>
+  </si>
+  <si>
+    <t>NP Theft</t>
+  </si>
+  <si>
+    <t>NP Theft,Adaptable,VP Gain,Growing Power</t>
+  </si>
+  <si>
+    <t>Matchup Reliant,Low Power,Setup Reliant</t>
+  </si>
+  <si>
+    <t>Matchup Reliant</t>
+  </si>
+  <si>
+    <t>VP Gain,VP Loss,Gank Protection</t>
+  </si>
+  <si>
+    <t>Low Power,High Risk,Setup Reliant</t>
+  </si>
+  <si>
+    <t>VP Theft,VP Gain</t>
+  </si>
+  <si>
+    <t>Setup Reliant,No Luck</t>
+  </si>
+  <si>
+    <t>Power Negation,VP Denial,High Mobility</t>
+  </si>
+  <si>
+    <t>Low Power,Recon Reliant</t>
+  </si>
+  <si>
+    <t>Recon Reliant</t>
+  </si>
+  <si>
+    <t>VP Gain,Mana Gain,Power Negation</t>
+  </si>
+  <si>
+    <t>Donates Mana,Setup Reliant,No Luck</t>
+  </si>
+  <si>
+    <t>VP Gain,Type Negation,Special Negation</t>
+  </si>
+  <si>
+    <t>Type Negation</t>
+  </si>
+  <si>
+    <t>Special Negation</t>
+  </si>
+  <si>
+    <t>VP Gain,High Power,Group Defeat</t>
+  </si>
+  <si>
+    <t>Setup Reliant,Donates Mana</t>
+  </si>
+  <si>
+    <t>VP Gain,High Power</t>
+  </si>
+  <si>
+    <t>Growing Power,Adaptable,VP Gain</t>
+  </si>
+  <si>
+    <t>Needs Combat Wins,Card Reliant,Setup Reliant</t>
+  </si>
+  <si>
+    <t>VP Gain,Reliable Defeat</t>
+  </si>
+  <si>
+    <t>Reliable Defeat</t>
+  </si>
+  <si>
+    <t>Buffs Opponents</t>
+  </si>
+  <si>
+    <t>Cheap Power,Adaptable,Target Defeat</t>
+  </si>
+  <si>
+    <t>Card Reliant,Buffs Opponents</t>
+  </si>
+  <si>
+    <t>Free Command Spells,Cheap Power</t>
+  </si>
+  <si>
+    <t>Free Command Spells</t>
+  </si>
+  <si>
+    <t>Group Defeat,VP Gain,Cheap Power</t>
+  </si>
+  <si>
+    <t>Positioning Reliant,Immobile,Mana Hungry</t>
+  </si>
+  <si>
+    <t>High Risk,Weak Duelist,NP Reliant</t>
+  </si>
+  <si>
+    <t>Control,Cheap Power,VP Gain</t>
+  </si>
+  <si>
+    <t>High Risk,Setup Reliant,Limited Use</t>
+  </si>
+  <si>
+    <t>VP Gain,Skill Negation</t>
+  </si>
+  <si>
+    <t>Low Power,Card Reliant</t>
+  </si>
+  <si>
+    <t>Skill Negation</t>
+  </si>
+  <si>
+    <t>Good Scaling,Ability Negation</t>
+  </si>
+  <si>
+    <t>VP Gain,Assassination,Target Defeat</t>
+  </si>
+  <si>
+    <t>Low Power,Limited Use,No Luck</t>
+  </si>
+  <si>
+    <t>Assassination</t>
+  </si>
+  <si>
+    <t>VP Gain,Assassination,High Mobility</t>
+  </si>
+  <si>
+    <t>Low Power,Buff Reliant,No Luck</t>
+  </si>
+  <si>
+    <t>Assassination,Basic Negation,High Mobility</t>
+  </si>
+  <si>
+    <t>Low Power,Weak Duelist</t>
+  </si>
+  <si>
+    <t>Basic Negation</t>
+  </si>
+  <si>
+    <t>Servant Removal,Group Defeat,High Power</t>
+  </si>
+  <si>
+    <t>Servant Removal</t>
+  </si>
+  <si>
+    <t>VP Gain,Assassination,Group Defeat</t>
+  </si>
+  <si>
+    <t>Low Power,Positioning Reliant</t>
+  </si>
+  <si>
+    <t>Combat Negation,Control,Assassination</t>
+  </si>
+  <si>
+    <t>Low Power,NP Reliant,No Luck</t>
+  </si>
+  <si>
+    <t>Target Defeat,Obscure Objectives,High Mobility</t>
+  </si>
+  <si>
+    <t>Obscure Objectives</t>
+  </si>
+  <si>
+    <t>Target Defeat,Combat Plays,High Mobility</t>
+  </si>
+  <si>
+    <t>Target Defeat,Deck Destruction,Control,VP Gain</t>
+  </si>
+  <si>
+    <t>Low Power,Setup Reliant,Immobile</t>
+  </si>
+  <si>
+    <t>Assassination,VP Gain</t>
+  </si>
+  <si>
+    <t>Alternating Abilities</t>
+  </si>
+  <si>
+    <t>Target Defeat,Assassination,VP Gain</t>
+  </si>
+  <si>
+    <t>Prediction Reliant,Positioning Reliant,Card Reliant</t>
+  </si>
+  <si>
+    <t>Target Defeat,Cheap Power,VP Gain</t>
+  </si>
+  <si>
+    <t>Requires Negotiation</t>
+  </si>
+  <si>
+    <t>Card Reliant,Setup Reliant,Chance Reliant</t>
+  </si>
+  <si>
+    <t>VP Gain,Assassination,Good Scaling</t>
+  </si>
+  <si>
+    <t>Assassination,Card Negation,VP Gain</t>
+  </si>
+  <si>
+    <t>Low Power,Card Reliant,Requires Negotiation</t>
+  </si>
+  <si>
+    <t>VP Theft,Assassination,Combat Plays</t>
+  </si>
+  <si>
+    <t>Good Scaling,Target Defeat,Assassination</t>
+  </si>
+  <si>
+    <t>Mana Hungry,Setup Reliant,High Risk</t>
+  </si>
+  <si>
+    <t>Assassination,VP Loss,Cheap Power</t>
+  </si>
+  <si>
+    <t>Setup Reliant,Reactive,No Luck</t>
+  </si>
+  <si>
+    <t>High Power,Cheap Power,Target Defeat</t>
+  </si>
+  <si>
+    <t>Mana Hungry,Limited Use,NP Reliant</t>
+  </si>
+  <si>
+    <t>VP Theft,Target Defeat,High Mobility</t>
+  </si>
+  <si>
+    <t>Positioning Reliant,Low Power,No Luck</t>
+  </si>
+  <si>
+    <t>VP Theft,Mana Theft,Control</t>
+  </si>
+  <si>
+    <t>Mana Theft</t>
+  </si>
+  <si>
+    <t>Low Power,Mana Hungry,Requires Negotiation</t>
+  </si>
+  <si>
+    <t>Cheap Power,Group Defeat,VP Theft</t>
+  </si>
+  <si>
+    <t>Limited Use,Card Reliant</t>
+  </si>
+  <si>
+    <t>Attack Theft,Skill Theft,Gank Protection</t>
+  </si>
+  <si>
+    <t>Attack Theft</t>
+  </si>
+  <si>
+    <t>VP Denial,Target Defeat,Gank Protection</t>
+  </si>
+  <si>
+    <t>VP Gain,Command Seal Hate</t>
+  </si>
+  <si>
+    <t>Command Seal Hate</t>
+  </si>
+  <si>
+    <t>VP Gain,Cheap Power,Gank Protection</t>
+  </si>
+  <si>
+    <t>Poor Matchups,Prediction Reliant</t>
+  </si>
+  <si>
+    <t>Cheap Power,High Power</t>
+  </si>
+  <si>
+    <t>Power Negation,VP Gain</t>
+  </si>
+  <si>
+    <t>Growing Power,High Power</t>
+  </si>
+  <si>
+    <t>Mana Hungry,Setup Reliant</t>
+  </si>
+  <si>
+    <t>Cheap Power,High Power,VP Gain</t>
+  </si>
+  <si>
+    <t>VP Loss,Limited Use</t>
+  </si>
+  <si>
+    <t>High Mobility,High Power</t>
+  </si>
+  <si>
+    <t>Cheap Power,High Power,Objective Manipulation</t>
+  </si>
+  <si>
+    <t>High Risk,Mana Hungry,NP Reliant</t>
+  </si>
+  <si>
+    <t>VP Gain,Cheap Power,Adapatable</t>
+  </si>
+  <si>
+    <t>VP Theft,Good Scaling</t>
+  </si>
+  <si>
+    <t>VP Gain,Cheap Power,VP Loss</t>
+  </si>
+  <si>
+    <t>Buffs Opponents,VP Loss</t>
+  </si>
+  <si>
+    <t>Mana Hungry,Card Reliant,Immobile</t>
+  </si>
+  <si>
+    <t>Enemy Displacement,VP Loss,High Power</t>
+  </si>
+  <si>
+    <t>Mana Hungry,Buffs Opponents,Card Reliant</t>
+  </si>
+  <si>
+    <t>Cheap Power,Control,Combat Plays</t>
+  </si>
+  <si>
+    <t>Setup Reliant,Card Reliant,Matchup Reliant</t>
+  </si>
+  <si>
+    <t>Gank Protection,Mana Loss,High Power</t>
+  </si>
+  <si>
+    <t>Mana Loss</t>
+  </si>
+  <si>
+    <t>Card Reliant,Setup Reliant,No Luck</t>
+  </si>
+  <si>
+    <t>Chance Reliant,Setup Reliant</t>
+  </si>
+  <si>
+    <t>Reactive,Setup Reliant,No Luck</t>
+  </si>
+  <si>
+    <t>Good Scaling,VP Loss,Group Defeat</t>
+  </si>
+  <si>
+    <t>Setup Reliant,High Risk,No Luck</t>
+  </si>
+  <si>
+    <t>Target Defeat,High Mobility,VP Loss</t>
+  </si>
+  <si>
+    <t>Reactive,Card Reliant,No Luck</t>
+  </si>
+  <si>
+    <t>Group Defeat,Control,Gank Protection</t>
+  </si>
+  <si>
+    <t>Enemy Displacement,VP Gain,Group Defeat</t>
+  </si>
+  <si>
+    <t>Enemy Displacement,VP Gain,VP Denial</t>
+  </si>
+  <si>
+    <t>Chance Reliant,Matchup Reliant</t>
+  </si>
+  <si>
+    <t>Prediction Reliant,High Risk</t>
+  </si>
+  <si>
+    <t>Enemy Displacement,High Power</t>
+  </si>
+  <si>
+    <t>Limited Use,NP Reliant,Mana Hungry</t>
+  </si>
+  <si>
+    <t>Alternate Win Con,Cheap Power,Adaptable</t>
+  </si>
+  <si>
+    <t>Poor Matchups,NP Reliant,Card Reliant</t>
+  </si>
+  <si>
+    <t>Low Power,NP Reliant,Mana Hungry</t>
+  </si>
+  <si>
+    <t>Power Reduction,Control</t>
+  </si>
+  <si>
+    <t>Low Power,Setup Reliant,NP Reliant</t>
+  </si>
+  <si>
+    <t>VP Gain,World Manipulation</t>
+  </si>
+  <si>
+    <t>World Manipulation</t>
+  </si>
+  <si>
+    <t>Chance Reliant,Card Reliant,Mana Hungry</t>
+  </si>
+  <si>
+    <t>Objective Manipulation,VP Denial,Mana Gain</t>
+  </si>
+  <si>
+    <t>Low Power,Mana Hungry</t>
+  </si>
+  <si>
+    <t>Setup Reliant,Chance Reliant,Mana Hungry</t>
+  </si>
+  <si>
+    <t>Card Negation,Type Manipulation</t>
+  </si>
+  <si>
+    <t>Type Manipulation</t>
+  </si>
+  <si>
+    <t>Cheap Power,Power Reduction,VP Gain</t>
+  </si>
+  <si>
+    <t>Setup Reliant,NP Reliant,Low Power</t>
+  </si>
+  <si>
+    <t>Setup Reliant,VP Loss,No Luck</t>
+  </si>
+  <si>
+    <t>High Power,Cheap Power,Combat Plays,Alternate Win Con</t>
+  </si>
+  <si>
+    <t>Limited Use,Mana Hungry</t>
+  </si>
+  <si>
+    <t>Kingmaking,VP Gain,Power Reduction</t>
   </si>
 </sst>
 </file>
@@ -4972,8 +6098,8 @@
     <col min="10" max="10" width="97" style="2" customWidth="1"/>
     <col min="11" max="11" width="12.59765625" customWidth="1"/>
     <col min="12" max="12" width="10.9296875" customWidth="1"/>
-    <col min="13" max="13" width="12" customWidth="1"/>
-    <col min="14" max="14" width="11.53125" customWidth="1"/>
+    <col min="13" max="13" width="45.6640625" customWidth="1"/>
+    <col min="14" max="14" width="41.33203125" customWidth="1"/>
     <col min="15" max="15" width="11.796875" customWidth="1"/>
     <col min="16" max="16" width="18.19921875" customWidth="1"/>
   </cols>
@@ -5015,8 +6141,12 @@
       <c r="L1" s="3" t="s">
         <v>1466</v>
       </c>
-      <c r="M1" s="3"/>
-      <c r="N1" s="3"/>
+      <c r="M1" s="3" t="s">
+        <v>1515</v>
+      </c>
+      <c r="N1" s="3" t="s">
+        <v>1516</v>
+      </c>
       <c r="O1" s="3"/>
       <c r="P1" s="3"/>
     </row>
@@ -5048,6 +6178,12 @@
       <c r="J2" s="2" t="s">
         <v>16</v>
       </c>
+      <c r="M2" s="2" t="s">
+        <v>1509</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>1510</v>
+      </c>
     </row>
     <row r="3" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
@@ -5077,6 +6213,12 @@
       <c r="J3" s="2" t="s">
         <v>177</v>
       </c>
+      <c r="M3" s="2" t="s">
+        <v>1511</v>
+      </c>
+      <c r="N3" s="2" t="s">
+        <v>1512</v>
+      </c>
     </row>
     <row r="4" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
@@ -5103,6 +6245,12 @@
       <c r="J4" s="2" t="s">
         <v>179</v>
       </c>
+      <c r="M4" t="s">
+        <v>1517</v>
+      </c>
+      <c r="N4" t="s">
+        <v>1518</v>
+      </c>
     </row>
     <row r="5" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
@@ -5132,6 +6280,12 @@
       <c r="L5" t="b">
         <v>1</v>
       </c>
+      <c r="M5" t="s">
+        <v>1528</v>
+      </c>
+      <c r="N5" t="s">
+        <v>1527</v>
+      </c>
     </row>
     <row r="6" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
@@ -5161,6 +6315,12 @@
       <c r="J6" s="2" t="s">
         <v>183</v>
       </c>
+      <c r="M6" s="2" t="s">
+        <v>1530</v>
+      </c>
+      <c r="N6" s="2" t="s">
+        <v>1525</v>
+      </c>
     </row>
     <row r="7" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
@@ -5190,6 +6350,12 @@
       <c r="J7" s="2" t="s">
         <v>186</v>
       </c>
+      <c r="M7" s="2" t="s">
+        <v>1531</v>
+      </c>
+      <c r="N7" s="2" t="s">
+        <v>1536</v>
+      </c>
     </row>
     <row r="8" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
@@ -5219,6 +6385,12 @@
       <c r="K8" t="b">
         <v>1</v>
       </c>
+      <c r="M8" s="2" t="s">
+        <v>1537</v>
+      </c>
+      <c r="N8" s="2" t="s">
+        <v>1538</v>
+      </c>
     </row>
     <row r="9" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
@@ -5245,6 +6417,12 @@
       <c r="J9" s="2" t="s">
         <v>186</v>
       </c>
+      <c r="M9" s="2" t="s">
+        <v>1540</v>
+      </c>
+      <c r="N9" s="2" t="s">
+        <v>1541</v>
+      </c>
     </row>
     <row r="10" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
@@ -5274,6 +6452,12 @@
       <c r="J10" s="2" t="s">
         <v>188</v>
       </c>
+      <c r="M10" s="2" t="s">
+        <v>1531</v>
+      </c>
+      <c r="N10" s="2" t="s">
+        <v>1542</v>
+      </c>
     </row>
     <row r="11" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
@@ -5303,6 +6487,12 @@
       <c r="J11" s="2" t="s">
         <v>188</v>
       </c>
+      <c r="M11" s="2" t="s">
+        <v>1545</v>
+      </c>
+      <c r="N11" s="2" t="s">
+        <v>1546</v>
+      </c>
     </row>
     <row r="12" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
@@ -5332,6 +6522,12 @@
       <c r="J12" s="2" t="s">
         <v>194</v>
       </c>
+      <c r="M12" s="2" t="s">
+        <v>1548</v>
+      </c>
+      <c r="N12" s="2" t="s">
+        <v>1549</v>
+      </c>
     </row>
     <row r="13" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
@@ -5358,6 +6554,12 @@
       <c r="J13" s="2" t="s">
         <v>188</v>
       </c>
+      <c r="M13" s="2" t="s">
+        <v>1554</v>
+      </c>
+      <c r="N13" s="2" t="s">
+        <v>1555</v>
+      </c>
     </row>
     <row r="14" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
@@ -5387,6 +6589,12 @@
       <c r="J14" s="2" t="s">
         <v>188</v>
       </c>
+      <c r="M14" s="2" t="s">
+        <v>1556</v>
+      </c>
+      <c r="N14" s="2" t="s">
+        <v>1557</v>
+      </c>
     </row>
     <row r="15" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
@@ -5416,6 +6624,12 @@
       <c r="J15" s="2" t="s">
         <v>197</v>
       </c>
+      <c r="M15" s="2" t="s">
+        <v>1560</v>
+      </c>
+      <c r="N15" s="2" t="s">
+        <v>1561</v>
+      </c>
     </row>
     <row r="16" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
@@ -5445,8 +6659,14 @@
       <c r="J16" s="2" t="s">
         <v>200</v>
       </c>
-    </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="M16" s="2" t="s">
+        <v>1562</v>
+      </c>
+      <c r="N16" s="2" t="s">
+        <v>1565</v>
+      </c>
+    </row>
+    <row r="17" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
         <v>125</v>
       </c>
@@ -5474,8 +6694,14 @@
       <c r="J17" s="2" t="s">
         <v>186</v>
       </c>
-    </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="M17" s="2" t="s">
+        <v>1567</v>
+      </c>
+      <c r="N17" s="2" t="s">
+        <v>1510</v>
+      </c>
+    </row>
+    <row r="18" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
         <v>126</v>
       </c>
@@ -5506,8 +6732,14 @@
       <c r="K18" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="M18" s="2" t="s">
+        <v>1568</v>
+      </c>
+      <c r="N18" s="2" t="s">
+        <v>1570</v>
+      </c>
+    </row>
+    <row r="19" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
         <v>127</v>
       </c>
@@ -5535,8 +6767,14 @@
       <c r="J19" s="2" t="s">
         <v>186</v>
       </c>
-    </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="M19" s="2" t="s">
+        <v>1571</v>
+      </c>
+      <c r="N19" s="2" t="s">
+        <v>1573</v>
+      </c>
+    </row>
+    <row r="20" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
         <v>128</v>
       </c>
@@ -5561,8 +6799,14 @@
       <c r="J20" s="2" t="s">
         <v>186</v>
       </c>
-    </row>
-    <row r="21" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="M20" s="2" t="s">
+        <v>1574</v>
+      </c>
+      <c r="N20" s="2" t="s">
+        <v>1575</v>
+      </c>
+    </row>
+    <row r="21" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
         <v>129</v>
       </c>
@@ -5590,8 +6834,14 @@
       <c r="J21" s="2" t="s">
         <v>205</v>
       </c>
-    </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="M21" s="2" t="s">
+        <v>1537</v>
+      </c>
+      <c r="N21" s="2" t="s">
+        <v>1577</v>
+      </c>
+    </row>
+    <row r="22" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
         <v>130</v>
       </c>
@@ -5622,8 +6872,14 @@
       <c r="K22" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="M22" s="2" t="s">
+        <v>1578</v>
+      </c>
+      <c r="N22" s="2" t="s">
+        <v>1583</v>
+      </c>
+    </row>
+    <row r="23" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
         <v>131</v>
       </c>
@@ -5651,8 +6907,14 @@
       <c r="J23" s="2" t="s">
         <v>188</v>
       </c>
-    </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="M23" s="2" t="s">
+        <v>1537</v>
+      </c>
+      <c r="N23" s="2" t="s">
+        <v>1584</v>
+      </c>
+    </row>
+    <row r="24" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
         <v>132</v>
       </c>
@@ -5680,8 +6942,14 @@
       <c r="J24" s="2" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="M24" s="2" t="s">
+        <v>1537</v>
+      </c>
+      <c r="N24" s="2" t="s">
+        <v>1586</v>
+      </c>
+    </row>
+    <row r="25" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
         <v>264</v>
       </c>
@@ -5709,8 +6977,14 @@
       <c r="J25" s="2" t="s">
         <v>270</v>
       </c>
-    </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="M25" s="2" t="s">
+        <v>1587</v>
+      </c>
+      <c r="N25" s="2" t="s">
+        <v>1590</v>
+      </c>
+    </row>
+    <row r="26" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
         <v>323</v>
       </c>
@@ -5735,8 +7009,14 @@
       <c r="J26" s="2" t="s">
         <v>328</v>
       </c>
-    </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="M26" s="2" t="s">
+        <v>1591</v>
+      </c>
+      <c r="N26" s="2" t="s">
+        <v>1592</v>
+      </c>
+    </row>
+    <row r="27" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
         <v>329</v>
       </c>
@@ -5764,8 +7044,14 @@
       <c r="J27" s="2" t="s">
         <v>200</v>
       </c>
-    </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="M27" s="2" t="s">
+        <v>1595</v>
+      </c>
+      <c r="N27" s="2" t="s">
+        <v>1596</v>
+      </c>
+    </row>
+    <row r="28" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
         <v>330</v>
       </c>
@@ -5790,8 +7076,14 @@
       <c r="J28" s="2" t="s">
         <v>396</v>
       </c>
-    </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="M28" s="2" t="s">
+        <v>1597</v>
+      </c>
+      <c r="N28" s="2" t="s">
+        <v>1581</v>
+      </c>
+    </row>
+    <row r="29" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
         <v>331</v>
       </c>
@@ -5819,8 +7111,14 @@
       <c r="J29" s="2" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="M29" s="2" t="s">
+        <v>1598</v>
+      </c>
+      <c r="N29" s="2" t="s">
+        <v>1599</v>
+      </c>
+    </row>
+    <row r="30" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
         <v>332</v>
       </c>
@@ -5845,8 +7143,14 @@
       <c r="J30" s="2" t="s">
         <v>200</v>
       </c>
-    </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="M30" s="2" t="s">
+        <v>1600</v>
+      </c>
+      <c r="N30" s="2" t="s">
+        <v>1518</v>
+      </c>
+    </row>
+    <row r="31" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A31" t="s">
         <v>333</v>
       </c>
@@ -5877,8 +7181,14 @@
       <c r="K31" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="M31" s="2" t="s">
+        <v>1604</v>
+      </c>
+      <c r="N31" s="2" t="s">
+        <v>1605</v>
+      </c>
+    </row>
+    <row r="32" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A32" t="s">
         <v>334</v>
       </c>
@@ -5905,6 +7215,12 @@
       </c>
       <c r="J32" s="2" t="s">
         <v>194</v>
+      </c>
+      <c r="M32" s="2" t="s">
+        <v>1606</v>
+      </c>
+      <c r="N32" s="2" t="s">
+        <v>1607</v>
       </c>
     </row>
     <row r="33" spans="1:16" x14ac:dyDescent="0.45">
@@ -5935,6 +7251,12 @@
       <c r="J33" s="2" t="s">
         <v>200</v>
       </c>
+      <c r="M33" s="2" t="s">
+        <v>1608</v>
+      </c>
+      <c r="N33" s="2" t="s">
+        <v>1609</v>
+      </c>
     </row>
     <row r="34" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A34" t="s">
@@ -5964,6 +7286,12 @@
       <c r="J34" s="2" t="s">
         <v>186</v>
       </c>
+      <c r="M34" s="2" t="s">
+        <v>1610</v>
+      </c>
+      <c r="N34" s="2" t="s">
+        <v>1612</v>
+      </c>
     </row>
     <row r="35" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A35" t="s">
@@ -5993,6 +7321,12 @@
       <c r="J35" s="2" t="s">
         <v>188</v>
       </c>
+      <c r="M35" s="2" t="s">
+        <v>1613</v>
+      </c>
+      <c r="N35" s="2" t="s">
+        <v>1614</v>
+      </c>
     </row>
     <row r="36" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A36" t="s">
@@ -6019,6 +7353,12 @@
       <c r="J36" s="2" t="s">
         <v>179</v>
       </c>
+      <c r="M36" s="2" t="s">
+        <v>1615</v>
+      </c>
+      <c r="N36" s="2" t="s">
+        <v>1526</v>
+      </c>
     </row>
     <row r="37" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A37" t="s">
@@ -6045,6 +7385,12 @@
       <c r="J37" s="2" t="s">
         <v>432</v>
       </c>
+      <c r="M37" s="2" t="s">
+        <v>1616</v>
+      </c>
+      <c r="N37" s="2" t="s">
+        <v>1617</v>
+      </c>
     </row>
     <row r="38" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A38" t="s">
@@ -6074,6 +7420,12 @@
       <c r="J38" s="2" t="s">
         <v>436</v>
       </c>
+      <c r="M38" s="2" t="s">
+        <v>1618</v>
+      </c>
+      <c r="N38" s="2" t="s">
+        <v>1518</v>
+      </c>
     </row>
     <row r="39" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A39" t="s">
@@ -6100,6 +7452,12 @@
       <c r="J39" s="2" t="s">
         <v>186</v>
       </c>
+      <c r="M39" s="2" t="s">
+        <v>1619</v>
+      </c>
+      <c r="N39" s="2" t="s">
+        <v>1620</v>
+      </c>
     </row>
     <row r="40" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A40" t="s">
@@ -6129,6 +7487,12 @@
       <c r="J40" s="2" t="s">
         <v>194</v>
       </c>
+      <c r="M40" s="2" t="s">
+        <v>1621</v>
+      </c>
+      <c r="N40" s="2" t="s">
+        <v>1622</v>
+      </c>
     </row>
     <row r="41" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A41" t="s">
@@ -6155,6 +7519,12 @@
       <c r="J41" s="2" t="s">
         <v>186</v>
       </c>
+      <c r="M41" s="2" t="s">
+        <v>1623</v>
+      </c>
+      <c r="N41" s="2" t="s">
+        <v>1624</v>
+      </c>
     </row>
     <row r="42" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A42" t="s">
@@ -6184,6 +7554,12 @@
       <c r="J42" s="2" t="s">
         <v>179</v>
       </c>
+      <c r="M42" s="2" t="s">
+        <v>1626</v>
+      </c>
+      <c r="N42" s="2" t="s">
+        <v>1627</v>
+      </c>
     </row>
     <row r="43" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A43" t="s">
@@ -6213,6 +7589,12 @@
       <c r="J43" s="2" t="s">
         <v>200</v>
       </c>
+      <c r="M43" s="2" t="s">
+        <v>1628</v>
+      </c>
+      <c r="N43" s="2" t="s">
+        <v>1630</v>
+      </c>
     </row>
     <row r="44" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A44" t="s">
@@ -6242,6 +7624,12 @@
       <c r="J44" s="2" t="s">
         <v>197</v>
       </c>
+      <c r="M44" s="2" t="s">
+        <v>1619</v>
+      </c>
+      <c r="N44" s="2" t="s">
+        <v>1631</v>
+      </c>
     </row>
     <row r="45" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A45" t="s">
@@ -6271,6 +7659,12 @@
       <c r="J45" s="2" t="s">
         <v>179</v>
       </c>
+      <c r="M45" s="2" t="s">
+        <v>1632</v>
+      </c>
+      <c r="N45" s="2" t="s">
+        <v>1633</v>
+      </c>
     </row>
     <row r="46" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A46" t="s">
@@ -6303,8 +7697,12 @@
       <c r="L46" t="b">
         <v>1</v>
       </c>
-      <c r="M46" s="2"/>
-      <c r="N46" s="2"/>
+      <c r="M46" s="2" t="s">
+        <v>1636</v>
+      </c>
+      <c r="N46" s="2" t="s">
+        <v>1637</v>
+      </c>
       <c r="O46" s="2"/>
       <c r="P46" s="2"/>
     </row>
@@ -6336,6 +7734,12 @@
       <c r="J47" s="2" t="s">
         <v>179</v>
       </c>
+      <c r="M47" s="2" t="s">
+        <v>1639</v>
+      </c>
+      <c r="N47" s="2" t="s">
+        <v>1561</v>
+      </c>
     </row>
     <row r="48" spans="1:16" x14ac:dyDescent="0.45">
       <c r="A48" t="s">
@@ -6365,8 +7769,14 @@
       <c r="J48" s="2" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M48" s="2" t="s">
+        <v>1641</v>
+      </c>
+      <c r="N48" s="2" t="s">
+        <v>1642</v>
+      </c>
+    </row>
+    <row r="49" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A49" t="s">
         <v>271</v>
       </c>
@@ -6394,8 +7804,14 @@
       <c r="J49" s="2" t="s">
         <v>274</v>
       </c>
-    </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M49" s="2" t="s">
+        <v>1530</v>
+      </c>
+      <c r="N49" s="2" t="s">
+        <v>1510</v>
+      </c>
+    </row>
+    <row r="50" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A50" t="s">
         <v>476</v>
       </c>
@@ -6420,8 +7836,14 @@
       <c r="J50" s="2" t="s">
         <v>558</v>
       </c>
-    </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M50" s="2" t="s">
+        <v>1644</v>
+      </c>
+      <c r="N50" s="2" t="s">
+        <v>1646</v>
+      </c>
+    </row>
+    <row r="51" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A51" t="s">
         <v>477</v>
       </c>
@@ -6446,8 +7868,14 @@
       <c r="J51" s="2" t="s">
         <v>560</v>
       </c>
-    </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M51" s="2" t="s">
+        <v>1647</v>
+      </c>
+      <c r="N51" s="2" t="s">
+        <v>1648</v>
+      </c>
+    </row>
+    <row r="52" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A52" t="s">
         <v>478</v>
       </c>
@@ -6475,8 +7903,14 @@
       <c r="J52" s="2" t="s">
         <v>188</v>
       </c>
-    </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M52" s="2" t="s">
+        <v>1649</v>
+      </c>
+      <c r="N52" s="2" t="s">
+        <v>1510</v>
+      </c>
+    </row>
+    <row r="53" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A53" t="s">
         <v>479</v>
       </c>
@@ -6501,8 +7935,14 @@
       <c r="J53" s="2" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M53" s="2" t="s">
+        <v>1650</v>
+      </c>
+      <c r="N53" s="2" t="s">
+        <v>1651</v>
+      </c>
+    </row>
+    <row r="54" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A54" t="s">
         <v>480</v>
       </c>
@@ -6530,8 +7970,14 @@
       <c r="J54" s="2" t="s">
         <v>200</v>
       </c>
-    </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M54" s="2" t="s">
+        <v>1652</v>
+      </c>
+      <c r="N54" s="2" t="s">
+        <v>1550</v>
+      </c>
+    </row>
+    <row r="55" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A55" t="s">
         <v>481</v>
       </c>
@@ -6559,8 +8005,14 @@
       <c r="J55" s="2" t="s">
         <v>564</v>
       </c>
-    </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M55" s="2" t="s">
+        <v>1653</v>
+      </c>
+      <c r="N55" s="2" t="s">
+        <v>1543</v>
+      </c>
+    </row>
+    <row r="56" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A56" t="s">
         <v>482</v>
       </c>
@@ -6588,8 +8040,14 @@
       <c r="J56" s="2" t="s">
         <v>186</v>
       </c>
-    </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M56" s="2" t="s">
+        <v>1654</v>
+      </c>
+      <c r="N56" s="2" t="s">
+        <v>1656</v>
+      </c>
+    </row>
+    <row r="57" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A57" t="s">
         <v>483</v>
       </c>
@@ -6614,8 +8072,14 @@
       <c r="J57" s="2" t="s">
         <v>186</v>
       </c>
-    </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M57" s="2" t="s">
+        <v>1657</v>
+      </c>
+      <c r="N57" s="2" t="s">
+        <v>1658</v>
+      </c>
+    </row>
+    <row r="58" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A58" t="s">
         <v>484</v>
       </c>
@@ -6643,8 +8107,14 @@
       <c r="J58" s="2" t="s">
         <v>183</v>
       </c>
-    </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M58" s="2" t="s">
+        <v>1660</v>
+      </c>
+      <c r="N58" s="2" t="s">
+        <v>1662</v>
+      </c>
+    </row>
+    <row r="59" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A59" t="s">
         <v>485</v>
       </c>
@@ -6669,8 +8139,14 @@
       <c r="J59" s="2" t="s">
         <v>200</v>
       </c>
-    </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M59" s="2" t="s">
+        <v>1663</v>
+      </c>
+      <c r="N59" s="2" t="s">
+        <v>1543</v>
+      </c>
+    </row>
+    <row r="60" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A60" t="s">
         <v>486</v>
       </c>
@@ -6695,8 +8171,14 @@
       <c r="J60" s="2" t="s">
         <v>200</v>
       </c>
-    </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M60" s="2" t="s">
+        <v>1664</v>
+      </c>
+      <c r="N60" s="2" t="s">
+        <v>1666</v>
+      </c>
+    </row>
+    <row r="61" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A61" t="s">
         <v>487</v>
       </c>
@@ -6724,8 +8206,14 @@
       <c r="J61" s="2" t="s">
         <v>200</v>
       </c>
-    </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M61" s="2" t="s">
+        <v>1667</v>
+      </c>
+      <c r="N61" s="2" t="s">
+        <v>1609</v>
+      </c>
+    </row>
+    <row r="62" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A62" t="s">
         <v>488</v>
       </c>
@@ -6753,8 +8241,14 @@
       <c r="J62" s="2" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M62" s="2" t="s">
+        <v>1668</v>
+      </c>
+      <c r="N62" s="2" t="s">
+        <v>1651</v>
+      </c>
+    </row>
+    <row r="63" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A63" t="s">
         <v>489</v>
       </c>
@@ -6782,8 +8276,14 @@
       <c r="J63" s="2" t="s">
         <v>188</v>
       </c>
-    </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M63" s="2" t="s">
+        <v>1669</v>
+      </c>
+      <c r="N63" s="2" t="s">
+        <v>1670</v>
+      </c>
+    </row>
+    <row r="64" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A64" t="s">
         <v>490</v>
       </c>
@@ -6811,8 +8311,14 @@
       <c r="J64" s="2" t="s">
         <v>564</v>
       </c>
-    </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="M64" s="2" t="s">
+        <v>1672</v>
+      </c>
+      <c r="N64" s="2" t="s">
+        <v>1673</v>
+      </c>
+    </row>
+    <row r="65" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A65" t="s">
         <v>491</v>
       </c>
@@ -6840,8 +8346,14 @@
       <c r="J65" s="2" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="M65" s="2" t="s">
+        <v>1674</v>
+      </c>
+      <c r="N65" s="2" t="s">
+        <v>1675</v>
+      </c>
+    </row>
+    <row r="66" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A66" t="s">
         <v>492</v>
       </c>
@@ -6866,8 +8378,14 @@
       <c r="J66" s="2" t="s">
         <v>200</v>
       </c>
-    </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="M66" s="2" t="s">
+        <v>1676</v>
+      </c>
+      <c r="N66" s="2" t="s">
+        <v>1677</v>
+      </c>
+    </row>
+    <row r="67" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A67" t="s">
         <v>493</v>
       </c>
@@ -6892,8 +8410,14 @@
       <c r="J67" s="2" t="s">
         <v>570</v>
       </c>
-    </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="M67" s="2" t="s">
+        <v>1678</v>
+      </c>
+      <c r="N67" s="2" t="s">
+        <v>1679</v>
+      </c>
+    </row>
+    <row r="68" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A68" t="s">
         <v>494</v>
       </c>
@@ -6921,8 +8445,14 @@
       <c r="J68" s="2" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="M68" s="2" t="s">
+        <v>1680</v>
+      </c>
+      <c r="N68" s="2" t="s">
+        <v>1681</v>
+      </c>
+    </row>
+    <row r="69" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A69" t="s">
         <v>495</v>
       </c>
@@ -6950,8 +8480,14 @@
       <c r="J69" s="2" t="s">
         <v>200</v>
       </c>
-    </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="M69" s="2" t="s">
+        <v>1682</v>
+      </c>
+      <c r="N69" s="2" t="s">
+        <v>1683</v>
+      </c>
+    </row>
+    <row r="70" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A70" t="s">
         <v>85</v>
       </c>
@@ -6979,8 +8515,14 @@
       <c r="K70" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="M70" s="2" t="s">
+        <v>1684</v>
+      </c>
+      <c r="N70" s="2" t="s">
+        <v>1685</v>
+      </c>
+    </row>
+    <row r="71" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A71" t="s">
         <v>275</v>
       </c>
@@ -7008,8 +8550,14 @@
       <c r="J71" s="2" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="M71" s="2" t="s">
+        <v>1686</v>
+      </c>
+      <c r="N71" s="2" t="s">
+        <v>1687</v>
+      </c>
+    </row>
+    <row r="72" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A72" t="s">
         <v>535</v>
       </c>
@@ -7037,8 +8585,14 @@
       <c r="J72" s="2" t="s">
         <v>181</v>
       </c>
-    </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="M72" s="2" t="s">
+        <v>1688</v>
+      </c>
+      <c r="N72" s="2" t="s">
+        <v>1689</v>
+      </c>
+    </row>
+    <row r="73" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A73" t="s">
         <v>536</v>
       </c>
@@ -7066,8 +8620,14 @@
       <c r="J73" s="2" t="s">
         <v>188</v>
       </c>
-    </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="M73" s="2" t="s">
+        <v>1547</v>
+      </c>
+      <c r="N73" s="2" t="s">
+        <v>1552</v>
+      </c>
+    </row>
+    <row r="74" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A74" t="s">
         <v>537</v>
       </c>
@@ -7092,8 +8652,14 @@
       <c r="J74" s="2" t="s">
         <v>186</v>
       </c>
-    </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="M74" s="2" t="s">
+        <v>1690</v>
+      </c>
+      <c r="N74" s="2" t="s">
+        <v>1691</v>
+      </c>
+    </row>
+    <row r="75" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A75" t="s">
         <v>538</v>
       </c>
@@ -7118,8 +8684,14 @@
       <c r="J75" s="2" t="s">
         <v>183</v>
       </c>
-    </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="M75" s="2" t="s">
+        <v>1693</v>
+      </c>
+      <c r="N75" s="2" t="s">
+        <v>1694</v>
+      </c>
+    </row>
+    <row r="76" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A76" t="s">
         <v>539</v>
       </c>
@@ -7144,8 +8716,14 @@
       <c r="J76" s="2" t="s">
         <v>649</v>
       </c>
-    </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="M76" s="2" t="s">
+        <v>1695</v>
+      </c>
+      <c r="N76" s="2" t="s">
+        <v>1561</v>
+      </c>
+    </row>
+    <row r="77" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A77" t="s">
         <v>540</v>
       </c>
@@ -7170,8 +8748,14 @@
       <c r="J77" s="2" t="s">
         <v>650</v>
       </c>
-    </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="M77" s="2" t="s">
+        <v>1696</v>
+      </c>
+      <c r="N77" s="2" t="s">
+        <v>1697</v>
+      </c>
+    </row>
+    <row r="78" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A78" t="s">
         <v>541</v>
       </c>
@@ -7199,8 +8783,14 @@
       <c r="J78" s="2" t="s">
         <v>436</v>
       </c>
-    </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="M78" s="2" t="s">
+        <v>1698</v>
+      </c>
+      <c r="N78" s="2" t="s">
+        <v>1699</v>
+      </c>
+    </row>
+    <row r="79" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A79" t="s">
         <v>542</v>
       </c>
@@ -7228,8 +8818,14 @@
       <c r="J79" s="2" t="s">
         <v>651</v>
       </c>
-    </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="M79" s="2" t="s">
+        <v>1700</v>
+      </c>
+      <c r="N79" s="2" t="s">
+        <v>1701</v>
+      </c>
+    </row>
+    <row r="80" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A80" t="s">
         <v>543</v>
       </c>
@@ -7257,8 +8853,14 @@
       <c r="J80" s="2" t="s">
         <v>653</v>
       </c>
-    </row>
-    <row r="81" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M80" s="2" t="s">
+        <v>1702</v>
+      </c>
+      <c r="N80" s="2" t="s">
+        <v>1703</v>
+      </c>
+    </row>
+    <row r="81" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A81" t="s">
         <v>544</v>
       </c>
@@ -7286,8 +8888,14 @@
       <c r="J81" s="2" t="s">
         <v>200</v>
       </c>
-    </row>
-    <row r="82" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M81" s="2" t="s">
+        <v>1700</v>
+      </c>
+      <c r="N81" s="2" t="s">
+        <v>1704</v>
+      </c>
+    </row>
+    <row r="82" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A82" t="s">
         <v>545</v>
       </c>
@@ -7312,8 +8920,14 @@
       <c r="J82" s="2" t="s">
         <v>186</v>
       </c>
-    </row>
-    <row r="83" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M82" s="2" t="s">
+        <v>1706</v>
+      </c>
+      <c r="N82" s="2" t="s">
+        <v>1707</v>
+      </c>
+    </row>
+    <row r="83" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A83" t="s">
         <v>546</v>
       </c>
@@ -7338,8 +8952,14 @@
       <c r="J83" s="2" t="s">
         <v>179</v>
       </c>
-    </row>
-    <row r="84" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M83" s="2" t="s">
+        <v>1708</v>
+      </c>
+      <c r="N83" s="2" t="s">
+        <v>1709</v>
+      </c>
+    </row>
+    <row r="84" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A84" t="s">
         <v>547</v>
       </c>
@@ -7367,8 +8987,14 @@
       <c r="J84" s="2" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="85" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M84" s="2" t="s">
+        <v>1710</v>
+      </c>
+      <c r="N84" s="2" t="s">
+        <v>1711</v>
+      </c>
+    </row>
+    <row r="85" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A85" t="s">
         <v>548</v>
       </c>
@@ -7396,8 +9022,14 @@
       <c r="J85" s="2" t="s">
         <v>200</v>
       </c>
-    </row>
-    <row r="86" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M85" s="2" t="s">
+        <v>1712</v>
+      </c>
+      <c r="N85" s="2" t="s">
+        <v>1713</v>
+      </c>
+    </row>
+    <row r="86" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A86" t="s">
         <v>549</v>
       </c>
@@ -7422,8 +9054,14 @@
       <c r="J86" s="2" t="s">
         <v>188</v>
       </c>
-    </row>
-    <row r="87" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M86" s="2" t="s">
+        <v>1667</v>
+      </c>
+      <c r="N86" s="2" t="s">
+        <v>1715</v>
+      </c>
+    </row>
+    <row r="87" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A87" t="s">
         <v>550</v>
       </c>
@@ -7448,8 +9086,14 @@
       <c r="J87" s="2" t="s">
         <v>188</v>
       </c>
-    </row>
-    <row r="88" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M87" s="2" t="s">
+        <v>1717</v>
+      </c>
+      <c r="N87" s="2" t="s">
+        <v>1718</v>
+      </c>
+    </row>
+    <row r="88" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A88" t="s">
         <v>551</v>
       </c>
@@ -7477,8 +9121,14 @@
       <c r="J88" s="2" t="s">
         <v>188</v>
       </c>
-    </row>
-    <row r="89" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M88" s="2" t="s">
+        <v>1719</v>
+      </c>
+      <c r="N88" s="2" t="s">
+        <v>1720</v>
+      </c>
+    </row>
+    <row r="89" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A89" t="s">
         <v>552</v>
       </c>
@@ -7506,8 +9156,14 @@
       <c r="J89" s="2" t="s">
         <v>179</v>
       </c>
-    </row>
-    <row r="90" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M89" s="2" t="s">
+        <v>1722</v>
+      </c>
+      <c r="N89" s="2" t="s">
+        <v>1527</v>
+      </c>
+    </row>
+    <row r="90" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A90" t="s">
         <v>553</v>
       </c>
@@ -7535,8 +9191,14 @@
       <c r="J90" s="2" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="91" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M90" s="2" t="s">
+        <v>1723</v>
+      </c>
+      <c r="N90" s="2" t="s">
+        <v>1724</v>
+      </c>
+    </row>
+    <row r="91" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A91" t="s">
         <v>554</v>
       </c>
@@ -7564,8 +9226,14 @@
       <c r="J91" s="2" t="s">
         <v>663</v>
       </c>
-    </row>
-    <row r="92" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M91" s="2" t="s">
+        <v>1725</v>
+      </c>
+      <c r="N91" s="2" t="s">
+        <v>1726</v>
+      </c>
+    </row>
+    <row r="92" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A92" t="s">
         <v>555</v>
       </c>
@@ -7593,8 +9261,14 @@
       <c r="J92" s="2" t="s">
         <v>665</v>
       </c>
-    </row>
-    <row r="93" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M92" s="2" t="s">
+        <v>1727</v>
+      </c>
+      <c r="N92" s="2" t="s">
+        <v>1729</v>
+      </c>
+    </row>
+    <row r="93" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A93" t="s">
         <v>556</v>
       </c>
@@ -7622,8 +9296,14 @@
       <c r="J93" s="2" t="s">
         <v>194</v>
       </c>
-    </row>
-    <row r="94" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M93" s="2" t="s">
+        <v>1730</v>
+      </c>
+      <c r="N93" s="2" t="s">
+        <v>1585</v>
+      </c>
+    </row>
+    <row r="94" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A94" t="s">
         <v>281</v>
       </c>
@@ -7648,8 +9328,14 @@
       <c r="J94" s="2" t="s">
         <v>283</v>
       </c>
-    </row>
-    <row r="95" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M94" s="2" t="s">
+        <v>1731</v>
+      </c>
+      <c r="N94" s="2" t="s">
+        <v>1552</v>
+      </c>
+    </row>
+    <row r="95" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A95" t="s">
         <v>738</v>
       </c>
@@ -7671,8 +9357,14 @@
       <c r="J95" s="2" t="s">
         <v>744</v>
       </c>
-    </row>
-    <row r="96" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M95" s="2" t="s">
+        <v>1732</v>
+      </c>
+      <c r="N95" s="2" t="s">
+        <v>1733</v>
+      </c>
+    </row>
+    <row r="96" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A96" t="s">
         <v>739</v>
       </c>
@@ -7700,8 +9392,14 @@
       <c r="J96" s="2" t="s">
         <v>183</v>
       </c>
-    </row>
-    <row r="97" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M96" s="2" t="s">
+        <v>1734</v>
+      </c>
+      <c r="N96" s="2" t="s">
+        <v>1736</v>
+      </c>
+    </row>
+    <row r="97" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A97" t="s">
         <v>740</v>
       </c>
@@ -7726,8 +9424,14 @@
       <c r="J97" s="2" t="s">
         <v>558</v>
       </c>
-    </row>
-    <row r="98" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M97" s="2" t="s">
+        <v>1737</v>
+      </c>
+      <c r="N97" s="2" t="s">
+        <v>1738</v>
+      </c>
+    </row>
+    <row r="98" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A98" t="s">
         <v>17</v>
       </c>
@@ -7752,8 +9456,14 @@
       <c r="K98" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="99" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M98" s="2" t="s">
+        <v>1740</v>
+      </c>
+      <c r="N98" s="2" t="s">
+        <v>1741</v>
+      </c>
+    </row>
+    <row r="99" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A99" t="s">
         <v>756</v>
       </c>
@@ -7781,8 +9491,14 @@
       <c r="J99" s="2" t="s">
         <v>762</v>
       </c>
-    </row>
-    <row r="100" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M99" s="2" t="s">
+        <v>1742</v>
+      </c>
+      <c r="N99" s="2" t="s">
+        <v>1582</v>
+      </c>
+    </row>
+    <row r="100" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A100" t="s">
         <v>757</v>
       </c>
@@ -7813,8 +9529,14 @@
       <c r="L100" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="101" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M100" s="2" t="s">
+        <v>1745</v>
+      </c>
+      <c r="N100" s="2" t="s">
+        <v>1746</v>
+      </c>
+    </row>
+    <row r="101" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A101" t="s">
         <v>758</v>
       </c>
@@ -7839,8 +9561,14 @@
       <c r="J101" s="2" t="s">
         <v>436</v>
       </c>
-    </row>
-    <row r="102" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M101" s="2" t="s">
+        <v>1748</v>
+      </c>
+      <c r="N101" s="2" t="s">
+        <v>1749</v>
+      </c>
+    </row>
+    <row r="102" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A102" t="s">
         <v>284</v>
       </c>
@@ -7865,8 +9593,14 @@
       <c r="K102" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="103" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M102" s="2" t="s">
+        <v>1566</v>
+      </c>
+      <c r="N102" s="2" t="s">
+        <v>1666</v>
+      </c>
+    </row>
+    <row r="103" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A103" t="s">
         <v>774</v>
       </c>
@@ -7891,8 +9625,14 @@
       <c r="J103" s="2" t="s">
         <v>564</v>
       </c>
-    </row>
-    <row r="104" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M103" s="2" t="s">
+        <v>1750</v>
+      </c>
+      <c r="N103" s="2" t="s">
+        <v>1751</v>
+      </c>
+    </row>
+    <row r="104" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A104" t="s">
         <v>775</v>
       </c>
@@ -7917,8 +9657,14 @@
       <c r="J104" s="2" t="s">
         <v>186</v>
       </c>
-    </row>
-    <row r="105" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M104" s="2" t="s">
+        <v>1752</v>
+      </c>
+      <c r="N104" s="2" t="s">
+        <v>1753</v>
+      </c>
+    </row>
+    <row r="105" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A105" t="s">
         <v>776</v>
       </c>
@@ -7943,8 +9689,14 @@
       <c r="J105" s="2" t="s">
         <v>558</v>
       </c>
-    </row>
-    <row r="106" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M105" s="2" t="s">
+        <v>1755</v>
+      </c>
+      <c r="N105" s="2" t="s">
+        <v>1756</v>
+      </c>
+    </row>
+    <row r="106" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A106" t="s">
         <v>777</v>
       </c>
@@ -7969,8 +9721,14 @@
       <c r="J106" s="2" t="s">
         <v>194</v>
       </c>
-    </row>
-    <row r="107" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M106" s="2" t="s">
+        <v>1757</v>
+      </c>
+      <c r="N106" s="2" t="s">
+        <v>1622</v>
+      </c>
+    </row>
+    <row r="107" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A107" t="s">
         <v>778</v>
       </c>
@@ -7998,8 +9756,14 @@
       <c r="J107" s="2" t="s">
         <v>194</v>
       </c>
-    </row>
-    <row r="108" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M107" s="2" t="s">
+        <v>1760</v>
+      </c>
+      <c r="N107" s="2" t="s">
+        <v>1761</v>
+      </c>
+    </row>
+    <row r="108" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A108" t="s">
         <v>779</v>
       </c>
@@ -8027,8 +9791,14 @@
       <c r="J108" s="2" t="s">
         <v>194</v>
       </c>
-    </row>
-    <row r="109" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M108" s="2" t="s">
+        <v>1762</v>
+      </c>
+      <c r="N108" s="2" t="s">
+        <v>1586</v>
+      </c>
+    </row>
+    <row r="109" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A109" t="s">
         <v>96</v>
       </c>
@@ -8053,8 +9823,14 @@
       <c r="K109" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="110" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M109" s="2" t="s">
+        <v>1763</v>
+      </c>
+      <c r="N109" s="2" t="s">
+        <v>1764</v>
+      </c>
+    </row>
+    <row r="110" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A110" t="s">
         <v>807</v>
       </c>
@@ -8082,8 +9858,14 @@
       <c r="J110" s="2" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="111" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M110" s="2" t="s">
+        <v>1765</v>
+      </c>
+      <c r="N110" s="2" t="s">
+        <v>1592</v>
+      </c>
+    </row>
+    <row r="111" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A111" t="s">
         <v>808</v>
       </c>
@@ -8108,8 +9890,14 @@
       <c r="J111" s="2" t="s">
         <v>436</v>
       </c>
-    </row>
-    <row r="112" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M111" s="2" t="s">
+        <v>1768</v>
+      </c>
+      <c r="N111" s="2" t="s">
+        <v>1769</v>
+      </c>
+    </row>
+    <row r="112" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A112" t="s">
         <v>809</v>
       </c>
@@ -8137,8 +9925,14 @@
       <c r="J112" s="2" t="s">
         <v>837</v>
       </c>
-    </row>
-    <row r="113" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M112" s="2" t="s">
+        <v>1770</v>
+      </c>
+      <c r="N112" s="2" t="s">
+        <v>1586</v>
+      </c>
+    </row>
+    <row r="113" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A113" t="s">
         <v>810</v>
       </c>
@@ -8163,8 +9957,14 @@
       <c r="J113" s="2" t="s">
         <v>744</v>
       </c>
-    </row>
-    <row r="114" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M113" s="2" t="s">
+        <v>1772</v>
+      </c>
+      <c r="N113" s="2" t="s">
+        <v>1773</v>
+      </c>
+    </row>
+    <row r="114" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A114" t="s">
         <v>811</v>
       </c>
@@ -8189,8 +9989,14 @@
       <c r="J114" s="2" t="s">
         <v>564</v>
       </c>
-    </row>
-    <row r="115" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M114" s="2" t="s">
+        <v>1712</v>
+      </c>
+      <c r="N114" s="2" t="s">
+        <v>1774</v>
+      </c>
+    </row>
+    <row r="115" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A115" t="s">
         <v>812</v>
       </c>
@@ -8218,8 +10024,14 @@
       <c r="J115" s="2" t="s">
         <v>186</v>
       </c>
-    </row>
-    <row r="116" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M115" s="2" t="s">
+        <v>1775</v>
+      </c>
+      <c r="N115" s="2" t="s">
+        <v>1776</v>
+      </c>
+    </row>
+    <row r="116" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A116" t="s">
         <v>813</v>
       </c>
@@ -8247,8 +10059,14 @@
       <c r="J116" s="2" t="s">
         <v>194</v>
       </c>
-    </row>
-    <row r="117" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M116" s="2" t="s">
+        <v>1777</v>
+      </c>
+      <c r="N116" s="2" t="s">
+        <v>1778</v>
+      </c>
+    </row>
+    <row r="117" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A117" t="s">
         <v>814</v>
       </c>
@@ -8273,8 +10091,11 @@
       <c r="J117" s="2" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="118" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M117" s="2" t="s">
+        <v>1780</v>
+      </c>
+    </row>
+    <row r="118" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A118" t="s">
         <v>815</v>
       </c>
@@ -8302,8 +10123,14 @@
       <c r="J118" s="2" t="s">
         <v>564</v>
       </c>
-    </row>
-    <row r="119" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M118" s="2" t="s">
+        <v>1781</v>
+      </c>
+      <c r="N118" s="2" t="s">
+        <v>1782</v>
+      </c>
+    </row>
+    <row r="119" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A119" t="s">
         <v>816</v>
       </c>
@@ -8331,8 +10158,14 @@
       <c r="J119" s="2" t="s">
         <v>866</v>
       </c>
-    </row>
-    <row r="120" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M119" s="2" t="s">
+        <v>1784</v>
+      </c>
+      <c r="N119" s="2" t="s">
+        <v>1785</v>
+      </c>
+    </row>
+    <row r="120" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A120" t="s">
         <v>817</v>
       </c>
@@ -8360,8 +10193,14 @@
       <c r="J120" s="2" t="s">
         <v>200</v>
       </c>
-    </row>
-    <row r="121" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M120" s="2" t="s">
+        <v>1786</v>
+      </c>
+      <c r="N120" s="2" t="s">
+        <v>1787</v>
+      </c>
+    </row>
+    <row r="121" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A121" t="s">
         <v>818</v>
       </c>
@@ -8389,8 +10228,14 @@
       <c r="J121" s="2" t="s">
         <v>837</v>
       </c>
-    </row>
-    <row r="122" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M121" s="2" t="s">
+        <v>1789</v>
+      </c>
+      <c r="N121" s="2" t="s">
+        <v>1679</v>
+      </c>
+    </row>
+    <row r="122" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A122" t="s">
         <v>314</v>
       </c>
@@ -8415,8 +10260,14 @@
       <c r="J122" s="2" t="s">
         <v>319</v>
       </c>
-    </row>
-    <row r="123" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M122" s="2" t="s">
+        <v>1791</v>
+      </c>
+      <c r="N122" s="2" t="s">
+        <v>1792</v>
+      </c>
+    </row>
+    <row r="123" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A123" t="s">
         <v>879</v>
       </c>
@@ -8444,8 +10295,14 @@
       <c r="J123" s="2" t="s">
         <v>564</v>
       </c>
-    </row>
-    <row r="124" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M123" s="2" t="s">
+        <v>1793</v>
+      </c>
+      <c r="N123" s="2" t="s">
+        <v>1794</v>
+      </c>
+    </row>
+    <row r="124" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A124" t="s">
         <v>880</v>
       </c>
@@ -8473,8 +10330,14 @@
       <c r="J124" s="2" t="s">
         <v>936</v>
       </c>
-    </row>
-    <row r="125" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M124" s="2" t="s">
+        <v>1795</v>
+      </c>
+      <c r="N124" s="2" t="s">
+        <v>1675</v>
+      </c>
+    </row>
+    <row r="125" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A125" t="s">
         <v>881</v>
       </c>
@@ -8499,8 +10362,14 @@
       <c r="J125" s="2" t="s">
         <v>270</v>
       </c>
-    </row>
-    <row r="126" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M125" s="2" t="s">
+        <v>1797</v>
+      </c>
+      <c r="N125" s="2" t="s">
+        <v>1592</v>
+      </c>
+    </row>
+    <row r="126" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A126" t="s">
         <v>882</v>
       </c>
@@ -8528,8 +10397,14 @@
       <c r="J126" s="2" t="s">
         <v>179</v>
       </c>
-    </row>
-    <row r="127" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M126" s="2" t="s">
+        <v>1798</v>
+      </c>
+      <c r="N126" s="2" t="s">
+        <v>1799</v>
+      </c>
+    </row>
+    <row r="127" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A127" t="s">
         <v>883</v>
       </c>
@@ -8554,8 +10429,14 @@
       <c r="J127" s="2" t="s">
         <v>938</v>
       </c>
-    </row>
-    <row r="128" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M127" s="2" t="s">
+        <v>1800</v>
+      </c>
+      <c r="N127" s="2" t="s">
+        <v>1801</v>
+      </c>
+    </row>
+    <row r="128" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A128" t="s">
         <v>884</v>
       </c>
@@ -8580,8 +10461,14 @@
       <c r="J128" s="2" t="s">
         <v>940</v>
       </c>
-    </row>
-    <row r="129" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="M128" s="2" t="s">
+        <v>1802</v>
+      </c>
+      <c r="N128" s="2" t="s">
+        <v>1803</v>
+      </c>
+    </row>
+    <row r="129" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A129" t="s">
         <v>885</v>
       </c>
@@ -8606,8 +10493,14 @@
       <c r="J129" s="2" t="s">
         <v>436</v>
       </c>
-    </row>
-    <row r="130" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="M129" s="2" t="s">
+        <v>1804</v>
+      </c>
+      <c r="N129" s="2" t="s">
+        <v>1805</v>
+      </c>
+    </row>
+    <row r="130" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A130" t="s">
         <v>886</v>
       </c>
@@ -8638,8 +10531,14 @@
       <c r="K130" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="131" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="M130" s="2" t="s">
+        <v>1730</v>
+      </c>
+      <c r="N130" s="2" t="s">
+        <v>1806</v>
+      </c>
+    </row>
+    <row r="131" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A131" t="s">
         <v>887</v>
       </c>
@@ -8667,8 +10566,14 @@
       <c r="J131" s="2" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="132" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="M131" s="2" t="s">
+        <v>1807</v>
+      </c>
+      <c r="N131" s="2" t="s">
+        <v>1526</v>
+      </c>
+    </row>
+    <row r="132" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A132" t="s">
         <v>888</v>
       </c>
@@ -8696,8 +10601,14 @@
       <c r="J132" s="2" t="s">
         <v>941</v>
       </c>
-    </row>
-    <row r="133" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="M132" s="2" t="s">
+        <v>1808</v>
+      </c>
+      <c r="N132" s="2" t="s">
+        <v>1809</v>
+      </c>
+    </row>
+    <row r="133" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A133" t="s">
         <v>889</v>
       </c>
@@ -8725,8 +10636,14 @@
       <c r="J133" s="2" t="s">
         <v>564</v>
       </c>
-    </row>
-    <row r="134" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="M133" s="2" t="s">
+        <v>1810</v>
+      </c>
+      <c r="N133" s="2" t="s">
+        <v>1552</v>
+      </c>
+    </row>
+    <row r="134" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A134" t="s">
         <v>890</v>
       </c>
@@ -8754,8 +10671,14 @@
       <c r="J134" s="2" t="s">
         <v>188</v>
       </c>
-    </row>
-    <row r="135" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="M134" s="2" t="s">
+        <v>1811</v>
+      </c>
+      <c r="N134" s="2" t="s">
+        <v>1812</v>
+      </c>
+    </row>
+    <row r="135" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A135" t="s">
         <v>891</v>
       </c>
@@ -8780,8 +10703,14 @@
       <c r="J135" s="2" t="s">
         <v>270</v>
       </c>
-    </row>
-    <row r="136" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="M135" s="2" t="s">
+        <v>1813</v>
+      </c>
+      <c r="N135" s="2" t="s">
+        <v>1814</v>
+      </c>
+    </row>
+    <row r="136" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A136" t="s">
         <v>892</v>
       </c>
@@ -8809,8 +10738,14 @@
       <c r="J136" s="2" t="s">
         <v>179</v>
       </c>
-    </row>
-    <row r="137" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="M136" s="2" t="s">
+        <v>1815</v>
+      </c>
+      <c r="N136" s="2" t="s">
+        <v>1816</v>
+      </c>
+    </row>
+    <row r="137" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A137" t="s">
         <v>893</v>
       </c>
@@ -8835,8 +10770,14 @@
       <c r="J137" s="2" t="s">
         <v>944</v>
       </c>
-    </row>
-    <row r="138" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="M137" s="2" t="s">
+        <v>1817</v>
+      </c>
+      <c r="N137" s="2" t="s">
+        <v>1818</v>
+      </c>
+    </row>
+    <row r="138" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A138" t="s">
         <v>894</v>
       </c>
@@ -8864,8 +10805,14 @@
       <c r="J138" s="2" t="s">
         <v>744</v>
       </c>
-    </row>
-    <row r="139" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="M138" s="2" t="s">
+        <v>1819</v>
+      </c>
+      <c r="N138" s="2" t="s">
+        <v>1821</v>
+      </c>
+    </row>
+    <row r="139" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A139" t="s">
         <v>895</v>
       </c>
@@ -8893,8 +10840,14 @@
       <c r="J139" s="2" t="s">
         <v>948</v>
       </c>
-    </row>
-    <row r="140" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="M139" s="2" t="s">
+        <v>1822</v>
+      </c>
+      <c r="N139" s="2" t="s">
+        <v>1525</v>
+      </c>
+    </row>
+    <row r="140" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A140" t="s">
         <v>896</v>
       </c>
@@ -8919,8 +10872,14 @@
       <c r="J140" s="2" t="s">
         <v>1056</v>
       </c>
-    </row>
-    <row r="141" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="M140" s="2" t="s">
+        <v>1589</v>
+      </c>
+      <c r="N140" s="2" t="s">
+        <v>1823</v>
+      </c>
+    </row>
+    <row r="141" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A141" t="s">
         <v>897</v>
       </c>
@@ -8945,8 +10904,14 @@
       <c r="J141" s="2" t="s">
         <v>1057</v>
       </c>
-    </row>
-    <row r="142" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="M141" s="2" t="s">
+        <v>1824</v>
+      </c>
+      <c r="N141" s="2" t="s">
+        <v>1550</v>
+      </c>
+    </row>
+    <row r="142" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A142" t="s">
         <v>898</v>
       </c>
@@ -8974,8 +10939,14 @@
       <c r="J142" s="2" t="s">
         <v>1058</v>
       </c>
-    </row>
-    <row r="143" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="M142" s="2" t="s">
+        <v>1826</v>
+      </c>
+      <c r="N142" s="2" t="s">
+        <v>1823</v>
+      </c>
+    </row>
+    <row r="143" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A143" t="s">
         <v>899</v>
       </c>
@@ -9000,8 +10971,14 @@
       <c r="J143" s="2" t="s">
         <v>188</v>
       </c>
-    </row>
-    <row r="144" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="M143" s="2" t="s">
+        <v>1660</v>
+      </c>
+      <c r="N143" s="2" t="s">
+        <v>1510</v>
+      </c>
+    </row>
+    <row r="144" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A144" t="s">
         <v>900</v>
       </c>
@@ -9026,8 +11003,14 @@
       <c r="J144" s="2" t="s">
         <v>1061</v>
       </c>
-    </row>
-    <row r="145" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M144" s="2" t="s">
+        <v>1827</v>
+      </c>
+      <c r="N144" s="2" t="s">
+        <v>1828</v>
+      </c>
+    </row>
+    <row r="145" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A145" t="s">
         <v>901</v>
       </c>
@@ -9052,8 +11035,14 @@
       <c r="J145" s="2" t="s">
         <v>1062</v>
       </c>
-    </row>
-    <row r="146" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M145" s="2" t="s">
+        <v>1829</v>
+      </c>
+      <c r="N145" s="2" t="s">
+        <v>1830</v>
+      </c>
+    </row>
+    <row r="146" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A146" t="s">
         <v>902</v>
       </c>
@@ -9078,8 +11067,14 @@
       <c r="J146" s="2" t="s">
         <v>1064</v>
       </c>
-    </row>
-    <row r="147" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M146" s="2" t="s">
+        <v>1520</v>
+      </c>
+      <c r="N146" s="2" t="s">
+        <v>1561</v>
+      </c>
+    </row>
+    <row r="147" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A147" t="s">
         <v>903</v>
       </c>
@@ -9104,8 +11099,11 @@
       <c r="J147" s="2" t="s">
         <v>197</v>
       </c>
-    </row>
-    <row r="148" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M147" s="2" t="s">
+        <v>1831</v>
+      </c>
+    </row>
+    <row r="148" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A148" t="s">
         <v>76</v>
       </c>
@@ -9133,8 +11131,14 @@
       <c r="J148" s="2" t="s">
         <v>322</v>
       </c>
-    </row>
-    <row r="149" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M148" s="2" t="s">
+        <v>1832</v>
+      </c>
+      <c r="N148" s="2" t="s">
+        <v>1526</v>
+      </c>
+    </row>
+    <row r="149" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A149" t="s">
         <v>995</v>
       </c>
@@ -9162,8 +11166,14 @@
       <c r="J149" s="2" t="s">
         <v>1066</v>
       </c>
-    </row>
-    <row r="150" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M149" s="2" t="s">
+        <v>1831</v>
+      </c>
+      <c r="N149" s="2" t="s">
+        <v>1550</v>
+      </c>
+    </row>
+    <row r="150" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A150" t="s">
         <v>996</v>
       </c>
@@ -9191,8 +11201,14 @@
       <c r="J150" s="2" t="s">
         <v>1067</v>
       </c>
-    </row>
-    <row r="151" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M150" s="2" t="s">
+        <v>1833</v>
+      </c>
+      <c r="N150" s="2" t="s">
+        <v>1834</v>
+      </c>
+    </row>
+    <row r="151" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A151" t="s">
         <v>997</v>
       </c>
@@ -9217,8 +11233,14 @@
       <c r="J151" s="2" t="s">
         <v>1068</v>
       </c>
-    </row>
-    <row r="152" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M151" s="2" t="s">
+        <v>1835</v>
+      </c>
+      <c r="N151" s="2" t="s">
+        <v>1836</v>
+      </c>
+    </row>
+    <row r="152" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A152" t="s">
         <v>998</v>
       </c>
@@ -9243,8 +11265,14 @@
       <c r="J152" s="2" t="s">
         <v>1069</v>
       </c>
-    </row>
-    <row r="153" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M152" s="2" t="s">
+        <v>1837</v>
+      </c>
+      <c r="N152" s="2" t="s">
+        <v>1580</v>
+      </c>
+    </row>
+    <row r="153" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A153" t="s">
         <v>999</v>
       </c>
@@ -9272,8 +11300,14 @@
       <c r="J153" s="2" t="s">
         <v>837</v>
       </c>
-    </row>
-    <row r="154" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M153" s="2" t="s">
+        <v>1838</v>
+      </c>
+      <c r="N153" s="2" t="s">
+        <v>1839</v>
+      </c>
+    </row>
+    <row r="154" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A154" t="s">
         <v>1000</v>
       </c>
@@ -9298,8 +11332,14 @@
       <c r="J154" s="2" t="s">
         <v>1066</v>
       </c>
-    </row>
-    <row r="155" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M154" s="2" t="s">
+        <v>1840</v>
+      </c>
+      <c r="N154" s="2" t="s">
+        <v>1544</v>
+      </c>
+    </row>
+    <row r="155" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A155" t="s">
         <v>1001</v>
       </c>
@@ -9327,8 +11367,14 @@
       <c r="J155" s="2" t="s">
         <v>1071</v>
       </c>
-    </row>
-    <row r="156" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M155" s="2" t="s">
+        <v>1841</v>
+      </c>
+      <c r="N155" s="2" t="s">
+        <v>1550</v>
+      </c>
+    </row>
+    <row r="156" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A156" t="s">
         <v>1002</v>
       </c>
@@ -9353,8 +11399,14 @@
       <c r="J156" s="2" t="s">
         <v>1072</v>
       </c>
-    </row>
-    <row r="157" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M156" s="2" t="s">
+        <v>1551</v>
+      </c>
+      <c r="N156" s="2" t="s">
+        <v>1526</v>
+      </c>
+    </row>
+    <row r="157" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A157" t="s">
         <v>1003</v>
       </c>
@@ -9382,8 +11434,14 @@
       <c r="J157" s="2" t="s">
         <v>183</v>
       </c>
-    </row>
-    <row r="158" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M157" s="2" t="s">
+        <v>1831</v>
+      </c>
+      <c r="N157" s="2" t="s">
+        <v>1586</v>
+      </c>
+    </row>
+    <row r="158" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A158" t="s">
         <v>1004</v>
       </c>
@@ -9411,8 +11469,14 @@
       <c r="J158" s="2" t="s">
         <v>744</v>
       </c>
-    </row>
-    <row r="159" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M158" s="2" t="s">
+        <v>1842</v>
+      </c>
+      <c r="N158" s="2" t="s">
+        <v>1843</v>
+      </c>
+    </row>
+    <row r="159" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A159" t="s">
         <v>1005</v>
       </c>
@@ -9437,8 +11501,14 @@
       <c r="J159" s="2" t="s">
         <v>179</v>
       </c>
-    </row>
-    <row r="160" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="M159" s="2" t="s">
+        <v>1831</v>
+      </c>
+      <c r="N159" s="2" t="s">
+        <v>1844</v>
+      </c>
+    </row>
+    <row r="160" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A160" t="s">
         <v>1006</v>
       </c>
@@ -9466,8 +11536,14 @@
       <c r="J160" s="2" t="s">
         <v>1507</v>
       </c>
-    </row>
-    <row r="161" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M160" s="2" t="s">
+        <v>1845</v>
+      </c>
+      <c r="N160" s="2" t="s">
+        <v>1846</v>
+      </c>
+    </row>
+    <row r="161" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A161" t="s">
         <v>1007</v>
       </c>
@@ -9492,8 +11568,14 @@
       <c r="J161" s="2" t="s">
         <v>1073</v>
       </c>
-    </row>
-    <row r="162" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M161" s="2" t="s">
+        <v>1847</v>
+      </c>
+      <c r="N161" s="2" t="s">
+        <v>1848</v>
+      </c>
+    </row>
+    <row r="162" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A162" t="s">
         <v>1008</v>
       </c>
@@ -9518,8 +11600,14 @@
       <c r="J162" s="2" t="s">
         <v>1074</v>
       </c>
-    </row>
-    <row r="163" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M162" s="2" t="s">
+        <v>1849</v>
+      </c>
+      <c r="N162" s="2" t="s">
+        <v>1561</v>
+      </c>
+    </row>
+    <row r="163" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A163" t="s">
         <v>1009</v>
       </c>
@@ -9547,8 +11635,14 @@
       <c r="J163" s="2" t="s">
         <v>1196</v>
       </c>
-    </row>
-    <row r="164" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M163" s="2" t="s">
+        <v>1589</v>
+      </c>
+      <c r="N163" s="2" t="s">
+        <v>1851</v>
+      </c>
+    </row>
+    <row r="164" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A164" t="s">
         <v>1010</v>
       </c>
@@ -9576,8 +11670,14 @@
       <c r="J164" s="2" t="s">
         <v>1197</v>
       </c>
-    </row>
-    <row r="165" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M164" s="2" t="s">
+        <v>1731</v>
+      </c>
+      <c r="N164" s="2" t="s">
+        <v>1852</v>
+      </c>
+    </row>
+    <row r="165" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A165" t="s">
         <v>1011</v>
       </c>
@@ -9602,8 +11702,14 @@
       <c r="J165" s="2" t="s">
         <v>1198</v>
       </c>
-    </row>
-    <row r="166" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M165" s="2" t="s">
+        <v>1762</v>
+      </c>
+      <c r="N165" s="2" t="s">
+        <v>1853</v>
+      </c>
+    </row>
+    <row r="166" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A166" t="s">
         <v>1012</v>
       </c>
@@ -9631,8 +11737,14 @@
       <c r="J166" s="2" t="s">
         <v>1196</v>
       </c>
-    </row>
-    <row r="167" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M166" s="2" t="s">
+        <v>1854</v>
+      </c>
+      <c r="N166" s="2" t="s">
+        <v>1855</v>
+      </c>
+    </row>
+    <row r="167" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A167" t="s">
         <v>1013</v>
       </c>
@@ -9660,8 +11772,14 @@
       <c r="J167" s="2" t="s">
         <v>1200</v>
       </c>
-    </row>
-    <row r="168" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M167" s="2" t="s">
+        <v>1856</v>
+      </c>
+      <c r="N167" s="2" t="s">
+        <v>1857</v>
+      </c>
+    </row>
+    <row r="168" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A168" t="s">
         <v>23</v>
       </c>
@@ -9686,8 +11804,14 @@
       <c r="J168" s="2" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="169" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M168" s="2" t="s">
+        <v>1663</v>
+      </c>
+      <c r="N168" s="2" t="s">
+        <v>1526</v>
+      </c>
+    </row>
+    <row r="169" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A169" t="s">
         <v>1139</v>
       </c>
@@ -9715,8 +11839,14 @@
       <c r="J169" s="2" t="s">
         <v>1196</v>
       </c>
-    </row>
-    <row r="170" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M169" s="2" t="s">
+        <v>1858</v>
+      </c>
+      <c r="N169" s="2" t="s">
+        <v>1834</v>
+      </c>
+    </row>
+    <row r="170" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A170" t="s">
         <v>1140</v>
       </c>
@@ -9747,8 +11877,14 @@
       <c r="L170" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="171" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M170" s="2" t="s">
+        <v>1859</v>
+      </c>
+      <c r="N170" s="2" t="s">
+        <v>1543</v>
+      </c>
+    </row>
+    <row r="171" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A171" t="s">
         <v>1141</v>
       </c>
@@ -9779,8 +11915,14 @@
       <c r="L171" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="172" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M171" s="2" t="s">
+        <v>1860</v>
+      </c>
+      <c r="N171" s="2" t="s">
+        <v>1861</v>
+      </c>
+    </row>
+    <row r="172" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A172" t="s">
         <v>1142</v>
       </c>
@@ -9805,8 +11947,14 @@
       <c r="J172" s="2" t="s">
         <v>1202</v>
       </c>
-    </row>
-    <row r="173" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M172" s="2" t="s">
+        <v>1731</v>
+      </c>
+      <c r="N172" s="2" t="s">
+        <v>1862</v>
+      </c>
+    </row>
+    <row r="173" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A173" t="s">
         <v>1143</v>
       </c>
@@ -9834,8 +11982,14 @@
       <c r="J173" s="2" t="s">
         <v>436</v>
       </c>
-    </row>
-    <row r="174" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M173" s="2" t="s">
+        <v>1556</v>
+      </c>
+      <c r="N173" s="2" t="s">
+        <v>1543</v>
+      </c>
+    </row>
+    <row r="174" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A174" t="s">
         <v>1144</v>
       </c>
@@ -9866,8 +12020,14 @@
       <c r="L174" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="175" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M174" s="2" t="s">
+        <v>1863</v>
+      </c>
+      <c r="N174" s="2" t="s">
+        <v>1864</v>
+      </c>
+    </row>
+    <row r="175" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A175" t="s">
         <v>1145</v>
       </c>
@@ -9898,8 +12058,14 @@
       <c r="L175" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="176" spans="1:12" x14ac:dyDescent="0.45">
+      <c r="M175" s="2" t="s">
+        <v>1865</v>
+      </c>
+      <c r="N175" s="2" t="s">
+        <v>1866</v>
+      </c>
+    </row>
+    <row r="176" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A176" t="s">
         <v>1146</v>
       </c>
@@ -9930,8 +12096,14 @@
       <c r="L176" t="b">
         <v>1</v>
       </c>
-    </row>
-    <row r="177" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="M176" s="2" t="s">
+        <v>1832</v>
+      </c>
+      <c r="N176" s="2" t="s">
+        <v>1867</v>
+      </c>
+    </row>
+    <row r="177" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A177" t="s">
         <v>1147</v>
       </c>
@@ -9959,8 +12131,14 @@
       <c r="J177" s="2" t="s">
         <v>436</v>
       </c>
-    </row>
-    <row r="178" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="M177" s="2" t="s">
+        <v>1868</v>
+      </c>
+      <c r="N177" s="2" t="s">
+        <v>1869</v>
+      </c>
+    </row>
+    <row r="178" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A178" t="s">
         <v>1148</v>
       </c>
@@ -9988,8 +12166,14 @@
       <c r="J178" s="2" t="s">
         <v>1206</v>
       </c>
-    </row>
-    <row r="179" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="M178" s="2" t="s">
+        <v>1870</v>
+      </c>
+      <c r="N178" s="2" t="s">
+        <v>1872</v>
+      </c>
+    </row>
+    <row r="179" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A179" t="s">
         <v>29</v>
       </c>
@@ -10017,8 +12201,14 @@
       <c r="J179" s="2" t="s">
         <v>35</v>
       </c>
-    </row>
-    <row r="180" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="M179" s="2" t="s">
+        <v>1873</v>
+      </c>
+      <c r="N179" s="2" t="s">
+        <v>1874</v>
+      </c>
+    </row>
+    <row r="180" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A180" t="s">
         <v>1149</v>
       </c>
@@ -10043,8 +12233,14 @@
       <c r="J180" s="2" t="s">
         <v>1207</v>
       </c>
-    </row>
-    <row r="181" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="M180" s="2" t="s">
+        <v>1686</v>
+      </c>
+      <c r="N180" s="2" t="s">
+        <v>1875</v>
+      </c>
+    </row>
+    <row r="181" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A181" t="s">
         <v>1150</v>
       </c>
@@ -10072,8 +12268,14 @@
       <c r="J181" s="2" t="s">
         <v>1208</v>
       </c>
-    </row>
-    <row r="182" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="M181" s="2" t="s">
+        <v>1876</v>
+      </c>
+      <c r="N181" s="2" t="s">
+        <v>1543</v>
+      </c>
+    </row>
+    <row r="182" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A182" t="s">
         <v>1151</v>
       </c>
@@ -10098,8 +12300,14 @@
       <c r="J182" s="2" t="s">
         <v>186</v>
       </c>
-    </row>
-    <row r="183" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="M182" s="2" t="s">
+        <v>1878</v>
+      </c>
+      <c r="N182" s="2" t="s">
+        <v>1879</v>
+      </c>
+    </row>
+    <row r="183" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A183" t="s">
         <v>1152</v>
       </c>
@@ -10127,8 +12335,14 @@
       <c r="J183" s="2" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="184" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="M183" s="2" t="s">
+        <v>1667</v>
+      </c>
+      <c r="N183" s="2" t="s">
+        <v>1880</v>
+      </c>
+    </row>
+    <row r="184" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A184" t="s">
         <v>1153</v>
       </c>
@@ -10156,8 +12370,14 @@
       <c r="J184" s="2" t="s">
         <v>179</v>
       </c>
-    </row>
-    <row r="185" spans="1:11" x14ac:dyDescent="0.45">
+      <c r="M184" s="2" t="s">
+        <v>1881</v>
+      </c>
+      <c r="N184" s="2" t="s">
+        <v>1882</v>
+      </c>
+    </row>
+    <row r="185" spans="1:14" x14ac:dyDescent="0.45">
       <c r="A185" t="s">
         <v>36</v>
       </c>
@@ -10184,6 +12404,12 @@
       </c>
       <c r="K185" t="b">
         <v>1</v>
+      </c>
+      <c r="M185" s="2" t="s">
+        <v>1883</v>
+      </c>
+      <c r="N185" s="2" t="s">
+        <v>1543</v>
       </c>
     </row>
   </sheetData>
@@ -10196,6 +12422,428 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{445C98DF-AF88-42FF-A8A5-2AB8831F51CC}">
+  <dimension ref="A1:B60"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <cols>
+    <col min="1" max="1" width="22.1328125" customWidth="1"/>
+    <col min="2" max="2" width="16.9296875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A1" s="1" t="s">
+        <v>1513</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1514</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
+        <v>1519</v>
+      </c>
+      <c r="B2" t="s">
+        <v>1510</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A3" t="s">
+        <v>1520</v>
+      </c>
+      <c r="B3" t="s">
+        <v>1525</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A4" t="s">
+        <v>1521</v>
+      </c>
+      <c r="B4" t="s">
+        <v>1526</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A5" t="s">
+        <v>1522</v>
+      </c>
+      <c r="B5" t="s">
+        <v>1527</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A6" t="s">
+        <v>1523</v>
+      </c>
+      <c r="B6" t="s">
+        <v>1534</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A7" t="s">
+        <v>1524</v>
+      </c>
+      <c r="B7" t="s">
+        <v>1535</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A8" t="s">
+        <v>1529</v>
+      </c>
+      <c r="B8" t="s">
+        <v>1538</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A9" t="s">
+        <v>1337</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>1541</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A10" t="s">
+        <v>1532</v>
+      </c>
+      <c r="B10" t="s">
+        <v>1543</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A11" t="s">
+        <v>1533</v>
+      </c>
+      <c r="B11" t="s">
+        <v>1544</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A12" t="s">
+        <v>1539</v>
+      </c>
+      <c r="B12" t="s">
+        <v>1550</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A13" t="s">
+        <v>1547</v>
+      </c>
+      <c r="B13" t="s">
+        <v>1552</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A14" t="s">
+        <v>1551</v>
+      </c>
+      <c r="B14" t="s">
+        <v>1553</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A15" t="s">
+        <v>1558</v>
+      </c>
+      <c r="B15" t="s">
+        <v>1572</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A16" t="s">
+        <v>1559</v>
+      </c>
+      <c r="B16" t="s">
+        <v>1576</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A17" t="s">
+        <v>1563</v>
+      </c>
+      <c r="B17" t="s">
+        <v>1580</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A18" t="s">
+        <v>1564</v>
+      </c>
+      <c r="B18" t="s">
+        <v>1581</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A19" t="s">
+        <v>1566</v>
+      </c>
+      <c r="B19" t="s">
+        <v>1582</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A20" t="s">
+        <v>1569</v>
+      </c>
+      <c r="B20" t="s">
+        <v>1585</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A21" t="s">
+        <v>1579</v>
+      </c>
+      <c r="B21" t="s">
+        <v>1603</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A22" t="s">
+        <v>1588</v>
+      </c>
+      <c r="B22" t="s">
+        <v>1634</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A23" t="s">
+        <v>1589</v>
+      </c>
+      <c r="B23" t="s">
+        <v>1635</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A24" t="s">
+        <v>1593</v>
+      </c>
+      <c r="B24" t="s">
+        <v>1659</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A25" t="s">
+        <v>1594</v>
+      </c>
+      <c r="B25" t="s">
+        <v>1661</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A26" t="s">
+        <v>1601</v>
+      </c>
+      <c r="B26" t="s">
+        <v>1705</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A27" t="s">
+        <v>1602</v>
+      </c>
+      <c r="B27" t="s">
+        <v>1714</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A28" t="s">
+        <v>1606</v>
+      </c>
+      <c r="B28" t="s">
+        <v>1716</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A29" t="s">
+        <v>1611</v>
+      </c>
+      <c r="B29" t="s">
+        <v>1721</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A30" t="s">
+        <v>1625</v>
+      </c>
+      <c r="B30" t="s">
+        <v>1728</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A31" t="s">
+        <v>1629</v>
+      </c>
+      <c r="B31" t="s">
+        <v>1747</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A32" t="s">
+        <v>1638</v>
+      </c>
+      <c r="B32" t="s">
+        <v>1754</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A33" t="s">
+        <v>1640</v>
+      </c>
+      <c r="B33" t="s">
+        <v>1767</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A34" t="s">
+        <v>1643</v>
+      </c>
+      <c r="B34" t="s">
+        <v>1801</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A35" t="s">
+        <v>1645</v>
+      </c>
+      <c r="B35" t="s">
+        <v>1805</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A36" t="s">
+        <v>1655</v>
+      </c>
+      <c r="B36" t="s">
+        <v>1828</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A37" t="s">
+        <v>1335</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A38" t="s">
+        <v>1665</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A39" t="s">
+        <v>1671</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A40" t="s">
+        <v>1692</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A41" t="s">
+        <v>1735</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A42" t="s">
+        <v>1739</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A43" t="s">
+        <v>1743</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A44" t="s">
+        <v>1744</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A45" t="s">
+        <v>1541</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A46" t="s">
+        <v>1758</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A47" t="s">
+        <v>1759</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A48" t="s">
+        <v>1766</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A49" t="s">
+        <v>1771</v>
+      </c>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A50" t="s">
+        <v>1779</v>
+      </c>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A51" t="s">
+        <v>1783</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A52" t="s">
+        <v>1788</v>
+      </c>
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A53" t="s">
+        <v>1790</v>
+      </c>
+    </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A54" t="s">
+        <v>1796</v>
+      </c>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A55" t="s">
+        <v>1820</v>
+      </c>
+    </row>
+    <row r="56" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A56" t="s">
+        <v>1825</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A57" t="s">
+        <v>1828</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A58" t="s">
+        <v>1850</v>
+      </c>
+    </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A59" t="s">
+        <v>1871</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A60" t="s">
+        <v>1877</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1BC60D8-44F3-478D-BCC0-4752624457AE}">
   <dimension ref="A1:F24"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -10625,7 +13273,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84E3BB0D-5578-4069-B1C9-C3864EB2A429}">
   <dimension ref="A1:G553"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -20050,7 +22698,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{494C60D6-2426-4CE0-9CA4-43EAAA3DD51B}">
   <dimension ref="A1:F26"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -20589,7 +23237,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32F3CD10-C054-4484-ABE2-D426F834FC22}">
   <dimension ref="A1:E67"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
@@ -21545,7 +24193,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{931309AC-3B5D-4169-8BD3-83BC320E154C}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>

</xml_diff>

<commit_message>
added all master images, still need to do ommand seals though
</commit_message>
<xml_diff>
--- a/data/Fate-Spreadsheet.xlsx
+++ b/data/Fate-Spreadsheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pixel\Documents\Projects\Fate-Wiki\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6975E217-4937-4962-9F68-2043D1A69F68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B248AF4-BF86-482E-9932-96EE6A1D4728}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" xr2:uid="{B05E798F-9EF6-4508-A0A4-311D06661AED}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" firstSheet="2" activeTab="5" xr2:uid="{B05E798F-9EF6-4508-A0A4-311D06661AED}"/>
   </bookViews>
   <sheets>
     <sheet name="Servants" sheetId="1" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4216" uniqueCount="1884">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4219" uniqueCount="1886">
   <si>
     <t>servant_id</t>
   </si>
@@ -5697,6 +5697,12 @@
   </si>
   <si>
     <t>Kingmaking,VP Gain,Power Reduction</t>
+  </si>
+  <si>
+    <t>has_attack_cards</t>
+  </si>
+  <si>
+    <t>has_abilities</t>
   </si>
 </sst>
 </file>
@@ -23239,16 +23245,17 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32F3CD10-C054-4484-ABE2-D426F834FC22}">
-  <dimension ref="A1:E67"/>
+  <dimension ref="A1:G67"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="13.3984375" customWidth="1"/>
     <col min="2" max="3" width="26" customWidth="1"/>
-    <col min="4" max="4" width="20.46484375" customWidth="1"/>
-    <col min="5" max="5" width="14.6640625" customWidth="1"/>
+    <col min="4" max="5" width="20.46484375" customWidth="1"/>
+    <col min="6" max="6" width="14.6640625" customWidth="1"/>
+    <col min="7" max="7" width="11.46484375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>1263</v>
       </c>
@@ -23261,9 +23268,17 @@
       <c r="D1" s="1" t="s">
         <v>1331</v>
       </c>
-      <c r="E1" s="1"/>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E1" s="1" t="s">
+        <v>1885</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>1884</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>1466</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>1264</v>
       </c>
@@ -23276,8 +23291,11 @@
       <c r="D2" t="s">
         <v>1333</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>1265</v>
       </c>
@@ -23290,8 +23308,14 @@
       <c r="D3" t="s">
         <v>1334</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E3" t="b">
+        <v>1</v>
+      </c>
+      <c r="F3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>1266</v>
       </c>
@@ -23304,8 +23328,11 @@
       <c r="D4" t="s">
         <v>1335</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>1267</v>
       </c>
@@ -23318,8 +23345,11 @@
       <c r="D5" t="s">
         <v>1336</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>1268</v>
       </c>
@@ -23332,8 +23362,11 @@
       <c r="D6" t="s">
         <v>1335</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>1269</v>
       </c>
@@ -23346,8 +23379,11 @@
       <c r="D7" t="s">
         <v>1337</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F7" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>1270</v>
       </c>
@@ -23360,8 +23396,11 @@
       <c r="D8" t="s">
         <v>1337</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E8" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>1271</v>
       </c>
@@ -23374,8 +23413,11 @@
       <c r="D9" t="s">
         <v>1335</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>1272</v>
       </c>
@@ -23389,7 +23431,7 @@
         <v>1337</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>1273</v>
       </c>
@@ -23402,8 +23444,14 @@
       <c r="D11" t="s">
         <v>1337</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E11" t="b">
+        <v>1</v>
+      </c>
+      <c r="F11" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>1274</v>
       </c>
@@ -23416,8 +23464,11 @@
       <c r="D12" t="s">
         <v>1337</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="E12" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>1275</v>
       </c>
@@ -23431,7 +23482,7 @@
         <v>1333</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
         <v>1276</v>
       </c>
@@ -23444,8 +23495,11 @@
       <c r="D14" t="s">
         <v>1333</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="F14" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
         <v>1277</v>
       </c>
@@ -23459,7 +23513,7 @@
         <v>1335</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
         <v>1278</v>
       </c>
@@ -23472,8 +23526,14 @@
       <c r="D16" t="s">
         <v>1337</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E16" t="b">
+        <v>1</v>
+      </c>
+      <c r="F16" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
         <v>1279</v>
       </c>
@@ -23486,8 +23546,11 @@
       <c r="D17" t="s">
         <v>1335</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E17" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
         <v>1280</v>
       </c>
@@ -23501,7 +23564,7 @@
         <v>1334</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
         <v>1281</v>
       </c>
@@ -23514,8 +23577,11 @@
       <c r="D19" t="s">
         <v>1333</v>
       </c>
-    </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="F19" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
         <v>1282</v>
       </c>
@@ -23528,8 +23594,11 @@
       <c r="D20" t="s">
         <v>1335</v>
       </c>
-    </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E20" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
         <v>1283</v>
       </c>
@@ -23542,8 +23611,11 @@
       <c r="D21" t="s">
         <v>1333</v>
       </c>
-    </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E21" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
         <v>1284</v>
       </c>
@@ -23556,8 +23628,11 @@
       <c r="D22" t="s">
         <v>1334</v>
       </c>
-    </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="F22" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
         <v>1285</v>
       </c>
@@ -23570,8 +23645,11 @@
       <c r="D23" t="s">
         <v>1337</v>
       </c>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E23" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
         <v>1286</v>
       </c>
@@ -23584,8 +23662,11 @@
       <c r="D24" t="s">
         <v>1333</v>
       </c>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E24" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
         <v>1287</v>
       </c>
@@ -23599,7 +23680,7 @@
         <v>1333</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
         <v>1288</v>
       </c>
@@ -23612,8 +23693,11 @@
       <c r="D26" t="s">
         <v>1337</v>
       </c>
-    </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E26" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
         <v>1289</v>
       </c>
@@ -23627,7 +23711,7 @@
         <v>1334</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
         <v>1290</v>
       </c>
@@ -23640,8 +23724,17 @@
       <c r="D28" t="s">
         <v>1333</v>
       </c>
-    </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="E28" t="b">
+        <v>1</v>
+      </c>
+      <c r="F28" t="b">
+        <v>1</v>
+      </c>
+      <c r="G28" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
         <v>1291</v>
       </c>
@@ -23655,7 +23748,7 @@
         <v>1336</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
         <v>1292</v>
       </c>
@@ -23669,7 +23762,7 @@
         <v>1334</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A31" t="s">
         <v>1293</v>
       </c>
@@ -23683,7 +23776,7 @@
         <v>1335</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A32" t="s">
         <v>1294</v>
       </c>
@@ -24190,6 +24283,7 @@
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
fixed json to include traits and traitslist
</commit_message>
<xml_diff>
--- a/data/Fate-Spreadsheet.xlsx
+++ b/data/Fate-Spreadsheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pixel\Documents\Projects\Fate-Wiki\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6FEAF3F0-9A7B-4665-AFC7-7E30F826BAAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E5DAD16-3B98-4A73-8020-619EA4DDD7CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" firstSheet="2" activeTab="2" xr2:uid="{B05E798F-9EF6-4508-A0A4-311D06661AED}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" firstSheet="1" activeTab="1" xr2:uid="{B05E798F-9EF6-4508-A0A4-311D06661AED}"/>
   </bookViews>
   <sheets>
     <sheet name="Servants" sheetId="1" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4218" uniqueCount="1885">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4219" uniqueCount="1885">
   <si>
     <t>servant_id</t>
   </si>
@@ -12426,7 +12426,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{445C98DF-AF88-42FF-A8A5-2AB8831F51CC}">
-  <dimension ref="A1:B60"/>
+  <dimension ref="A1:B61"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="22.1328125" customWidth="1"/>
@@ -12839,6 +12839,11 @@
     <row r="60" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A60" t="s">
         <v>1877</v>
+      </c>
+    </row>
+    <row r="61" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A61" t="s">
+        <v>1534</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
worked on master modals
</commit_message>
<xml_diff>
--- a/data/Fate-Spreadsheet.xlsx
+++ b/data/Fate-Spreadsheet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Important\Python\Fate-Wiki\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE9E610C-D5D3-4347-8319-DA44D04AEDD4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AECEEA88-4C6A-4D9C-BF5B-579B066E645F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="7" xr2:uid="{B05E798F-9EF6-4508-A0A4-311D06661AED}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="2" activeTab="7" xr2:uid="{B05E798F-9EF6-4508-A0A4-311D06661AED}"/>
   </bookViews>
   <sheets>
     <sheet name="Servants" sheetId="1" r:id="rId1"/>
@@ -20,8 +20,8 @@
     <sheet name="Servant Misc Cards" sheetId="7" r:id="rId5"/>
     <sheet name="Masters" sheetId="5" r:id="rId6"/>
     <sheet name="Master Abilities" sheetId="6" r:id="rId7"/>
-    <sheet name="Master Ascensions" sheetId="10" r:id="rId8"/>
-    <sheet name="Master Assets" sheetId="9" r:id="rId9"/>
+    <sheet name="Master Assets" sheetId="9" r:id="rId8"/>
+    <sheet name="Master Ascensions" sheetId="10" r:id="rId9"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -47,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5761" uniqueCount="2507">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5762" uniqueCount="2507">
   <si>
     <t>servant_id</t>
   </si>
@@ -25700,7 +25700,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{32F3CD10-C054-4484-ABE2-D426F834FC22}">
-  <dimension ref="A1:J67"/>
+  <dimension ref="A1:K67"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.42578125" customWidth="1"/>
@@ -25711,9 +25711,10 @@
     <col min="8" max="8" width="19.85546875" customWidth="1"/>
     <col min="9" max="9" width="16" customWidth="1"/>
     <col min="10" max="10" width="13.140625" customWidth="1"/>
+    <col min="11" max="11" width="13.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>1263</v>
       </c>
@@ -25744,8 +25745,11 @@
       <c r="J1" s="1" t="s">
         <v>1887</v>
       </c>
-    </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="K1" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1264</v>
       </c>
@@ -25762,7 +25766,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>1265</v>
       </c>
@@ -25779,7 +25783,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>1266</v>
       </c>
@@ -25796,7 +25800,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>1267</v>
       </c>
@@ -25813,7 +25817,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>1268</v>
       </c>
@@ -25830,7 +25834,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>1269</v>
       </c>
@@ -25847,7 +25851,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>1270</v>
       </c>
@@ -25864,7 +25868,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>1271</v>
       </c>
@@ -25881,7 +25885,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>1272</v>
       </c>
@@ -25895,7 +25899,7 @@
         <v>1337</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>1273</v>
       </c>
@@ -25912,7 +25916,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>1274</v>
       </c>
@@ -25929,7 +25933,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>1275</v>
       </c>
@@ -25943,7 +25947,7 @@
         <v>1333</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>1276</v>
       </c>
@@ -25960,7 +25964,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>1277</v>
       </c>
@@ -25974,7 +25978,7 @@
         <v>1335</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>1278</v>
       </c>
@@ -30163,6 +30167,1302 @@
 </file>
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{01AAAE8C-814F-43DB-A5DB-B841E00BE266}">
+  <dimension ref="A1:F64"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12.5703125" customWidth="1"/>
+    <col min="2" max="2" width="24.5703125" customWidth="1"/>
+    <col min="3" max="5" width="20.28515625" customWidth="1"/>
+    <col min="6" max="6" width="11.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>1263</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1330</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>2150</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>1467</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>1291</v>
+      </c>
+      <c r="B2" t="s">
+        <v>1362</v>
+      </c>
+      <c r="C2" t="s">
+        <v>2086</v>
+      </c>
+      <c r="D2" t="s">
+        <v>2087</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2" t="s">
+        <v>1503</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>1291</v>
+      </c>
+      <c r="B3" t="s">
+        <v>1362</v>
+      </c>
+      <c r="C3" t="s">
+        <v>2088</v>
+      </c>
+      <c r="D3" t="s">
+        <v>2089</v>
+      </c>
+      <c r="E3">
+        <v>2</v>
+      </c>
+      <c r="F3" t="s">
+        <v>1503</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>1291</v>
+      </c>
+      <c r="B4" t="s">
+        <v>1362</v>
+      </c>
+      <c r="C4" t="s">
+        <v>2090</v>
+      </c>
+      <c r="D4" t="s">
+        <v>2091</v>
+      </c>
+      <c r="E4">
+        <v>3</v>
+      </c>
+      <c r="F4" t="s">
+        <v>1503</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>1291</v>
+      </c>
+      <c r="B5" t="s">
+        <v>1362</v>
+      </c>
+      <c r="C5" t="s">
+        <v>2092</v>
+      </c>
+      <c r="D5" t="s">
+        <v>2093</v>
+      </c>
+      <c r="E5">
+        <v>4</v>
+      </c>
+      <c r="F5" t="s">
+        <v>1503</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>1291</v>
+      </c>
+      <c r="B6" t="s">
+        <v>1362</v>
+      </c>
+      <c r="C6" t="s">
+        <v>2094</v>
+      </c>
+      <c r="D6" t="s">
+        <v>2096</v>
+      </c>
+      <c r="E6">
+        <v>5</v>
+      </c>
+      <c r="F6" t="s">
+        <v>1503</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>1291</v>
+      </c>
+      <c r="B7" t="s">
+        <v>1362</v>
+      </c>
+      <c r="C7" t="s">
+        <v>2095</v>
+      </c>
+      <c r="D7" t="s">
+        <v>2097</v>
+      </c>
+      <c r="E7">
+        <v>6</v>
+      </c>
+      <c r="F7" t="s">
+        <v>1503</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>1302</v>
+      </c>
+      <c r="B8" t="s">
+        <v>1374</v>
+      </c>
+      <c r="C8" t="s">
+        <v>2151</v>
+      </c>
+      <c r="D8" t="s">
+        <v>2165</v>
+      </c>
+      <c r="E8">
+        <v>1</v>
+      </c>
+      <c r="F8" t="s">
+        <v>1949</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>1302</v>
+      </c>
+      <c r="B9" t="s">
+        <v>1374</v>
+      </c>
+      <c r="C9" t="s">
+        <v>1333</v>
+      </c>
+      <c r="D9" t="s">
+        <v>2166</v>
+      </c>
+      <c r="E9">
+        <v>2</v>
+      </c>
+      <c r="F9" t="s">
+        <v>1949</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>1302</v>
+      </c>
+      <c r="B10" t="s">
+        <v>1374</v>
+      </c>
+      <c r="C10" t="s">
+        <v>2152</v>
+      </c>
+      <c r="D10" t="s">
+        <v>2167</v>
+      </c>
+      <c r="E10">
+        <v>3</v>
+      </c>
+      <c r="F10" t="s">
+        <v>1949</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>1302</v>
+      </c>
+      <c r="B11" t="s">
+        <v>1374</v>
+      </c>
+      <c r="C11" t="s">
+        <v>2153</v>
+      </c>
+      <c r="D11" t="s">
+        <v>2168</v>
+      </c>
+      <c r="E11">
+        <v>4</v>
+      </c>
+      <c r="F11" t="s">
+        <v>1949</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>1302</v>
+      </c>
+      <c r="B12" t="s">
+        <v>1374</v>
+      </c>
+      <c r="C12" t="s">
+        <v>2154</v>
+      </c>
+      <c r="D12" t="s">
+        <v>2169</v>
+      </c>
+      <c r="E12">
+        <v>5</v>
+      </c>
+      <c r="F12" t="s">
+        <v>1949</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>1302</v>
+      </c>
+      <c r="B13" t="s">
+        <v>1374</v>
+      </c>
+      <c r="C13" t="s">
+        <v>2155</v>
+      </c>
+      <c r="D13" t="s">
+        <v>2170</v>
+      </c>
+      <c r="E13">
+        <v>6</v>
+      </c>
+      <c r="F13" t="s">
+        <v>1949</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>1302</v>
+      </c>
+      <c r="B14" t="s">
+        <v>1374</v>
+      </c>
+      <c r="C14" t="s">
+        <v>2156</v>
+      </c>
+      <c r="D14" t="s">
+        <v>2171</v>
+      </c>
+      <c r="E14">
+        <v>7</v>
+      </c>
+      <c r="F14" t="s">
+        <v>1949</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>1302</v>
+      </c>
+      <c r="B15" t="s">
+        <v>1374</v>
+      </c>
+      <c r="C15" t="s">
+        <v>2157</v>
+      </c>
+      <c r="D15" t="s">
+        <v>2179</v>
+      </c>
+      <c r="E15">
+        <v>8</v>
+      </c>
+      <c r="F15" t="s">
+        <v>1949</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>1302</v>
+      </c>
+      <c r="B16" t="s">
+        <v>1374</v>
+      </c>
+      <c r="C16" t="s">
+        <v>2158</v>
+      </c>
+      <c r="D16" t="s">
+        <v>2172</v>
+      </c>
+      <c r="E16">
+        <v>9</v>
+      </c>
+      <c r="F16" t="s">
+        <v>1949</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>1302</v>
+      </c>
+      <c r="B17" t="s">
+        <v>1374</v>
+      </c>
+      <c r="C17" t="s">
+        <v>2159</v>
+      </c>
+      <c r="D17" t="s">
+        <v>2178</v>
+      </c>
+      <c r="E17">
+        <v>10</v>
+      </c>
+      <c r="F17" t="s">
+        <v>1949</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>1302</v>
+      </c>
+      <c r="B18" t="s">
+        <v>1374</v>
+      </c>
+      <c r="C18" t="s">
+        <v>2160</v>
+      </c>
+      <c r="D18" t="s">
+        <v>2173</v>
+      </c>
+      <c r="E18">
+        <v>11</v>
+      </c>
+      <c r="F18" t="s">
+        <v>1949</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>1302</v>
+      </c>
+      <c r="B19" t="s">
+        <v>1374</v>
+      </c>
+      <c r="C19" t="s">
+        <v>2161</v>
+      </c>
+      <c r="D19" t="s">
+        <v>2174</v>
+      </c>
+      <c r="E19">
+        <v>12</v>
+      </c>
+      <c r="F19" t="s">
+        <v>1949</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>1302</v>
+      </c>
+      <c r="B20" t="s">
+        <v>1374</v>
+      </c>
+      <c r="C20" t="s">
+        <v>2162</v>
+      </c>
+      <c r="D20" t="s">
+        <v>2175</v>
+      </c>
+      <c r="E20">
+        <v>13</v>
+      </c>
+      <c r="F20" t="s">
+        <v>1949</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>1302</v>
+      </c>
+      <c r="B21" t="s">
+        <v>1374</v>
+      </c>
+      <c r="C21" t="s">
+        <v>2163</v>
+      </c>
+      <c r="D21" t="s">
+        <v>2176</v>
+      </c>
+      <c r="E21">
+        <v>14</v>
+      </c>
+      <c r="F21" t="s">
+        <v>1949</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" t="s">
+        <v>1302</v>
+      </c>
+      <c r="B22" t="s">
+        <v>1374</v>
+      </c>
+      <c r="C22" t="s">
+        <v>2164</v>
+      </c>
+      <c r="D22" t="s">
+        <v>2177</v>
+      </c>
+      <c r="E22">
+        <v>15</v>
+      </c>
+      <c r="F22" t="s">
+        <v>1949</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>1304</v>
+      </c>
+      <c r="B23" t="s">
+        <v>1376</v>
+      </c>
+      <c r="C23" t="s">
+        <v>2194</v>
+      </c>
+      <c r="D23" t="s">
+        <v>2207</v>
+      </c>
+      <c r="E23">
+        <v>1</v>
+      </c>
+      <c r="F23" t="s">
+        <v>1468</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>1304</v>
+      </c>
+      <c r="B24" t="s">
+        <v>1376</v>
+      </c>
+      <c r="C24" t="s">
+        <v>2195</v>
+      </c>
+      <c r="D24" t="s">
+        <v>2208</v>
+      </c>
+      <c r="E24">
+        <v>2</v>
+      </c>
+      <c r="F24" t="s">
+        <v>1468</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>1304</v>
+      </c>
+      <c r="B25" t="s">
+        <v>1376</v>
+      </c>
+      <c r="C25" t="s">
+        <v>2196</v>
+      </c>
+      <c r="D25" t="s">
+        <v>2209</v>
+      </c>
+      <c r="E25">
+        <v>3</v>
+      </c>
+      <c r="F25" t="s">
+        <v>1468</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>1304</v>
+      </c>
+      <c r="B26" t="s">
+        <v>1376</v>
+      </c>
+      <c r="C26" t="s">
+        <v>2197</v>
+      </c>
+      <c r="D26" t="s">
+        <v>2210</v>
+      </c>
+      <c r="E26">
+        <v>4</v>
+      </c>
+      <c r="F26" t="s">
+        <v>1468</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>1304</v>
+      </c>
+      <c r="B27" t="s">
+        <v>1376</v>
+      </c>
+      <c r="C27" t="s">
+        <v>2198</v>
+      </c>
+      <c r="D27" t="s">
+        <v>2218</v>
+      </c>
+      <c r="E27">
+        <v>5</v>
+      </c>
+      <c r="F27" t="s">
+        <v>1468</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>1304</v>
+      </c>
+      <c r="B28" t="s">
+        <v>1376</v>
+      </c>
+      <c r="C28" t="s">
+        <v>2199</v>
+      </c>
+      <c r="D28" t="s">
+        <v>2211</v>
+      </c>
+      <c r="E28">
+        <v>6</v>
+      </c>
+      <c r="F28" t="s">
+        <v>1468</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>1304</v>
+      </c>
+      <c r="B29" t="s">
+        <v>1376</v>
+      </c>
+      <c r="C29" t="s">
+        <v>2200</v>
+      </c>
+      <c r="D29" t="s">
+        <v>2212</v>
+      </c>
+      <c r="E29">
+        <v>7</v>
+      </c>
+      <c r="F29" t="s">
+        <v>1468</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>1304</v>
+      </c>
+      <c r="B30" t="s">
+        <v>1376</v>
+      </c>
+      <c r="C30" t="s">
+        <v>2201</v>
+      </c>
+      <c r="D30" t="s">
+        <v>2213</v>
+      </c>
+      <c r="E30">
+        <v>8</v>
+      </c>
+      <c r="F30" t="s">
+        <v>1468</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>1304</v>
+      </c>
+      <c r="B31" t="s">
+        <v>1376</v>
+      </c>
+      <c r="C31" t="s">
+        <v>2202</v>
+      </c>
+      <c r="D31" t="s">
+        <v>2214</v>
+      </c>
+      <c r="E31">
+        <v>9</v>
+      </c>
+      <c r="F31" t="s">
+        <v>1949</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>1304</v>
+      </c>
+      <c r="B32" t="s">
+        <v>1376</v>
+      </c>
+      <c r="C32" t="s">
+        <v>2203</v>
+      </c>
+      <c r="D32" t="s">
+        <v>2215</v>
+      </c>
+      <c r="E32">
+        <v>10</v>
+      </c>
+      <c r="F32" t="s">
+        <v>1949</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>1304</v>
+      </c>
+      <c r="B33" t="s">
+        <v>1376</v>
+      </c>
+      <c r="C33" t="s">
+        <v>2204</v>
+      </c>
+      <c r="D33" t="s">
+        <v>2216</v>
+      </c>
+      <c r="E33">
+        <v>11</v>
+      </c>
+      <c r="F33" t="s">
+        <v>1468</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>1304</v>
+      </c>
+      <c r="B34" t="s">
+        <v>1376</v>
+      </c>
+      <c r="C34" t="s">
+        <v>2205</v>
+      </c>
+      <c r="D34" t="s">
+        <v>2219</v>
+      </c>
+      <c r="E34">
+        <v>12</v>
+      </c>
+      <c r="F34" t="s">
+        <v>1949</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>1304</v>
+      </c>
+      <c r="B35" t="s">
+        <v>1376</v>
+      </c>
+      <c r="C35" t="s">
+        <v>2206</v>
+      </c>
+      <c r="D35" t="s">
+        <v>2217</v>
+      </c>
+      <c r="E35">
+        <v>13</v>
+      </c>
+      <c r="F35" t="s">
+        <v>1468</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>1306</v>
+      </c>
+      <c r="B36" t="s">
+        <v>1378</v>
+      </c>
+      <c r="C36" t="s">
+        <v>2226</v>
+      </c>
+      <c r="D36" t="s">
+        <v>2229</v>
+      </c>
+      <c r="E36">
+        <v>1</v>
+      </c>
+      <c r="F36" t="s">
+        <v>1503</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" t="s">
+        <v>1306</v>
+      </c>
+      <c r="B37" t="s">
+        <v>1378</v>
+      </c>
+      <c r="C37" t="s">
+        <v>2227</v>
+      </c>
+      <c r="D37" t="s">
+        <v>2230</v>
+      </c>
+      <c r="E37">
+        <v>2</v>
+      </c>
+      <c r="F37" t="s">
+        <v>1503</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" t="s">
+        <v>1306</v>
+      </c>
+      <c r="B38" t="s">
+        <v>1378</v>
+      </c>
+      <c r="C38" t="s">
+        <v>2228</v>
+      </c>
+      <c r="D38" t="s">
+        <v>2231</v>
+      </c>
+      <c r="E38">
+        <v>3</v>
+      </c>
+      <c r="F38" t="s">
+        <v>1503</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" t="s">
+        <v>1307</v>
+      </c>
+      <c r="B39" t="s">
+        <v>1379</v>
+      </c>
+      <c r="C39" t="s">
+        <v>2238</v>
+      </c>
+      <c r="D39" t="s">
+        <v>2239</v>
+      </c>
+      <c r="E39">
+        <v>1</v>
+      </c>
+      <c r="F39" t="s">
+        <v>1503</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" t="s">
+        <v>1307</v>
+      </c>
+      <c r="B40" t="s">
+        <v>1379</v>
+      </c>
+      <c r="C40" t="s">
+        <v>2240</v>
+      </c>
+      <c r="D40" t="s">
+        <v>2245</v>
+      </c>
+      <c r="E40">
+        <v>2</v>
+      </c>
+      <c r="F40" t="s">
+        <v>1503</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>1307</v>
+      </c>
+      <c r="B41" t="s">
+        <v>1379</v>
+      </c>
+      <c r="C41" t="s">
+        <v>2241</v>
+      </c>
+      <c r="D41" t="s">
+        <v>2244</v>
+      </c>
+      <c r="E41">
+        <v>3</v>
+      </c>
+      <c r="F41" t="s">
+        <v>1503</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>1307</v>
+      </c>
+      <c r="B42" t="s">
+        <v>1379</v>
+      </c>
+      <c r="C42" t="s">
+        <v>2242</v>
+      </c>
+      <c r="D42" t="s">
+        <v>2243</v>
+      </c>
+      <c r="E42">
+        <v>4</v>
+      </c>
+      <c r="F42" t="s">
+        <v>1503</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>1308</v>
+      </c>
+      <c r="B43" t="s">
+        <v>1380</v>
+      </c>
+      <c r="C43" t="s">
+        <v>2254</v>
+      </c>
+      <c r="D43" t="s">
+        <v>2263</v>
+      </c>
+      <c r="E43">
+        <v>1</v>
+      </c>
+      <c r="F43" t="s">
+        <v>1503</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" t="s">
+        <v>1308</v>
+      </c>
+      <c r="B44" t="s">
+        <v>1380</v>
+      </c>
+      <c r="C44" t="s">
+        <v>2255</v>
+      </c>
+      <c r="D44" t="s">
+        <v>2264</v>
+      </c>
+      <c r="E44">
+        <v>2</v>
+      </c>
+      <c r="F44" t="s">
+        <v>1503</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" t="s">
+        <v>1308</v>
+      </c>
+      <c r="B45" t="s">
+        <v>1380</v>
+      </c>
+      <c r="C45" t="s">
+        <v>2256</v>
+      </c>
+      <c r="D45" t="s">
+        <v>2266</v>
+      </c>
+      <c r="E45">
+        <v>3</v>
+      </c>
+      <c r="F45" t="s">
+        <v>1503</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" t="s">
+        <v>1308</v>
+      </c>
+      <c r="B46" t="s">
+        <v>1380</v>
+      </c>
+      <c r="C46" t="s">
+        <v>2257</v>
+      </c>
+      <c r="D46" t="s">
+        <v>2267</v>
+      </c>
+      <c r="E46">
+        <v>4</v>
+      </c>
+      <c r="F46" t="s">
+        <v>1503</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" t="s">
+        <v>1308</v>
+      </c>
+      <c r="B47" t="s">
+        <v>1380</v>
+      </c>
+      <c r="C47" t="s">
+        <v>2258</v>
+      </c>
+      <c r="D47" t="s">
+        <v>2268</v>
+      </c>
+      <c r="E47">
+        <v>5</v>
+      </c>
+      <c r="F47" t="s">
+        <v>1503</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" t="s">
+        <v>1308</v>
+      </c>
+      <c r="B48" t="s">
+        <v>1380</v>
+      </c>
+      <c r="C48" t="s">
+        <v>2259</v>
+      </c>
+      <c r="D48" t="s">
+        <v>2269</v>
+      </c>
+      <c r="E48">
+        <v>6</v>
+      </c>
+      <c r="F48" t="s">
+        <v>1503</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A49" t="s">
+        <v>1308</v>
+      </c>
+      <c r="B49" t="s">
+        <v>1380</v>
+      </c>
+      <c r="C49" t="s">
+        <v>2260</v>
+      </c>
+      <c r="D49" t="s">
+        <v>2270</v>
+      </c>
+      <c r="E49">
+        <v>7</v>
+      </c>
+      <c r="F49" t="s">
+        <v>1503</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A50" t="s">
+        <v>1308</v>
+      </c>
+      <c r="B50" t="s">
+        <v>1380</v>
+      </c>
+      <c r="C50" t="s">
+        <v>2261</v>
+      </c>
+      <c r="D50" t="s">
+        <v>2271</v>
+      </c>
+      <c r="E50">
+        <v>8</v>
+      </c>
+      <c r="F50" t="s">
+        <v>1503</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A51" t="s">
+        <v>1308</v>
+      </c>
+      <c r="B51" t="s">
+        <v>1380</v>
+      </c>
+      <c r="C51" t="s">
+        <v>2262</v>
+      </c>
+      <c r="D51" t="s">
+        <v>2265</v>
+      </c>
+      <c r="E51">
+        <v>9</v>
+      </c>
+      <c r="F51" t="s">
+        <v>1503</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A52" t="s">
+        <v>1309</v>
+      </c>
+      <c r="B52" t="s">
+        <v>1381</v>
+      </c>
+      <c r="C52" t="s">
+        <v>2288</v>
+      </c>
+      <c r="D52" t="s">
+        <v>2295</v>
+      </c>
+      <c r="E52">
+        <v>1</v>
+      </c>
+      <c r="F52" t="s">
+        <v>1503</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A53" t="s">
+        <v>1309</v>
+      </c>
+      <c r="B53" t="s">
+        <v>1381</v>
+      </c>
+      <c r="C53" t="s">
+        <v>2289</v>
+      </c>
+      <c r="D53" t="s">
+        <v>2296</v>
+      </c>
+      <c r="E53">
+        <v>2</v>
+      </c>
+      <c r="F53" t="s">
+        <v>1503</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A54" t="s">
+        <v>1309</v>
+      </c>
+      <c r="B54" t="s">
+        <v>1381</v>
+      </c>
+      <c r="C54" t="s">
+        <v>2290</v>
+      </c>
+      <c r="D54" t="s">
+        <v>2297</v>
+      </c>
+      <c r="E54">
+        <v>3</v>
+      </c>
+      <c r="F54" t="s">
+        <v>1503</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A55" t="s">
+        <v>1309</v>
+      </c>
+      <c r="B55" t="s">
+        <v>1381</v>
+      </c>
+      <c r="C55" t="s">
+        <v>2291</v>
+      </c>
+      <c r="D55" t="s">
+        <v>2300</v>
+      </c>
+      <c r="E55">
+        <v>4</v>
+      </c>
+      <c r="F55" t="s">
+        <v>1503</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A56" t="s">
+        <v>1309</v>
+      </c>
+      <c r="B56" t="s">
+        <v>1381</v>
+      </c>
+      <c r="C56" t="s">
+        <v>2292</v>
+      </c>
+      <c r="D56" t="s">
+        <v>2298</v>
+      </c>
+      <c r="E56">
+        <v>5</v>
+      </c>
+      <c r="F56" t="s">
+        <v>1503</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>1309</v>
+      </c>
+      <c r="B57" t="s">
+        <v>1381</v>
+      </c>
+      <c r="C57" t="s">
+        <v>2293</v>
+      </c>
+      <c r="D57" t="s">
+        <v>2299</v>
+      </c>
+      <c r="E57">
+        <v>6</v>
+      </c>
+      <c r="F57" t="s">
+        <v>1503</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A58" t="s">
+        <v>1309</v>
+      </c>
+      <c r="B58" t="s">
+        <v>1381</v>
+      </c>
+      <c r="C58" t="s">
+        <v>2294</v>
+      </c>
+      <c r="D58" t="s">
+        <v>2301</v>
+      </c>
+      <c r="E58">
+        <v>7</v>
+      </c>
+      <c r="F58" t="s">
+        <v>1503</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A59" t="s">
+        <v>1310</v>
+      </c>
+      <c r="B59" t="s">
+        <v>1382</v>
+      </c>
+      <c r="C59" t="s">
+        <v>2314</v>
+      </c>
+      <c r="D59" t="s">
+        <v>2318</v>
+      </c>
+      <c r="E59">
+        <v>1</v>
+      </c>
+      <c r="F59" t="s">
+        <v>1503</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A60" t="s">
+        <v>1310</v>
+      </c>
+      <c r="B60" t="s">
+        <v>1382</v>
+      </c>
+      <c r="C60" t="s">
+        <v>2315</v>
+      </c>
+      <c r="D60" t="s">
+        <v>2319</v>
+      </c>
+      <c r="E60">
+        <v>2</v>
+      </c>
+      <c r="F60" t="s">
+        <v>1503</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A61" t="s">
+        <v>1310</v>
+      </c>
+      <c r="B61" t="s">
+        <v>1382</v>
+      </c>
+      <c r="C61" t="s">
+        <v>2316</v>
+      </c>
+      <c r="D61" t="s">
+        <v>2320</v>
+      </c>
+      <c r="E61">
+        <v>3</v>
+      </c>
+      <c r="F61" t="s">
+        <v>1503</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A62" t="s">
+        <v>1310</v>
+      </c>
+      <c r="B62" t="s">
+        <v>1382</v>
+      </c>
+      <c r="C62" t="s">
+        <v>2317</v>
+      </c>
+      <c r="D62" t="s">
+        <v>2321</v>
+      </c>
+      <c r="E62">
+        <v>4</v>
+      </c>
+      <c r="F62" t="s">
+        <v>1503</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A63" t="s">
+        <v>1323</v>
+      </c>
+      <c r="B63" t="s">
+        <v>1393</v>
+      </c>
+      <c r="C63" t="s">
+        <v>2439</v>
+      </c>
+      <c r="D63" t="s">
+        <v>2440</v>
+      </c>
+      <c r="E63">
+        <v>1</v>
+      </c>
+      <c r="F63" t="s">
+        <v>1506</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A64" t="s">
+        <v>1326</v>
+      </c>
+      <c r="B64" t="s">
+        <v>1396</v>
+      </c>
+      <c r="C64" t="s">
+        <v>2473</v>
+      </c>
+      <c r="D64" t="s">
+        <v>2474</v>
+      </c>
+      <c r="E64">
+        <v>1</v>
+      </c>
+      <c r="F64" t="s">
+        <v>1503</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F134C8BE-E9AE-4B7A-9200-034BBD6B89FF}">
   <dimension ref="A1:D67"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -31114,1300 +32414,4 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{01AAAE8C-814F-43DB-A5DB-B841E00BE266}">
-  <dimension ref="A1:F64"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="12.5703125" customWidth="1"/>
-    <col min="2" max="2" width="24.5703125" customWidth="1"/>
-    <col min="3" max="5" width="20.28515625" customWidth="1"/>
-    <col min="6" max="6" width="11.140625" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A1" s="1" t="s">
-        <v>1263</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1330</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>44</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>2150</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>1467</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>1291</v>
-      </c>
-      <c r="B2" t="s">
-        <v>1362</v>
-      </c>
-      <c r="C2" t="s">
-        <v>2086</v>
-      </c>
-      <c r="D2" t="s">
-        <v>2087</v>
-      </c>
-      <c r="E2">
-        <v>1</v>
-      </c>
-      <c r="F2" t="s">
-        <v>1503</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>1291</v>
-      </c>
-      <c r="B3" t="s">
-        <v>1362</v>
-      </c>
-      <c r="C3" t="s">
-        <v>2088</v>
-      </c>
-      <c r="D3" t="s">
-        <v>2089</v>
-      </c>
-      <c r="E3">
-        <v>2</v>
-      </c>
-      <c r="F3" t="s">
-        <v>1503</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>1291</v>
-      </c>
-      <c r="B4" t="s">
-        <v>1362</v>
-      </c>
-      <c r="C4" t="s">
-        <v>2090</v>
-      </c>
-      <c r="D4" t="s">
-        <v>2091</v>
-      </c>
-      <c r="E4">
-        <v>3</v>
-      </c>
-      <c r="F4" t="s">
-        <v>1503</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>1291</v>
-      </c>
-      <c r="B5" t="s">
-        <v>1362</v>
-      </c>
-      <c r="C5" t="s">
-        <v>2092</v>
-      </c>
-      <c r="D5" t="s">
-        <v>2093</v>
-      </c>
-      <c r="E5">
-        <v>4</v>
-      </c>
-      <c r="F5" t="s">
-        <v>1503</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>1291</v>
-      </c>
-      <c r="B6" t="s">
-        <v>1362</v>
-      </c>
-      <c r="C6" t="s">
-        <v>2094</v>
-      </c>
-      <c r="D6" t="s">
-        <v>2096</v>
-      </c>
-      <c r="E6">
-        <v>5</v>
-      </c>
-      <c r="F6" t="s">
-        <v>1503</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>1291</v>
-      </c>
-      <c r="B7" t="s">
-        <v>1362</v>
-      </c>
-      <c r="C7" t="s">
-        <v>2095</v>
-      </c>
-      <c r="D7" t="s">
-        <v>2097</v>
-      </c>
-      <c r="E7">
-        <v>6</v>
-      </c>
-      <c r="F7" t="s">
-        <v>1503</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>1302</v>
-      </c>
-      <c r="B8" t="s">
-        <v>1374</v>
-      </c>
-      <c r="C8" t="s">
-        <v>2151</v>
-      </c>
-      <c r="D8" t="s">
-        <v>2165</v>
-      </c>
-      <c r="E8">
-        <v>1</v>
-      </c>
-      <c r="F8" t="s">
-        <v>1949</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>1302</v>
-      </c>
-      <c r="B9" t="s">
-        <v>1374</v>
-      </c>
-      <c r="C9" t="s">
-        <v>1333</v>
-      </c>
-      <c r="D9" t="s">
-        <v>2166</v>
-      </c>
-      <c r="E9">
-        <v>2</v>
-      </c>
-      <c r="F9" t="s">
-        <v>1949</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>1302</v>
-      </c>
-      <c r="B10" t="s">
-        <v>1374</v>
-      </c>
-      <c r="C10" t="s">
-        <v>2152</v>
-      </c>
-      <c r="D10" t="s">
-        <v>2167</v>
-      </c>
-      <c r="E10">
-        <v>3</v>
-      </c>
-      <c r="F10" t="s">
-        <v>1949</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>1302</v>
-      </c>
-      <c r="B11" t="s">
-        <v>1374</v>
-      </c>
-      <c r="C11" t="s">
-        <v>2153</v>
-      </c>
-      <c r="D11" t="s">
-        <v>2168</v>
-      </c>
-      <c r="E11">
-        <v>4</v>
-      </c>
-      <c r="F11" t="s">
-        <v>1949</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>1302</v>
-      </c>
-      <c r="B12" t="s">
-        <v>1374</v>
-      </c>
-      <c r="C12" t="s">
-        <v>2154</v>
-      </c>
-      <c r="D12" t="s">
-        <v>2169</v>
-      </c>
-      <c r="E12">
-        <v>5</v>
-      </c>
-      <c r="F12" t="s">
-        <v>1949</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>1302</v>
-      </c>
-      <c r="B13" t="s">
-        <v>1374</v>
-      </c>
-      <c r="C13" t="s">
-        <v>2155</v>
-      </c>
-      <c r="D13" t="s">
-        <v>2170</v>
-      </c>
-      <c r="E13">
-        <v>6</v>
-      </c>
-      <c r="F13" t="s">
-        <v>1949</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>1302</v>
-      </c>
-      <c r="B14" t="s">
-        <v>1374</v>
-      </c>
-      <c r="C14" t="s">
-        <v>2156</v>
-      </c>
-      <c r="D14" t="s">
-        <v>2171</v>
-      </c>
-      <c r="E14">
-        <v>7</v>
-      </c>
-      <c r="F14" t="s">
-        <v>1949</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>1302</v>
-      </c>
-      <c r="B15" t="s">
-        <v>1374</v>
-      </c>
-      <c r="C15" t="s">
-        <v>2157</v>
-      </c>
-      <c r="D15" t="s">
-        <v>2179</v>
-      </c>
-      <c r="E15">
-        <v>8</v>
-      </c>
-      <c r="F15" t="s">
-        <v>1949</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>1302</v>
-      </c>
-      <c r="B16" t="s">
-        <v>1374</v>
-      </c>
-      <c r="C16" t="s">
-        <v>2158</v>
-      </c>
-      <c r="D16" t="s">
-        <v>2172</v>
-      </c>
-      <c r="E16">
-        <v>9</v>
-      </c>
-      <c r="F16" t="s">
-        <v>1949</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>1302</v>
-      </c>
-      <c r="B17" t="s">
-        <v>1374</v>
-      </c>
-      <c r="C17" t="s">
-        <v>2159</v>
-      </c>
-      <c r="D17" t="s">
-        <v>2178</v>
-      </c>
-      <c r="E17">
-        <v>10</v>
-      </c>
-      <c r="F17" t="s">
-        <v>1949</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>1302</v>
-      </c>
-      <c r="B18" t="s">
-        <v>1374</v>
-      </c>
-      <c r="C18" t="s">
-        <v>2160</v>
-      </c>
-      <c r="D18" t="s">
-        <v>2173</v>
-      </c>
-      <c r="E18">
-        <v>11</v>
-      </c>
-      <c r="F18" t="s">
-        <v>1949</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>1302</v>
-      </c>
-      <c r="B19" t="s">
-        <v>1374</v>
-      </c>
-      <c r="C19" t="s">
-        <v>2161</v>
-      </c>
-      <c r="D19" t="s">
-        <v>2174</v>
-      </c>
-      <c r="E19">
-        <v>12</v>
-      </c>
-      <c r="F19" t="s">
-        <v>1949</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>1302</v>
-      </c>
-      <c r="B20" t="s">
-        <v>1374</v>
-      </c>
-      <c r="C20" t="s">
-        <v>2162</v>
-      </c>
-      <c r="D20" t="s">
-        <v>2175</v>
-      </c>
-      <c r="E20">
-        <v>13</v>
-      </c>
-      <c r="F20" t="s">
-        <v>1949</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>1302</v>
-      </c>
-      <c r="B21" t="s">
-        <v>1374</v>
-      </c>
-      <c r="C21" t="s">
-        <v>2163</v>
-      </c>
-      <c r="D21" t="s">
-        <v>2176</v>
-      </c>
-      <c r="E21">
-        <v>14</v>
-      </c>
-      <c r="F21" t="s">
-        <v>1949</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>1302</v>
-      </c>
-      <c r="B22" t="s">
-        <v>1374</v>
-      </c>
-      <c r="C22" t="s">
-        <v>2164</v>
-      </c>
-      <c r="D22" t="s">
-        <v>2177</v>
-      </c>
-      <c r="E22">
-        <v>15</v>
-      </c>
-      <c r="F22" t="s">
-        <v>1949</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>1304</v>
-      </c>
-      <c r="B23" t="s">
-        <v>1376</v>
-      </c>
-      <c r="C23" t="s">
-        <v>2194</v>
-      </c>
-      <c r="D23" t="s">
-        <v>2207</v>
-      </c>
-      <c r="E23">
-        <v>1</v>
-      </c>
-      <c r="F23" t="s">
-        <v>1468</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>1304</v>
-      </c>
-      <c r="B24" t="s">
-        <v>1376</v>
-      </c>
-      <c r="C24" t="s">
-        <v>2195</v>
-      </c>
-      <c r="D24" t="s">
-        <v>2208</v>
-      </c>
-      <c r="E24">
-        <v>2</v>
-      </c>
-      <c r="F24" t="s">
-        <v>1468</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>1304</v>
-      </c>
-      <c r="B25" t="s">
-        <v>1376</v>
-      </c>
-      <c r="C25" t="s">
-        <v>2196</v>
-      </c>
-      <c r="D25" t="s">
-        <v>2209</v>
-      </c>
-      <c r="E25">
-        <v>3</v>
-      </c>
-      <c r="F25" t="s">
-        <v>1468</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>1304</v>
-      </c>
-      <c r="B26" t="s">
-        <v>1376</v>
-      </c>
-      <c r="C26" t="s">
-        <v>2197</v>
-      </c>
-      <c r="D26" t="s">
-        <v>2210</v>
-      </c>
-      <c r="E26">
-        <v>4</v>
-      </c>
-      <c r="F26" t="s">
-        <v>1468</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>1304</v>
-      </c>
-      <c r="B27" t="s">
-        <v>1376</v>
-      </c>
-      <c r="C27" t="s">
-        <v>2198</v>
-      </c>
-      <c r="D27" t="s">
-        <v>2218</v>
-      </c>
-      <c r="E27">
-        <v>5</v>
-      </c>
-      <c r="F27" t="s">
-        <v>1468</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>1304</v>
-      </c>
-      <c r="B28" t="s">
-        <v>1376</v>
-      </c>
-      <c r="C28" t="s">
-        <v>2199</v>
-      </c>
-      <c r="D28" t="s">
-        <v>2211</v>
-      </c>
-      <c r="E28">
-        <v>6</v>
-      </c>
-      <c r="F28" t="s">
-        <v>1468</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>1304</v>
-      </c>
-      <c r="B29" t="s">
-        <v>1376</v>
-      </c>
-      <c r="C29" t="s">
-        <v>2200</v>
-      </c>
-      <c r="D29" t="s">
-        <v>2212</v>
-      </c>
-      <c r="E29">
-        <v>7</v>
-      </c>
-      <c r="F29" t="s">
-        <v>1468</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>1304</v>
-      </c>
-      <c r="B30" t="s">
-        <v>1376</v>
-      </c>
-      <c r="C30" t="s">
-        <v>2201</v>
-      </c>
-      <c r="D30" t="s">
-        <v>2213</v>
-      </c>
-      <c r="E30">
-        <v>8</v>
-      </c>
-      <c r="F30" t="s">
-        <v>1468</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>1304</v>
-      </c>
-      <c r="B31" t="s">
-        <v>1376</v>
-      </c>
-      <c r="C31" t="s">
-        <v>2202</v>
-      </c>
-      <c r="D31" t="s">
-        <v>2214</v>
-      </c>
-      <c r="E31">
-        <v>9</v>
-      </c>
-      <c r="F31" t="s">
-        <v>1949</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>1304</v>
-      </c>
-      <c r="B32" t="s">
-        <v>1376</v>
-      </c>
-      <c r="C32" t="s">
-        <v>2203</v>
-      </c>
-      <c r="D32" t="s">
-        <v>2215</v>
-      </c>
-      <c r="E32">
-        <v>10</v>
-      </c>
-      <c r="F32" t="s">
-        <v>1949</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>1304</v>
-      </c>
-      <c r="B33" t="s">
-        <v>1376</v>
-      </c>
-      <c r="C33" t="s">
-        <v>2204</v>
-      </c>
-      <c r="D33" t="s">
-        <v>2216</v>
-      </c>
-      <c r="E33">
-        <v>11</v>
-      </c>
-      <c r="F33" t="s">
-        <v>1468</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>1304</v>
-      </c>
-      <c r="B34" t="s">
-        <v>1376</v>
-      </c>
-      <c r="C34" t="s">
-        <v>2205</v>
-      </c>
-      <c r="D34" t="s">
-        <v>2219</v>
-      </c>
-      <c r="E34">
-        <v>12</v>
-      </c>
-      <c r="F34" t="s">
-        <v>1949</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>1304</v>
-      </c>
-      <c r="B35" t="s">
-        <v>1376</v>
-      </c>
-      <c r="C35" t="s">
-        <v>2206</v>
-      </c>
-      <c r="D35" t="s">
-        <v>2217</v>
-      </c>
-      <c r="E35">
-        <v>13</v>
-      </c>
-      <c r="F35" t="s">
-        <v>1468</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>1306</v>
-      </c>
-      <c r="B36" t="s">
-        <v>1378</v>
-      </c>
-      <c r="C36" t="s">
-        <v>2226</v>
-      </c>
-      <c r="D36" t="s">
-        <v>2229</v>
-      </c>
-      <c r="E36">
-        <v>1</v>
-      </c>
-      <c r="F36" t="s">
-        <v>1503</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>1306</v>
-      </c>
-      <c r="B37" t="s">
-        <v>1378</v>
-      </c>
-      <c r="C37" t="s">
-        <v>2227</v>
-      </c>
-      <c r="D37" t="s">
-        <v>2230</v>
-      </c>
-      <c r="E37">
-        <v>2</v>
-      </c>
-      <c r="F37" t="s">
-        <v>1503</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>1306</v>
-      </c>
-      <c r="B38" t="s">
-        <v>1378</v>
-      </c>
-      <c r="C38" t="s">
-        <v>2228</v>
-      </c>
-      <c r="D38" t="s">
-        <v>2231</v>
-      </c>
-      <c r="E38">
-        <v>3</v>
-      </c>
-      <c r="F38" t="s">
-        <v>1503</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
-        <v>1307</v>
-      </c>
-      <c r="B39" t="s">
-        <v>1379</v>
-      </c>
-      <c r="C39" t="s">
-        <v>2238</v>
-      </c>
-      <c r="D39" t="s">
-        <v>2239</v>
-      </c>
-      <c r="E39">
-        <v>1</v>
-      </c>
-      <c r="F39" t="s">
-        <v>1503</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
-        <v>1307</v>
-      </c>
-      <c r="B40" t="s">
-        <v>1379</v>
-      </c>
-      <c r="C40" t="s">
-        <v>2240</v>
-      </c>
-      <c r="D40" t="s">
-        <v>2245</v>
-      </c>
-      <c r="E40">
-        <v>2</v>
-      </c>
-      <c r="F40" t="s">
-        <v>1503</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
-        <v>1307</v>
-      </c>
-      <c r="B41" t="s">
-        <v>1379</v>
-      </c>
-      <c r="C41" t="s">
-        <v>2241</v>
-      </c>
-      <c r="D41" t="s">
-        <v>2244</v>
-      </c>
-      <c r="E41">
-        <v>3</v>
-      </c>
-      <c r="F41" t="s">
-        <v>1503</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
-        <v>1307</v>
-      </c>
-      <c r="B42" t="s">
-        <v>1379</v>
-      </c>
-      <c r="C42" t="s">
-        <v>2242</v>
-      </c>
-      <c r="D42" t="s">
-        <v>2243</v>
-      </c>
-      <c r="E42">
-        <v>4</v>
-      </c>
-      <c r="F42" t="s">
-        <v>1503</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
-        <v>1308</v>
-      </c>
-      <c r="B43" t="s">
-        <v>1380</v>
-      </c>
-      <c r="C43" t="s">
-        <v>2254</v>
-      </c>
-      <c r="D43" t="s">
-        <v>2263</v>
-      </c>
-      <c r="E43">
-        <v>1</v>
-      </c>
-      <c r="F43" t="s">
-        <v>1503</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
-        <v>1308</v>
-      </c>
-      <c r="B44" t="s">
-        <v>1380</v>
-      </c>
-      <c r="C44" t="s">
-        <v>2255</v>
-      </c>
-      <c r="D44" t="s">
-        <v>2264</v>
-      </c>
-      <c r="E44">
-        <v>2</v>
-      </c>
-      <c r="F44" t="s">
-        <v>1503</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
-        <v>1308</v>
-      </c>
-      <c r="B45" t="s">
-        <v>1380</v>
-      </c>
-      <c r="C45" t="s">
-        <v>2256</v>
-      </c>
-      <c r="D45" t="s">
-        <v>2266</v>
-      </c>
-      <c r="E45">
-        <v>3</v>
-      </c>
-      <c r="F45" t="s">
-        <v>1503</v>
-      </c>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
-        <v>1308</v>
-      </c>
-      <c r="B46" t="s">
-        <v>1380</v>
-      </c>
-      <c r="C46" t="s">
-        <v>2257</v>
-      </c>
-      <c r="D46" t="s">
-        <v>2267</v>
-      </c>
-      <c r="E46">
-        <v>4</v>
-      </c>
-      <c r="F46" t="s">
-        <v>1503</v>
-      </c>
-    </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
-        <v>1308</v>
-      </c>
-      <c r="B47" t="s">
-        <v>1380</v>
-      </c>
-      <c r="C47" t="s">
-        <v>2258</v>
-      </c>
-      <c r="D47" t="s">
-        <v>2268</v>
-      </c>
-      <c r="E47">
-        <v>5</v>
-      </c>
-      <c r="F47" t="s">
-        <v>1503</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
-        <v>1308</v>
-      </c>
-      <c r="B48" t="s">
-        <v>1380</v>
-      </c>
-      <c r="C48" t="s">
-        <v>2259</v>
-      </c>
-      <c r="D48" t="s">
-        <v>2269</v>
-      </c>
-      <c r="E48">
-        <v>6</v>
-      </c>
-      <c r="F48" t="s">
-        <v>1503</v>
-      </c>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A49" t="s">
-        <v>1308</v>
-      </c>
-      <c r="B49" t="s">
-        <v>1380</v>
-      </c>
-      <c r="C49" t="s">
-        <v>2260</v>
-      </c>
-      <c r="D49" t="s">
-        <v>2270</v>
-      </c>
-      <c r="E49">
-        <v>7</v>
-      </c>
-      <c r="F49" t="s">
-        <v>1503</v>
-      </c>
-    </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
-        <v>1308</v>
-      </c>
-      <c r="B50" t="s">
-        <v>1380</v>
-      </c>
-      <c r="C50" t="s">
-        <v>2261</v>
-      </c>
-      <c r="D50" t="s">
-        <v>2271</v>
-      </c>
-      <c r="E50">
-        <v>8</v>
-      </c>
-      <c r="F50" t="s">
-        <v>1503</v>
-      </c>
-    </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
-        <v>1308</v>
-      </c>
-      <c r="B51" t="s">
-        <v>1380</v>
-      </c>
-      <c r="C51" t="s">
-        <v>2262</v>
-      </c>
-      <c r="D51" t="s">
-        <v>2265</v>
-      </c>
-      <c r="E51">
-        <v>9</v>
-      </c>
-      <c r="F51" t="s">
-        <v>1503</v>
-      </c>
-    </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
-        <v>1309</v>
-      </c>
-      <c r="B52" t="s">
-        <v>1381</v>
-      </c>
-      <c r="C52" t="s">
-        <v>2288</v>
-      </c>
-      <c r="D52" t="s">
-        <v>2295</v>
-      </c>
-      <c r="E52">
-        <v>1</v>
-      </c>
-      <c r="F52" t="s">
-        <v>1503</v>
-      </c>
-    </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
-        <v>1309</v>
-      </c>
-      <c r="B53" t="s">
-        <v>1381</v>
-      </c>
-      <c r="C53" t="s">
-        <v>2289</v>
-      </c>
-      <c r="D53" t="s">
-        <v>2296</v>
-      </c>
-      <c r="E53">
-        <v>2</v>
-      </c>
-      <c r="F53" t="s">
-        <v>1503</v>
-      </c>
-    </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A54" t="s">
-        <v>1309</v>
-      </c>
-      <c r="B54" t="s">
-        <v>1381</v>
-      </c>
-      <c r="C54" t="s">
-        <v>2290</v>
-      </c>
-      <c r="D54" t="s">
-        <v>2297</v>
-      </c>
-      <c r="E54">
-        <v>3</v>
-      </c>
-      <c r="F54" t="s">
-        <v>1503</v>
-      </c>
-    </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A55" t="s">
-        <v>1309</v>
-      </c>
-      <c r="B55" t="s">
-        <v>1381</v>
-      </c>
-      <c r="C55" t="s">
-        <v>2291</v>
-      </c>
-      <c r="D55" t="s">
-        <v>2300</v>
-      </c>
-      <c r="E55">
-        <v>4</v>
-      </c>
-      <c r="F55" t="s">
-        <v>1503</v>
-      </c>
-    </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A56" t="s">
-        <v>1309</v>
-      </c>
-      <c r="B56" t="s">
-        <v>1381</v>
-      </c>
-      <c r="C56" t="s">
-        <v>2292</v>
-      </c>
-      <c r="D56" t="s">
-        <v>2298</v>
-      </c>
-      <c r="E56">
-        <v>5</v>
-      </c>
-      <c r="F56" t="s">
-        <v>1503</v>
-      </c>
-    </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A57" t="s">
-        <v>1309</v>
-      </c>
-      <c r="B57" t="s">
-        <v>1381</v>
-      </c>
-      <c r="C57" t="s">
-        <v>2293</v>
-      </c>
-      <c r="D57" t="s">
-        <v>2299</v>
-      </c>
-      <c r="E57">
-        <v>6</v>
-      </c>
-      <c r="F57" t="s">
-        <v>1503</v>
-      </c>
-    </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A58" t="s">
-        <v>1309</v>
-      </c>
-      <c r="B58" t="s">
-        <v>1381</v>
-      </c>
-      <c r="C58" t="s">
-        <v>2294</v>
-      </c>
-      <c r="D58" t="s">
-        <v>2301</v>
-      </c>
-      <c r="E58">
-        <v>7</v>
-      </c>
-      <c r="F58" t="s">
-        <v>1503</v>
-      </c>
-    </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A59" t="s">
-        <v>1310</v>
-      </c>
-      <c r="B59" t="s">
-        <v>1382</v>
-      </c>
-      <c r="C59" t="s">
-        <v>2314</v>
-      </c>
-      <c r="D59" t="s">
-        <v>2318</v>
-      </c>
-      <c r="E59">
-        <v>1</v>
-      </c>
-      <c r="F59" t="s">
-        <v>1503</v>
-      </c>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A60" t="s">
-        <v>1310</v>
-      </c>
-      <c r="B60" t="s">
-        <v>1382</v>
-      </c>
-      <c r="C60" t="s">
-        <v>2315</v>
-      </c>
-      <c r="D60" t="s">
-        <v>2319</v>
-      </c>
-      <c r="E60">
-        <v>2</v>
-      </c>
-      <c r="F60" t="s">
-        <v>1503</v>
-      </c>
-    </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A61" t="s">
-        <v>1310</v>
-      </c>
-      <c r="B61" t="s">
-        <v>1382</v>
-      </c>
-      <c r="C61" t="s">
-        <v>2316</v>
-      </c>
-      <c r="D61" t="s">
-        <v>2320</v>
-      </c>
-      <c r="E61">
-        <v>3</v>
-      </c>
-      <c r="F61" t="s">
-        <v>1503</v>
-      </c>
-    </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A62" t="s">
-        <v>1310</v>
-      </c>
-      <c r="B62" t="s">
-        <v>1382</v>
-      </c>
-      <c r="C62" t="s">
-        <v>2317</v>
-      </c>
-      <c r="D62" t="s">
-        <v>2321</v>
-      </c>
-      <c r="E62">
-        <v>4</v>
-      </c>
-      <c r="F62" t="s">
-        <v>1503</v>
-      </c>
-    </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A63" t="s">
-        <v>1323</v>
-      </c>
-      <c r="B63" t="s">
-        <v>1393</v>
-      </c>
-      <c r="C63" t="s">
-        <v>2439</v>
-      </c>
-      <c r="D63" t="s">
-        <v>2440</v>
-      </c>
-      <c r="E63">
-        <v>1</v>
-      </c>
-      <c r="F63" t="s">
-        <v>1506</v>
-      </c>
-    </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A64" t="s">
-        <v>1326</v>
-      </c>
-      <c r="B64" t="s">
-        <v>1396</v>
-      </c>
-      <c r="C64" t="s">
-        <v>2473</v>
-      </c>
-      <c r="D64" t="s">
-        <v>2474</v>
-      </c>
-      <c r="E64">
-        <v>1</v>
-      </c>
-      <c r="F64" t="s">
-        <v>1503</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
fixing filters for masters
</commit_message>
<xml_diff>
--- a/data/Fate-Spreadsheet.xlsx
+++ b/data/Fate-Spreadsheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Important\Python\Fate-Wiki\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AECEEA88-4C6A-4D9C-BF5B-579B066E645F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C5EBDEB-3EBE-4AC4-B87C-81898D0D729E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="2" activeTab="7" xr2:uid="{B05E798F-9EF6-4508-A0A4-311D06661AED}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="1" activeTab="1" xr2:uid="{B05E798F-9EF6-4508-A0A4-311D06661AED}"/>
   </bookViews>
   <sheets>
     <sheet name="Servants" sheetId="1" r:id="rId1"/>
@@ -22,6 +22,7 @@
     <sheet name="Master Abilities" sheetId="6" r:id="rId7"/>
     <sheet name="Master Assets" sheetId="9" r:id="rId8"/>
     <sheet name="Master Ascensions" sheetId="10" r:id="rId9"/>
+    <sheet name="Master Mechanics List" sheetId="12" r:id="rId10"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -47,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5762" uniqueCount="2507">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5769" uniqueCount="2508">
   <si>
     <t>servant_id</t>
   </si>
@@ -7568,6 +7569,9 @@
   </si>
   <si>
     <t>old-acquaintances</t>
+  </si>
+  <si>
+    <t>mechanics</t>
   </si>
 </sst>
 </file>
@@ -7959,6 +7963,7 @@
   <dimension ref="A1:R189"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="1" max="1" width="14.85546875" customWidth="1"/>
     <col min="2" max="3" width="22" customWidth="1"/>
     <col min="4" max="4" width="12.5703125" customWidth="1"/>
     <col min="5" max="5" width="11.28515625" customWidth="1"/>
@@ -14450,6 +14455,55 @@
   <ignoredErrors>
     <ignoredError sqref="H2 I6:I7 I10 I12 H14 I18 I22 I24 I27 G34 I40 I42 I45 I52 I62 I72 H79 I80 I84 I88 I90 G91 H100 I119 I124 I121:I123 G130:I139 G142:I148 G164:I185 G187:I187" numberStoredAsText="1"/>
   </ignoredErrors>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{41E57DE0-A26F-4023-BFBB-B4D5A6C17F78}">
+  <dimension ref="A1:A7"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="21" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>2507</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>1333</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>1334</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>1335</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>1336</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>1337</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>1373</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>